<commit_message>
Process pending data updates (2026-08-26T21:03:59Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18043,7 +18043,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>96</v>
@@ -21193,30 +21193,74 @@
       <c r="C183" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D183" s="52"/>
-      <c r="E183" s="52"/>
-      <c r="F183" s="52"/>
-      <c r="G183" s="53"/>
-      <c r="H183" s="52"/>
-      <c r="I183" s="52"/>
-      <c r="J183" s="52"/>
-      <c r="K183" s="52"/>
-      <c r="L183" s="52"/>
-      <c r="M183" s="53"/>
+      <c r="D183" s="52">
+        <v>16897.53</v>
+      </c>
+      <c r="E183" s="52">
+        <v>5491.7</v>
+      </c>
+      <c r="F183" s="52">
+        <v>11405.829999999998</v>
+      </c>
+      <c r="G183" s="53">
+        <v>0.6749998372543206</v>
+      </c>
+      <c r="H183" s="52">
+        <v>9226.27</v>
+      </c>
+      <c r="I183" s="52">
+        <v>3702.78</v>
+      </c>
+      <c r="J183" s="52">
+        <v>2977.1100000000006</v>
+      </c>
+      <c r="K183" s="52">
+        <v>2335.9700000000003</v>
+      </c>
+      <c r="L183" s="52">
+        <v>641.1400000000003</v>
+      </c>
+      <c r="M183" s="53">
+        <v>0.2153565034546927</v>
+      </c>
       <c r="N183" s="53"/>
-      <c r="O183" s="52"/>
-      <c r="P183" s="52"/>
-      <c r="Q183" s="52"/>
-      <c r="R183" s="53"/>
-      <c r="S183" s="54"/>
-      <c r="T183" s="54"/>
-      <c r="U183" s="54"/>
-      <c r="V183" s="53"/>
+      <c r="O183" s="52">
+        <v>6249.16</v>
+      </c>
+      <c r="P183" s="52">
+        <v>1366.81</v>
+      </c>
+      <c r="Q183" s="52">
+        <v>4882.35</v>
+      </c>
+      <c r="R183" s="53">
+        <v>0.7812810041669601</v>
+      </c>
+      <c r="S183" s="54">
+        <v>125.17</v>
+      </c>
+      <c r="T183" s="54">
+        <v>23.75</v>
+      </c>
+      <c r="U183" s="54">
+        <v>101.42</v>
+      </c>
+      <c r="V183" s="53">
+        <v>0.8102580490532876</v>
+      </c>
       <c r="W183" s="53"/>
-      <c r="X183" s="55"/>
-      <c r="Y183" s="55"/>
-      <c r="Z183" s="53"/>
-      <c r="AA183" s="56"/>
+      <c r="X183" s="55">
+        <v>75.32294736842105</v>
+      </c>
+      <c r="Y183" s="55">
+        <v>61.286703843093385</v>
+      </c>
+      <c r="Z183" s="53">
+        <v>0.3257</v>
+      </c>
+      <c r="AA183" s="56">
+        <v>0.454</v>
+      </c>
       <c r="AB183" s="57"/>
       <c r="AD183" s="35"/>
       <c r="AE183" s="35"/>
@@ -21596,32 +21640,74 @@
       <c r="C190" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D190" s="52"/>
-      <c r="E190" s="52"/>
-      <c r="F190" s="52"/>
-      <c r="G190" s="53"/>
-      <c r="H190" s="52"/>
-      <c r="I190" s="52"/>
-      <c r="J190" s="52"/>
+      <c r="D190" s="52">
+        <v>20992.12</v>
+      </c>
+      <c r="E190" s="52">
+        <v>14169.68</v>
+      </c>
+      <c r="F190" s="52">
+        <v>6822.439999999999</v>
+      </c>
+      <c r="G190" s="53">
+        <v>0.32500004763692275</v>
+      </c>
+      <c r="H190" s="52">
+        <v>16299.09</v>
+      </c>
+      <c r="I190" s="52">
+        <v>9699.51</v>
+      </c>
+      <c r="J190" s="52">
+        <v>9784.33</v>
+      </c>
       <c r="K190" s="52">
-        <v>0</v>
-      </c>
-      <c r="L190" s="52"/>
-      <c r="M190" s="53"/>
+        <v>8137.88</v>
+      </c>
+      <c r="L190" s="52">
+        <v>1646.4499999999998</v>
+      </c>
+      <c r="M190" s="53">
+        <v>0.16827416900288522</v>
+      </c>
       <c r="N190" s="53"/>
-      <c r="O190" s="52"/>
-      <c r="P190" s="52"/>
-      <c r="Q190" s="52"/>
-      <c r="R190" s="53"/>
-      <c r="S190" s="54"/>
-      <c r="T190" s="54"/>
-      <c r="U190" s="54"/>
-      <c r="V190" s="53"/>
+      <c r="O190" s="52">
+        <v>6514.76</v>
+      </c>
+      <c r="P190" s="52">
+        <v>1561.63</v>
+      </c>
+      <c r="Q190" s="52">
+        <v>4953.13</v>
+      </c>
+      <c r="R190" s="53">
+        <v>0.7602935488030257</v>
+      </c>
+      <c r="S190" s="54">
+        <v>130.62</v>
+      </c>
+      <c r="T190" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U190" s="54">
+        <v>95.87</v>
+      </c>
+      <c r="V190" s="53">
+        <v>0.7339611085591793</v>
+      </c>
       <c r="W190" s="53"/>
-      <c r="X190" s="55"/>
-      <c r="Y190" s="55"/>
-      <c r="Z190" s="53"/>
-      <c r="AA190" s="56"/>
+      <c r="X190" s="55">
+        <v>128.6379856115108</v>
+      </c>
+      <c r="Y190" s="55">
+        <v>35.92887828502527</v>
+      </c>
+      <c r="Z190" s="53">
+        <v>0.3155</v>
+      </c>
+      <c r="AA190" s="56">
+        <v>0.2236</v>
+      </c>
       <c r="AB190" s="57"/>
       <c r="AD190" s="35"/>
       <c r="AE190" s="35"/>
@@ -21995,32 +22081,74 @@
       <c r="C197" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D197" s="52"/>
-      <c r="E197" s="52"/>
-      <c r="F197" s="52"/>
-      <c r="G197" s="53"/>
-      <c r="H197" s="52"/>
-      <c r="I197" s="52"/>
-      <c r="J197" s="52"/>
+      <c r="D197" s="52">
+        <v>23770.95</v>
+      </c>
+      <c r="E197" s="52">
+        <v>10204.54</v>
+      </c>
+      <c r="F197" s="52">
+        <v>13566.41</v>
+      </c>
+      <c r="G197" s="53">
+        <v>0.5707138334816235</v>
+      </c>
+      <c r="H197" s="52">
+        <v>14310.96</v>
+      </c>
+      <c r="I197" s="52">
+        <v>6935.96</v>
+      </c>
+      <c r="J197" s="52">
+        <v>7389.339999999999</v>
+      </c>
       <c r="K197" s="52">
-        <v>0</v>
-      </c>
-      <c r="L197" s="52"/>
-      <c r="M197" s="53"/>
+        <v>6605.05</v>
+      </c>
+      <c r="L197" s="52">
+        <v>784.289999999999</v>
+      </c>
+      <c r="M197" s="53">
+        <v>0.1061380312720756</v>
+      </c>
       <c r="N197" s="53"/>
-      <c r="O197" s="52"/>
-      <c r="P197" s="52"/>
-      <c r="Q197" s="52"/>
-      <c r="R197" s="53"/>
-      <c r="S197" s="54"/>
-      <c r="T197" s="54"/>
-      <c r="U197" s="54"/>
-      <c r="V197" s="53"/>
+      <c r="O197" s="52">
+        <v>6921.62</v>
+      </c>
+      <c r="P197" s="52">
+        <v>330.91</v>
+      </c>
+      <c r="Q197" s="52">
+        <v>6590.71</v>
+      </c>
+      <c r="R197" s="53">
+        <v>0.9521918279246766</v>
+      </c>
+      <c r="S197" s="54">
+        <v>140.15</v>
+      </c>
+      <c r="T197" s="54">
+        <v>5.75</v>
+      </c>
+      <c r="U197" s="54">
+        <v>134.4</v>
+      </c>
+      <c r="V197" s="53">
+        <v>0.9589725294327506</v>
+      </c>
       <c r="W197" s="53"/>
-      <c r="X197" s="55"/>
-      <c r="Y197" s="55"/>
-      <c r="Z197" s="53"/>
-      <c r="AA197" s="56"/>
+      <c r="X197" s="55">
+        <v>568.4486956521739</v>
+      </c>
+      <c r="Y197" s="55">
+        <v>67.49902570438813</v>
+      </c>
+      <c r="Z197" s="53">
+        <v>0.32030000000000003</v>
+      </c>
+      <c r="AA197" s="56">
+        <v>0.398</v>
+      </c>
       <c r="AB197" s="57"/>
       <c r="AD197" s="35"/>
       <c r="AE197" s="35"/>
@@ -22968,30 +23096,74 @@
       <c r="C218" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D218" s="52"/>
-      <c r="E218" s="52"/>
-      <c r="F218" s="52"/>
-      <c r="G218" s="53"/>
-      <c r="H218" s="52"/>
-      <c r="I218" s="52"/>
-      <c r="J218" s="52"/>
-      <c r="K218" s="52"/>
-      <c r="L218" s="52"/>
-      <c r="M218" s="53"/>
+      <c r="D218" s="52">
+        <v>137109.56</v>
+      </c>
+      <c r="E218" s="52">
+        <v>30174.75</v>
+      </c>
+      <c r="F218" s="52">
+        <v>106934.81</v>
+      </c>
+      <c r="G218" s="53">
+        <v>0.7799223482301307</v>
+      </c>
+      <c r="H218" s="52">
+        <v>117394.57</v>
+      </c>
+      <c r="I218" s="52">
+        <v>26124</v>
+      </c>
+      <c r="J218" s="52">
+        <v>99479.62000000001</v>
+      </c>
+      <c r="K218" s="52">
+        <v>26124</v>
+      </c>
+      <c r="L218" s="52">
+        <v>73355.62000000001</v>
+      </c>
+      <c r="M218" s="53">
+        <v>0.7373934480248316</v>
+      </c>
       <c r="N218" s="53"/>
-      <c r="O218" s="52"/>
-      <c r="P218" s="52"/>
-      <c r="Q218" s="52"/>
-      <c r="R218" s="53"/>
-      <c r="S218" s="54"/>
-      <c r="T218" s="54"/>
-      <c r="U218" s="54"/>
-      <c r="V218" s="53"/>
+      <c r="O218" s="52">
+        <v>17914.95</v>
+      </c>
+      <c r="P218" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q218" s="52">
+        <v>17914.95</v>
+      </c>
+      <c r="R218" s="53">
+        <v>1</v>
+      </c>
+      <c r="S218" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="T218" s="54">
+        <v>0</v>
+      </c>
+      <c r="U218" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="V218" s="53">
+        <v>1</v>
+      </c>
       <c r="W218" s="53"/>
-      <c r="X218" s="55"/>
-      <c r="Y218" s="55"/>
-      <c r="Z218" s="53"/>
-      <c r="AA218" s="56"/>
+      <c r="X218" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y218" s="55">
+        <v>54.93783457863793</v>
+      </c>
+      <c r="Z218" s="53">
+        <v>0.13419999999999999</v>
+      </c>
+      <c r="AA218" s="56">
+        <v>0.1438</v>
+      </c>
       <c r="AB218" s="57"/>
       <c r="AD218" s="35"/>
       <c r="AE218" s="35"/>
@@ -23369,34 +23541,74 @@
       <c r="C225" s="51" t="s">
         <v>98</v>
       </c>
-      <c r="D225" s="52"/>
-      <c r="E225" s="52"/>
-      <c r="F225" s="52"/>
-      <c r="G225" s="53"/>
-      <c r="H225" s="52"/>
-      <c r="I225" s="52"/>
+      <c r="D225" s="52">
+        <v>396453.46</v>
+      </c>
+      <c r="E225" s="52">
+        <v>271388.15</v>
+      </c>
+      <c r="F225" s="52">
+        <v>125065.31</v>
+      </c>
+      <c r="G225" s="53">
+        <v>0.3154602560411504</v>
+      </c>
+      <c r="H225" s="52">
+        <v>295569.99</v>
+      </c>
+      <c r="I225" s="52">
+        <v>234322.81</v>
+      </c>
       <c r="J225" s="52">
-        <v>0</v>
+        <v>178700.37</v>
       </c>
       <c r="K225" s="52">
-        <v>0</v>
-      </c>
-      <c r="L225" s="52"/>
-      <c r="M225" s="53"/>
+        <v>177071.47999999998</v>
+      </c>
+      <c r="L225" s="52">
+        <v>1628.890000000014</v>
+      </c>
+      <c r="M225" s="53">
+        <v>0.009115202167740415</v>
+      </c>
       <c r="N225" s="53"/>
-      <c r="O225" s="52"/>
-      <c r="P225" s="52"/>
-      <c r="Q225" s="52"/>
-      <c r="R225" s="53"/>
-      <c r="S225" s="54"/>
-      <c r="T225" s="54"/>
-      <c r="U225" s="54"/>
-      <c r="V225" s="53"/>
+      <c r="O225" s="52">
+        <v>116869.62</v>
+      </c>
+      <c r="P225" s="52">
+        <v>57251.33</v>
+      </c>
+      <c r="Q225" s="52">
+        <v>59618.28999999999</v>
+      </c>
+      <c r="R225" s="53">
+        <v>0.5101264982293944</v>
+      </c>
+      <c r="S225" s="54">
+        <v>2344.68</v>
+      </c>
+      <c r="T225" s="54">
+        <v>1212</v>
+      </c>
+      <c r="U225" s="54">
+        <v>1132.6799999999998</v>
+      </c>
+      <c r="V225" s="53">
+        <v>0.48308511182762676</v>
+      </c>
       <c r="W225" s="53"/>
-      <c r="X225" s="55"/>
-      <c r="Y225" s="55"/>
-      <c r="Z225" s="53"/>
-      <c r="AA225" s="56"/>
+      <c r="X225" s="55">
+        <v>30.581963696369634</v>
+      </c>
+      <c r="Y225" s="55">
+        <v>43.0265399367206</v>
+      </c>
+      <c r="Z225" s="53">
+        <v>0.1366</v>
+      </c>
+      <c r="AA225" s="56">
+        <v>0.2545</v>
+      </c>
       <c r="AB225" s="57"/>
       <c r="AD225" s="35"/>
       <c r="AE225" s="35"/>
@@ -24013,7 +24225,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:AD70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -24027,7 +24239,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -24049,7 +24261,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>101</v>
       </c>
@@ -24097,7 +24309,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -24115,7 +24327,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -24162,7 +24374,7 @@
         <v>-726.0072857142857</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -24179,7 +24391,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -24199,7 +24411,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="53">
-        <v>0.2556317756411565</v>
+        <v>0.25548771651006935</v>
       </c>
       <c r="H6" s="53">
         <v>0.239214585617637</v>
@@ -24214,22 +24426,22 @@
         <v>1872.6</v>
       </c>
       <c r="L6" s="53">
-        <v>0.2016787498663849</v>
+        <v>0.20153469073529773</v>
       </c>
       <c r="M6" s="52">
-        <v>6999.8599999999915</v>
+        <v>6994.8599999999915</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>-559.9887999999993</v>
+        <v>-559.5887999999993</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -24246,7 +24458,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -24289,7 +24501,7 @@
         <v>-232.53333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -24306,7 +24518,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -24353,7 +24565,7 @@
         <v>-50.95312270389416</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -24370,7 +24582,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -24418,7 +24630,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -24435,7 +24647,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -24482,7 +24694,7 @@
         <v>-42.80544642857142</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -24499,7 +24711,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -24544,7 +24756,7 @@
         <v>7.380864553314173</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -24561,7 +24773,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -24611,7 +24823,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -24628,7 +24840,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -24667,7 +24879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -24684,7 +24896,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -24725,7 +24937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -24742,7 +24954,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24779,7 +24991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -24796,7 +25008,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24841,7 +25053,7 @@
         <v>0.2554973821989554</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -24858,7 +25070,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24901,7 +25113,7 @@
         <v>7.589966329966334</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -24918,7 +25130,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24961,7 +25173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -24978,7 +25190,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -25025,7 +25237,7 @@
         <v>4.666337611056268</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -25042,7 +25254,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -25087,7 +25299,7 @@
         <v>285.64884004884004</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -25104,7 +25316,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -25147,7 +25359,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -25164,7 +25376,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -25205,7 +25417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -25222,7 +25434,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -25267,7 +25479,7 @@
         <v>561.1049999999996</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -25284,7 +25496,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25327,7 +25539,7 @@
         <v>-9.801274601686979</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -25344,7 +25556,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25381,7 +25593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -25398,7 +25610,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25439,7 +25651,7 @@
         <v>0.05940556088207709</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -25456,7 +25668,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -25499,7 +25711,7 @@
         <v>-179.9832402234637</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -25516,7 +25728,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -25558,7 +25770,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -25575,7 +25787,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -25620,7 +25832,7 @@
         <v>-9.106177818515201</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -25637,7 +25849,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -25682,7 +25894,7 @@
         <v>862.1199999999999</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -25699,7 +25911,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -25710,14 +25922,14 @@
         <v>12937.1</v>
       </c>
       <c r="D56" s="99">
-        <v>4850.19</v>
+        <v>4794.2300000000005</v>
       </c>
       <c r="E56" s="99">
-        <v>8086.910000000001</v>
+        <v>8142.87</v>
       </c>
       <c r="F56" s="99"/>
       <c r="G56" s="100">
-        <v>0.6250944956752287</v>
+        <v>0.6294200400398853</v>
       </c>
       <c r="H56" s="100">
         <v>0.22356150784199</v>
@@ -25732,19 +25944,19 @@
         <v>5400</v>
       </c>
       <c r="L56" s="100">
-        <v>0.20769028607647777</v>
+        <v>0.2120158304411344</v>
       </c>
       <c r="M56" s="99">
-        <v>2686.9100000000008</v>
+        <v>2742.87</v>
       </c>
       <c r="N56" s="98">
         <v>-32.25</v>
       </c>
       <c r="O56" s="60">
-        <v>-120.76000000000003</v>
-      </c>
-    </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>-123.27505617977528</v>
+      </c>
+    </row>
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25761,7 +25973,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -25769,17 +25981,17 @@
         <v>60</v>
       </c>
       <c r="C58" s="99">
-        <v>0</v>
+        <v>10204.54</v>
       </c>
       <c r="D58" s="99">
-        <v>6849.16</v>
+        <v>6605.05</v>
       </c>
       <c r="E58" s="99">
-        <v>-6849.16</v>
+        <v>3599.4900000000007</v>
       </c>
       <c r="F58" s="99"/>
       <c r="G58" s="100">
-        <v>0</v>
+        <v>0.35273417518085093</v>
       </c>
       <c r="H58" s="100"/>
       <c r="I58" s="98"/>
@@ -25788,17 +26000,17 @@
         <v>0</v>
       </c>
       <c r="L58" s="100">
-        <v>0</v>
+        <v>0.35273417518085093</v>
       </c>
       <c r="M58" s="99">
-        <v>-6849.16</v>
+        <v>3599.4900000000007</v>
       </c>
       <c r="N58" s="98"/>
       <c r="O58" s="60">
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -25815,7 +26027,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -25832,7 +26044,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -25849,7 +26061,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>61</v>
@@ -25870,7 +26082,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -25887,7 +26099,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -25895,17 +26107,17 @@
         <v>62</v>
       </c>
       <c r="C64" s="99">
-        <v>0</v>
+        <v>30174.75</v>
       </c>
       <c r="D64" s="99">
-        <v>1749.8</v>
+        <v>26124</v>
       </c>
       <c r="E64" s="99">
-        <v>-1749.8</v>
+        <v>4050.75</v>
       </c>
       <c r="F64" s="99"/>
       <c r="G64" s="100">
-        <v>0</v>
+        <v>0.13424303432505655</v>
       </c>
       <c r="H64" s="100">
         <v>0.143790046441692</v>
@@ -25918,17 +26130,17 @@
         <v>1750</v>
       </c>
       <c r="L64" s="100">
-        <v>0</v>
+        <v>0.07624752483450567</v>
       </c>
       <c r="M64" s="99">
-        <v>-3499.8</v>
+        <v>2300.75</v>
       </c>
       <c r="N64" s="98"/>
       <c r="O64" s="60">
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -25945,7 +26157,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -25956,10 +26168,10 @@
         <v>0</v>
       </c>
       <c r="D66" s="99">
-        <v>2584.2399999999907</v>
+        <v>9863.48999999999</v>
       </c>
       <c r="E66" s="99">
-        <v>-2584.2399999999907</v>
+        <v>-9863.48999999999</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
@@ -25981,16 +26193,16 @@
         <v>0</v>
       </c>
       <c r="M66" s="99">
-        <v>-5784.239999999991</v>
+        <v>-13063.48999999999</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>6.191319240032102</v>
-      </c>
-    </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>13.982863259298894</v>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -26007,7 +26219,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -26024,7 +26236,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>121</v>
       </c>
@@ -26032,25 +26244,25 @@
         <v>122</v>
       </c>
       <c r="C69" s="104">
-        <v>308475.47</v>
+        <v>348854.75999999995</v>
       </c>
       <c r="D69" s="104">
-        <v>345627.75999999995</v>
+        <v>376981.13999999996</v>
       </c>
       <c r="E69" s="105">
-        <v>-37152.289999999986</v>
+        <v>-28126.379999999983</v>
       </c>
       <c r="F69" s="106" t="s">
         <v>123</v>
       </c>
       <c r="G69" s="107">
-        <v>-0.12043839336722621</v>
+        <v>-0.08062489960005129</v>
       </c>
       <c r="H69" s="108" t="s">
         <v>124</v>
       </c>
       <c r="I69" s="109">
-        <v>-0.2884666647886135</v>
+        <v>-0.2292042109444056</v>
       </c>
       <c r="J69" s="36"/>
       <c r="K69" s="36"/>
@@ -26059,7 +26271,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>125</v>
@@ -26442,7 +26654,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB109"/>
+  <dimension ref="A1:AD109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -26453,7 +26665,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -26474,7 +26686,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>126</v>
@@ -26536,7 +26748,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>142</v>
       </c>
@@ -26594,7 +26806,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -26628,7 +26840,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -26647,7 +26859,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -26681,7 +26893,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -26700,7 +26912,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26734,7 +26946,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26753,7 +26965,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -26789,7 +27001,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -26808,7 +27020,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -26846,7 +27058,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -26865,7 +27077,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -26903,7 +27115,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -26922,7 +27134,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -26955,7 +27167,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -26974,7 +27186,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -27007,7 +27219,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -27026,7 +27238,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -27057,7 +27269,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -27076,7 +27288,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -27111,7 +27323,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -27130,7 +27342,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -27163,7 +27375,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -27182,7 +27394,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -27213,7 +27425,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -27232,7 +27444,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27264,7 +27476,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -27283,7 +27495,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27319,7 +27531,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -27338,7 +27550,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27367,7 +27579,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -27386,7 +27598,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27417,7 +27629,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -27436,7 +27648,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27469,7 +27681,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -27488,7 +27700,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27524,7 +27736,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -27543,7 +27755,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27578,7 +27790,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -27597,7 +27809,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27627,7 +27839,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -27646,7 +27858,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27686,7 +27898,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -27705,7 +27917,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27734,7 +27946,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27753,7 +27965,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -27786,7 +27998,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -27805,7 +28017,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -27838,7 +28050,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -27857,7 +28069,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -27893,7 +28105,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -27912,7 +28124,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -27948,7 +28160,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -27967,7 +28179,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -28001,7 +28213,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -28020,7 +28232,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -28055,7 +28267,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -28074,7 +28286,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -28093,7 +28305,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -28112,7 +28324,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>61</v>
@@ -28133,7 +28345,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -28152,7 +28364,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -28185,7 +28397,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -28204,7 +28416,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -28212,13 +28424,13 @@
         <v>63</v>
       </c>
       <c r="C66" s="54">
-        <v>2312.68</v>
+        <v>2344.68</v>
       </c>
       <c r="D66" s="54">
-        <v>1120.5</v>
+        <v>1212</v>
       </c>
       <c r="E66" s="54">
-        <v>1192.1799999999998</v>
+        <v>1132.6799999999998</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>
@@ -28243,7 +28455,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -28262,7 +28474,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -28281,7 +28493,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -28300,7 +28512,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>146</v>
@@ -28345,7 +28557,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>147</v>
@@ -28384,7 +28596,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -28413,7 +28625,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>149</v>
@@ -28458,7 +28670,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>150</v>
@@ -28503,7 +28715,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -28522,7 +28734,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>151</v>
@@ -28569,7 +28781,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>153</v>
@@ -28614,7 +28826,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -28633,7 +28845,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>154</v>
@@ -28656,7 +28868,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>156</v>
@@ -28679,7 +28891,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>157</v>
@@ -28702,7 +28914,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28725,7 +28937,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28748,7 +28960,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28771,7 +28983,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -28794,7 +29006,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -28817,7 +29029,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -28840,7 +29052,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -28863,7 +29075,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -28886,7 +29098,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -28909,7 +29121,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -28930,7 +29142,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -28951,7 +29163,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -28972,7 +29184,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -28993,7 +29205,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -29014,7 +29226,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -29035,7 +29247,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -29056,7 +29268,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>167</v>
@@ -29079,7 +29291,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -29102,7 +29314,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -29125,7 +29337,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -29148,7 +29360,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -29171,7 +29383,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -29194,7 +29406,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -29217,7 +29429,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -29236,7 +29448,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -29255,7 +29467,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -29274,7 +29486,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -29293,7 +29505,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>174</v>
@@ -29367,10 +29579,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>175</v>
       </c>
@@ -29402,7 +29615,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>176</v>
       </c>
@@ -29435,7 +29648,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>177</v>
       </c>
@@ -29468,7 +29681,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>178</v>
       </c>
@@ -29501,7 +29714,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>179</v>
       </c>
@@ -29534,7 +29747,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>180</v>
       </c>
@@ -29567,7 +29780,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>181</v>
       </c>
@@ -29600,7 +29813,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>182</v>
       </c>
@@ -29633,7 +29846,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -29664,7 +29877,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29695,7 +29908,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>183</v>
       </c>
@@ -29728,7 +29941,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>184</v>
       </c>
@@ -29761,7 +29974,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>185</v>
       </c>
@@ -29794,7 +30007,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>186</v>
       </c>
@@ -29827,7 +30040,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>187</v>
       </c>
@@ -29860,7 +30073,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>188</v>
       </c>
@@ -29893,7 +30106,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>189</v>
       </c>
@@ -29926,7 +30139,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>190</v>
       </c>
@@ -29959,7 +30172,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>191</v>
       </c>
@@ -29992,7 +30205,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>192</v>
       </c>
@@ -30025,7 +30238,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>193</v>
       </c>
@@ -30058,7 +30271,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>194</v>
       </c>
@@ -30091,7 +30304,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>195</v>
       </c>
@@ -30124,7 +30337,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>196</v>
       </c>
@@ -30157,7 +30370,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>197</v>
       </c>
@@ -30190,7 +30403,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>198</v>
       </c>
@@ -30223,7 +30436,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>199</v>
       </c>
@@ -30255,7 +30468,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>200</v>
       </c>
@@ -30287,7 +30500,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>201</v>
       </c>
@@ -30319,7 +30532,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>202</v>
       </c>
@@ -30351,7 +30564,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>203</v>
       </c>
@@ -30383,7 +30596,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -30413,7 +30626,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -30443,7 +30656,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>204</v>
       </c>
@@ -30475,7 +30688,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>205</v>
       </c>
@@ -30507,7 +30720,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>206</v>
       </c>
@@ -30539,7 +30752,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>207</v>
       </c>
@@ -30571,7 +30784,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>208</v>
       </c>
@@ -30603,7 +30816,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -30633,7 +30846,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>209</v>
       </c>
@@ -30665,7 +30878,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>210</v>
       </c>
@@ -30697,7 +30910,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>211</v>
       </c>
@@ -30729,7 +30942,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>212</v>
       </c>
@@ -30761,7 +30974,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -30791,7 +31004,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -30821,7 +31034,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -30851,7 +31064,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -30881,7 +31094,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>213</v>
       </c>
@@ -30913,7 +31126,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>214</v>
       </c>
@@ -30945,7 +31158,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -30975,7 +31188,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -31005,7 +31218,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -31035,7 +31248,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -31065,7 +31278,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -31095,7 +31308,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -31190,10 +31403,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>215</v>
       </c>
@@ -31225,7 +31439,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -31256,7 +31470,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -31287,7 +31501,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -31318,7 +31532,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -31349,7 +31563,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -31380,7 +31594,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -31411,7 +31625,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -31442,7 +31656,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -31473,7 +31687,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -31504,7 +31718,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -31535,7 +31749,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -31566,7 +31780,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -31597,7 +31811,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -31628,7 +31842,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -31659,7 +31873,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31690,7 +31904,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31721,7 +31935,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31752,7 +31966,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31783,7 +31997,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -31814,7 +32028,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -31844,7 +32058,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -31874,7 +32088,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -31904,7 +32118,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -31934,7 +32148,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -31964,7 +32178,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -31994,7 +32208,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -32024,7 +32238,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -32054,7 +32268,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -32084,7 +32298,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -32114,7 +32328,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -32144,7 +32358,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -32174,7 +32388,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -32204,7 +32418,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -32234,7 +32448,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -32264,7 +32478,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -32294,7 +32508,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>213</v>
       </c>
@@ -32326,7 +32540,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>214</v>
       </c>
@@ -32358,7 +32572,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -32388,7 +32602,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -32418,7 +32632,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -32448,7 +32662,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -32478,7 +32692,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -32508,7 +32722,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -54251,19 +54465,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -54277,7 +54491,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>222</v>
       </c>
@@ -54289,7 +54503,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>223</v>
       </c>
@@ -54300,7 +54514,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>224</v>
       </c>
@@ -54311,7 +54525,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>225</v>
       </c>
@@ -54322,13 +54536,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-26T21:15:42Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18043,7 +18043,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>96</v>
@@ -24225,7 +24225,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD70"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -24239,7 +24239,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -24261,7 +24261,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>101</v>
       </c>
@@ -24309,7 +24309,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -24327,7 +24327,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -24374,7 +24374,7 @@
         <v>-726.0072857142857</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -24391,7 +24391,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -24441,7 +24441,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -24458,7 +24458,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -24501,7 +24501,7 @@
         <v>-232.53333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -24518,7 +24518,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -24565,7 +24565,7 @@
         <v>-50.95312270389416</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -24582,7 +24582,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -24630,7 +24630,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -24647,7 +24647,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -24694,7 +24694,7 @@
         <v>-42.80544642857142</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -24711,7 +24711,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -24756,7 +24756,7 @@
         <v>7.380864553314173</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -24773,7 +24773,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -24823,7 +24823,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -24840,7 +24840,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -24879,7 +24879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -24896,7 +24896,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -24937,7 +24937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -24954,7 +24954,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24991,7 +24991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -25008,7 +25008,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25053,7 +25053,7 @@
         <v>0.2554973821989554</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -25070,7 +25070,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25113,7 +25113,7 @@
         <v>7.589966329966334</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -25130,7 +25130,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -25173,7 +25173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -25190,7 +25190,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -25237,7 +25237,7 @@
         <v>4.666337611056268</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -25254,7 +25254,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -25299,7 +25299,7 @@
         <v>285.64884004884004</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -25316,7 +25316,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -25359,7 +25359,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -25376,7 +25376,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -25417,7 +25417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -25434,7 +25434,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -25479,7 +25479,7 @@
         <v>561.1049999999996</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -25496,7 +25496,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25539,7 +25539,7 @@
         <v>-9.801274601686979</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -25556,7 +25556,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25593,7 +25593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -25610,7 +25610,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25651,7 +25651,7 @@
         <v>0.05940556088207709</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -25668,7 +25668,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -25711,7 +25711,7 @@
         <v>-179.9832402234637</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -25728,7 +25728,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -25770,7 +25770,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -25787,7 +25787,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -25832,7 +25832,7 @@
         <v>-9.106177818515201</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -25849,7 +25849,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -25894,7 +25894,7 @@
         <v>862.1199999999999</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -25911,7 +25911,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -25956,7 +25956,7 @@
         <v>-123.27505617977528</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25973,7 +25973,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -26010,7 +26010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -26027,7 +26027,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -26044,7 +26044,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -26061,7 +26061,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>61</v>
@@ -26082,7 +26082,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -26099,7 +26099,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -26140,7 +26140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -26157,7 +26157,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -26202,7 +26202,7 @@
         <v>13.982863259298894</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -26219,7 +26219,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -26236,7 +26236,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>121</v>
       </c>
@@ -26271,7 +26271,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>125</v>
@@ -26654,7 +26654,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -26665,7 +26665,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -26686,7 +26686,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>126</v>
@@ -26748,7 +26748,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>142</v>
       </c>
@@ -26806,7 +26806,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -26840,7 +26840,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -26859,7 +26859,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -26893,7 +26893,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -26912,7 +26912,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26946,7 +26946,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26965,7 +26965,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -27001,7 +27001,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -27020,7 +27020,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -27058,7 +27058,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -27077,7 +27077,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -27115,7 +27115,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -27134,7 +27134,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -27167,7 +27167,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -27186,7 +27186,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -27219,7 +27219,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -27238,7 +27238,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -27269,7 +27269,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -27288,7 +27288,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -27323,7 +27323,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -27342,7 +27342,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -27375,7 +27375,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -27394,7 +27394,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -27425,7 +27425,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -27444,7 +27444,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27476,7 +27476,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -27495,7 +27495,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27531,7 +27531,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -27550,7 +27550,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27579,7 +27579,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -27598,7 +27598,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27629,7 +27629,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -27648,7 +27648,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27681,7 +27681,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -27700,7 +27700,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27736,7 +27736,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -27755,7 +27755,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27790,7 +27790,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -27809,7 +27809,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27839,7 +27839,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -27858,7 +27858,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27898,7 +27898,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -27917,7 +27917,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27946,7 +27946,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27965,7 +27965,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -27998,7 +27998,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -28017,7 +28017,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -28050,7 +28050,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -28069,7 +28069,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -28105,7 +28105,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -28124,7 +28124,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -28160,7 +28160,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -28179,7 +28179,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -28213,7 +28213,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -28232,7 +28232,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -28267,7 +28267,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -28286,7 +28286,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -28305,7 +28305,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -28324,7 +28324,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>61</v>
@@ -28345,7 +28345,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -28364,7 +28364,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -28397,7 +28397,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -28416,7 +28416,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -28455,7 +28455,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -28474,7 +28474,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -28493,7 +28493,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -28512,7 +28512,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>146</v>
@@ -28557,7 +28557,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>147</v>
@@ -28596,7 +28596,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -28625,7 +28625,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>149</v>
@@ -28670,7 +28670,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>150</v>
@@ -28715,7 +28715,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -28734,7 +28734,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>151</v>
@@ -28781,7 +28781,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>153</v>
@@ -28826,7 +28826,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -28845,7 +28845,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>154</v>
@@ -28868,7 +28868,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>156</v>
@@ -28891,7 +28891,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>157</v>
@@ -28914,7 +28914,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28937,7 +28937,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28960,7 +28960,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28983,7 +28983,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -29006,7 +29006,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -29029,7 +29029,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -29052,7 +29052,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -29075,7 +29075,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -29098,7 +29098,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -29121,7 +29121,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -29142,7 +29142,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -29163,7 +29163,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -29184,7 +29184,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -29205,7 +29205,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -29226,7 +29226,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -29247,7 +29247,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -29268,7 +29268,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>167</v>
@@ -29291,7 +29291,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -29314,7 +29314,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -29337,7 +29337,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -29360,7 +29360,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -29383,7 +29383,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -29406,7 +29406,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -29429,7 +29429,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -29448,7 +29448,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -29467,7 +29467,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -29486,7 +29486,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -29505,7 +29505,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>174</v>
@@ -29579,11 +29579,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>175</v>
       </c>
@@ -29615,7 +29614,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>176</v>
       </c>
@@ -29648,7 +29647,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>177</v>
       </c>
@@ -29681,7 +29680,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>178</v>
       </c>
@@ -29714,7 +29713,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>179</v>
       </c>
@@ -29747,7 +29746,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>180</v>
       </c>
@@ -29780,7 +29779,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>181</v>
       </c>
@@ -29813,7 +29812,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>182</v>
       </c>
@@ -29846,7 +29845,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -29877,7 +29876,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29908,7 +29907,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>183</v>
       </c>
@@ -29941,7 +29940,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>184</v>
       </c>
@@ -29974,7 +29973,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>185</v>
       </c>
@@ -30007,7 +30006,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>186</v>
       </c>
@@ -30040,7 +30039,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>187</v>
       </c>
@@ -30073,7 +30072,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>188</v>
       </c>
@@ -30106,7 +30105,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>189</v>
       </c>
@@ -30139,7 +30138,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>190</v>
       </c>
@@ -30172,7 +30171,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>191</v>
       </c>
@@ -30205,7 +30204,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>192</v>
       </c>
@@ -30238,7 +30237,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>193</v>
       </c>
@@ -30271,7 +30270,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>194</v>
       </c>
@@ -30304,7 +30303,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>195</v>
       </c>
@@ -30337,7 +30336,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>196</v>
       </c>
@@ -30370,7 +30369,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>197</v>
       </c>
@@ -30403,7 +30402,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>198</v>
       </c>
@@ -30436,7 +30435,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>199</v>
       </c>
@@ -30468,7 +30467,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>200</v>
       </c>
@@ -30500,7 +30499,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>201</v>
       </c>
@@ -30532,7 +30531,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>202</v>
       </c>
@@ -30564,7 +30563,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>203</v>
       </c>
@@ -30596,7 +30595,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -30626,7 +30625,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -30656,7 +30655,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>204</v>
       </c>
@@ -30688,7 +30687,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>205</v>
       </c>
@@ -30720,7 +30719,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>206</v>
       </c>
@@ -30752,7 +30751,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>207</v>
       </c>
@@ -30784,7 +30783,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>208</v>
       </c>
@@ -30816,7 +30815,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -30846,7 +30845,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>209</v>
       </c>
@@ -30878,7 +30877,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>210</v>
       </c>
@@ -30910,7 +30909,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>211</v>
       </c>
@@ -30942,7 +30941,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>212</v>
       </c>
@@ -30974,7 +30973,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -31004,7 +31003,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -31034,7 +31033,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -31064,7 +31063,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -31094,7 +31093,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>213</v>
       </c>
@@ -31126,7 +31125,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>214</v>
       </c>
@@ -31158,7 +31157,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -31188,7 +31187,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -31218,7 +31217,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -31248,7 +31247,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -31278,7 +31277,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -31308,7 +31307,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -31403,11 +31402,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>215</v>
       </c>
@@ -31439,7 +31437,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -31470,7 +31468,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -31501,7 +31499,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -31532,7 +31530,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -31563,7 +31561,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -31594,7 +31592,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -31625,7 +31623,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -31656,7 +31654,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -31687,7 +31685,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -31718,7 +31716,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -31749,7 +31747,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -31780,7 +31778,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -31811,7 +31809,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -31842,7 +31840,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -31873,7 +31871,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31904,7 +31902,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31935,7 +31933,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31966,7 +31964,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31997,7 +31995,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -32028,7 +32026,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -32058,7 +32056,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -32088,7 +32086,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -32118,7 +32116,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -32148,7 +32146,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -32178,7 +32176,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -32208,7 +32206,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -32238,7 +32236,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -32268,7 +32266,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -32298,7 +32296,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -32328,7 +32326,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -32358,7 +32356,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -32388,7 +32386,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -32418,7 +32416,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -32448,7 +32446,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -32478,7 +32476,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -32508,7 +32506,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>213</v>
       </c>
@@ -32540,7 +32538,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>214</v>
       </c>
@@ -32572,7 +32570,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -32602,7 +32600,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -32632,7 +32630,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -32662,7 +32660,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -32692,7 +32690,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -32722,7 +32720,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -54465,19 +54463,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -54491,7 +54489,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>222</v>
       </c>
@@ -54503,7 +54501,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>223</v>
       </c>
@@ -54514,7 +54512,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>224</v>
       </c>
@@ -54525,7 +54523,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>225</v>
       </c>
@@ -54536,13 +54534,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-26T23:19:57Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18043,7 +18043,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>96</v>
@@ -24225,7 +24225,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:AD70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -24239,7 +24239,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -24261,7 +24261,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>101</v>
       </c>
@@ -24309,7 +24309,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -24327,7 +24327,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -24374,7 +24374,7 @@
         <v>-726.0072857142857</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -24391,7 +24391,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -24441,7 +24441,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -24458,7 +24458,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -24501,7 +24501,7 @@
         <v>-232.53333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -24518,7 +24518,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -24565,7 +24565,7 @@
         <v>-50.95312270389416</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -24582,7 +24582,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -24630,7 +24630,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -24647,7 +24647,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -24694,7 +24694,7 @@
         <v>-42.80544642857142</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -24711,7 +24711,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -24756,7 +24756,7 @@
         <v>7.380864553314173</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -24773,7 +24773,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -24823,7 +24823,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -24840,7 +24840,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -24879,7 +24879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -24896,7 +24896,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -24937,7 +24937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -24954,7 +24954,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24991,7 +24991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -25008,7 +25008,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25053,7 +25053,7 @@
         <v>0.2554973821989554</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -25070,7 +25070,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25113,7 +25113,7 @@
         <v>7.589966329966334</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -25130,7 +25130,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -25173,7 +25173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -25190,7 +25190,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -25237,7 +25237,7 @@
         <v>4.666337611056268</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -25254,7 +25254,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -25299,7 +25299,7 @@
         <v>285.64884004884004</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -25316,7 +25316,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -25359,7 +25359,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -25376,7 +25376,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -25417,7 +25417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -25434,7 +25434,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -25479,7 +25479,7 @@
         <v>561.1049999999996</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -25496,7 +25496,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25539,7 +25539,7 @@
         <v>-9.801274601686979</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -25556,7 +25556,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25593,7 +25593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -25610,7 +25610,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25651,7 +25651,7 @@
         <v>0.05940556088207709</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -25668,7 +25668,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -25711,7 +25711,7 @@
         <v>-179.9832402234637</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -25728,7 +25728,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -25770,7 +25770,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -25787,7 +25787,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -25832,7 +25832,7 @@
         <v>-9.106177818515201</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -25849,7 +25849,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -25894,7 +25894,7 @@
         <v>862.1199999999999</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -25911,7 +25911,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -25956,7 +25956,7 @@
         <v>-123.27505617977528</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25973,7 +25973,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -26010,7 +26010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -26027,7 +26027,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -26044,7 +26044,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -26061,7 +26061,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>61</v>
@@ -26082,7 +26082,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -26099,7 +26099,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -26140,7 +26140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -26157,7 +26157,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -26202,7 +26202,7 @@
         <v>13.982863259298894</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -26219,7 +26219,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -26236,7 +26236,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>121</v>
       </c>
@@ -26271,7 +26271,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>125</v>
@@ -26654,7 +26654,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB109"/>
+  <dimension ref="A1:AD109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -26665,7 +26665,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -26686,7 +26686,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>126</v>
@@ -26748,7 +26748,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>142</v>
       </c>
@@ -26806,7 +26806,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -26840,7 +26840,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -26859,7 +26859,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -26893,7 +26893,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -26912,7 +26912,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26946,7 +26946,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26965,7 +26965,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -27001,7 +27001,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -27020,7 +27020,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -27058,7 +27058,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -27077,7 +27077,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -27115,7 +27115,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -27134,7 +27134,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -27167,7 +27167,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -27186,7 +27186,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -27219,7 +27219,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -27238,7 +27238,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -27269,7 +27269,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -27288,7 +27288,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -27323,7 +27323,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -27342,7 +27342,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -27375,7 +27375,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -27394,7 +27394,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -27425,7 +27425,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -27444,7 +27444,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27476,7 +27476,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -27495,7 +27495,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27531,7 +27531,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -27550,7 +27550,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27579,7 +27579,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -27598,7 +27598,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27629,7 +27629,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -27648,7 +27648,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27681,7 +27681,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -27700,7 +27700,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27736,7 +27736,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -27755,7 +27755,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27790,7 +27790,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -27809,7 +27809,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27839,7 +27839,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -27858,7 +27858,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27898,7 +27898,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -27917,7 +27917,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27946,7 +27946,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27965,7 +27965,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -27998,7 +27998,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -28017,7 +28017,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -28050,7 +28050,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -28069,7 +28069,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -28105,7 +28105,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -28124,7 +28124,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -28160,7 +28160,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -28179,7 +28179,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -28213,7 +28213,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -28232,7 +28232,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -28267,7 +28267,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -28286,7 +28286,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -28305,7 +28305,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -28324,7 +28324,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>61</v>
@@ -28345,7 +28345,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -28364,7 +28364,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -28397,7 +28397,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -28416,7 +28416,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -28455,7 +28455,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -28474,7 +28474,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -28493,7 +28493,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -28512,7 +28512,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>146</v>
@@ -28557,7 +28557,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>147</v>
@@ -28596,7 +28596,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -28625,7 +28625,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>149</v>
@@ -28670,7 +28670,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>150</v>
@@ -28715,7 +28715,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -28734,7 +28734,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>151</v>
@@ -28781,7 +28781,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>153</v>
@@ -28826,7 +28826,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -28845,7 +28845,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>154</v>
@@ -28868,7 +28868,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>156</v>
@@ -28891,7 +28891,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>157</v>
@@ -28914,7 +28914,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28937,7 +28937,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28960,7 +28960,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28983,7 +28983,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -29006,7 +29006,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -29029,7 +29029,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -29052,7 +29052,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -29075,7 +29075,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -29098,7 +29098,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -29121,7 +29121,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -29142,7 +29142,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -29163,7 +29163,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -29184,7 +29184,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -29205,7 +29205,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -29226,7 +29226,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -29247,7 +29247,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -29268,7 +29268,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>167</v>
@@ -29291,7 +29291,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -29314,7 +29314,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -29337,7 +29337,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -29360,7 +29360,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -29383,7 +29383,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -29406,7 +29406,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -29429,7 +29429,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -29448,7 +29448,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -29467,7 +29467,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -29486,7 +29486,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -29505,7 +29505,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>174</v>
@@ -29579,10 +29579,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>175</v>
       </c>
@@ -29614,7 +29615,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>176</v>
       </c>
@@ -29647,7 +29648,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>177</v>
       </c>
@@ -29680,7 +29681,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>178</v>
       </c>
@@ -29713,7 +29714,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>179</v>
       </c>
@@ -29746,7 +29747,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>180</v>
       </c>
@@ -29779,7 +29780,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>181</v>
       </c>
@@ -29812,7 +29813,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>182</v>
       </c>
@@ -29845,7 +29846,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -29876,7 +29877,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29907,7 +29908,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>183</v>
       </c>
@@ -29940,7 +29941,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>184</v>
       </c>
@@ -29973,7 +29974,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>185</v>
       </c>
@@ -30006,7 +30007,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>186</v>
       </c>
@@ -30039,7 +30040,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>187</v>
       </c>
@@ -30072,7 +30073,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>188</v>
       </c>
@@ -30105,7 +30106,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>189</v>
       </c>
@@ -30138,7 +30139,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>190</v>
       </c>
@@ -30171,7 +30172,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>191</v>
       </c>
@@ -30204,7 +30205,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>192</v>
       </c>
@@ -30237,7 +30238,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>193</v>
       </c>
@@ -30270,7 +30271,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>194</v>
       </c>
@@ -30303,7 +30304,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>195</v>
       </c>
@@ -30336,7 +30337,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>196</v>
       </c>
@@ -30369,7 +30370,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>197</v>
       </c>
@@ -30402,7 +30403,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>198</v>
       </c>
@@ -30435,7 +30436,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>199</v>
       </c>
@@ -30467,7 +30468,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>200</v>
       </c>
@@ -30499,7 +30500,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>201</v>
       </c>
@@ -30531,7 +30532,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>202</v>
       </c>
@@ -30563,7 +30564,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>203</v>
       </c>
@@ -30595,7 +30596,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -30625,7 +30626,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -30655,7 +30656,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>204</v>
       </c>
@@ -30687,7 +30688,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>205</v>
       </c>
@@ -30719,7 +30720,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>206</v>
       </c>
@@ -30751,7 +30752,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>207</v>
       </c>
@@ -30783,7 +30784,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>208</v>
       </c>
@@ -30815,7 +30816,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -30845,7 +30846,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>209</v>
       </c>
@@ -30877,7 +30878,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>210</v>
       </c>
@@ -30909,7 +30910,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>211</v>
       </c>
@@ -30941,7 +30942,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>212</v>
       </c>
@@ -30973,7 +30974,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -31003,7 +31004,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -31033,7 +31034,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -31063,7 +31064,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -31093,7 +31094,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>213</v>
       </c>
@@ -31125,7 +31126,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>214</v>
       </c>
@@ -31157,7 +31158,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -31187,7 +31188,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -31217,7 +31218,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -31247,7 +31248,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -31277,7 +31278,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -31307,7 +31308,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -31402,10 +31403,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>215</v>
       </c>
@@ -31437,7 +31439,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -31468,7 +31470,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -31499,7 +31501,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -31530,7 +31532,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -31561,7 +31563,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -31592,7 +31594,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -31623,7 +31625,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -31654,7 +31656,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -31685,7 +31687,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -31716,7 +31718,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -31747,7 +31749,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -31778,7 +31780,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -31809,7 +31811,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -31840,7 +31842,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -31871,7 +31873,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31902,7 +31904,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31933,7 +31935,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31964,7 +31966,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31995,7 +31997,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -32026,7 +32028,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -32056,7 +32058,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -32086,7 +32088,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -32116,7 +32118,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -32146,7 +32148,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -32176,7 +32178,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -32206,7 +32208,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -32236,7 +32238,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -32266,7 +32268,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -32296,7 +32298,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -32326,7 +32328,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -32356,7 +32358,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -32386,7 +32388,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -32416,7 +32418,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -32446,7 +32448,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -32476,7 +32478,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -32506,7 +32508,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>213</v>
       </c>
@@ -32538,7 +32540,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>214</v>
       </c>
@@ -32570,7 +32572,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -32600,7 +32602,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -32630,7 +32632,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -32660,7 +32662,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -32690,7 +32692,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -32720,7 +32722,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -54463,19 +54465,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -54489,7 +54491,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>222</v>
       </c>
@@ -54501,7 +54503,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>223</v>
       </c>
@@ -54512,7 +54514,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>224</v>
       </c>
@@ -54523,7 +54525,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>225</v>
       </c>
@@ -54534,13 +54536,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-08-26T23:23:40Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -18043,7 +18043,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>96</v>
@@ -24225,7 +24225,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD70"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -24239,7 +24239,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -24261,7 +24261,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>101</v>
       </c>
@@ -24309,7 +24309,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -24327,7 +24327,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -24374,7 +24374,7 @@
         <v>-726.0072857142857</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -24391,7 +24391,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -24441,7 +24441,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -24458,7 +24458,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -24501,7 +24501,7 @@
         <v>-232.53333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -24518,7 +24518,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -24565,7 +24565,7 @@
         <v>-50.95312270389416</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -24582,7 +24582,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -24630,7 +24630,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -24647,7 +24647,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -24694,7 +24694,7 @@
         <v>-42.80544642857142</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -24711,7 +24711,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -24756,7 +24756,7 @@
         <v>7.380864553314173</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -24773,7 +24773,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -24823,7 +24823,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -24840,7 +24840,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -24879,7 +24879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -24896,7 +24896,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -24937,7 +24937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -24954,7 +24954,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24991,7 +24991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -25008,7 +25008,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25053,7 +25053,7 @@
         <v>0.2554973821989554</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -25070,7 +25070,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25113,7 +25113,7 @@
         <v>7.589966329966334</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -25130,7 +25130,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -25173,7 +25173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -25190,7 +25190,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -25237,7 +25237,7 @@
         <v>4.666337611056268</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -25254,7 +25254,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -25299,7 +25299,7 @@
         <v>285.64884004884004</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -25316,7 +25316,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -25359,7 +25359,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -25376,7 +25376,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -25417,7 +25417,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -25434,7 +25434,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -25479,7 +25479,7 @@
         <v>561.1049999999996</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -25496,7 +25496,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25539,7 +25539,7 @@
         <v>-9.801274601686979</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -25556,7 +25556,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25593,7 +25593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -25610,7 +25610,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25651,7 +25651,7 @@
         <v>0.05940556088207709</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -25668,7 +25668,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -25711,7 +25711,7 @@
         <v>-179.9832402234637</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -25728,7 +25728,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -25770,7 +25770,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -25787,7 +25787,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -25832,7 +25832,7 @@
         <v>-9.106177818515201</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -25849,7 +25849,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -25894,7 +25894,7 @@
         <v>862.1199999999999</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -25911,7 +25911,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -25956,7 +25956,7 @@
         <v>-123.27505617977528</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25973,7 +25973,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -26010,7 +26010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -26027,7 +26027,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -26044,7 +26044,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -26061,7 +26061,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>61</v>
@@ -26082,7 +26082,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -26099,7 +26099,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -26140,7 +26140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -26157,7 +26157,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -26202,7 +26202,7 @@
         <v>13.982863259298894</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -26219,7 +26219,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -26236,7 +26236,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>121</v>
       </c>
@@ -26271,7 +26271,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>125</v>
@@ -26654,7 +26654,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -26665,7 +26665,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -26686,7 +26686,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>126</v>
@@ -26748,7 +26748,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>142</v>
       </c>
@@ -26806,7 +26806,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -26840,7 +26840,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -26859,7 +26859,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -26893,7 +26893,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -26912,7 +26912,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26946,7 +26946,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26965,7 +26965,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -26994,14 +26994,16 @@
       <c r="N10" s="54">
         <v>80</v>
       </c>
-      <c r="O10" s="54"/>
+      <c r="O10" s="54">
+        <v>0</v>
+      </c>
       <c r="P10" s="54"/>
       <c r="Q10" s="131"/>
       <c r="S10" s="35" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -27020,7 +27022,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -27058,7 +27060,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -27077,7 +27079,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -27115,7 +27117,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -27134,7 +27136,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -27167,7 +27169,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -27186,7 +27188,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -27219,7 +27221,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -27238,7 +27240,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -27269,7 +27271,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -27288,7 +27290,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -27323,7 +27325,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -27342,7 +27344,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -27375,7 +27377,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -27394,7 +27396,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -27425,7 +27427,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -27444,7 +27446,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -27476,7 +27478,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -27495,7 +27497,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -27531,7 +27533,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -27550,7 +27552,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -27579,7 +27581,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -27598,7 +27600,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -27629,7 +27631,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -27648,7 +27650,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -27681,7 +27683,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -27700,7 +27702,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -27736,7 +27738,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -27755,7 +27757,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -27790,7 +27792,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -27809,7 +27811,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -27839,7 +27841,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -27858,7 +27860,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -27898,7 +27900,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -27917,7 +27919,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27946,7 +27948,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27965,7 +27967,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -27998,7 +28000,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -28017,7 +28019,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -28050,7 +28052,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -28069,7 +28071,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -28105,7 +28107,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -28124,7 +28126,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -28160,7 +28162,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -28179,7 +28181,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -28213,7 +28215,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -28232,7 +28234,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -28267,7 +28269,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -28286,7 +28288,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -28305,7 +28307,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -28324,7 +28326,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>61</v>
@@ -28345,7 +28347,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -28364,7 +28366,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -28397,7 +28399,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -28416,7 +28418,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -28455,7 +28457,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -28474,7 +28476,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -28493,7 +28495,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -28512,7 +28514,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>146</v>
@@ -28557,7 +28559,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>147</v>
@@ -28596,7 +28598,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -28625,7 +28627,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>149</v>
@@ -28670,7 +28672,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>150</v>
@@ -28715,7 +28717,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -28734,7 +28736,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>151</v>
@@ -28781,7 +28783,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>153</v>
@@ -28826,7 +28828,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -28845,7 +28847,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>154</v>
@@ -28868,7 +28870,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>156</v>
@@ -28891,7 +28893,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>157</v>
@@ -28914,7 +28916,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28937,7 +28939,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28960,7 +28962,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28983,7 +28985,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -29006,7 +29008,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -29029,7 +29031,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -29052,7 +29054,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -29075,7 +29077,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -29098,7 +29100,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -29121,7 +29123,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -29142,7 +29144,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -29163,7 +29165,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -29184,7 +29186,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -29205,7 +29207,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -29226,7 +29228,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -29247,7 +29249,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -29268,7 +29270,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>167</v>
@@ -29291,7 +29293,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -29314,7 +29316,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -29337,7 +29339,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -29360,7 +29362,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -29383,7 +29385,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -29406,7 +29408,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -29429,7 +29431,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -29448,7 +29450,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -29467,7 +29469,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -29486,7 +29488,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -29505,7 +29507,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>174</v>
@@ -29579,11 +29581,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>175</v>
       </c>
@@ -29615,7 +29616,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>176</v>
       </c>
@@ -29648,7 +29649,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>177</v>
       </c>
@@ -29681,7 +29682,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>178</v>
       </c>
@@ -29714,7 +29715,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>179</v>
       </c>
@@ -29747,7 +29748,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>180</v>
       </c>
@@ -29780,7 +29781,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>181</v>
       </c>
@@ -29813,7 +29814,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>182</v>
       </c>
@@ -29846,7 +29847,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -29877,7 +29878,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29908,7 +29909,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>183</v>
       </c>
@@ -29941,7 +29942,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>184</v>
       </c>
@@ -29974,7 +29975,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>185</v>
       </c>
@@ -30007,7 +30008,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>186</v>
       </c>
@@ -30040,7 +30041,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>187</v>
       </c>
@@ -30073,7 +30074,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>188</v>
       </c>
@@ -30106,7 +30107,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>189</v>
       </c>
@@ -30139,7 +30140,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>190</v>
       </c>
@@ -30172,7 +30173,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>191</v>
       </c>
@@ -30205,7 +30206,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>192</v>
       </c>
@@ -30238,7 +30239,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>193</v>
       </c>
@@ -30271,7 +30272,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>194</v>
       </c>
@@ -30304,7 +30305,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>195</v>
       </c>
@@ -30337,7 +30338,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>196</v>
       </c>
@@ -30370,7 +30371,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>197</v>
       </c>
@@ -30403,7 +30404,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>198</v>
       </c>
@@ -30436,7 +30437,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>199</v>
       </c>
@@ -30468,7 +30469,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>200</v>
       </c>
@@ -30500,7 +30501,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>201</v>
       </c>
@@ -30532,7 +30533,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>202</v>
       </c>
@@ -30564,7 +30565,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>203</v>
       </c>
@@ -30596,7 +30597,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -30626,7 +30627,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -30656,7 +30657,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>204</v>
       </c>
@@ -30688,7 +30689,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>205</v>
       </c>
@@ -30720,7 +30721,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>206</v>
       </c>
@@ -30752,7 +30753,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>207</v>
       </c>
@@ -30784,7 +30785,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>208</v>
       </c>
@@ -30816,7 +30817,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -30846,7 +30847,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>209</v>
       </c>
@@ -30878,7 +30879,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>210</v>
       </c>
@@ -30910,7 +30911,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>211</v>
       </c>
@@ -30942,7 +30943,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>212</v>
       </c>
@@ -30974,7 +30975,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -31004,7 +31005,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -31034,7 +31035,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -31064,7 +31065,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -31094,7 +31095,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>213</v>
       </c>
@@ -31126,7 +31127,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>214</v>
       </c>
@@ -31158,7 +31159,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -31188,7 +31189,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -31218,7 +31219,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -31248,7 +31249,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -31278,7 +31279,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -31308,7 +31309,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -31403,11 +31404,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>215</v>
       </c>
@@ -31439,7 +31439,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -31470,7 +31470,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -31501,7 +31501,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -31532,7 +31532,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -31563,7 +31563,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -31594,7 +31594,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -31625,7 +31625,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -31656,7 +31656,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -31687,7 +31687,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -31718,7 +31718,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -31749,7 +31749,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -31780,7 +31780,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -31811,7 +31811,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -31842,7 +31842,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -31873,7 +31873,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31904,7 +31904,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31935,7 +31935,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31966,7 +31966,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31997,7 +31997,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -32028,7 +32028,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -32058,7 +32058,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -32088,7 +32088,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -32118,7 +32118,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -32148,7 +32148,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -32178,7 +32178,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -32208,7 +32208,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -32238,7 +32238,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -32268,7 +32268,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -32298,7 +32298,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -32328,7 +32328,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -32358,7 +32358,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -32388,7 +32388,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -32418,7 +32418,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -32448,7 +32448,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -32478,7 +32478,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -32508,7 +32508,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>213</v>
       </c>
@@ -32540,7 +32540,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>214</v>
       </c>
@@ -32572,7 +32572,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -32602,7 +32602,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -32632,7 +32632,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -32662,7 +32662,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -32692,7 +32692,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -32722,7 +32722,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -54465,19 +54465,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -54491,7 +54491,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>222</v>
       </c>
@@ -54503,7 +54503,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>223</v>
       </c>
@@ -54514,7 +54514,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>224</v>
       </c>
@@ -54525,7 +54525,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>225</v>
       </c>
@@ -54536,13 +54536,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T00:21:25Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -9939,54 +9939,54 @@
         <v>101420.72</v>
       </c>
       <c r="I12" s="52">
-        <v>75109.37</v>
+        <v>76488.35</v>
       </c>
       <c r="J12" s="52">
         <v>83645.65</v>
       </c>
       <c r="K12" s="52">
-        <v>70211.29</v>
+        <v>70758.46</v>
       </c>
       <c r="L12" s="52">
-        <v>13434.36</v>
+        <v>12887.189999999988</v>
       </c>
       <c r="M12" s="53">
-        <v>0.16061038440134068</v>
+        <v>0.1540688607237793</v>
       </c>
       <c r="N12" s="53"/>
       <c r="O12" s="52">
         <v>17775.07</v>
       </c>
       <c r="P12" s="52">
-        <v>4898.08</v>
+        <v>5729.89</v>
       </c>
       <c r="Q12" s="52">
-        <v>12876.99</v>
+        <v>12045.18</v>
       </c>
       <c r="R12" s="53">
-        <v>0.724441028924218</v>
+        <v>0.6776445887414227</v>
       </c>
       <c r="S12" s="54">
         <v>356.07</v>
       </c>
       <c r="T12" s="54">
-        <v>100.75</v>
+        <v>117.75</v>
       </c>
       <c r="U12" s="54">
-        <v>255.32</v>
+        <v>238.32</v>
       </c>
       <c r="V12" s="53">
-        <v>0.7170500182548375</v>
+        <v>0.6693065970174403</v>
       </c>
       <c r="W12" s="53"/>
       <c r="X12" s="55">
-        <v>106.74650124069478</v>
+        <v>79.624033970276</v>
       </c>
       <c r="Y12" s="55">
         <v>77.66490997775718</v>
       </c>
       <c r="Z12" s="53">
-        <v>0.1253</v>
+        <v>0.1092</v>
       </c>
       <c r="AA12" s="56">
         <v>0.2142</v>
@@ -10302,19 +10302,19 @@
         <v>19565.83</v>
       </c>
       <c r="I19" s="52">
-        <v>7621.92</v>
+        <v>7921.92</v>
       </c>
       <c r="J19" s="52">
         <v>13767.340000000002</v>
       </c>
       <c r="K19" s="52">
-        <v>5911.24</v>
+        <v>6211.24</v>
       </c>
       <c r="L19" s="52">
-        <v>7856.100000000002</v>
+        <v>7556.100000000002</v>
       </c>
       <c r="M19" s="53">
-        <v>0.5706331070490016</v>
+        <v>0.5488424052867149</v>
       </c>
       <c r="N19" s="53"/>
       <c r="O19" s="52">
@@ -10343,13 +10343,13 @@
       </c>
       <c r="W19" s="53"/>
       <c r="X19" s="55">
-        <v>125.96143884892086</v>
+        <v>117.328345323741</v>
       </c>
       <c r="Y19" s="55">
         <v>63.27846478985563</v>
       </c>
       <c r="Z19" s="53">
-        <v>0.36479999999999996</v>
+        <v>0.3398</v>
       </c>
       <c r="AA19" s="56">
         <v>0.2885</v>
@@ -10667,19 +10667,19 @@
         <v>102178.42</v>
       </c>
       <c r="I26" s="52">
-        <v>87230.67</v>
+        <v>87101.11</v>
       </c>
       <c r="J26" s="52">
         <v>62464.86</v>
       </c>
       <c r="K26" s="52">
-        <v>58028.31</v>
+        <v>57898.75</v>
       </c>
       <c r="L26" s="52">
-        <v>4436.550000000003</v>
+        <v>4566.110000000001</v>
       </c>
       <c r="M26" s="53">
-        <v>0.07102473294585152</v>
+        <v>0.07309885910254182</v>
       </c>
       <c r="N26" s="53"/>
       <c r="O26" s="52">
@@ -10708,13 +10708,13 @@
       </c>
       <c r="W26" s="53"/>
       <c r="X26" s="55">
-        <v>96.11460050462573</v>
+        <v>96.3325315391085</v>
       </c>
       <c r="Y26" s="55">
         <v>61.20621468124544</v>
       </c>
       <c r="Z26" s="53">
-        <v>0.3958</v>
+        <v>0.3967</v>
       </c>
       <c r="AA26" s="56">
         <v>0.3227</v>
@@ -11030,54 +11030,54 @@
         <v>327431.12</v>
       </c>
       <c r="I33" s="65">
-        <v>219182.25</v>
+        <v>220187.84</v>
       </c>
       <c r="J33" s="52">
         <v>271519.78</v>
       </c>
       <c r="K33" s="52">
-        <v>196853</v>
+        <v>196879.33</v>
       </c>
       <c r="L33" s="52">
-        <v>74666.78000000003</v>
+        <v>74640.45000000004</v>
       </c>
       <c r="M33" s="53">
-        <v>0.2749957295928865</v>
+        <v>0.27489875691561044</v>
       </c>
       <c r="N33" s="53"/>
       <c r="O33" s="52">
         <v>55911.34</v>
       </c>
       <c r="P33" s="52">
-        <v>22329.25</v>
+        <v>23308.51</v>
       </c>
       <c r="Q33" s="52">
-        <v>33582.09</v>
+        <v>32602.829999999998</v>
       </c>
       <c r="R33" s="53">
-        <v>0.6006311063193978</v>
+        <v>0.5831165913748445</v>
       </c>
       <c r="S33" s="54">
         <v>1120.27</v>
       </c>
       <c r="T33" s="54">
-        <v>522.25</v>
+        <v>543.5</v>
       </c>
       <c r="U33" s="54">
-        <v>598.02</v>
+        <v>576.77</v>
       </c>
       <c r="V33" s="53">
-        <v>0.5338177403661617</v>
+        <v>0.514849098877949</v>
       </c>
       <c r="W33" s="53"/>
       <c r="X33" s="55">
-        <v>76.90849210148396</v>
+        <v>72.05127874885005</v>
       </c>
       <c r="Y33" s="55">
         <v>61.5841822414239</v>
       </c>
       <c r="Z33" s="53">
-        <v>0.1549</v>
+        <v>0.151</v>
       </c>
       <c r="AA33" s="56">
         <v>0.174</v>
@@ -11393,54 +11393,54 @@
         <v>94098.32</v>
       </c>
       <c r="I40" s="52">
-        <v>45499.87</v>
+        <v>46289.42</v>
       </c>
       <c r="J40" s="52">
         <v>69042.09000000001</v>
       </c>
       <c r="K40" s="52">
-        <v>35731.93</v>
+        <v>35507.08</v>
       </c>
       <c r="L40" s="52">
-        <v>33310.16000000001</v>
+        <v>33535.01000000001</v>
       </c>
       <c r="M40" s="53">
-        <v>0.4824616404283243</v>
+        <v>0.4857183494879718</v>
       </c>
       <c r="N40" s="53"/>
       <c r="O40" s="52">
         <v>25056.23</v>
       </c>
       <c r="P40" s="52">
-        <v>9767.94</v>
+        <v>10782.34</v>
       </c>
       <c r="Q40" s="52">
-        <v>15288.289999999999</v>
+        <v>14273.89</v>
       </c>
       <c r="R40" s="53">
-        <v>0.6101592298601984</v>
+        <v>0.5696742885901032</v>
       </c>
       <c r="S40" s="54">
         <v>501.83</v>
       </c>
       <c r="T40" s="54">
-        <v>205.75</v>
+        <v>232.25</v>
       </c>
       <c r="U40" s="54">
-        <v>296.08</v>
+        <v>269.58</v>
       </c>
       <c r="V40" s="53">
-        <v>0.5900005978120081</v>
+        <v>0.5371938704342107</v>
       </c>
       <c r="W40" s="53"/>
       <c r="X40" s="55">
-        <v>41.0447630619684</v>
+        <v>32.96193756727664</v>
       </c>
       <c r="Y40" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z40" s="53">
-        <v>0.1565</v>
+        <v>0.1419</v>
       </c>
       <c r="AA40" s="56">
         <v>0.2663</v>
@@ -11758,19 +11758,19 @@
         <v>50582.37</v>
       </c>
       <c r="I47" s="52">
-        <v>25337.26</v>
+        <v>25187.36</v>
       </c>
       <c r="J47" s="52">
         <v>39438.990000000005</v>
       </c>
       <c r="K47" s="52">
-        <v>20582.32</v>
+        <v>20432.420000000002</v>
       </c>
       <c r="L47" s="52">
-        <v>18856.670000000006</v>
+        <v>19006.570000000003</v>
       </c>
       <c r="M47" s="53">
-        <v>0.4781225381278781</v>
+        <v>0.48192334540007237</v>
       </c>
       <c r="N47" s="53"/>
       <c r="O47" s="52">
@@ -11799,13 +11799,13 @@
       </c>
       <c r="W47" s="53"/>
       <c r="X47" s="55">
-        <v>76.63529976019184</v>
+        <v>78.07318944844125</v>
       </c>
       <c r="Y47" s="55">
         <v>67.69550512136009</v>
       </c>
       <c r="Z47" s="53">
-        <v>0.2397</v>
+        <v>0.24420000000000003</v>
       </c>
       <c r="AA47" s="56">
         <v>0.23</v>
@@ -12121,19 +12121,19 @@
         <v>109364.97</v>
       </c>
       <c r="I54" s="52">
-        <v>95642.03</v>
+        <v>95597.19</v>
       </c>
       <c r="J54" s="52">
         <v>75135.01000000001</v>
       </c>
       <c r="K54" s="52">
-        <v>71188.63</v>
+        <v>71143.79000000001</v>
       </c>
       <c r="L54" s="52">
-        <v>3946.3800000000047</v>
+        <v>3991.220000000001</v>
       </c>
       <c r="M54" s="53">
-        <v>0.05252385006669999</v>
+        <v>0.05312064242754477</v>
       </c>
       <c r="N54" s="53"/>
       <c r="O54" s="52">
@@ -12162,13 +12162,13 @@
       </c>
       <c r="W54" s="53"/>
       <c r="X54" s="55">
-        <v>62.138966682761954</v>
+        <v>62.22557218734911</v>
       </c>
       <c r="Y54" s="55">
         <v>67.00679527854935</v>
       </c>
       <c r="Z54" s="53">
-        <v>0.25170000000000003</v>
+        <v>0.2521</v>
       </c>
       <c r="AA54" s="56">
         <v>0.2958</v>
@@ -12841,19 +12841,19 @@
         <v>35572.59</v>
       </c>
       <c r="I68" s="52">
-        <v>9981.43</v>
+        <v>10547.08</v>
       </c>
       <c r="J68" s="52">
         <v>27136.549999999996</v>
       </c>
       <c r="K68" s="52">
-        <v>9832.65</v>
+        <v>10398.3</v>
       </c>
       <c r="L68" s="52">
-        <v>17303.899999999994</v>
+        <v>16738.249999999996</v>
       </c>
       <c r="M68" s="53">
-        <v>0.6376602773749794</v>
+        <v>0.6168156969106242</v>
       </c>
       <c r="N68" s="53"/>
       <c r="O68" s="52">
@@ -12882,13 +12882,13 @@
       </c>
       <c r="W68" s="53"/>
       <c r="X68" s="55">
-        <v>243.27272727272728</v>
+        <v>37.58181818181818</v>
       </c>
       <c r="Y68" s="55">
         <v>72.22475431425701</v>
       </c>
       <c r="Z68" s="53">
-        <v>0.06280000000000001</v>
+        <v>0.0097</v>
       </c>
       <c r="AA68" s="56">
         <v>0.2558</v>
@@ -13916,19 +13916,19 @@
         <v>27002.93</v>
       </c>
       <c r="I89" s="52">
-        <v>26005.99</v>
+        <v>24950.27</v>
       </c>
       <c r="J89" s="52">
         <v>15440.32</v>
       </c>
       <c r="K89" s="52">
-        <v>14988.440000000002</v>
+        <v>13932.720000000001</v>
       </c>
       <c r="L89" s="52">
-        <v>451.8799999999974</v>
+        <v>1507.5999999999985</v>
       </c>
       <c r="M89" s="53">
-        <v>0.029266232824190004</v>
+        <v>0.09764046341008467</v>
       </c>
       <c r="N89" s="53"/>
       <c r="O89" s="52">
@@ -13957,13 +13957,13 @@
       </c>
       <c r="W89" s="53"/>
       <c r="X89" s="55">
-        <v>46.26684503901895</v>
+        <v>50.9746265328874</v>
       </c>
       <c r="Y89" s="55">
         <v>43.49557070636461</v>
       </c>
       <c r="Z89" s="53">
-        <v>0.2852</v>
+        <v>0.31420000000000003</v>
       </c>
       <c r="AA89" s="56">
         <v>0.2718</v>
@@ -14626,30 +14626,74 @@
       <c r="C103" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="D103" s="52"/>
-      <c r="E103" s="69"/>
-      <c r="F103" s="52"/>
-      <c r="G103" s="53"/>
-      <c r="H103" s="52"/>
-      <c r="I103" s="52"/>
-      <c r="J103" s="52"/>
-      <c r="K103" s="52"/>
-      <c r="L103" s="52"/>
-      <c r="M103" s="53"/>
+      <c r="D103" s="52">
+        <v>32473.02</v>
+      </c>
+      <c r="E103" s="69">
+        <v>33188.03</v>
+      </c>
+      <c r="F103" s="52">
+        <v>-715.0099999999984</v>
+      </c>
+      <c r="G103" s="53">
+        <v>-0.022018586506582952</v>
+      </c>
+      <c r="H103" s="52">
+        <v>23075.07</v>
+      </c>
+      <c r="I103" s="52">
+        <v>30925.21</v>
+      </c>
+      <c r="J103" s="52">
+        <v>12691.21</v>
+      </c>
+      <c r="K103" s="52">
+        <v>15184.269999999999</v>
+      </c>
+      <c r="L103" s="52">
+        <v>-2493.0599999999995</v>
+      </c>
+      <c r="M103" s="53">
+        <v>-0.1964398981657383</v>
+      </c>
       <c r="N103" s="53"/>
-      <c r="O103" s="52"/>
-      <c r="P103" s="52"/>
-      <c r="Q103" s="52"/>
-      <c r="R103" s="53"/>
-      <c r="S103" s="54"/>
-      <c r="T103" s="54"/>
-      <c r="U103" s="54"/>
-      <c r="V103" s="53"/>
+      <c r="O103" s="52">
+        <v>10383.86</v>
+      </c>
+      <c r="P103" s="52">
+        <v>15740.94</v>
+      </c>
+      <c r="Q103" s="52">
+        <v>-5357.08</v>
+      </c>
+      <c r="R103" s="53">
+        <v>-0.5159044902377343</v>
+      </c>
+      <c r="S103" s="54">
+        <v>208.2</v>
+      </c>
+      <c r="T103" s="54">
+        <v>317.25</v>
+      </c>
+      <c r="U103" s="54">
+        <v>-109.05000000000001</v>
+      </c>
+      <c r="V103" s="53">
+        <v>-0.5237752161383286</v>
+      </c>
       <c r="W103" s="53"/>
-      <c r="X103" s="55"/>
-      <c r="Y103" s="55"/>
-      <c r="Z103" s="53"/>
-      <c r="AA103" s="56"/>
+      <c r="X103" s="55">
+        <v>7.132608353033885</v>
+      </c>
+      <c r="Y103" s="55">
+        <v>45.139084580403456</v>
+      </c>
+      <c r="Z103" s="53">
+        <v>0.0682</v>
+      </c>
+      <c r="AA103" s="56">
+        <v>0.2894</v>
+      </c>
       <c r="AB103" s="57"/>
       <c r="AD103" s="35" t="s">
         <v>93</v>
@@ -14963,19 +15007,19 @@
         <v>37601.88</v>
       </c>
       <c r="I110" s="52">
-        <v>45837.23</v>
+        <v>45817.77</v>
       </c>
       <c r="J110" s="52">
         <v>21415.85</v>
       </c>
       <c r="K110" s="52">
-        <v>23958.850000000002</v>
+        <v>23939.389999999996</v>
       </c>
       <c r="L110" s="52">
-        <v>-2543.0000000000036</v>
+        <v>-2523.5399999999972</v>
       </c>
       <c r="M110" s="53">
-        <v>-0.11874382758564352</v>
+        <v>-0.11783515480356826</v>
       </c>
       <c r="N110" s="53"/>
       <c r="O110" s="52">
@@ -15004,13 +15048,13 @@
       </c>
       <c r="W110" s="53"/>
       <c r="X110" s="55">
-        <v>48.93201480698043</v>
+        <v>48.973178212585935</v>
       </c>
       <c r="Y110" s="55">
         <v>65.70431400737223</v>
       </c>
       <c r="Z110" s="53">
-        <v>0.3354</v>
+        <v>0.3357</v>
       </c>
       <c r="AA110" s="56">
         <v>0.3616</v>
@@ -15673,19 +15717,19 @@
         <v>82694.87</v>
       </c>
       <c r="I124" s="52">
-        <v>56983.56</v>
+        <v>56763.31</v>
       </c>
       <c r="J124" s="52">
         <v>68214.25</v>
       </c>
       <c r="K124" s="52">
-        <v>52178.049999999996</v>
+        <v>51957.799999999996</v>
       </c>
       <c r="L124" s="52">
-        <v>16036.200000000004</v>
+        <v>16256.450000000004</v>
       </c>
       <c r="M124" s="53">
-        <v>0.23508577753182075</v>
+        <v>0.23831457503380898</v>
       </c>
       <c r="N124" s="53"/>
       <c r="O124" s="52">
@@ -15714,13 +15758,13 @@
       </c>
       <c r="W124" s="53"/>
       <c r="X124" s="55">
-        <v>99.27371428571428</v>
+        <v>101.37133333333333</v>
       </c>
       <c r="Y124" s="55">
         <v>63.04545035767707</v>
       </c>
       <c r="Z124" s="53">
-        <v>0.15460000000000002</v>
+        <v>0.15789999999999998</v>
       </c>
       <c r="AA124" s="56">
         <v>0.1811</v>
@@ -18141,30 +18185,74 @@
       <c r="C173" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="D173" s="52"/>
-      <c r="E173" s="52"/>
-      <c r="F173" s="52"/>
-      <c r="G173" s="53"/>
-      <c r="H173" s="52"/>
-      <c r="I173" s="52"/>
-      <c r="J173" s="52"/>
-      <c r="K173" s="52"/>
-      <c r="L173" s="52"/>
-      <c r="M173" s="53"/>
+      <c r="D173" s="52">
+        <v>146237.11</v>
+      </c>
+      <c r="E173" s="52">
+        <v>125386.21</v>
+      </c>
+      <c r="F173" s="52">
+        <v>20850.89999999998</v>
+      </c>
+      <c r="G173" s="53">
+        <v>0.14258282319720336</v>
+      </c>
+      <c r="H173" s="52">
+        <v>114651.87</v>
+      </c>
+      <c r="I173" s="52">
+        <v>105511.63</v>
+      </c>
+      <c r="J173" s="52">
+        <v>82888.07999999999</v>
+      </c>
+      <c r="K173" s="52">
+        <v>78161.06</v>
+      </c>
+      <c r="L173" s="52">
+        <v>4727.0199999999895</v>
+      </c>
+      <c r="M173" s="53">
+        <v>0.05702894795005495</v>
+      </c>
       <c r="N173" s="53"/>
-      <c r="O173" s="52"/>
-      <c r="P173" s="52"/>
-      <c r="Q173" s="52"/>
-      <c r="R173" s="53"/>
-      <c r="S173" s="54"/>
-      <c r="T173" s="54"/>
-      <c r="U173" s="54"/>
-      <c r="V173" s="53"/>
+      <c r="O173" s="52">
+        <v>31763.79</v>
+      </c>
+      <c r="P173" s="52">
+        <v>27350.57</v>
+      </c>
+      <c r="Q173" s="52">
+        <v>4413.220000000001</v>
+      </c>
+      <c r="R173" s="53">
+        <v>0.13893870976983544</v>
+      </c>
+      <c r="S173" s="54">
+        <v>659.73</v>
+      </c>
+      <c r="T173" s="54">
+        <v>548.75</v>
+      </c>
+      <c r="U173" s="54">
+        <v>110.98000000000002</v>
+      </c>
+      <c r="V173" s="53">
+        <v>0.16822033256028984</v>
+      </c>
       <c r="W173" s="53"/>
-      <c r="X173" s="55"/>
-      <c r="Y173" s="55"/>
-      <c r="Z173" s="53"/>
-      <c r="AA173" s="56"/>
+      <c r="X173" s="55">
+        <v>36.21791343963554</v>
+      </c>
+      <c r="Y173" s="55">
+        <v>47.87601261940491</v>
+      </c>
+      <c r="Z173" s="53">
+        <v>0.1585</v>
+      </c>
+      <c r="AA173" s="56">
+        <v>0.216</v>
+      </c>
       <c r="AB173" s="57"/>
       <c r="AD173" s="35" t="s">
         <v>93</v>
@@ -18771,30 +18859,74 @@
       <c r="C187" s="51" t="s">
         <v>92</v>
       </c>
-      <c r="D187" s="52"/>
-      <c r="E187" s="52"/>
-      <c r="F187" s="52"/>
-      <c r="G187" s="53"/>
-      <c r="H187" s="52"/>
-      <c r="I187" s="52"/>
-      <c r="J187" s="52"/>
-      <c r="K187" s="52"/>
-      <c r="L187" s="52"/>
-      <c r="M187" s="53"/>
+      <c r="D187" s="52">
+        <v>20992.12</v>
+      </c>
+      <c r="E187" s="52">
+        <v>14169.68</v>
+      </c>
+      <c r="F187" s="52">
+        <v>6822.439999999999</v>
+      </c>
+      <c r="G187" s="53">
+        <v>0.32500004763692275</v>
+      </c>
+      <c r="H187" s="52">
+        <v>16299.09</v>
+      </c>
+      <c r="I187" s="52">
+        <v>9699.51</v>
+      </c>
+      <c r="J187" s="52">
+        <v>9784.33</v>
+      </c>
+      <c r="K187" s="52">
+        <v>8137.88</v>
+      </c>
+      <c r="L187" s="52">
+        <v>1646.4499999999998</v>
+      </c>
+      <c r="M187" s="53">
+        <v>0.16827416900288522</v>
+      </c>
       <c r="N187" s="53"/>
-      <c r="O187" s="52"/>
-      <c r="P187" s="52"/>
-      <c r="Q187" s="52"/>
-      <c r="R187" s="53"/>
-      <c r="S187" s="54"/>
-      <c r="T187" s="54"/>
-      <c r="U187" s="54"/>
-      <c r="V187" s="53"/>
+      <c r="O187" s="52">
+        <v>6514.76</v>
+      </c>
+      <c r="P187" s="52">
+        <v>1561.63</v>
+      </c>
+      <c r="Q187" s="52">
+        <v>4953.13</v>
+      </c>
+      <c r="R187" s="53">
+        <v>0.7602935488030257</v>
+      </c>
+      <c r="S187" s="54">
+        <v>130.62</v>
+      </c>
+      <c r="T187" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U187" s="54">
+        <v>95.87</v>
+      </c>
+      <c r="V187" s="53">
+        <v>0.7339611085591793</v>
+      </c>
       <c r="W187" s="53"/>
-      <c r="X187" s="55"/>
-      <c r="Y187" s="55"/>
-      <c r="Z187" s="53"/>
-      <c r="AA187" s="56"/>
+      <c r="X187" s="55">
+        <v>128.6379856115108</v>
+      </c>
+      <c r="Y187" s="55">
+        <v>35.92887828502527</v>
+      </c>
+      <c r="Z187" s="53">
+        <v>0.3155</v>
+      </c>
+      <c r="AA187" s="56">
+        <v>0.2236</v>
+      </c>
       <c r="AB187" s="57"/>
       <c r="AD187" s="35" t="s">
         <v>93</v>
@@ -20023,19 +20155,19 @@
         <v>117394.57</v>
       </c>
       <c r="I215" s="52">
-        <v>26124</v>
+        <v>30594.96</v>
       </c>
       <c r="J215" s="52">
         <v>99479.62000000001</v>
       </c>
       <c r="K215" s="52">
-        <v>26124</v>
+        <v>30594.96</v>
       </c>
       <c r="L215" s="52">
-        <v>73355.62000000001</v>
+        <v>68884.66</v>
       </c>
       <c r="M215" s="53">
-        <v>0.7373934480248316</v>
+        <v>0.692449971159922</v>
       </c>
       <c r="N215" s="53"/>
       <c r="O215" s="52">
@@ -20070,7 +20202,7 @@
         <v>54.93783457863793</v>
       </c>
       <c r="Z215" s="53">
-        <v>0.13419999999999999</v>
+        <v>-0.0139</v>
       </c>
       <c r="AA215" s="56">
         <v>0.1438</v>
@@ -20376,54 +20508,54 @@
         <v>295569.99</v>
       </c>
       <c r="I222" s="52">
-        <v>240067.38</v>
+        <v>241753.24</v>
       </c>
       <c r="J222" s="52">
         <v>178700.37</v>
       </c>
       <c r="K222" s="52">
-        <v>178119.89</v>
+        <v>178956.15</v>
       </c>
       <c r="L222" s="52">
-        <v>580.4799999999814</v>
+        <v>-255.77999999999884</v>
       </c>
       <c r="M222" s="53">
-        <v>0.003248342462861053</v>
+        <v>-0.0014313344734540776</v>
       </c>
       <c r="N222" s="53"/>
       <c r="O222" s="52">
         <v>116869.62</v>
       </c>
       <c r="P222" s="52">
-        <v>61947.49</v>
+        <v>62797.09</v>
       </c>
       <c r="Q222" s="52">
-        <v>54922.13</v>
+        <v>54072.53</v>
       </c>
       <c r="R222" s="53">
-        <v>0.4699436003984611</v>
+        <v>0.4626739609489618</v>
       </c>
       <c r="S222" s="54">
         <v>2344.68</v>
       </c>
       <c r="T222" s="54">
-        <v>1315</v>
+        <v>1335</v>
       </c>
       <c r="U222" s="54">
-        <v>1029.6799999999998</v>
+        <v>1009.6799999999998</v>
       </c>
       <c r="V222" s="53">
-        <v>0.4391558762816247</v>
+        <v>0.4306259276319156</v>
       </c>
       <c r="W222" s="53"/>
       <c r="X222" s="55">
-        <v>50.16819011406844</v>
+        <v>48.153790262172286</v>
       </c>
       <c r="Y222" s="55">
         <v>43.0265399367206</v>
       </c>
       <c r="Z222" s="53">
-        <v>0.21559999999999999</v>
+        <v>0.2101</v>
       </c>
       <c r="AA222" s="56">
         <v>0.2545</v>
@@ -21331,10 +21463,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="52">
-        <v>972.0499999999884</v>
+        <v>2351.029999999999</v>
       </c>
       <c r="E6" s="52">
-        <v>-972.0499999999884</v>
+        <v>-2351.029999999999</v>
       </c>
       <c r="F6" s="52">
         <v>0</v>
@@ -21358,13 +21490,13 @@
         <v>0</v>
       </c>
       <c r="M6" s="52">
-        <v>-2844.6499999999883</v>
+        <v>-4223.629999999999</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>227.57199999999906</v>
+        <v>337.89039999999994</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>115</v>
@@ -21398,10 +21530,10 @@
         <v>0</v>
       </c>
       <c r="D8" s="52">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="E8" s="52">
-        <v>0</v>
+        <v>-300</v>
       </c>
       <c r="F8" s="52"/>
       <c r="G8" s="53">
@@ -21421,13 +21553,13 @@
         <v>0</v>
       </c>
       <c r="M8" s="52">
-        <v>-640</v>
+        <v>-940</v>
       </c>
       <c r="N8" s="54">
         <v>-34.75</v>
       </c>
       <c r="O8" s="58">
-        <v>34.13333333333333</v>
+        <v>50.13333333333333</v>
       </c>
     </row>
     <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -21458,10 +21590,10 @@
         <v>0</v>
       </c>
       <c r="D10" s="52">
-        <v>1382.2599999999948</v>
+        <v>1252.699999999997</v>
       </c>
       <c r="E10" s="52">
-        <v>-1382.2599999999948</v>
+        <v>-1252.699999999997</v>
       </c>
       <c r="F10" s="52">
         <v>0</v>
@@ -21485,13 +21617,13 @@
         <v>0</v>
       </c>
       <c r="M10" s="52">
-        <v>-6302.259999999995</v>
+        <v>-6172.699999999997</v>
       </c>
       <c r="N10" s="54">
         <v>-388.25</v>
       </c>
       <c r="O10" s="58">
-        <v>18.522439382806745</v>
+        <v>18.141660543717848</v>
       </c>
     </row>
     <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -21522,10 +21654,10 @@
         <v>0</v>
       </c>
       <c r="D12" s="52">
-        <v>2837.649999999994</v>
+        <v>3843.2399999999907</v>
       </c>
       <c r="E12" s="52">
-        <v>-2837.649999999994</v>
+        <v>-3843.2399999999907</v>
       </c>
       <c r="F12" s="52"/>
       <c r="G12" s="53">
@@ -21547,13 +21679,13 @@
         <v>0</v>
       </c>
       <c r="M12" s="52">
-        <v>-5477.649999999994</v>
+        <v>-6483.239999999991</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>-79.38623188405789</v>
+        <v>-93.95999999999987</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>117</v>
@@ -21587,10 +21719,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="52">
-        <v>3226.1800000000003</v>
+        <v>4015.729999999996</v>
       </c>
       <c r="E14" s="52">
-        <v>-3226.1800000000003</v>
+        <v>-4015.729999999996</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
@@ -21614,13 +21746,13 @@
         <v>0</v>
       </c>
       <c r="M14" s="52">
-        <v>-6226.18</v>
+        <v>-7015.729999999996</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>55.59089285714286</v>
+        <v>62.640446428571394</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -21651,10 +21783,10 @@
         <v>0</v>
       </c>
       <c r="D16" s="52">
-        <v>125.67999999999665</v>
+        <v>-24.220000000001164</v>
       </c>
       <c r="E16" s="52">
-        <v>-125.67999999999665</v>
+        <v>24.220000000001164</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="53">
@@ -21676,13 +21808,13 @@
         <v>0</v>
       </c>
       <c r="M16" s="52">
-        <v>-3125.6799999999967</v>
+        <v>-2975.779999999999</v>
       </c>
       <c r="N16" s="54">
         <v>-86.75</v>
       </c>
       <c r="O16" s="58">
-        <v>36.030893371757884</v>
+        <v>34.302939481268</v>
       </c>
     </row>
     <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -21713,10 +21845,10 @@
         <v>0</v>
       </c>
       <c r="D18" s="52">
-        <v>321.5200000000041</v>
+        <v>276.68000000000757</v>
       </c>
       <c r="E18" s="52">
-        <v>-321.5200000000041</v>
+        <v>-276.68000000000757</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
@@ -21740,13 +21872,13 @@
         <v>0</v>
       </c>
       <c r="M18" s="52">
-        <v>-8521.520000000004</v>
+        <v>-8476.680000000008</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>45.087407407407426</v>
+        <v>44.85015873015877</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>118</v>
@@ -21836,10 +21968,10 @@
         <v>0</v>
       </c>
       <c r="D22" s="52">
-        <v>0</v>
+        <v>565.6499999999996</v>
       </c>
       <c r="E22" s="52">
-        <v>0</v>
+        <v>-565.6499999999996</v>
       </c>
       <c r="F22" s="52">
         <v>0</v>
@@ -21859,7 +21991,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="52">
-        <v>0</v>
+        <v>-565.6499999999996</v>
       </c>
       <c r="N22" s="54"/>
       <c r="O22" s="58">
@@ -22010,10 +22142,10 @@
         <v>0</v>
       </c>
       <c r="D28" s="52">
-        <v>0</v>
+        <v>-1055.7200000000012</v>
       </c>
       <c r="E28" s="52">
-        <v>0</v>
+        <v>1055.7200000000012</v>
       </c>
       <c r="F28" s="52">
         <v>0</v>
@@ -22033,13 +22165,13 @@
         <v>0</v>
       </c>
       <c r="M28" s="52">
-        <v>0</v>
+        <v>1055.7200000000012</v>
       </c>
       <c r="N28" s="54">
         <v>-148.5</v>
       </c>
       <c r="O28" s="58">
-        <v>0</v>
+        <v>-7.109225589225597</v>
       </c>
     </row>
     <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22194,10 +22326,10 @@
         <v>0</v>
       </c>
       <c r="D34" s="52">
-        <v>943.3400000000038</v>
+        <v>923.8799999999974</v>
       </c>
       <c r="E34" s="52">
-        <v>-943.3400000000038</v>
+        <v>-923.8799999999974</v>
       </c>
       <c r="F34" s="52">
         <v>0</v>
@@ -22219,13 +22351,13 @@
         <v>0</v>
       </c>
       <c r="M34" s="52">
-        <v>-943.3400000000038</v>
+        <v>-923.8799999999974</v>
       </c>
       <c r="N34" s="54">
         <v>-204.75</v>
       </c>
       <c r="O34" s="58">
-        <v>4.607277167277186</v>
+        <v>4.512234432234419</v>
       </c>
     </row>
     <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22316,16 +22448,16 @@
         <v>52040.560000000005</v>
       </c>
       <c r="D38" s="52">
-        <v>746.3099999999977</v>
+        <v>526.0599999999977</v>
       </c>
       <c r="E38" s="52">
-        <v>51294.25000000001</v>
+        <v>51514.50000000001</v>
       </c>
       <c r="F38" s="52">
         <v>0</v>
       </c>
       <c r="G38" s="53">
-        <v>0.9856590705403632</v>
+        <v>0.9898913462883566</v>
       </c>
       <c r="H38" s="53">
         <v>0.1750921737769</v>
@@ -22336,10 +22468,10 @@
         <v>0</v>
       </c>
       <c r="L38" s="53">
-        <v>0.9856590705403632</v>
+        <v>0.9898913462883566</v>
       </c>
       <c r="M38" s="52">
-        <v>51294.25000000001</v>
+        <v>51514.50000000001</v>
       </c>
       <c r="N38" s="54"/>
       <c r="O38" s="58">
@@ -22727,10 +22859,10 @@
         <v>0</v>
       </c>
       <c r="D52" s="99">
-        <v>0</v>
+        <v>2629.5100000000093</v>
       </c>
       <c r="E52" s="99">
-        <v>0</v>
+        <v>-2629.5100000000093</v>
       </c>
       <c r="F52" s="99"/>
       <c r="G52" s="100">
@@ -22752,13 +22884,13 @@
         <v>0</v>
       </c>
       <c r="M52" s="99">
-        <v>-1280</v>
+        <v>-3909.5100000000093</v>
       </c>
       <c r="N52" s="98">
         <v>-304.75</v>
       </c>
       <c r="O52" s="60">
-        <v>4.692942254812099</v>
+        <v>14.333675527039448</v>
       </c>
     </row>
     <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23039,10 +23171,10 @@
         <v>0</v>
       </c>
       <c r="D64" s="99">
-        <v>0</v>
+        <v>4470.959999999999</v>
       </c>
       <c r="E64" s="99">
-        <v>0</v>
+        <v>-4470.959999999999</v>
       </c>
       <c r="F64" s="99"/>
       <c r="G64" s="100">
@@ -23062,7 +23194,7 @@
         <v>0</v>
       </c>
       <c r="M64" s="99">
-        <v>-1750</v>
+        <v>-6220.959999999999</v>
       </c>
       <c r="N64" s="98"/>
       <c r="O64" s="60">
@@ -23097,14 +23229,14 @@
         <v>34650.399999999965</v>
       </c>
       <c r="D66" s="99">
-        <v>5744.570000000007</v>
+        <v>7430.429999999993</v>
       </c>
       <c r="E66" s="99">
-        <v>28905.829999999958</v>
+        <v>27219.969999999972</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
-        <v>0.8342134578533</v>
+        <v>0.7855600512548195</v>
       </c>
       <c r="H66" s="100">
         <v>0.256265521519856</v>
@@ -23119,16 +23251,16 @@
         <v>3200</v>
       </c>
       <c r="L66" s="100">
-        <v>0.7418624316025207</v>
+        <v>0.6932090250040402</v>
       </c>
       <c r="M66" s="99">
-        <v>25705.829999999958</v>
+        <v>24019.969999999972</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>-27.51493711533311</v>
+        <v>-25.71043082686644</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23176,22 +23308,22 @@
         <v>88818.76999999996</v>
       </c>
       <c r="D69" s="104">
-        <v>18681.369999999988</v>
+        <v>29887.739999999983</v>
       </c>
       <c r="E69" s="105">
-        <v>70137.39999999998</v>
+        <v>58931.02999999998</v>
       </c>
       <c r="F69" s="106" t="s">
         <v>122</v>
       </c>
       <c r="G69" s="107">
-        <v>0.7896686702596761</v>
+        <v>0.6634974791927427</v>
       </c>
       <c r="H69" s="108" t="s">
         <v>123</v>
       </c>
       <c r="I69" s="109">
-        <v>0.20609157276102777</v>
+        <v>0.0799203816940944</v>
       </c>
       <c r="J69" s="36"/>
       <c r="K69" s="36"/>
@@ -23799,10 +23931,10 @@
         <v>356.07</v>
       </c>
       <c r="D6" s="54">
-        <v>100.75</v>
+        <v>117.75</v>
       </c>
       <c r="E6" s="54">
-        <v>255.32</v>
+        <v>238.32</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -23962,10 +24094,10 @@
         <v>1120.27</v>
       </c>
       <c r="D12" s="54">
-        <v>522.25</v>
+        <v>543.5</v>
       </c>
       <c r="E12" s="54">
-        <v>598.02</v>
+        <v>576.77</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -24019,10 +24151,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>205.75</v>
+        <v>232.25</v>
       </c>
       <c r="E14" s="54">
-        <v>296.08</v>
+        <v>269.58</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -25011,10 +25143,10 @@
         <v>659.73</v>
       </c>
       <c r="D52" s="54">
-        <v>505.25</v>
+        <v>548.75</v>
       </c>
       <c r="E52" s="54">
-        <v>154.48000000000002</v>
+        <v>110.98000000000002</v>
       </c>
       <c r="F52" s="54"/>
       <c r="G52" s="54"/>
@@ -25358,10 +25490,10 @@
         <v>2344.68</v>
       </c>
       <c r="D66" s="54">
-        <v>1315</v>
+        <v>1335</v>
       </c>
       <c r="E66" s="54">
-        <v>1029.6799999999998</v>
+        <v>1009.6799999999998</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T01:53:58Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16176,7 +16176,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -21286,7 +21286,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD70"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21300,7 +21300,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21322,7 +21322,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -21370,7 +21370,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21388,7 +21388,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21435,7 +21435,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21452,7 +21452,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -21502,7 +21502,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -21519,7 +21519,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -21562,7 +21562,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -21579,7 +21579,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -21626,7 +21626,7 @@
         <v>18.141660543717848</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -21643,7 +21643,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -21659,7 +21659,9 @@
       <c r="E12" s="52">
         <v>-3843.2399999999907</v>
       </c>
-      <c r="F12" s="52"/>
+      <c r="F12" s="52">
+        <v>3</v>
+      </c>
       <c r="G12" s="53">
         <v>0</v>
       </c>
@@ -21691,7 +21693,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -21708,7 +21710,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -21755,7 +21757,7 @@
         <v>62.640446428571394</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -21772,7 +21774,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -21817,7 +21819,7 @@
         <v>34.302939481268</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -21834,7 +21836,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -21884,7 +21886,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -21901,7 +21903,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -21940,7 +21942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -21957,7 +21959,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -21998,7 +22000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22015,7 +22017,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22052,7 +22054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22069,7 +22071,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22114,7 +22116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22131,7 +22133,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22174,7 +22176,7 @@
         <v>-7.109225589225597</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22191,7 +22193,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22234,7 +22236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22251,7 +22253,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22298,7 +22300,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22315,7 +22317,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22360,7 +22362,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22377,7 +22379,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22420,7 +22422,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22437,7 +22439,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22478,7 +22480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -22495,7 +22497,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -22540,7 +22542,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -22557,7 +22559,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -22600,7 +22602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -22617,7 +22619,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -22654,7 +22656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -22671,7 +22673,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -22712,7 +22714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -22729,7 +22731,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -22772,7 +22774,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -22789,7 +22791,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -22831,7 +22833,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -22848,7 +22850,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -22893,7 +22895,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -22910,7 +22912,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -22955,7 +22957,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -22972,7 +22974,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23017,7 +23019,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23034,7 +23036,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23071,7 +23073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23088,7 +23090,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23105,7 +23107,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23122,7 +23124,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23143,7 +23145,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23160,7 +23162,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23201,7 +23203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23218,7 +23220,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23263,7 +23265,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -23280,7 +23282,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23297,7 +23299,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -23332,7 +23334,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -23715,7 +23717,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -23726,7 +23728,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -23747,7 +23749,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -23809,7 +23811,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -23867,7 +23869,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -23901,7 +23903,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -23920,7 +23922,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -23954,7 +23956,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -23973,7 +23975,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24007,7 +24009,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24026,7 +24028,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24064,7 +24066,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24083,7 +24085,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24121,7 +24123,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24140,7 +24142,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24178,7 +24180,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24197,7 +24199,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24230,7 +24232,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24249,7 +24251,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24282,7 +24284,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24301,7 +24303,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24332,7 +24334,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24351,7 +24353,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24386,7 +24388,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24405,7 +24407,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24438,7 +24440,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -24457,7 +24459,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24488,7 +24490,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -24507,7 +24509,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24539,7 +24541,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -24558,7 +24560,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24594,7 +24596,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -24613,7 +24615,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24642,7 +24644,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -24661,7 +24663,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24692,7 +24694,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -24711,7 +24713,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24744,7 +24746,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -24763,7 +24765,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24799,7 +24801,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -24818,7 +24820,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24853,7 +24855,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -24872,7 +24874,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24902,7 +24904,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -24921,7 +24923,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24961,7 +24963,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -24980,7 +24982,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25009,7 +25011,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25028,7 +25030,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25061,7 +25063,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25080,7 +25082,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25113,7 +25115,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25132,7 +25134,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25168,7 +25170,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25187,7 +25189,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25223,7 +25225,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25242,7 +25244,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25276,7 +25278,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25295,7 +25297,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25330,7 +25332,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25349,7 +25351,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25368,7 +25370,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25387,7 +25389,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25408,7 +25410,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25427,7 +25429,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -25460,7 +25462,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -25479,7 +25481,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -25518,7 +25520,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -25537,7 +25539,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -25556,7 +25558,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -25575,7 +25577,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -25620,7 +25622,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -25659,7 +25661,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -25688,7 +25690,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -25733,7 +25735,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -25778,7 +25780,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -25797,7 +25799,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -25844,7 +25846,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -25889,7 +25891,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -25908,7 +25910,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -25931,7 +25933,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -25954,7 +25956,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -25977,7 +25979,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -26000,7 +26002,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -26023,7 +26025,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -26046,7 +26048,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -26069,7 +26071,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -26092,7 +26094,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -26115,7 +26117,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -26138,7 +26140,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -26161,7 +26163,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -26184,7 +26186,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -26205,7 +26207,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26226,7 +26228,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26247,7 +26249,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26268,7 +26270,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26289,7 +26291,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26310,7 +26312,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26331,7 +26333,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -26354,7 +26356,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -26377,7 +26379,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -26400,7 +26402,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -26423,7 +26425,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -26446,7 +26448,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -26469,7 +26471,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -26492,7 +26494,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -26511,7 +26513,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -26530,7 +26532,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -26549,7 +26551,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -26568,7 +26570,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -26642,11 +26644,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -26678,7 +26679,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -26711,7 +26712,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -26744,7 +26745,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -26777,7 +26778,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -26810,7 +26811,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -26843,7 +26844,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -26876,7 +26877,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -26909,7 +26910,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -26940,7 +26941,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -26971,7 +26972,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -27004,7 +27005,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -27037,7 +27038,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -27070,7 +27071,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -27103,7 +27104,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -27136,7 +27137,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -27169,7 +27170,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -27202,7 +27203,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -27235,7 +27236,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -27268,7 +27269,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -27301,7 +27302,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -27334,7 +27335,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -27367,7 +27368,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -27400,7 +27401,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -27433,7 +27434,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -27466,7 +27467,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -27499,7 +27500,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -27531,7 +27532,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -27563,7 +27564,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -27595,7 +27596,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -27627,7 +27628,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -27659,7 +27660,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -27689,7 +27690,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -27719,7 +27720,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -27751,7 +27752,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -27783,7 +27784,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -27815,7 +27816,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -27847,7 +27848,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -27879,7 +27880,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -27909,7 +27910,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -27941,7 +27942,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -27973,7 +27974,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -28005,7 +28006,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -28037,7 +28038,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28067,7 +28068,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28097,7 +28098,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28127,7 +28128,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28157,7 +28158,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -28189,7 +28190,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -28221,7 +28222,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28251,7 +28252,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28281,7 +28282,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28311,7 +28312,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28341,7 +28342,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28371,7 +28372,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -28466,11 +28467,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -28502,7 +28502,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -28533,7 +28533,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -28564,7 +28564,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -28595,7 +28595,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -28626,7 +28626,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -28657,7 +28657,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -28688,7 +28688,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -28719,7 +28719,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -28750,7 +28750,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -28781,7 +28781,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -28812,7 +28812,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -28843,7 +28843,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -28874,7 +28874,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -28905,7 +28905,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -28936,7 +28936,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -28967,7 +28967,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -28998,7 +28998,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29029,7 +29029,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29060,7 +29060,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29091,7 +29091,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29121,7 +29121,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29151,7 +29151,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29181,7 +29181,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29211,7 +29211,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29241,7 +29241,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29271,7 +29271,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29301,7 +29301,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29331,7 +29331,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29361,7 +29361,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29391,7 +29391,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -29421,7 +29421,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -29451,7 +29451,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -29481,7 +29481,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -29511,7 +29511,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -29541,7 +29541,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -29571,7 +29571,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -29603,7 +29603,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -29635,7 +29635,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -29665,7 +29665,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -29695,7 +29695,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -29725,7 +29725,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -29755,7 +29755,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -29785,7 +29785,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -51528,19 +51528,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -51554,7 +51554,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -51566,7 +51566,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -51577,7 +51577,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -51588,7 +51588,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -51599,13 +51599,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T01:58:02Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1061" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="226">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6757,7 +6757,9 @@
       <c r="R32" s="13"/>
       <c r="S32" s="13"/>
       <c r="T32" s="16"/>
-      <c r="U32" s="1"/>
+      <c r="U32" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="V32" s="1"/>
       <c r="W32" s="1"/>
       <c r="X32" s="1"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T01:59:17Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1062" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="226">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -5974,18 +5974,30 @@
       <c r="K12" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="L12" s="13"/>
+      <c r="L12" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="M12" s="13" t="s">
         <v>27</v>
       </c>
       <c r="N12" s="14"/>
       <c r="O12" s="18"/>
-      <c r="P12" s="13"/>
-      <c r="Q12" s="15"/>
-      <c r="R12" s="13"/>
-      <c r="S12" s="13"/>
+      <c r="P12" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q12" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="R12" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="S12" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="T12" s="16"/>
-      <c r="U12" s="1"/>
+      <c r="U12" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="V12" s="1"/>
       <c r="W12" s="1"/>
       <c r="X12" s="1"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:08:09Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1070" uniqueCount="226">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -5798,8 +5798,12 @@
       </c>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="14"/>
+      <c r="F8" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>28</v>
+      </c>
       <c r="H8" s="13"/>
       <c r="I8" s="13"/>
       <c r="J8" s="13"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:10:47Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -6758,7 +6758,7 @@
         <v>28</v>
       </c>
       <c r="L32" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M32" s="13"/>
       <c r="N32" s="14"/>
@@ -21701,13 +21701,13 @@
         <v>0</v>
       </c>
       <c r="M12" s="52">
-        <v>-6483.239999999991</v>
+        <v>-6480.239999999991</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>-93.95999999999987</v>
+        <v>-93.9165217391303</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>117</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:11:31Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1071" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6760,8 +6760,12 @@
       <c r="L32" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="M32" s="13"/>
-      <c r="N32" s="14"/>
+      <c r="M32" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="N32" s="14" t="s">
+        <v>28</v>
+      </c>
       <c r="O32" s="13" t="s">
         <v>33</v>
       </c>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:12:40Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1073" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -5804,13 +5804,25 @@
       <c r="H8" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="I8" s="13"/>
-      <c r="J8" s="13"/>
+      <c r="I8" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="K8" s="13"/>
-      <c r="L8" s="13"/>
-      <c r="M8" s="13"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="13"/>
+      <c r="L8" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="M8" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="N8" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="O8" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="P8" s="13"/>
       <c r="Q8" s="15"/>
       <c r="R8" s="13"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:13:15Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1079" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -5824,9 +5824,15 @@
         <v>27</v>
       </c>
       <c r="P8" s="13"/>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="13"/>
-      <c r="S8" s="13"/>
+      <c r="Q8" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="R8" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="T8" s="16"/>
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:16:45Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1082" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -5834,7 +5834,9 @@
         <v>27</v>
       </c>
       <c r="T8" s="16"/>
-      <c r="U8" s="1"/>
+      <c r="U8" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="V8" s="1"/>
       <c r="W8" s="1"/>
       <c r="X8" s="1"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:17:43Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -7977,10 +7977,18 @@
       <c r="C64" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="D64" s="29"/>
-      <c r="E64" s="13"/>
-      <c r="F64" s="13"/>
-      <c r="G64" s="14"/>
+      <c r="D64" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="E64" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F64" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G64" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="H64" s="13"/>
       <c r="I64" s="13"/>
       <c r="J64" s="13"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:18:40Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -7990,9 +7990,15 @@
         <v>27</v>
       </c>
       <c r="H64" s="13"/>
-      <c r="I64" s="13"/>
-      <c r="J64" s="13"/>
-      <c r="K64" s="13"/>
+      <c r="I64" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="J64" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="K64" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="L64" s="13"/>
       <c r="M64" s="13"/>
       <c r="N64" s="14"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:22:22Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1090" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -8001,7 +8001,9 @@
       </c>
       <c r="L64" s="13"/>
       <c r="M64" s="13"/>
-      <c r="N64" s="14"/>
+      <c r="N64" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="O64" s="13"/>
       <c r="P64" s="18"/>
       <c r="Q64" s="15"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:23:05Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1091" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -8006,7 +8006,9 @@
       </c>
       <c r="O64" s="13"/>
       <c r="P64" s="18"/>
-      <c r="Q64" s="15"/>
+      <c r="Q64" s="15" t="s">
+        <v>27</v>
+      </c>
       <c r="R64" s="13"/>
       <c r="S64" s="13"/>
       <c r="T64" s="16"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:29:54Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1092" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1094" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -7989,7 +7989,9 @@
       <c r="G64" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="H64" s="13"/>
+      <c r="H64" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="I64" s="13" t="s">
         <v>27</v>
       </c>
@@ -7999,7 +8001,9 @@
       <c r="K64" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="L64" s="13"/>
+      <c r="L64" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="M64" s="13"/>
       <c r="N64" s="14" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:30:28Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1094" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -8014,7 +8014,9 @@
         <v>27</v>
       </c>
       <c r="R64" s="13"/>
-      <c r="S64" s="13"/>
+      <c r="S64" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="T64" s="16"/>
       <c r="U64" s="1"/>
       <c r="V64" s="1"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:31:40Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16244,7 +16244,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -21354,7 +21354,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:AD70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21368,7 +21368,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21390,7 +21390,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -21438,7 +21438,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21456,7 +21456,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21503,7 +21503,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21520,7 +21520,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -21570,7 +21570,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -21587,7 +21587,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -21630,7 +21630,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -21647,7 +21647,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -21694,7 +21694,7 @@
         <v>18.141660543717848</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -21711,7 +21711,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -21761,7 +21761,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -21778,7 +21778,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -21825,7 +21825,7 @@
         <v>62.640446428571394</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -21842,7 +21842,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -21887,7 +21887,7 @@
         <v>34.302939481268</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -21904,7 +21904,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -21954,7 +21954,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -21971,7 +21971,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -22010,7 +22010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -22027,7 +22027,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -22068,7 +22068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22085,7 +22085,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22122,7 +22122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22139,7 +22139,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22184,7 +22184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22201,7 +22201,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22244,7 +22244,7 @@
         <v>-7.109225589225597</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22261,7 +22261,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22304,7 +22304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22321,7 +22321,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22368,7 +22368,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22385,7 +22385,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22430,7 +22430,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22447,7 +22447,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22490,7 +22490,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22507,7 +22507,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22548,7 +22548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -22565,7 +22565,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -22610,7 +22610,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -22627,7 +22627,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -22670,7 +22670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -22687,7 +22687,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -22724,7 +22724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -22741,7 +22741,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -22782,7 +22782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -22799,7 +22799,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -22842,7 +22842,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -22859,7 +22859,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -22901,7 +22901,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -22918,7 +22918,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -22963,7 +22963,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -22980,7 +22980,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -23025,7 +23025,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -23042,7 +23042,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23087,7 +23087,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23104,7 +23104,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23141,7 +23141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23158,7 +23158,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23175,7 +23175,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23192,7 +23192,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23213,7 +23213,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23230,7 +23230,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23271,7 +23271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23288,7 +23288,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23333,7 +23333,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -23350,7 +23350,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23367,7 +23367,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -23402,7 +23402,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -23785,7 +23785,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB109"/>
+  <dimension ref="A1:AD109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -23796,7 +23796,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -23817,7 +23817,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -23879,7 +23879,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -23937,7 +23937,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -23971,7 +23971,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -23990,7 +23990,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -24024,7 +24024,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -24043,7 +24043,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24077,7 +24077,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24096,7 +24096,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24134,7 +24134,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24153,7 +24153,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24191,7 +24191,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24210,7 +24210,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24248,7 +24248,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24267,7 +24267,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24300,7 +24300,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24319,7 +24319,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24352,7 +24352,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24371,7 +24371,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24402,7 +24402,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24421,7 +24421,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24456,7 +24456,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24475,7 +24475,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24508,7 +24508,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -24527,7 +24527,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24558,7 +24558,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -24577,7 +24577,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24609,7 +24609,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -24628,7 +24628,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24664,7 +24664,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -24683,7 +24683,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24712,7 +24712,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -24731,7 +24731,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24762,7 +24762,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -24781,7 +24781,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24814,7 +24814,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -24833,7 +24833,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24869,7 +24869,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -24888,7 +24888,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24923,7 +24923,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -24942,7 +24942,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24972,7 +24972,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -24991,7 +24991,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25031,7 +25031,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -25050,7 +25050,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25079,7 +25079,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25098,7 +25098,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25131,7 +25131,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25150,7 +25150,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25183,7 +25183,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25202,7 +25202,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25238,7 +25238,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25257,7 +25257,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25293,7 +25293,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25312,7 +25312,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25346,7 +25346,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25365,7 +25365,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25400,7 +25400,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25419,7 +25419,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25438,7 +25438,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25457,7 +25457,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25478,7 +25478,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25497,7 +25497,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -25530,7 +25530,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -25549,7 +25549,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -25588,7 +25588,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -25607,7 +25607,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -25626,7 +25626,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -25645,7 +25645,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -25690,7 +25690,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -25729,7 +25729,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -25758,7 +25758,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -25803,7 +25803,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -25848,7 +25848,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -25867,7 +25867,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -25914,7 +25914,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -25959,7 +25959,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -25978,7 +25978,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -26001,7 +26001,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -26024,7 +26024,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -26047,7 +26047,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -26070,7 +26070,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -26093,7 +26093,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -26116,7 +26116,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -26139,7 +26139,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -26162,7 +26162,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -26185,7 +26185,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -26208,7 +26208,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -26231,7 +26231,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -26254,7 +26254,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -26275,7 +26275,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26296,7 +26296,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26317,7 +26317,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26338,7 +26338,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26359,7 +26359,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26380,7 +26380,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26401,7 +26401,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -26424,7 +26424,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -26447,7 +26447,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -26470,7 +26470,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -26493,7 +26493,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -26516,7 +26516,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -26539,7 +26539,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -26562,7 +26562,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -26581,7 +26581,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -26600,7 +26600,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -26619,7 +26619,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -26638,7 +26638,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -26712,10 +26712,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -26747,7 +26748,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -26780,7 +26781,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -26813,7 +26814,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -26846,7 +26847,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -26879,7 +26880,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -26912,7 +26913,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -26945,7 +26946,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -26978,7 +26979,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -27009,7 +27010,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -27040,7 +27041,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -27073,7 +27074,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -27106,7 +27107,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -27139,7 +27140,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -27172,7 +27173,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -27205,7 +27206,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -27238,7 +27239,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -27271,7 +27272,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -27304,7 +27305,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -27337,7 +27338,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -27370,7 +27371,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -27403,7 +27404,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -27436,7 +27437,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -27469,7 +27470,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -27502,7 +27503,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -27535,7 +27536,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -27568,7 +27569,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -27600,7 +27601,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -27632,7 +27633,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -27664,7 +27665,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -27696,7 +27697,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -27728,7 +27729,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -27758,7 +27759,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -27788,7 +27789,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -27820,7 +27821,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -27852,7 +27853,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -27884,7 +27885,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -27916,7 +27917,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -27948,7 +27949,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -27978,7 +27979,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -28010,7 +28011,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -28042,7 +28043,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -28074,7 +28075,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -28106,7 +28107,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28136,7 +28137,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28166,7 +28167,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28196,7 +28197,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28226,7 +28227,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -28258,7 +28259,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -28290,7 +28291,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28320,7 +28321,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28350,7 +28351,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28380,7 +28381,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28410,7 +28411,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28440,7 +28441,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -28535,10 +28536,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -28570,7 +28572,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -28601,7 +28603,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -28632,7 +28634,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -28663,7 +28665,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -28694,7 +28696,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -28725,7 +28727,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -28756,7 +28758,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -28787,7 +28789,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -28818,7 +28820,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -28849,7 +28851,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -28880,7 +28882,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -28911,7 +28913,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -28942,7 +28944,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -28973,7 +28975,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -29004,7 +29006,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -29035,7 +29037,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -29066,7 +29068,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29097,7 +29099,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29128,7 +29130,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29159,7 +29161,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29189,7 +29191,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29219,7 +29221,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29249,7 +29251,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29279,7 +29281,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29309,7 +29311,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29339,7 +29341,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29369,7 +29371,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29399,7 +29401,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29429,7 +29431,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29459,7 +29461,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -29489,7 +29491,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -29519,7 +29521,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -29549,7 +29551,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -29579,7 +29581,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -29609,7 +29611,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -29639,7 +29641,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -29671,7 +29673,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -29703,7 +29705,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -29733,7 +29735,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -29763,7 +29765,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -29793,7 +29795,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -29823,7 +29825,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -29853,7 +29855,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -51596,19 +51598,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -51622,7 +51624,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -51634,7 +51636,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -51645,7 +51647,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -51656,7 +51658,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -51667,13 +51669,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:32:46Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16244,7 +16244,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -21354,7 +21354,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD70"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21368,7 +21368,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21390,7 +21390,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -21438,7 +21438,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21456,7 +21456,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21503,7 +21503,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21520,7 +21520,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -21570,7 +21570,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -21587,7 +21587,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -21630,7 +21630,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -21647,7 +21647,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -21694,7 +21694,7 @@
         <v>18.141660543717848</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -21711,7 +21711,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -21761,7 +21761,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -21778,7 +21778,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -21825,7 +21825,7 @@
         <v>62.640446428571394</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -21842,7 +21842,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -21887,7 +21887,7 @@
         <v>34.302939481268</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -21904,7 +21904,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -21954,7 +21954,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -21971,7 +21971,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -22010,7 +22010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -22027,7 +22027,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -22068,7 +22068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22085,7 +22085,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22122,7 +22122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22139,7 +22139,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22184,7 +22184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22201,7 +22201,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22244,7 +22244,7 @@
         <v>-7.109225589225597</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22261,7 +22261,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22304,7 +22304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22321,7 +22321,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22368,7 +22368,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22385,7 +22385,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22430,7 +22430,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22447,7 +22447,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22490,7 +22490,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22507,7 +22507,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22548,7 +22548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -22565,7 +22565,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -22610,7 +22610,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -22627,7 +22627,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -22670,7 +22670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -22687,7 +22687,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -22724,7 +22724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -22741,7 +22741,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -22782,7 +22782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -22799,7 +22799,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -22842,7 +22842,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -22859,7 +22859,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -22901,7 +22901,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -22918,7 +22918,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -22963,7 +22963,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -22980,7 +22980,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -23025,7 +23025,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -23042,7 +23042,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23087,7 +23087,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23104,7 +23104,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23141,7 +23141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23158,7 +23158,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23175,7 +23175,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23192,7 +23192,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23213,7 +23213,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23230,7 +23230,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23271,7 +23271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23288,7 +23288,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23333,7 +23333,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -23350,7 +23350,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23367,7 +23367,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -23402,7 +23402,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -23785,7 +23785,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -23796,7 +23796,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -23817,7 +23817,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -23879,7 +23879,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -23937,7 +23937,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -23971,7 +23971,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -23990,7 +23990,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -24024,7 +24024,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -24043,7 +24043,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24077,7 +24077,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24096,7 +24096,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24134,7 +24134,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24153,7 +24153,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24191,7 +24191,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24210,7 +24210,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24248,7 +24248,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24267,7 +24267,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24300,7 +24300,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24319,7 +24319,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24352,7 +24352,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24371,7 +24371,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24402,7 +24402,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24421,7 +24421,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24456,7 +24456,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24475,7 +24475,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24508,7 +24508,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -24527,7 +24527,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24558,7 +24558,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -24577,7 +24577,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24609,7 +24609,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -24628,7 +24628,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24664,7 +24664,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -24683,7 +24683,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24712,7 +24712,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -24731,7 +24731,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24762,7 +24762,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -24781,7 +24781,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24814,7 +24814,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -24833,7 +24833,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24869,7 +24869,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -24888,7 +24888,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24923,7 +24923,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -24942,7 +24942,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24972,7 +24972,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -24991,7 +24991,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25031,7 +25031,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -25050,7 +25050,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25079,7 +25079,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25098,7 +25098,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25131,7 +25131,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25150,7 +25150,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25183,7 +25183,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25202,7 +25202,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25238,7 +25238,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25257,7 +25257,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25293,7 +25293,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25312,7 +25312,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25346,7 +25346,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25365,7 +25365,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25400,7 +25400,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25419,7 +25419,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25438,7 +25438,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25457,7 +25457,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25478,7 +25478,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25497,7 +25497,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -25530,7 +25530,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -25549,7 +25549,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -25588,7 +25588,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -25607,7 +25607,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -25626,7 +25626,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -25645,7 +25645,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -25690,7 +25690,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -25729,7 +25729,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -25758,7 +25758,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -25803,7 +25803,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -25848,7 +25848,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -25867,7 +25867,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -25914,7 +25914,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -25959,7 +25959,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -25978,7 +25978,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -26001,7 +26001,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -26024,7 +26024,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -26047,7 +26047,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -26070,7 +26070,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -26093,7 +26093,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -26116,7 +26116,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -26139,7 +26139,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -26162,7 +26162,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -26185,7 +26185,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -26208,7 +26208,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -26231,7 +26231,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -26254,7 +26254,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -26275,7 +26275,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26296,7 +26296,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26317,7 +26317,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26338,7 +26338,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26359,7 +26359,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26380,7 +26380,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26401,7 +26401,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -26424,7 +26424,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -26447,7 +26447,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -26470,7 +26470,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -26493,7 +26493,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -26516,7 +26516,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -26539,7 +26539,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -26562,7 +26562,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -26581,7 +26581,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -26600,7 +26600,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -26619,7 +26619,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -26638,7 +26638,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -26712,11 +26712,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -26748,7 +26747,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -26781,7 +26780,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -26814,7 +26813,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -26847,7 +26846,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -26880,7 +26879,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -26913,7 +26912,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -26946,7 +26945,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -26979,7 +26978,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -27010,7 +27009,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -27041,7 +27040,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -27074,7 +27073,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -27107,7 +27106,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -27140,7 +27139,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -27173,7 +27172,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -27206,7 +27205,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -27239,7 +27238,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -27272,7 +27271,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -27305,7 +27304,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -27338,7 +27337,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -27371,7 +27370,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -27404,7 +27403,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -27437,7 +27436,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -27470,7 +27469,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -27503,7 +27502,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -27536,7 +27535,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -27569,7 +27568,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -27601,7 +27600,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -27633,7 +27632,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -27665,7 +27664,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -27697,7 +27696,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -27729,7 +27728,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -27759,7 +27758,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -27789,7 +27788,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -27821,7 +27820,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -27853,7 +27852,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -27885,7 +27884,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -27917,7 +27916,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -27949,7 +27948,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -27979,7 +27978,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -28011,7 +28010,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -28043,7 +28042,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -28075,7 +28074,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -28107,7 +28106,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28137,7 +28136,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28167,7 +28166,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28197,7 +28196,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28227,7 +28226,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -28259,7 +28258,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -28291,7 +28290,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28321,7 +28320,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28351,7 +28350,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28381,7 +28380,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28411,7 +28410,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28441,7 +28440,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -28536,11 +28535,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -28572,7 +28570,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -28603,7 +28601,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -28634,7 +28632,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -28665,7 +28663,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -28696,7 +28694,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -28727,7 +28725,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -28758,7 +28756,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -28789,7 +28787,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -28820,7 +28818,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -28851,7 +28849,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -28882,7 +28880,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -28913,7 +28911,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -28944,7 +28942,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -28975,7 +28973,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -29006,7 +29004,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -29037,7 +29035,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -29068,7 +29066,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29099,7 +29097,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29130,7 +29128,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29161,7 +29159,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29191,7 +29189,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29221,7 +29219,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29251,7 +29249,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29281,7 +29279,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29311,7 +29309,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29341,7 +29339,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29371,7 +29369,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29401,7 +29399,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29431,7 +29429,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29461,7 +29459,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -29491,7 +29489,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -29521,7 +29519,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -29551,7 +29549,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -29581,7 +29579,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -29611,7 +29609,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -29641,7 +29639,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -29673,7 +29671,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -29705,7 +29703,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -29735,7 +29733,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -29765,7 +29763,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -29795,7 +29793,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -29825,7 +29823,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -29855,7 +29853,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -51598,19 +51596,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -51624,7 +51622,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -51636,7 +51634,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -51647,7 +51645,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -51658,7 +51656,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -51669,13 +51667,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:33:56Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1097" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -8013,12 +8013,16 @@
       <c r="Q64" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="R64" s="13"/>
+      <c r="R64" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="S64" s="13" t="s">
         <v>27</v>
       </c>
       <c r="T64" s="16"/>
-      <c r="U64" s="1"/>
+      <c r="U64" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="V64" s="1"/>
       <c r="W64" s="1"/>
       <c r="X64" s="1"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:36:07Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1097" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6381,9 +6381,13 @@
       <c r="C22" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="13"/>
+      <c r="D22" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="E22" s="13"/>
-      <c r="F22" s="13"/>
+      <c r="F22" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="G22" s="14"/>
       <c r="H22" s="13"/>
       <c r="I22" s="13"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:36:42Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1099" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6388,11 +6388,21 @@
       <c r="F22" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="G22" s="14"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="13"/>
-      <c r="J22" s="13"/>
-      <c r="K22" s="13"/>
+      <c r="G22" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H22" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="I22" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="J22" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="K22" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="L22" s="13"/>
       <c r="M22" s="13"/>
       <c r="N22" s="14"/>
@@ -22052,7 +22062,7 @@
         <v>-565.6499999999996</v>
       </c>
       <c r="F22" s="52">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G22" s="53">
         <v>0</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:37:19Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6403,7 +6403,9 @@
       <c r="K22" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="L22" s="13"/>
+      <c r="L22" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="M22" s="13"/>
       <c r="N22" s="14"/>
       <c r="O22" s="13"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:39:42Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6406,13 +6406,23 @@
       <c r="L22" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="M22" s="13"/>
-      <c r="N22" s="14"/>
+      <c r="M22" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="N22" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="O22" s="13"/>
       <c r="P22" s="13"/>
-      <c r="Q22" s="15"/>
-      <c r="R22" s="13"/>
-      <c r="S22" s="13"/>
+      <c r="Q22" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="R22" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="S22" s="13" t="s">
+        <v>28</v>
+      </c>
       <c r="T22" s="16"/>
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:42:00Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6424,7 +6424,9 @@
         <v>28</v>
       </c>
       <c r="T22" s="16"/>
-      <c r="U22" s="1"/>
+      <c r="U22" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="V22" s="1"/>
       <c r="W22" s="1"/>
       <c r="X22" s="1"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:42:42Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6479,7 +6479,9 @@
       <c r="C24" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="D24" s="13"/>
+      <c r="D24" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="E24" s="13"/>
       <c r="F24" s="13"/>
       <c r="G24" s="14"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:43:37Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1112" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6483,10 +6483,18 @@
         <v>27</v>
       </c>
       <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="13"/>
+      <c r="F24" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G24" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="H24" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="I24" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="J24" s="13"/>
       <c r="K24" s="13"/>
       <c r="L24" s="13"/>
@@ -22135,7 +22143,9 @@
       <c r="E24" s="52">
         <v>-1528.260000000002</v>
       </c>
-      <c r="F24" s="52"/>
+      <c r="F24" s="52">
+        <v>3</v>
+      </c>
       <c r="G24" s="53">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:44:21Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1116" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1119" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6495,9 +6495,15 @@
       <c r="I24" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="J24" s="13"/>
-      <c r="K24" s="13"/>
-      <c r="L24" s="13"/>
+      <c r="J24" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="K24" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="L24" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="M24" s="13"/>
       <c r="N24" s="14"/>
       <c r="O24" s="13"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:45:17Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1119" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6504,7 +6504,9 @@
       <c r="L24" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="M24" s="13"/>
+      <c r="M24" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="13"/>
       <c r="P24" s="13"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:46:38Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1120" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6507,11 +6507,21 @@
       <c r="M24" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="N24" s="14"/>
-      <c r="O24" s="13"/>
-      <c r="P24" s="13"/>
-      <c r="Q24" s="15"/>
-      <c r="R24" s="13"/>
+      <c r="N24" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="O24" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="P24" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q24" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="R24" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="S24" s="13"/>
       <c r="T24" s="16"/>
       <c r="U24" s="1"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:47:04Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1125" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1126" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6522,7 +6522,9 @@
       <c r="R24" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="S24" s="13"/>
+      <c r="S24" s="13" t="s">
+        <v>28</v>
+      </c>
       <c r="T24" s="16"/>
       <c r="U24" s="1"/>
       <c r="V24" s="1"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T02:49:50Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1126" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1127" uniqueCount="225">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6526,7 +6526,9 @@
         <v>28</v>
       </c>
       <c r="T24" s="16"/>
-      <c r="U24" s="1"/>
+      <c r="U24" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="V24" s="1"/>
       <c r="W24" s="1"/>
       <c r="X24" s="1"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-03T03:50:30Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16308,7 +16308,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -21418,7 +21418,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R70"/>
+  <dimension ref="A1:AD70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21432,7 +21432,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21454,7 +21454,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -21502,7 +21502,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21520,7 +21520,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21567,7 +21567,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21584,7 +21584,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -21634,7 +21634,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -21651,7 +21651,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -21694,7 +21694,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -21711,7 +21711,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -21758,7 +21758,7 @@
         <v>18.141660543717848</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -21775,7 +21775,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -21825,7 +21825,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -21842,7 +21842,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -21889,7 +21889,7 @@
         <v>62.640446428571394</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -21906,7 +21906,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -21951,7 +21951,7 @@
         <v>34.302939481268</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -21968,7 +21968,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -22018,7 +22018,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -22035,7 +22035,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -22074,7 +22074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -22091,7 +22091,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -22125,14 +22125,14 @@
         <v>0</v>
       </c>
       <c r="M22" s="52">
-        <v>-565.6499999999996</v>
+        <v>-562.6499999999996</v>
       </c>
       <c r="N22" s="54"/>
       <c r="O22" s="58">
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22149,7 +22149,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22181,14 +22181,14 @@
         <v>0</v>
       </c>
       <c r="M24" s="52">
-        <v>-1528.260000000002</v>
+        <v>-1525.260000000002</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22205,7 +22205,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22250,7 +22250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22267,7 +22267,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22310,7 +22310,7 @@
         <v>-7.109225589225597</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22327,7 +22327,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22370,7 +22370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22387,7 +22387,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22434,7 +22434,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22451,7 +22451,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22496,7 +22496,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22513,7 +22513,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22556,7 +22556,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22573,7 +22573,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22614,7 +22614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -22631,7 +22631,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -22676,7 +22676,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -22693,7 +22693,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -22736,7 +22736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -22753,7 +22753,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -22790,7 +22790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -22807,7 +22807,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -22848,7 +22848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -22865,7 +22865,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -22908,7 +22908,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -22925,7 +22925,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -22967,7 +22967,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -22984,7 +22984,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -23029,7 +23029,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -23046,7 +23046,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -23091,7 +23091,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -23108,7 +23108,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23153,7 +23153,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23170,7 +23170,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23207,7 +23207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23224,7 +23224,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23241,7 +23241,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23258,7 +23258,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23279,7 +23279,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23296,7 +23296,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23337,7 +23337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23354,7 +23354,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23399,7 +23399,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -23416,7 +23416,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23433,7 +23433,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -23468,7 +23468,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -23851,7 +23851,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB109"/>
+  <dimension ref="A1:AD109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -23862,7 +23862,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -23883,7 +23883,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -23945,7 +23945,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -24003,7 +24003,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -24037,7 +24037,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -24056,7 +24056,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -24090,7 +24090,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -24109,7 +24109,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24143,7 +24143,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24162,7 +24162,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24200,7 +24200,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24219,7 +24219,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24257,7 +24257,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24276,7 +24276,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24314,7 +24314,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24333,7 +24333,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24366,7 +24366,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24385,7 +24385,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24418,7 +24418,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24437,7 +24437,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24468,7 +24468,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24487,7 +24487,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24522,7 +24522,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24541,7 +24541,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24574,7 +24574,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -24593,7 +24593,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24624,7 +24624,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -24643,7 +24643,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24675,7 +24675,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -24694,7 +24694,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24730,7 +24730,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -24749,7 +24749,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24778,7 +24778,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -24797,7 +24797,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24828,7 +24828,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -24847,7 +24847,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24880,7 +24880,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -24899,7 +24899,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24935,7 +24935,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -24954,7 +24954,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24989,7 +24989,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -25008,7 +25008,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25038,7 +25038,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -25057,7 +25057,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25097,7 +25097,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -25116,7 +25116,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25145,7 +25145,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25164,7 +25164,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25197,7 +25197,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25216,7 +25216,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25249,7 +25249,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25268,7 +25268,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25304,7 +25304,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25323,7 +25323,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25359,7 +25359,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25378,7 +25378,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25412,7 +25412,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25431,7 +25431,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25466,7 +25466,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25485,7 +25485,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25504,7 +25504,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25523,7 +25523,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25544,7 +25544,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25563,7 +25563,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -25596,7 +25596,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -25615,7 +25615,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -25654,7 +25654,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -25673,7 +25673,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -25692,7 +25692,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -25711,7 +25711,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -25756,7 +25756,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -25795,7 +25795,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -25824,7 +25824,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -25869,7 +25869,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -25914,7 +25914,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -25933,7 +25933,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -25980,7 +25980,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -26025,7 +26025,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -26044,7 +26044,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -26067,7 +26067,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -26090,7 +26090,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -26113,7 +26113,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -26136,7 +26136,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -26159,7 +26159,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -26182,7 +26182,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -26205,7 +26205,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -26228,7 +26228,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -26251,7 +26251,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -26274,7 +26274,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -26297,7 +26297,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -26320,7 +26320,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -26341,7 +26341,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26362,7 +26362,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26383,7 +26383,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26404,7 +26404,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26425,7 +26425,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26446,7 +26446,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26467,7 +26467,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -26490,7 +26490,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -26513,7 +26513,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -26536,7 +26536,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -26559,7 +26559,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -26582,7 +26582,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -26605,7 +26605,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -26628,7 +26628,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -26647,7 +26647,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -26666,7 +26666,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -26685,7 +26685,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -26704,7 +26704,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -26778,10 +26778,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -26813,7 +26814,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -26846,7 +26847,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -26879,7 +26880,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -26912,7 +26913,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -26945,7 +26946,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -26978,7 +26979,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -27011,7 +27012,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -27044,7 +27045,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -27075,7 +27076,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -27106,7 +27107,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -27139,7 +27140,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -27172,7 +27173,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -27205,7 +27206,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -27238,7 +27239,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -27271,7 +27272,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -27304,7 +27305,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -27337,7 +27338,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -27370,7 +27371,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -27403,7 +27404,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -27436,7 +27437,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -27469,7 +27470,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -27502,7 +27503,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -27535,7 +27536,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -27568,7 +27569,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -27601,7 +27602,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -27634,7 +27635,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -27666,7 +27667,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -27698,7 +27699,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -27730,7 +27731,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -27762,7 +27763,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -27794,7 +27795,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -27824,7 +27825,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -27854,7 +27855,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -27886,7 +27887,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -27918,7 +27919,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -27950,7 +27951,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -27982,7 +27983,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -28014,7 +28015,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -28044,7 +28045,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -28076,7 +28077,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -28108,7 +28109,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -28140,7 +28141,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -28172,7 +28173,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28202,7 +28203,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28232,7 +28233,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28262,7 +28263,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28292,7 +28293,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -28324,7 +28325,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -28356,7 +28357,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28386,7 +28387,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28416,7 +28417,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28446,7 +28447,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28476,7 +28477,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28506,7 +28507,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -28601,10 +28602,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -28636,7 +28638,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -28667,7 +28669,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -28698,7 +28700,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -28729,7 +28731,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -28760,7 +28762,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -28791,7 +28793,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -28822,7 +28824,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -28853,7 +28855,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -28884,7 +28886,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -28915,7 +28917,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -28946,7 +28948,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -28977,7 +28979,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -29008,7 +29010,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -29039,7 +29041,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -29070,7 +29072,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -29101,7 +29103,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -29132,7 +29134,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29163,7 +29165,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29194,7 +29196,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29225,7 +29227,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29255,7 +29257,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29285,7 +29287,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29315,7 +29317,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29345,7 +29347,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29375,7 +29377,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29405,7 +29407,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29435,7 +29437,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29465,7 +29467,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29495,7 +29497,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29525,7 +29527,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -29555,7 +29557,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -29585,7 +29587,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -29615,7 +29617,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -29645,7 +29647,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -29675,7 +29677,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -29705,7 +29707,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -29737,7 +29739,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -29769,7 +29771,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -29799,7 +29801,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -29829,7 +29831,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -29859,7 +29861,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -29889,7 +29891,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -29919,7 +29921,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -51662,19 +51664,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -51688,7 +51690,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -51700,7 +51702,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -51711,7 +51713,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -51722,7 +51724,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -51733,13 +51735,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-06T22:09:36Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16308,7 +16308,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>95</v>
@@ -21418,7 +21418,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD70"/>
+  <dimension ref="A1:R70"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21432,7 +21432,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21454,7 +21454,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>100</v>
       </c>
@@ -21502,7 +21502,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21520,7 +21520,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21567,7 +21567,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21584,7 +21584,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -21634,7 +21634,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -21651,7 +21651,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -21694,7 +21694,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -21711,7 +21711,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -21758,7 +21758,7 @@
         <v>18.141660543717848</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -21775,7 +21775,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -21825,7 +21825,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -21842,7 +21842,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -21889,7 +21889,7 @@
         <v>62.640446428571394</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -21906,7 +21906,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -21951,7 +21951,7 @@
         <v>34.302939481268</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -21968,7 +21968,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -22018,7 +22018,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -22035,7 +22035,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -22074,7 +22074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -22091,7 +22091,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -22132,7 +22132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22149,7 +22149,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22188,7 +22188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22205,7 +22205,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22250,7 +22250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22267,7 +22267,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22310,7 +22310,7 @@
         <v>-7.109225589225597</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22327,7 +22327,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22370,7 +22370,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22387,7 +22387,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22434,7 +22434,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22451,7 +22451,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22496,7 +22496,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22513,7 +22513,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22556,7 +22556,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22573,7 +22573,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22614,7 +22614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -22631,7 +22631,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -22676,7 +22676,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -22693,7 +22693,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -22736,7 +22736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -22753,7 +22753,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -22790,7 +22790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -22807,7 +22807,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -22848,7 +22848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -22865,7 +22865,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -22908,7 +22908,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -22925,7 +22925,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -22967,7 +22967,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -22984,7 +22984,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -23029,7 +23029,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -23046,7 +23046,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -23091,7 +23091,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -23108,7 +23108,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23153,7 +23153,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23170,7 +23170,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23207,7 +23207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23224,7 +23224,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23241,7 +23241,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23258,7 +23258,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23279,7 +23279,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23296,7 +23296,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23337,7 +23337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23354,7 +23354,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23399,7 +23399,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="35"/>
       <c r="B67" s="35"/>
       <c r="C67" s="36"/>
@@ -23416,7 +23416,7 @@
       <c r="N67" s="35"/>
       <c r="O67" s="36"/>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23433,7 +23433,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="35"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="49" t="s">
         <v>120</v>
       </c>
@@ -23468,7 +23468,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="59"/>
       <c r="B70" s="98" t="s">
         <v>124</v>
@@ -23851,7 +23851,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD109"/>
+  <dimension ref="A1:AB109"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -23862,7 +23862,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -23883,7 +23883,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>125</v>
@@ -23945,7 +23945,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>141</v>
       </c>
@@ -24003,7 +24003,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -24037,7 +24037,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -24056,7 +24056,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -24090,7 +24090,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -24109,7 +24109,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24143,7 +24143,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24162,7 +24162,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24200,7 +24200,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24219,7 +24219,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24257,7 +24257,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24276,7 +24276,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24314,7 +24314,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24333,7 +24333,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24366,7 +24366,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24385,7 +24385,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24418,7 +24418,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24437,7 +24437,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24468,7 +24468,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24487,7 +24487,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24522,7 +24522,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24541,7 +24541,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24574,7 +24574,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -24593,7 +24593,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24624,7 +24624,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -24643,7 +24643,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24675,7 +24675,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -24694,7 +24694,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24730,7 +24730,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -24749,7 +24749,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24778,7 +24778,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -24797,7 +24797,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24828,7 +24828,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -24847,7 +24847,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24880,7 +24880,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -24899,7 +24899,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24935,7 +24935,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -24954,7 +24954,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24989,7 +24989,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -25008,7 +25008,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25038,7 +25038,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -25057,7 +25057,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25097,7 +25097,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -25116,7 +25116,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25145,7 +25145,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25164,7 +25164,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25197,7 +25197,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25216,7 +25216,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25249,7 +25249,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25268,7 +25268,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25304,7 +25304,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25323,7 +25323,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25359,7 +25359,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25378,7 +25378,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25412,7 +25412,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25431,7 +25431,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25466,7 +25466,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25485,7 +25485,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25504,7 +25504,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25523,7 +25523,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25544,7 +25544,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25563,7 +25563,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -25596,7 +25596,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -25615,7 +25615,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -25654,7 +25654,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="142"/>
       <c r="B67" s="143"/>
       <c r="C67" s="35"/>
@@ -25673,7 +25673,7 @@
       <c r="P67" s="35"/>
       <c r="Q67" s="144"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -25692,7 +25692,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="145"/>
       <c r="B69" s="145"/>
       <c r="C69" s="145"/>
@@ -25711,7 +25711,7 @@
       <c r="P69" s="145"/>
       <c r="Q69" s="145"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="142"/>
       <c r="B70" s="146" t="s">
         <v>145</v>
@@ -25756,7 +25756,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="77" t="s">
         <v>146</v>
@@ -25795,7 +25795,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>147</v>
@@ -25824,7 +25824,7 @@
       <c r="P72" s="20"/>
       <c r="Q72" s="20"/>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="148" t="s">
         <v>148</v>
@@ -25869,7 +25869,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="151" t="s">
         <v>149</v>
@@ -25914,7 +25914,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="35"/>
       <c r="C75" s="35"/>
@@ -25933,7 +25933,7 @@
       <c r="P75" s="35"/>
       <c r="Q75" s="144"/>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="156" t="s">
         <v>150</v>
@@ -25980,7 +25980,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="161"/>
       <c r="B77" s="162" t="s">
         <v>152</v>
@@ -26025,7 +26025,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="35"/>
       <c r="B78" s="35"/>
       <c r="C78" s="35"/>
@@ -26044,7 +26044,7 @@
       <c r="P78" s="35"/>
       <c r="Q78" s="35"/>
     </row>
-    <row r="79" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="164" t="s">
         <v>153</v>
@@ -26067,7 +26067,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="167" t="s">
         <v>155</v>
@@ -26090,7 +26090,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="19" t="s">
         <v>156</v>
@@ -26113,7 +26113,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>157</v>
@@ -26136,7 +26136,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>158</v>
@@ -26159,7 +26159,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>159</v>
@@ -26182,7 +26182,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>160</v>
@@ -26205,7 +26205,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>161</v>
@@ -26228,7 +26228,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>162</v>
@@ -26251,7 +26251,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>163</v>
@@ -26274,7 +26274,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>164</v>
@@ -26297,7 +26297,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>165</v>
@@ -26320,7 +26320,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19"/>
       <c r="C91" s="131">
@@ -26341,7 +26341,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26362,7 +26362,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26383,7 +26383,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26404,7 +26404,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26425,7 +26425,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26446,7 +26446,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26467,7 +26467,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19" t="s">
         <v>166</v>
@@ -26490,7 +26490,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>167</v>
@@ -26513,7 +26513,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>168</v>
@@ -26536,7 +26536,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>169</v>
@@ -26559,7 +26559,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>170</v>
@@ -26582,7 +26582,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>171</v>
@@ -26605,7 +26605,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>172</v>
@@ -26628,7 +26628,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19"/>
       <c r="C105" s="131"/>
@@ -26647,7 +26647,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -26666,7 +26666,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -26685,7 +26685,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="169"/>
       <c r="C108" s="150"/>
@@ -26704,7 +26704,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="164" t="s">
         <v>173</v>
@@ -26778,11 +26778,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>174</v>
       </c>
@@ -26814,7 +26813,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>175</v>
       </c>
@@ -26847,7 +26846,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>176</v>
       </c>
@@ -26880,7 +26879,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>177</v>
       </c>
@@ -26913,7 +26912,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>178</v>
       </c>
@@ -26946,7 +26945,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>179</v>
       </c>
@@ -26979,7 +26978,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>180</v>
       </c>
@@ -27012,7 +27011,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>181</v>
       </c>
@@ -27045,7 +27044,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -27076,7 +27075,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -27107,7 +27106,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>182</v>
       </c>
@@ -27140,7 +27139,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>183</v>
       </c>
@@ -27173,7 +27172,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>184</v>
       </c>
@@ -27206,7 +27205,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>185</v>
       </c>
@@ -27239,7 +27238,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>186</v>
       </c>
@@ -27272,7 +27271,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>187</v>
       </c>
@@ -27305,7 +27304,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>188</v>
       </c>
@@ -27338,7 +27337,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>189</v>
       </c>
@@ -27371,7 +27370,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>190</v>
       </c>
@@ -27404,7 +27403,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>191</v>
       </c>
@@ -27437,7 +27436,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>192</v>
       </c>
@@ -27470,7 +27469,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>193</v>
       </c>
@@ -27503,7 +27502,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>194</v>
       </c>
@@ -27536,7 +27535,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>195</v>
       </c>
@@ -27569,7 +27568,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>196</v>
       </c>
@@ -27602,7 +27601,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>197</v>
       </c>
@@ -27635,7 +27634,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>198</v>
       </c>
@@ -27667,7 +27666,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>199</v>
       </c>
@@ -27699,7 +27698,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>200</v>
       </c>
@@ -27731,7 +27730,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>201</v>
       </c>
@@ -27763,7 +27762,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>202</v>
       </c>
@@ -27795,7 +27794,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -27825,7 +27824,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -27855,7 +27854,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>203</v>
       </c>
@@ -27887,7 +27886,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>204</v>
       </c>
@@ -27919,7 +27918,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>205</v>
       </c>
@@ -27951,7 +27950,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>206</v>
       </c>
@@ -27983,7 +27982,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>207</v>
       </c>
@@ -28015,7 +28014,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -28045,7 +28044,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>208</v>
       </c>
@@ -28077,7 +28076,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>209</v>
       </c>
@@ -28109,7 +28108,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>210</v>
       </c>
@@ -28141,7 +28140,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>211</v>
       </c>
@@ -28173,7 +28172,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28203,7 +28202,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28233,7 +28232,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28263,7 +28262,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28293,7 +28292,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>212</v>
       </c>
@@ -28325,7 +28324,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>213</v>
       </c>
@@ -28357,7 +28356,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28387,7 +28386,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28417,7 +28416,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28447,7 +28446,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28477,7 +28476,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28507,7 +28506,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -28602,11 +28601,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>214</v>
       </c>
@@ -28638,7 +28636,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -28669,7 +28667,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -28700,7 +28698,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -28731,7 +28729,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -28762,7 +28760,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -28793,7 +28791,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -28824,7 +28822,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -28855,7 +28853,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -28886,7 +28884,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -28917,7 +28915,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -28948,7 +28946,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -28979,7 +28977,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -29010,7 +29008,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -29041,7 +29039,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -29072,7 +29070,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -29103,7 +29101,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -29134,7 +29132,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29165,7 +29163,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29196,7 +29194,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29227,7 +29225,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29257,7 +29255,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29287,7 +29285,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29317,7 +29315,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29347,7 +29345,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29377,7 +29375,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29407,7 +29405,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29437,7 +29435,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29467,7 +29465,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29497,7 +29495,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29527,7 +29525,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -29557,7 +29555,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -29587,7 +29585,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -29617,7 +29615,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -29647,7 +29645,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -29677,7 +29675,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -29707,7 +29705,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>212</v>
       </c>
@@ -29739,7 +29737,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>213</v>
       </c>
@@ -29771,7 +29769,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -29801,7 +29799,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -29831,7 +29829,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -29861,7 +29859,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -29891,7 +29889,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -29921,7 +29919,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -51664,19 +51662,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -51690,7 +51688,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>221</v>
       </c>
@@ -51702,7 +51700,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>222</v>
       </c>
@@ -51713,7 +51711,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>223</v>
       </c>
@@ -51724,7 +51722,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>224</v>
       </c>
@@ -51735,13 +51733,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-07T20:10:03Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -6835,13 +6835,13 @@
         <v>27</v>
       </c>
       <c r="K32" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L32" s="13" t="s">
         <v>27</v>
       </c>
       <c r="M32" s="13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N32" s="14" t="s">
         <v>27</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-07T20:44:28Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -6841,7 +6841,7 @@
         <v>27</v>
       </c>
       <c r="M32" s="13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N32" s="14" t="s">
         <v>27</v>
@@ -24019,7 +24019,9 @@
       <c r="E4" s="54">
         <v>-22.799999999999955</v>
       </c>
-      <c r="F4" s="54"/>
+      <c r="F4" s="54">
+        <v>0</v>
+      </c>
       <c r="G4" s="54"/>
       <c r="H4" s="54"/>
       <c r="I4" s="54"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-07T20:48:10Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -9780,30 +9780,74 @@
       <c r="C5" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
-      <c r="F5" s="52"/>
-      <c r="G5" s="53"/>
-      <c r="H5" s="52"/>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="52"/>
-      <c r="L5" s="52"/>
-      <c r="M5" s="53"/>
+      <c r="D5" s="52">
+        <v>245679.5</v>
+      </c>
+      <c r="E5" s="52">
+        <v>216530.08</v>
+      </c>
+      <c r="F5" s="52">
+        <v>29149.420000000013</v>
+      </c>
+      <c r="G5" s="53">
+        <v>0.11864815745717495</v>
+      </c>
+      <c r="H5" s="52">
+        <v>208360.5</v>
+      </c>
+      <c r="I5" s="52">
+        <v>168361.6</v>
+      </c>
+      <c r="J5" s="52">
+        <v>180366.49</v>
+      </c>
+      <c r="K5" s="52">
+        <v>138438.46000000002</v>
+      </c>
+      <c r="L5" s="52">
+        <v>41928.02999999997</v>
+      </c>
+      <c r="M5" s="53">
+        <v>0.23246019812216767</v>
+      </c>
       <c r="N5" s="53"/>
-      <c r="O5" s="52"/>
-      <c r="P5" s="52"/>
-      <c r="Q5" s="52"/>
-      <c r="R5" s="53"/>
-      <c r="S5" s="54"/>
-      <c r="T5" s="54"/>
-      <c r="U5" s="54"/>
-      <c r="V5" s="53"/>
+      <c r="O5" s="52">
+        <v>27994.01</v>
+      </c>
+      <c r="P5" s="52">
+        <v>29923.14</v>
+      </c>
+      <c r="Q5" s="52">
+        <v>-1929.130000000001</v>
+      </c>
+      <c r="R5" s="53">
+        <v>-0.06891224229754869</v>
+      </c>
+      <c r="S5" s="54">
+        <v>565.45</v>
+      </c>
+      <c r="T5" s="54">
+        <v>600.25</v>
+      </c>
+      <c r="U5" s="54">
+        <v>-34.799999999999955</v>
+      </c>
+      <c r="V5" s="53">
+        <v>-0.061543903086037584</v>
+      </c>
       <c r="W5" s="53"/>
-      <c r="X5" s="55"/>
-      <c r="Y5" s="55"/>
-      <c r="Z5" s="53"/>
-      <c r="AA5" s="56"/>
+      <c r="X5" s="55">
+        <v>80.24736359850063</v>
+      </c>
+      <c r="Y5" s="55">
+        <v>65.99877634098505</v>
+      </c>
+      <c r="Z5" s="53">
+        <v>0.2225</v>
+      </c>
+      <c r="AA5" s="56">
+        <v>0.1519</v>
+      </c>
       <c r="AB5" s="57"/>
       <c r="AD5" s="35" t="s">
         <v>95</v>
@@ -10115,54 +10159,54 @@
         <v>101420.72</v>
       </c>
       <c r="I12" s="52">
-        <v>76488.35</v>
+        <v>79791.03</v>
       </c>
       <c r="J12" s="52">
         <v>83645.65</v>
       </c>
       <c r="K12" s="52">
-        <v>70758.46</v>
+        <v>71604.5</v>
       </c>
       <c r="L12" s="52">
-        <v>12887.189999999988</v>
+        <v>12041.149999999994</v>
       </c>
       <c r="M12" s="53">
-        <v>0.1540688607237793</v>
+        <v>0.1439542881189876</v>
       </c>
       <c r="N12" s="53"/>
       <c r="O12" s="52">
         <v>17775.07</v>
       </c>
       <c r="P12" s="52">
-        <v>5729.89</v>
+        <v>8186.53</v>
       </c>
       <c r="Q12" s="52">
-        <v>12045.18</v>
+        <v>9588.54</v>
       </c>
       <c r="R12" s="53">
-        <v>0.6776445887414227</v>
+        <v>0.5394375380800188</v>
       </c>
       <c r="S12" s="54">
         <v>356.07</v>
       </c>
       <c r="T12" s="54">
-        <v>117.75</v>
+        <v>168.25</v>
       </c>
       <c r="U12" s="54">
-        <v>238.32</v>
+        <v>187.82</v>
       </c>
       <c r="V12" s="53">
-        <v>0.6693065970174403</v>
+        <v>0.5274805515769371</v>
       </c>
       <c r="W12" s="53"/>
       <c r="X12" s="55">
-        <v>79.624033970276</v>
+        <v>36.09539375928678</v>
       </c>
       <c r="Y12" s="55">
         <v>77.66490997775718</v>
       </c>
       <c r="Z12" s="53">
-        <v>0.1092</v>
+        <v>0.0707</v>
       </c>
       <c r="AA12" s="56">
         <v>0.2142</v>
@@ -10843,54 +10887,54 @@
         <v>102178.42</v>
       </c>
       <c r="I26" s="52">
-        <v>87101.11</v>
+        <v>89222.05</v>
       </c>
       <c r="J26" s="52">
         <v>62464.86</v>
       </c>
       <c r="K26" s="52">
-        <v>57898.75</v>
+        <v>58984</v>
       </c>
       <c r="L26" s="52">
-        <v>4566.110000000001</v>
+        <v>3480.8600000000006</v>
       </c>
       <c r="M26" s="53">
-        <v>0.07309885910254182</v>
+        <v>0.05572509087509362</v>
       </c>
       <c r="N26" s="53"/>
       <c r="O26" s="52">
         <v>39713.56</v>
       </c>
       <c r="P26" s="52">
-        <v>29202.36</v>
+        <v>30238.05</v>
       </c>
       <c r="Q26" s="52">
-        <v>10511.199999999997</v>
+        <v>9475.509999999998</v>
       </c>
       <c r="R26" s="53">
-        <v>0.26467534011053145</v>
+        <v>0.23859633837913294</v>
       </c>
       <c r="S26" s="54">
         <v>795.22</v>
       </c>
       <c r="T26" s="54">
-        <v>594.5</v>
+        <v>615</v>
       </c>
       <c r="U26" s="54">
-        <v>200.72000000000003</v>
+        <v>180.22000000000003</v>
       </c>
       <c r="V26" s="53">
-        <v>0.25240813862830414</v>
+        <v>0.22662910892583188</v>
       </c>
       <c r="W26" s="53"/>
       <c r="X26" s="55">
-        <v>96.3325315391085</v>
+        <v>89.67276422764228</v>
       </c>
       <c r="Y26" s="55">
         <v>61.20621468124544</v>
       </c>
       <c r="Z26" s="53">
-        <v>0.3967</v>
+        <v>0.382</v>
       </c>
       <c r="AA26" s="56">
         <v>0.3227</v>
@@ -11206,54 +11250,54 @@
         <v>327431.12</v>
       </c>
       <c r="I33" s="65">
-        <v>220187.84</v>
+        <v>223659.54</v>
       </c>
       <c r="J33" s="52">
         <v>271519.78</v>
       </c>
       <c r="K33" s="52">
-        <v>196879.33</v>
+        <v>197370.72</v>
       </c>
       <c r="L33" s="52">
-        <v>74640.45000000004</v>
+        <v>74149.06000000003</v>
       </c>
       <c r="M33" s="53">
-        <v>0.27489875691561044</v>
+        <v>0.27308898084699396</v>
       </c>
       <c r="N33" s="53"/>
       <c r="O33" s="52">
         <v>55911.34</v>
       </c>
       <c r="P33" s="52">
-        <v>23308.51</v>
+        <v>26288.82</v>
       </c>
       <c r="Q33" s="52">
-        <v>32602.829999999998</v>
+        <v>29622.519999999997</v>
       </c>
       <c r="R33" s="53">
-        <v>0.5831165913748445</v>
+        <v>0.5298123779540966</v>
       </c>
       <c r="S33" s="54">
         <v>1120.27</v>
       </c>
       <c r="T33" s="54">
-        <v>543.5</v>
+        <v>607.75</v>
       </c>
       <c r="U33" s="54">
-        <v>576.77</v>
+        <v>512.52</v>
       </c>
       <c r="V33" s="53">
-        <v>0.514849098877949</v>
+        <v>0.4574968534371178</v>
       </c>
       <c r="W33" s="53"/>
       <c r="X33" s="55">
-        <v>72.05127874885005</v>
+        <v>58.721793500617025</v>
       </c>
       <c r="Y33" s="55">
         <v>61.5841822414239</v>
       </c>
       <c r="Z33" s="53">
-        <v>0.151</v>
+        <v>0.1376</v>
       </c>
       <c r="AA33" s="56">
         <v>0.174</v>
@@ -11569,54 +11613,54 @@
         <v>94098.32</v>
       </c>
       <c r="I40" s="52">
-        <v>46289.42</v>
+        <v>49261.61</v>
       </c>
       <c r="J40" s="52">
         <v>69042.09000000001</v>
       </c>
       <c r="K40" s="52">
-        <v>35507.08</v>
+        <v>35683.74</v>
       </c>
       <c r="L40" s="52">
-        <v>33535.01000000001</v>
+        <v>33358.35000000001</v>
       </c>
       <c r="M40" s="53">
-        <v>0.4857183494879718</v>
+        <v>0.4831596204576079</v>
       </c>
       <c r="N40" s="53"/>
       <c r="O40" s="52">
         <v>25056.23</v>
       </c>
       <c r="P40" s="52">
-        <v>10782.34</v>
+        <v>13577.87</v>
       </c>
       <c r="Q40" s="52">
-        <v>14273.89</v>
+        <v>11478.359999999999</v>
       </c>
       <c r="R40" s="53">
-        <v>0.5696742885901032</v>
+        <v>0.45810403241030273</v>
       </c>
       <c r="S40" s="54">
         <v>501.83</v>
       </c>
       <c r="T40" s="54">
-        <v>232.25</v>
+        <v>299.5</v>
       </c>
       <c r="U40" s="54">
-        <v>269.58</v>
+        <v>202.32999999999998</v>
       </c>
       <c r="V40" s="53">
-        <v>0.5371938704342107</v>
+        <v>0.40318434529621583</v>
       </c>
       <c r="W40" s="53"/>
       <c r="X40" s="55">
-        <v>32.96193756727664</v>
+        <v>15.63679465776294</v>
       </c>
       <c r="Y40" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z40" s="53">
-        <v>0.1419</v>
+        <v>0.0868</v>
       </c>
       <c r="AA40" s="56">
         <v>0.2663</v>
@@ -11934,54 +11978,54 @@
         <v>50582.37</v>
       </c>
       <c r="I47" s="52">
-        <v>25187.36</v>
+        <v>25196.36</v>
       </c>
       <c r="J47" s="52">
         <v>39438.990000000005</v>
       </c>
       <c r="K47" s="52">
-        <v>20432.420000000002</v>
+        <v>20036.420000000002</v>
       </c>
       <c r="L47" s="52">
-        <v>19006.570000000003</v>
+        <v>19402.570000000003</v>
       </c>
       <c r="M47" s="53">
-        <v>0.48192334540007237</v>
+        <v>0.49196417048205343</v>
       </c>
       <c r="N47" s="53"/>
       <c r="O47" s="52">
         <v>11143.38</v>
       </c>
       <c r="P47" s="52">
-        <v>4754.94</v>
+        <v>5159.94</v>
       </c>
       <c r="Q47" s="52">
-        <v>6388.44</v>
+        <v>5983.44</v>
       </c>
       <c r="R47" s="53">
-        <v>0.5732946377131535</v>
+        <v>0.5369501892603501</v>
       </c>
       <c r="S47" s="54">
         <v>223.22</v>
       </c>
       <c r="T47" s="54">
-        <v>104.25</v>
+        <v>113.25</v>
       </c>
       <c r="U47" s="54">
-        <v>118.97</v>
+        <v>109.97</v>
       </c>
       <c r="V47" s="53">
-        <v>0.5329719559179285</v>
+        <v>0.49265298808350505</v>
       </c>
       <c r="W47" s="53"/>
       <c r="X47" s="55">
-        <v>78.07318944844125</v>
+        <v>71.78922737306843</v>
       </c>
       <c r="Y47" s="55">
         <v>67.69550512136009</v>
       </c>
       <c r="Z47" s="53">
-        <v>0.24420000000000003</v>
+        <v>0.244</v>
       </c>
       <c r="AA47" s="56">
         <v>0.23</v>
@@ -12297,54 +12341,54 @@
         <v>109364.97</v>
       </c>
       <c r="I54" s="52">
-        <v>95597.19</v>
+        <v>96483.38</v>
       </c>
       <c r="J54" s="52">
         <v>75135.01000000001</v>
       </c>
       <c r="K54" s="52">
-        <v>71143.79000000001</v>
+        <v>71221.34</v>
       </c>
       <c r="L54" s="52">
-        <v>3991.220000000001</v>
+        <v>3913.670000000013</v>
       </c>
       <c r="M54" s="53">
-        <v>0.05312064242754477</v>
+        <v>0.05208850042077604</v>
       </c>
       <c r="N54" s="53"/>
       <c r="O54" s="52">
         <v>34229.96</v>
       </c>
       <c r="P54" s="52">
-        <v>24453.4</v>
+        <v>25262.04</v>
       </c>
       <c r="Q54" s="52">
-        <v>9776.559999999998</v>
+        <v>8967.919999999998</v>
       </c>
       <c r="R54" s="53">
-        <v>0.28561412283274645</v>
+        <v>0.2619903733454552</v>
       </c>
       <c r="S54" s="54">
         <v>685.48</v>
       </c>
       <c r="T54" s="54">
-        <v>517.75</v>
+        <v>533.75</v>
       </c>
       <c r="U54" s="54">
-        <v>167.73000000000002</v>
+        <v>151.73000000000002</v>
       </c>
       <c r="V54" s="53">
-        <v>0.24468985236622515</v>
+        <v>0.22134854408589605</v>
       </c>
       <c r="W54" s="53"/>
       <c r="X54" s="55">
-        <v>62.22557218734911</v>
+        <v>58.699953161592504</v>
       </c>
       <c r="Y54" s="55">
         <v>67.00679527854935</v>
       </c>
       <c r="Z54" s="53">
-        <v>0.2521</v>
+        <v>0.2451</v>
       </c>
       <c r="AA54" s="56">
         <v>0.2958</v>
@@ -13372,19 +13416,19 @@
         <v>54302.66</v>
       </c>
       <c r="I75" s="52">
-        <v>33447.19</v>
+        <v>29696.65</v>
       </c>
       <c r="J75" s="52">
         <v>31383.390000000003</v>
       </c>
       <c r="K75" s="52">
-        <v>27343.140000000003</v>
+        <v>23592.600000000002</v>
       </c>
       <c r="L75" s="52">
-        <v>4040.25</v>
+        <v>7790.790000000001</v>
       </c>
       <c r="M75" s="53">
-        <v>0.128738482362804</v>
+        <v>0.24824564841465502</v>
       </c>
       <c r="N75" s="53"/>
       <c r="O75" s="52">
@@ -13413,13 +13457,13 @@
       </c>
       <c r="W75" s="53"/>
       <c r="X75" s="55">
-        <v>94.11891891891891</v>
+        <v>125.30844074844074</v>
       </c>
       <c r="Y75" s="55">
         <v>48.58165977967362</v>
       </c>
       <c r="Z75" s="53">
-        <v>0.2528</v>
+        <v>0.33659999999999995</v>
       </c>
       <c r="AA75" s="56">
         <v>0.2963</v>
@@ -14092,54 +14136,54 @@
         <v>27002.93</v>
       </c>
       <c r="I89" s="52">
-        <v>24950.27</v>
+        <v>25060.53</v>
       </c>
       <c r="J89" s="52">
         <v>15440.32</v>
       </c>
       <c r="K89" s="52">
-        <v>13932.720000000001</v>
+        <v>13974.73</v>
       </c>
       <c r="L89" s="52">
-        <v>1507.5999999999985</v>
+        <v>1465.5900000000001</v>
       </c>
       <c r="M89" s="53">
-        <v>0.09764046341008467</v>
+        <v>0.09491966487741188</v>
       </c>
       <c r="N89" s="53"/>
       <c r="O89" s="52">
         <v>11562.61</v>
       </c>
       <c r="P89" s="52">
-        <v>11017.55</v>
+        <v>11085.8</v>
       </c>
       <c r="Q89" s="52">
-        <v>545.0600000000013</v>
+        <v>476.8100000000013</v>
       </c>
       <c r="R89" s="53">
-        <v>0.04713987585847843</v>
+        <v>0.041237229310683424</v>
       </c>
       <c r="S89" s="68">
         <v>231.75</v>
       </c>
       <c r="T89" s="68">
-        <v>224.25</v>
+        <v>225.5</v>
       </c>
       <c r="U89" s="54">
-        <v>7.5</v>
+        <v>6.25</v>
       </c>
       <c r="V89" s="53">
-        <v>0.032362459546925564</v>
+        <v>0.02696871628910464</v>
       </c>
       <c r="W89" s="53"/>
       <c r="X89" s="55">
-        <v>50.9746265328874</v>
+        <v>50.20310421286031</v>
       </c>
       <c r="Y89" s="55">
         <v>43.49557070636461</v>
       </c>
       <c r="Z89" s="53">
-        <v>0.31420000000000003</v>
+        <v>0.31120000000000003</v>
       </c>
       <c r="AA89" s="56">
         <v>0.2718</v>
@@ -21872,10 +21916,10 @@
         <v>0</v>
       </c>
       <c r="D4" s="52">
-        <v>0</v>
+        <v>403.9200000000128</v>
       </c>
       <c r="E4" s="52">
-        <v>0</v>
+        <v>-403.9200000000128</v>
       </c>
       <c r="F4" s="52">
         <v>0</v>
@@ -21899,13 +21943,13 @@
         <v>0</v>
       </c>
       <c r="M4" s="52">
-        <v>-7000</v>
+        <v>-7403.920000000013</v>
       </c>
       <c r="N4" s="54">
         <v>20</v>
       </c>
       <c r="O4" s="58">
-        <v>-100</v>
+        <v>-105.77028571428589</v>
       </c>
     </row>
     <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -21936,10 +21980,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="52">
-        <v>2351.029999999999</v>
+        <v>5653.709999999992</v>
       </c>
       <c r="E6" s="52">
-        <v>-2351.029999999999</v>
+        <v>-5653.709999999992</v>
       </c>
       <c r="F6" s="52">
         <v>0</v>
@@ -21963,13 +22007,13 @@
         <v>0</v>
       </c>
       <c r="M6" s="52">
-        <v>-4223.629999999999</v>
+        <v>-7526.309999999992</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>337.89039999999994</v>
+        <v>602.1047999999994</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>117</v>
@@ -22063,10 +22107,10 @@
         <v>0</v>
       </c>
       <c r="D10" s="52">
-        <v>1252.699999999997</v>
+        <v>3373.6399999999994</v>
       </c>
       <c r="E10" s="52">
-        <v>-1252.699999999997</v>
+        <v>-3373.6399999999994</v>
       </c>
       <c r="F10" s="52">
         <v>0</v>
@@ -22090,13 +22134,13 @@
         <v>0</v>
       </c>
       <c r="M10" s="52">
-        <v>-6172.699999999997</v>
+        <v>-8293.64</v>
       </c>
       <c r="N10" s="54">
         <v>-388.25</v>
       </c>
       <c r="O10" s="58">
-        <v>18.141660543717848</v>
+        <v>24.375135929463628</v>
       </c>
     </row>
     <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22127,10 +22171,10 @@
         <v>0</v>
       </c>
       <c r="D12" s="52">
-        <v>3843.2399999999907</v>
+        <v>7314.940000000002</v>
       </c>
       <c r="E12" s="52">
-        <v>-3843.2399999999907</v>
+        <v>-7314.940000000002</v>
       </c>
       <c r="F12" s="52">
         <v>3</v>
@@ -22154,13 +22198,13 @@
         <v>0</v>
       </c>
       <c r="M12" s="52">
-        <v>-6480.239999999991</v>
+        <v>-9951.940000000002</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>-93.9165217391303</v>
+        <v>-144.23101449275364</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>119</v>
@@ -22194,10 +22238,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="52">
-        <v>4015.729999999996</v>
+        <v>6987.919999999998</v>
       </c>
       <c r="E14" s="52">
-        <v>-4015.729999999996</v>
+        <v>-6987.919999999998</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
@@ -22221,13 +22265,13 @@
         <v>0</v>
       </c>
       <c r="M14" s="52">
-        <v>-7015.729999999996</v>
+        <v>-9987.919999999998</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>62.640446428571394</v>
+        <v>89.17785714285712</v>
       </c>
     </row>
     <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22258,10 +22302,10 @@
         <v>0</v>
       </c>
       <c r="D16" s="52">
-        <v>-24.220000000001164</v>
+        <v>-15.220000000001164</v>
       </c>
       <c r="E16" s="52">
-        <v>24.220000000001164</v>
+        <v>15.220000000001164</v>
       </c>
       <c r="F16" s="52"/>
       <c r="G16" s="53">
@@ -22283,13 +22327,13 @@
         <v>0</v>
       </c>
       <c r="M16" s="52">
-        <v>-2975.779999999999</v>
+        <v>-2984.779999999999</v>
       </c>
       <c r="N16" s="54">
         <v>-86.75</v>
       </c>
       <c r="O16" s="58">
-        <v>34.302939481268</v>
+        <v>34.40668587896252</v>
       </c>
     </row>
     <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -22320,10 +22364,10 @@
         <v>0</v>
       </c>
       <c r="D18" s="52">
-        <v>276.68000000000757</v>
+        <v>1162.87000000001</v>
       </c>
       <c r="E18" s="52">
-        <v>-276.68000000000757</v>
+        <v>-1162.87000000001</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
@@ -22347,13 +22391,13 @@
         <v>0</v>
       </c>
       <c r="M18" s="52">
-        <v>-8476.680000000008</v>
+        <v>-9362.87000000001</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>44.85015873015877</v>
+        <v>49.538994708994764</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>120</v>
@@ -22501,10 +22545,10 @@
         <v>0</v>
       </c>
       <c r="D24" s="52">
-        <v>1528.260000000002</v>
+        <v>-2222.279999999999</v>
       </c>
       <c r="E24" s="52">
-        <v>-1528.260000000002</v>
+        <v>2222.279999999999</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
@@ -22522,7 +22566,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="52">
-        <v>-1525.260000000002</v>
+        <v>2225.279999999999</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -22619,10 +22663,10 @@
         <v>0</v>
       </c>
       <c r="D28" s="52">
-        <v>-1055.7200000000012</v>
+        <v>-945.4600000000028</v>
       </c>
       <c r="E28" s="52">
-        <v>1055.7200000000012</v>
+        <v>945.4600000000028</v>
       </c>
       <c r="F28" s="52">
         <v>0</v>
@@ -22642,13 +22686,13 @@
         <v>0</v>
       </c>
       <c r="M28" s="52">
-        <v>1055.7200000000012</v>
+        <v>945.4600000000028</v>
       </c>
       <c r="N28" s="54">
         <v>-148.5</v>
       </c>
       <c r="O28" s="58">
-        <v>-7.109225589225597</v>
+        <v>-6.366734006734025</v>
       </c>
     </row>
     <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
@@ -23820,22 +23864,22 @@
         <v>88818.76999999996</v>
       </c>
       <c r="D70" s="104">
-        <v>29887.739999999983</v>
+        <v>39414.08000000001</v>
       </c>
       <c r="E70" s="105">
-        <v>58931.02999999998</v>
+        <v>49404.68999999996</v>
       </c>
       <c r="F70" s="106" t="s">
         <v>124</v>
       </c>
       <c r="G70" s="107">
-        <v>0.6634974791927427</v>
+        <v>0.5562415466910877</v>
       </c>
       <c r="H70" s="108" t="s">
         <v>125</v>
       </c>
       <c r="I70" s="109">
-        <v>0.0799203816940944</v>
+        <v>-0.02733555080756062</v>
       </c>
       <c r="J70" s="36"/>
       <c r="K70" s="36"/>
@@ -24390,10 +24434,10 @@
         <v>565.45</v>
       </c>
       <c r="D4" s="54">
-        <v>588.25</v>
+        <v>600.25</v>
       </c>
       <c r="E4" s="54">
-        <v>-22.799999999999955</v>
+        <v>-34.799999999999955</v>
       </c>
       <c r="F4" s="54">
         <v>0</v>
@@ -24445,10 +24489,10 @@
         <v>356.07</v>
       </c>
       <c r="D6" s="54">
-        <v>117.75</v>
+        <v>168.25</v>
       </c>
       <c r="E6" s="54">
-        <v>238.32</v>
+        <v>187.82</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -24551,10 +24595,10 @@
         <v>795.22</v>
       </c>
       <c r="D10" s="54">
-        <v>594.5</v>
+        <v>615</v>
       </c>
       <c r="E10" s="54">
-        <v>200.72000000000003</v>
+        <v>180.22000000000003</v>
       </c>
       <c r="F10" s="54"/>
       <c r="G10" s="54"/>
@@ -24608,10 +24652,10 @@
         <v>1120.27</v>
       </c>
       <c r="D12" s="54">
-        <v>543.5</v>
+        <v>607.75</v>
       </c>
       <c r="E12" s="54">
-        <v>576.77</v>
+        <v>512.52</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -24665,10 +24709,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>232.25</v>
+        <v>299.5</v>
       </c>
       <c r="E14" s="54">
-        <v>269.58</v>
+        <v>202.32999999999998</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -24722,10 +24766,10 @@
         <v>223.22</v>
       </c>
       <c r="D16" s="54">
-        <v>104.25</v>
+        <v>113.25</v>
       </c>
       <c r="E16" s="54">
-        <v>118.97</v>
+        <v>109.97</v>
       </c>
       <c r="F16" s="54"/>
       <c r="G16" s="54"/>
@@ -24774,10 +24818,10 @@
         <v>685.48</v>
       </c>
       <c r="D18" s="54">
-        <v>517.75</v>
+        <v>533.75</v>
       </c>
       <c r="E18" s="54">
-        <v>167.73000000000002</v>
+        <v>151.73000000000002</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -25032,10 +25076,10 @@
         <v>231.75</v>
       </c>
       <c r="D28" s="54">
-        <v>224.25</v>
+        <v>225.5</v>
       </c>
       <c r="E28" s="54">
-        <v>7.5</v>
+        <v>6.25</v>
       </c>
       <c r="F28" s="54"/>
       <c r="G28" s="54"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-07T20:53:50Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16396,7 +16396,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>97</v>
@@ -21803,7 +21803,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD71"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21817,7 +21817,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21839,7 +21839,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>102</v>
       </c>
@@ -21887,7 +21887,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21905,7 +21905,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21952,7 +21952,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21969,7 +21969,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -22019,7 +22019,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -22036,7 +22036,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -22079,7 +22079,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -22096,7 +22096,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -22143,7 +22143,7 @@
         <v>24.375135929463628</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -22160,7 +22160,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -22210,7 +22210,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -22227,7 +22227,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -22274,7 +22274,7 @@
         <v>89.17785714285712</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -22291,7 +22291,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -22336,7 +22336,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -22353,7 +22353,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -22403,7 +22403,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -22420,7 +22420,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -22459,7 +22459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -22476,7 +22476,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -22517,7 +22517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22534,7 +22534,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22573,7 +22573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22590,7 +22590,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22635,7 +22635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22652,7 +22652,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22695,7 +22695,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22712,7 +22712,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22755,7 +22755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22772,7 +22772,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22819,7 +22819,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22836,7 +22836,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22881,7 +22881,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22898,7 +22898,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22941,7 +22941,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22958,7 +22958,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22999,7 +22999,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -23016,7 +23016,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -23061,7 +23061,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -23078,7 +23078,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -23121,7 +23121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -23138,7 +23138,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -23175,7 +23175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -23192,7 +23192,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -23233,7 +23233,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -23250,7 +23250,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -23293,7 +23293,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -23310,7 +23310,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -23352,7 +23352,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -23369,7 +23369,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -23414,7 +23414,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -23431,7 +23431,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -23476,7 +23476,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -23493,7 +23493,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23538,7 +23538,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23555,7 +23555,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23592,7 +23592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23609,7 +23609,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23626,7 +23626,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23643,7 +23643,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23664,7 +23664,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23681,7 +23681,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23722,7 +23722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23739,7 +23739,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23784,7 +23784,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -23819,7 +23819,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23836,7 +23836,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -23853,7 +23853,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>122</v>
       </c>
@@ -23888,7 +23888,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>126</v>
@@ -24271,7 +24271,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD110"/>
+  <dimension ref="A1:AB110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -24282,7 +24282,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -24303,7 +24303,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>127</v>
@@ -24365,7 +24365,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>143</v>
       </c>
@@ -24423,7 +24423,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -24459,7 +24459,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -24478,7 +24478,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -24512,7 +24512,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -24531,7 +24531,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24565,7 +24565,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24584,7 +24584,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24622,7 +24622,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24641,7 +24641,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24679,7 +24679,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24698,7 +24698,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24736,7 +24736,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24755,7 +24755,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24788,7 +24788,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24807,7 +24807,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24840,7 +24840,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24859,7 +24859,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24890,7 +24890,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24909,7 +24909,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24944,7 +24944,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24963,7 +24963,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24996,7 +24996,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -25015,7 +25015,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25046,7 +25046,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -25065,7 +25065,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25097,7 +25097,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -25116,7 +25116,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -25152,7 +25152,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -25171,7 +25171,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -25200,7 +25200,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -25219,7 +25219,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -25250,7 +25250,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -25269,7 +25269,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -25302,7 +25302,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -25321,7 +25321,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -25357,7 +25357,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -25376,7 +25376,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -25411,7 +25411,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -25430,7 +25430,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25460,7 +25460,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -25479,7 +25479,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25519,7 +25519,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -25538,7 +25538,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25567,7 +25567,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25586,7 +25586,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25619,7 +25619,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25638,7 +25638,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25671,7 +25671,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25690,7 +25690,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25726,7 +25726,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25745,7 +25745,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25781,7 +25781,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25800,7 +25800,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25834,7 +25834,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25853,7 +25853,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25888,7 +25888,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25907,7 +25907,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25926,7 +25926,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25945,7 +25945,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25966,7 +25966,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25985,7 +25985,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -26018,7 +26018,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -26037,7 +26037,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -26076,7 +26076,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -26105,7 +26105,7 @@
       <c r="P67" s="54"/>
       <c r="Q67" s="54"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -26124,7 +26124,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="142"/>
       <c r="B69" s="143"/>
       <c r="C69" s="35"/>
@@ -26143,7 +26143,7 @@
       <c r="P69" s="35"/>
       <c r="Q69" s="144"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="145"/>
       <c r="B70" s="145"/>
       <c r="C70" s="145"/>
@@ -26162,7 +26162,7 @@
       <c r="P70" s="145"/>
       <c r="Q70" s="145"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="146" t="s">
         <v>147</v>
@@ -26207,7 +26207,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -26246,7 +26246,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="77" t="s">
         <v>149</v>
@@ -26275,7 +26275,7 @@
       <c r="P73" s="20"/>
       <c r="Q73" s="20"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="148" t="s">
         <v>150</v>
@@ -26320,7 +26320,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="151" t="s">
         <v>151</v>
@@ -26365,7 +26365,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
@@ -26384,7 +26384,7 @@
       <c r="P76" s="35"/>
       <c r="Q76" s="144"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="156" t="s">
         <v>152</v>
@@ -26431,7 +26431,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="161"/>
       <c r="B78" s="162" t="s">
         <v>154</v>
@@ -26476,7 +26476,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -26495,7 +26495,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="164" t="s">
         <v>155</v>
@@ -26518,7 +26518,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="167" t="s">
         <v>157</v>
@@ -26541,7 +26541,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -26564,7 +26564,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -26587,7 +26587,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -26610,7 +26610,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -26633,7 +26633,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -26656,7 +26656,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -26679,7 +26679,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -26702,7 +26702,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -26725,7 +26725,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -26748,7 +26748,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -26771,7 +26771,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26792,7 +26792,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26813,7 +26813,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26834,7 +26834,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26855,7 +26855,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26876,7 +26876,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26897,7 +26897,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -26918,7 +26918,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -26941,7 +26941,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -26964,7 +26964,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -26987,7 +26987,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -27010,7 +27010,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -27033,7 +27033,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -27056,7 +27056,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -27079,7 +27079,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -27098,7 +27098,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -27117,7 +27117,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19"/>
       <c r="C108" s="131"/>
@@ -27136,7 +27136,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="169"/>
       <c r="C109" s="150"/>
@@ -27155,7 +27155,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="164" t="s">
         <v>175</v>
@@ -27229,11 +27229,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>176</v>
       </c>
@@ -27265,7 +27264,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>177</v>
       </c>
@@ -27298,7 +27297,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>178</v>
       </c>
@@ -27331,7 +27330,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>179</v>
       </c>
@@ -27364,7 +27363,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>180</v>
       </c>
@@ -27397,7 +27396,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>181</v>
       </c>
@@ -27430,7 +27429,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>182</v>
       </c>
@@ -27463,7 +27462,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>183</v>
       </c>
@@ -27496,7 +27495,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -27527,7 +27526,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -27558,7 +27557,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>184</v>
       </c>
@@ -27591,7 +27590,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>185</v>
       </c>
@@ -27624,7 +27623,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>186</v>
       </c>
@@ -27657,7 +27656,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>187</v>
       </c>
@@ -27690,7 +27689,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>188</v>
       </c>
@@ -27723,7 +27722,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>189</v>
       </c>
@@ -27756,7 +27755,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>190</v>
       </c>
@@ -27789,7 +27788,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>191</v>
       </c>
@@ -27822,7 +27821,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>192</v>
       </c>
@@ -27855,7 +27854,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>193</v>
       </c>
@@ -27888,7 +27887,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>194</v>
       </c>
@@ -27921,7 +27920,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>195</v>
       </c>
@@ -27954,7 +27953,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>196</v>
       </c>
@@ -27987,7 +27986,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>197</v>
       </c>
@@ -28020,7 +28019,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>198</v>
       </c>
@@ -28053,7 +28052,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>199</v>
       </c>
@@ -28086,7 +28085,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>200</v>
       </c>
@@ -28118,7 +28117,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>201</v>
       </c>
@@ -28150,7 +28149,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>202</v>
       </c>
@@ -28182,7 +28181,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>203</v>
       </c>
@@ -28214,7 +28213,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>204</v>
       </c>
@@ -28246,7 +28245,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -28276,7 +28275,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -28306,7 +28305,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>205</v>
       </c>
@@ -28338,7 +28337,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>206</v>
       </c>
@@ -28370,7 +28369,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>207</v>
       </c>
@@ -28402,7 +28401,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>208</v>
       </c>
@@ -28434,7 +28433,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>209</v>
       </c>
@@ -28466,7 +28465,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -28496,7 +28495,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>210</v>
       </c>
@@ -28528,7 +28527,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>211</v>
       </c>
@@ -28560,7 +28559,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>212</v>
       </c>
@@ -28592,7 +28591,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>213</v>
       </c>
@@ -28624,7 +28623,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28654,7 +28653,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28684,7 +28683,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28714,7 +28713,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28744,7 +28743,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>214</v>
       </c>
@@ -28776,7 +28775,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>215</v>
       </c>
@@ -28808,7 +28807,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28838,7 +28837,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28868,7 +28867,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28898,7 +28897,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28928,7 +28927,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28958,7 +28957,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -29053,11 +29052,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>216</v>
       </c>
@@ -29089,7 +29087,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -29120,7 +29118,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -29151,7 +29149,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -29182,7 +29180,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -29213,7 +29211,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -29244,7 +29242,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -29275,7 +29273,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -29306,7 +29304,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -29337,7 +29335,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -29368,7 +29366,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -29399,7 +29397,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -29430,7 +29428,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -29461,7 +29459,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -29492,7 +29490,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -29523,7 +29521,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -29554,7 +29552,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -29585,7 +29583,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29616,7 +29614,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29647,7 +29645,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29678,7 +29676,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29708,7 +29706,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29738,7 +29736,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29768,7 +29766,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29798,7 +29796,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29828,7 +29826,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29858,7 +29856,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29888,7 +29886,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29918,7 +29916,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29948,7 +29946,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29978,7 +29976,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -30008,7 +30006,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -30038,7 +30036,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -30068,7 +30066,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -30098,7 +30096,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -30128,7 +30126,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -30158,7 +30156,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>214</v>
       </c>
@@ -30190,7 +30188,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>215</v>
       </c>
@@ -30222,7 +30220,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -30252,7 +30250,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -30282,7 +30280,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -30312,7 +30310,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -30342,7 +30340,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -30372,7 +30370,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -52115,19 +52113,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -52141,7 +52139,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>223</v>
       </c>
@@ -52153,7 +52151,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>224</v>
       </c>
@@ -52164,7 +52162,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>225</v>
       </c>
@@ -52175,7 +52173,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>226</v>
       </c>
@@ -52186,13 +52184,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-07T20:56:21Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16396,7 +16396,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>97</v>
@@ -18764,30 +18764,74 @@
       <c r="C180" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D180" s="52"/>
-      <c r="E180" s="52"/>
-      <c r="F180" s="52"/>
-      <c r="G180" s="53"/>
-      <c r="H180" s="52"/>
-      <c r="I180" s="52"/>
-      <c r="J180" s="52"/>
-      <c r="K180" s="52"/>
-      <c r="L180" s="52"/>
-      <c r="M180" s="53"/>
+      <c r="D180" s="52">
+        <v>16897.53</v>
+      </c>
+      <c r="E180" s="52">
+        <v>5491.7</v>
+      </c>
+      <c r="F180" s="52">
+        <v>11405.829999999998</v>
+      </c>
+      <c r="G180" s="53">
+        <v>0.6749998372543206</v>
+      </c>
+      <c r="H180" s="52">
+        <v>9226.27</v>
+      </c>
+      <c r="I180" s="52">
+        <v>3702.78</v>
+      </c>
+      <c r="J180" s="52">
+        <v>2977.1100000000006</v>
+      </c>
+      <c r="K180" s="52">
+        <v>2335.9700000000003</v>
+      </c>
+      <c r="L180" s="52">
+        <v>641.1400000000003</v>
+      </c>
+      <c r="M180" s="53">
+        <v>0.2153565034546927</v>
+      </c>
       <c r="N180" s="53"/>
-      <c r="O180" s="52"/>
-      <c r="P180" s="52"/>
-      <c r="Q180" s="52"/>
-      <c r="R180" s="53"/>
-      <c r="S180" s="54"/>
-      <c r="T180" s="54"/>
-      <c r="U180" s="54"/>
-      <c r="V180" s="53"/>
+      <c r="O180" s="52">
+        <v>6249.16</v>
+      </c>
+      <c r="P180" s="52">
+        <v>1366.81</v>
+      </c>
+      <c r="Q180" s="52">
+        <v>4882.35</v>
+      </c>
+      <c r="R180" s="53">
+        <v>0.7812810041669601</v>
+      </c>
+      <c r="S180" s="54">
+        <v>125.17</v>
+      </c>
+      <c r="T180" s="54">
+        <v>23.75</v>
+      </c>
+      <c r="U180" s="54">
+        <v>101.42</v>
+      </c>
+      <c r="V180" s="53">
+        <v>0.8102580490532876</v>
+      </c>
       <c r="W180" s="53"/>
-      <c r="X180" s="55"/>
-      <c r="Y180" s="55"/>
-      <c r="Z180" s="53"/>
-      <c r="AA180" s="56"/>
+      <c r="X180" s="55">
+        <v>75.32294736842105</v>
+      </c>
+      <c r="Y180" s="55">
+        <v>61.286703843093385</v>
+      </c>
+      <c r="Z180" s="53">
+        <v>0.3257</v>
+      </c>
+      <c r="AA180" s="56">
+        <v>0.454</v>
+      </c>
       <c r="AB180" s="57"/>
       <c r="AD180" s="35" t="s">
         <v>95</v>
@@ -21061,30 +21105,74 @@
       <c r="C229" s="51" t="s">
         <v>94</v>
       </c>
-      <c r="D229" s="52"/>
-      <c r="E229" s="52"/>
-      <c r="F229" s="52"/>
-      <c r="G229" s="53"/>
-      <c r="H229" s="52"/>
-      <c r="I229" s="52"/>
-      <c r="J229" s="52"/>
-      <c r="K229" s="52"/>
-      <c r="L229" s="52"/>
-      <c r="M229" s="53"/>
+      <c r="D229" s="52">
+        <v>8795.03</v>
+      </c>
+      <c r="E229" s="52">
+        <v>0</v>
+      </c>
+      <c r="F229" s="52">
+        <v>8795.03</v>
+      </c>
+      <c r="G229" s="53">
+        <v>1</v>
+      </c>
+      <c r="H229" s="52">
+        <v>6369.12</v>
+      </c>
+      <c r="I229" s="52">
+        <v>0</v>
+      </c>
+      <c r="J229" s="52">
+        <v>4527.889999999999</v>
+      </c>
+      <c r="K229" s="52">
+        <v>0</v>
+      </c>
+      <c r="L229" s="52">
+        <v>4527.889999999999</v>
+      </c>
+      <c r="M229" s="53">
+        <v>1</v>
+      </c>
       <c r="N229" s="53"/>
-      <c r="O229" s="52"/>
-      <c r="P229" s="52"/>
-      <c r="Q229" s="52"/>
-      <c r="R229" s="53"/>
-      <c r="S229" s="54"/>
-      <c r="T229" s="54"/>
-      <c r="U229" s="54"/>
-      <c r="V229" s="53"/>
+      <c r="O229" s="52">
+        <v>1841.23</v>
+      </c>
+      <c r="P229" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q229" s="52">
+        <v>1841.23</v>
+      </c>
+      <c r="R229" s="53">
+        <v>1</v>
+      </c>
+      <c r="S229" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="T229" s="54">
+        <v>0</v>
+      </c>
+      <c r="U229" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="V229" s="53">
+        <v>1</v>
+      </c>
       <c r="W229" s="53"/>
-      <c r="X229" s="55"/>
-      <c r="Y229" s="55"/>
-      <c r="Z229" s="53"/>
-      <c r="AA229" s="56"/>
+      <c r="X229" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y229" s="55">
+        <v>65.70711175027087</v>
+      </c>
+      <c r="Z229" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA229" s="56">
+        <v>0.2758</v>
+      </c>
       <c r="AB229" s="57"/>
       <c r="AD229" s="35"/>
       <c r="AE229" s="36"/>
@@ -21803,7 +21891,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R71"/>
+  <dimension ref="A1:AD71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -21817,7 +21905,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -21839,7 +21927,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>102</v>
       </c>
@@ -21887,7 +21975,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -21905,7 +21993,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -21952,7 +22040,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -21969,7 +22057,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -22019,7 +22107,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -22036,7 +22124,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -22079,7 +22167,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -22096,7 +22184,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -22143,7 +22231,7 @@
         <v>24.375135929463628</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -22160,7 +22248,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -22210,7 +22298,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -22227,7 +22315,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -22274,7 +22362,7 @@
         <v>89.17785714285712</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -22291,7 +22379,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -22336,7 +22424,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -22353,7 +22441,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -22403,7 +22491,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -22420,7 +22508,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -22459,7 +22547,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -22476,7 +22564,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -22517,7 +22605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -22534,7 +22622,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -22573,7 +22661,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -22590,7 +22678,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -22635,7 +22723,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -22652,7 +22740,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -22695,7 +22783,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -22712,7 +22800,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -22755,7 +22843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -22772,7 +22860,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -22819,7 +22907,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -22836,7 +22924,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -22881,7 +22969,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -22898,7 +22986,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -22941,7 +23029,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -22958,7 +23046,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -22999,7 +23087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -23016,7 +23104,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -23061,7 +23149,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -23078,7 +23166,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -23121,7 +23209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -23138,7 +23226,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -23175,7 +23263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -23192,7 +23280,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -23233,7 +23321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -23250,7 +23338,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -23293,7 +23381,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -23310,7 +23398,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -23352,7 +23440,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -23369,7 +23457,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -23414,7 +23502,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -23431,7 +23519,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -23476,7 +23564,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -23493,7 +23581,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -23538,7 +23626,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -23555,7 +23643,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -23592,7 +23680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -23609,7 +23697,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -23626,7 +23714,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -23643,7 +23731,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -23664,7 +23752,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -23681,7 +23769,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -23722,7 +23810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -23739,7 +23827,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -23784,7 +23872,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -23819,7 +23907,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -23836,7 +23924,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -23853,7 +23941,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>122</v>
       </c>
@@ -23888,7 +23976,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>126</v>
@@ -24271,7 +24359,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB110"/>
+  <dimension ref="A1:AD110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -24282,7 +24370,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -24303,7 +24391,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>127</v>
@@ -24365,7 +24453,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>143</v>
       </c>
@@ -24423,7 +24511,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -24459,7 +24547,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -24478,7 +24566,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -24512,7 +24600,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -24531,7 +24619,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -24565,7 +24653,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -24584,7 +24672,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -24622,7 +24710,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -24641,7 +24729,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -24679,7 +24767,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -24698,7 +24786,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -24736,7 +24824,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -24755,7 +24843,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -24788,7 +24876,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -24807,7 +24895,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -24840,7 +24928,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -24859,7 +24947,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -24890,7 +24978,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -24909,7 +24997,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -24944,7 +25032,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -24963,7 +25051,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24996,7 +25084,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -25015,7 +25103,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25046,7 +25134,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -25065,7 +25153,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25097,7 +25185,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -25116,7 +25204,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -25152,7 +25240,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -25171,7 +25259,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -25200,7 +25288,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -25219,7 +25307,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -25250,7 +25338,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -25269,7 +25357,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -25302,7 +25390,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -25321,7 +25409,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -25357,7 +25445,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -25376,7 +25464,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -25411,7 +25499,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -25430,7 +25518,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -25460,7 +25548,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -25479,7 +25567,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -25519,7 +25607,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -25538,7 +25626,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -25567,7 +25655,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -25586,7 +25674,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -25619,7 +25707,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -25638,7 +25726,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -25671,7 +25759,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -25690,7 +25778,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -25726,7 +25814,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -25745,7 +25833,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -25781,7 +25869,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -25800,7 +25888,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -25834,7 +25922,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -25853,7 +25941,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -25888,7 +25976,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -25907,7 +25995,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -25926,7 +26014,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -25945,7 +26033,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -25966,7 +26054,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -25985,7 +26073,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -26018,7 +26106,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -26037,7 +26125,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -26076,7 +26164,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -26105,7 +26193,7 @@
       <c r="P67" s="54"/>
       <c r="Q67" s="54"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -26124,7 +26212,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="142"/>
       <c r="B69" s="143"/>
       <c r="C69" s="35"/>
@@ -26143,7 +26231,7 @@
       <c r="P69" s="35"/>
       <c r="Q69" s="144"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="145"/>
       <c r="B70" s="145"/>
       <c r="C70" s="145"/>
@@ -26162,7 +26250,7 @@
       <c r="P70" s="145"/>
       <c r="Q70" s="145"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="146" t="s">
         <v>147</v>
@@ -26207,7 +26295,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -26246,7 +26334,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="77" t="s">
         <v>149</v>
@@ -26275,7 +26363,7 @@
       <c r="P73" s="20"/>
       <c r="Q73" s="20"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="148" t="s">
         <v>150</v>
@@ -26320,7 +26408,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="151" t="s">
         <v>151</v>
@@ -26365,7 +26453,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
@@ -26384,7 +26472,7 @@
       <c r="P76" s="35"/>
       <c r="Q76" s="144"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="156" t="s">
         <v>152</v>
@@ -26431,7 +26519,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="161"/>
       <c r="B78" s="162" t="s">
         <v>154</v>
@@ -26476,7 +26564,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -26495,7 +26583,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="164" t="s">
         <v>155</v>
@@ -26518,7 +26606,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="167" t="s">
         <v>157</v>
@@ -26541,7 +26629,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -26564,7 +26652,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -26587,7 +26675,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -26610,7 +26698,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -26633,7 +26721,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -26656,7 +26744,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -26679,7 +26767,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -26702,7 +26790,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -26725,7 +26813,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -26748,7 +26836,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -26771,7 +26859,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -26792,7 +26880,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -26813,7 +26901,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -26834,7 +26922,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -26855,7 +26943,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -26876,7 +26964,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -26897,7 +26985,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -26918,7 +27006,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -26941,7 +27029,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -26964,7 +27052,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -26987,7 +27075,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -27010,7 +27098,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -27033,7 +27121,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -27056,7 +27144,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -27079,7 +27167,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -27098,7 +27186,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -27117,7 +27205,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19"/>
       <c r="C108" s="131"/>
@@ -27136,7 +27224,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="169"/>
       <c r="C109" s="150"/>
@@ -27155,7 +27243,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="164" t="s">
         <v>175</v>
@@ -27229,10 +27317,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>176</v>
       </c>
@@ -27264,7 +27353,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>177</v>
       </c>
@@ -27297,7 +27386,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>178</v>
       </c>
@@ -27330,7 +27419,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>179</v>
       </c>
@@ -27363,7 +27452,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>180</v>
       </c>
@@ -27396,7 +27485,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>181</v>
       </c>
@@ -27429,7 +27518,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>182</v>
       </c>
@@ -27462,7 +27551,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>183</v>
       </c>
@@ -27495,7 +27584,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -27526,7 +27615,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -27557,7 +27646,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>184</v>
       </c>
@@ -27590,7 +27679,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>185</v>
       </c>
@@ -27623,7 +27712,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>186</v>
       </c>
@@ -27656,7 +27745,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>187</v>
       </c>
@@ -27689,7 +27778,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>188</v>
       </c>
@@ -27722,7 +27811,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>189</v>
       </c>
@@ -27755,7 +27844,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>190</v>
       </c>
@@ -27788,7 +27877,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>191</v>
       </c>
@@ -27821,7 +27910,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>192</v>
       </c>
@@ -27854,7 +27943,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>193</v>
       </c>
@@ -27887,7 +27976,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>194</v>
       </c>
@@ -27920,7 +28009,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>195</v>
       </c>
@@ -27953,7 +28042,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>196</v>
       </c>
@@ -27986,7 +28075,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>197</v>
       </c>
@@ -28019,7 +28108,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>198</v>
       </c>
@@ -28052,7 +28141,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>199</v>
       </c>
@@ -28085,7 +28174,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>200</v>
       </c>
@@ -28117,7 +28206,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>201</v>
       </c>
@@ -28149,7 +28238,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>202</v>
       </c>
@@ -28181,7 +28270,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>203</v>
       </c>
@@ -28213,7 +28302,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>204</v>
       </c>
@@ -28245,7 +28334,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -28275,7 +28364,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -28305,7 +28394,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>205</v>
       </c>
@@ -28337,7 +28426,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>206</v>
       </c>
@@ -28369,7 +28458,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>207</v>
       </c>
@@ -28401,7 +28490,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>208</v>
       </c>
@@ -28433,7 +28522,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>209</v>
       </c>
@@ -28465,7 +28554,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -28495,7 +28584,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>210</v>
       </c>
@@ -28527,7 +28616,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>211</v>
       </c>
@@ -28559,7 +28648,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>212</v>
       </c>
@@ -28591,7 +28680,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>213</v>
       </c>
@@ -28623,7 +28712,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -28653,7 +28742,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -28683,7 +28772,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -28713,7 +28802,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -28743,7 +28832,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>214</v>
       </c>
@@ -28775,7 +28864,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>215</v>
       </c>
@@ -28807,7 +28896,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -28837,7 +28926,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -28867,7 +28956,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -28897,7 +28986,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -28927,7 +29016,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -28957,7 +29046,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -29052,10 +29141,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>216</v>
       </c>
@@ -29087,7 +29177,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -29118,7 +29208,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -29149,7 +29239,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -29180,7 +29270,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -29211,7 +29301,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -29242,7 +29332,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -29273,7 +29363,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -29304,7 +29394,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -29335,7 +29425,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -29366,7 +29456,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -29397,7 +29487,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -29428,7 +29518,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -29459,7 +29549,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -29490,7 +29580,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -29521,7 +29611,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -29552,7 +29642,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -29583,7 +29673,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -29614,7 +29704,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -29645,7 +29735,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -29676,7 +29766,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -29706,7 +29796,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -29736,7 +29826,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -29766,7 +29856,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -29796,7 +29886,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -29826,7 +29916,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -29856,7 +29946,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -29886,7 +29976,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -29916,7 +30006,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -29946,7 +30036,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -29976,7 +30066,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -30006,7 +30096,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -30036,7 +30126,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -30066,7 +30156,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -30096,7 +30186,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -30126,7 +30216,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -30156,7 +30246,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>214</v>
       </c>
@@ -30188,7 +30278,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>215</v>
       </c>
@@ -30220,7 +30310,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -30250,7 +30340,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -30280,7 +30370,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -30310,7 +30400,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -30340,7 +30430,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -30370,7 +30460,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -52113,19 +52203,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -52139,7 +52229,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>223</v>
       </c>
@@ -52151,7 +52241,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>224</v>
       </c>
@@ -52162,7 +52252,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>225</v>
       </c>
@@ -52173,7 +52263,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>226</v>
       </c>
@@ -52184,13 +52274,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-07T21:11:33Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -9864,30 +9864,74 @@
       <c r="C6" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D6" s="52"/>
-      <c r="E6" s="52"/>
-      <c r="F6" s="52"/>
-      <c r="G6" s="53"/>
-      <c r="H6" s="52"/>
-      <c r="I6" s="52"/>
-      <c r="J6" s="52"/>
-      <c r="K6" s="52"/>
-      <c r="L6" s="52"/>
-      <c r="M6" s="53"/>
+      <c r="D6" s="52">
+        <v>245679.5</v>
+      </c>
+      <c r="E6" s="52">
+        <v>216530.08</v>
+      </c>
+      <c r="F6" s="52">
+        <v>29149.420000000013</v>
+      </c>
+      <c r="G6" s="53">
+        <v>0.11864815745717495</v>
+      </c>
+      <c r="H6" s="52">
+        <v>208360.5</v>
+      </c>
+      <c r="I6" s="52">
+        <v>168361.6</v>
+      </c>
+      <c r="J6" s="52">
+        <v>180366.49</v>
+      </c>
+      <c r="K6" s="52">
+        <v>138438.46000000002</v>
+      </c>
+      <c r="L6" s="52">
+        <v>41928.02999999997</v>
+      </c>
+      <c r="M6" s="53">
+        <v>0.23246019812216767</v>
+      </c>
       <c r="N6" s="53"/>
-      <c r="O6" s="52"/>
-      <c r="P6" s="52"/>
-      <c r="Q6" s="52"/>
-      <c r="R6" s="53"/>
-      <c r="S6" s="54"/>
-      <c r="T6" s="54"/>
-      <c r="U6" s="54"/>
-      <c r="V6" s="53"/>
+      <c r="O6" s="52">
+        <v>27994.01</v>
+      </c>
+      <c r="P6" s="52">
+        <v>29923.14</v>
+      </c>
+      <c r="Q6" s="52">
+        <v>-1929.130000000001</v>
+      </c>
+      <c r="R6" s="53">
+        <v>-0.06891224229754869</v>
+      </c>
+      <c r="S6" s="54">
+        <v>565.45</v>
+      </c>
+      <c r="T6" s="54">
+        <v>600.25</v>
+      </c>
+      <c r="U6" s="54">
+        <v>-34.799999999999955</v>
+      </c>
+      <c r="V6" s="53">
+        <v>-0.061543903086037584</v>
+      </c>
       <c r="W6" s="53"/>
-      <c r="X6" s="55"/>
-      <c r="Y6" s="55"/>
-      <c r="Z6" s="53"/>
-      <c r="AA6" s="56"/>
+      <c r="X6" s="55">
+        <v>80.24736359850063</v>
+      </c>
+      <c r="Y6" s="55">
+        <v>65.99877634098505</v>
+      </c>
+      <c r="Z6" s="53">
+        <v>0.2225</v>
+      </c>
+      <c r="AA6" s="56">
+        <v>0.1519</v>
+      </c>
       <c r="AB6" s="57"/>
       <c r="AD6" s="35"/>
       <c r="AE6" s="35"/>
@@ -10227,30 +10271,74 @@
       <c r="C13" s="63" t="s">
         <v>96</v>
       </c>
-      <c r="D13" s="52"/>
-      <c r="E13" s="62"/>
-      <c r="F13" s="52"/>
-      <c r="G13" s="53"/>
-      <c r="H13" s="52"/>
-      <c r="I13" s="52"/>
-      <c r="J13" s="52"/>
-      <c r="K13" s="52"/>
-      <c r="L13" s="52"/>
-      <c r="M13" s="53"/>
+      <c r="D13" s="52">
+        <v>129074.86</v>
+      </c>
+      <c r="E13" s="62">
+        <v>85864.08</v>
+      </c>
+      <c r="F13" s="52">
+        <v>43210.78</v>
+      </c>
+      <c r="G13" s="53">
+        <v>0.3347730146676123</v>
+      </c>
+      <c r="H13" s="52">
+        <v>101420.72</v>
+      </c>
+      <c r="I13" s="52">
+        <v>79791.03</v>
+      </c>
+      <c r="J13" s="52">
+        <v>83645.65</v>
+      </c>
+      <c r="K13" s="52">
+        <v>71604.5</v>
+      </c>
+      <c r="L13" s="52">
+        <v>12041.149999999994</v>
+      </c>
+      <c r="M13" s="53">
+        <v>0.1439542881189876</v>
+      </c>
       <c r="N13" s="53"/>
-      <c r="O13" s="52"/>
-      <c r="P13" s="52"/>
-      <c r="Q13" s="52"/>
-      <c r="R13" s="53"/>
-      <c r="S13" s="54"/>
-      <c r="T13" s="54"/>
-      <c r="U13" s="54"/>
-      <c r="V13" s="53"/>
+      <c r="O13" s="52">
+        <v>17775.07</v>
+      </c>
+      <c r="P13" s="52">
+        <v>8186.53</v>
+      </c>
+      <c r="Q13" s="52">
+        <v>9588.54</v>
+      </c>
+      <c r="R13" s="53">
+        <v>0.5394375380800188</v>
+      </c>
+      <c r="S13" s="54">
+        <v>356.07</v>
+      </c>
+      <c r="T13" s="54">
+        <v>168.25</v>
+      </c>
+      <c r="U13" s="54">
+        <v>187.82</v>
+      </c>
+      <c r="V13" s="53">
+        <v>0.5274805515769371</v>
+      </c>
       <c r="W13" s="53"/>
-      <c r="X13" s="55"/>
-      <c r="Y13" s="55"/>
-      <c r="Z13" s="53"/>
-      <c r="AA13" s="56"/>
+      <c r="X13" s="55">
+        <v>36.09539375928678</v>
+      </c>
+      <c r="Y13" s="55">
+        <v>77.66490997775718</v>
+      </c>
+      <c r="Z13" s="53">
+        <v>0.0707</v>
+      </c>
+      <c r="AA13" s="56">
+        <v>0.2142</v>
+      </c>
       <c r="AB13" s="57"/>
       <c r="AD13" s="35"/>
       <c r="AE13" s="35"/>
@@ -10590,30 +10678,74 @@
       <c r="C20" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D20" s="52"/>
-      <c r="E20" s="52"/>
-      <c r="F20" s="52"/>
-      <c r="G20" s="53"/>
-      <c r="H20" s="52"/>
-      <c r="I20" s="52"/>
-      <c r="J20" s="52"/>
-      <c r="K20" s="52"/>
-      <c r="L20" s="52"/>
-      <c r="M20" s="53"/>
+      <c r="D20" s="52">
+        <v>27500.32</v>
+      </c>
+      <c r="E20" s="52">
+        <v>11999.08</v>
+      </c>
+      <c r="F20" s="52">
+        <v>15501.24</v>
+      </c>
+      <c r="G20" s="53">
+        <v>0.5636748954193987</v>
+      </c>
+      <c r="H20" s="52">
+        <v>19565.83</v>
+      </c>
+      <c r="I20" s="52">
+        <v>7921.92</v>
+      </c>
+      <c r="J20" s="52">
+        <v>13767.340000000002</v>
+      </c>
+      <c r="K20" s="52">
+        <v>6211.24</v>
+      </c>
+      <c r="L20" s="52">
+        <v>7556.100000000002</v>
+      </c>
+      <c r="M20" s="53">
+        <v>0.5488424052867149</v>
+      </c>
       <c r="N20" s="53"/>
-      <c r="O20" s="52"/>
-      <c r="P20" s="52"/>
-      <c r="Q20" s="52"/>
-      <c r="R20" s="53"/>
-      <c r="S20" s="54"/>
-      <c r="T20" s="54"/>
-      <c r="U20" s="54"/>
-      <c r="V20" s="53"/>
+      <c r="O20" s="52">
+        <v>5798.49</v>
+      </c>
+      <c r="P20" s="52">
+        <v>1710.68</v>
+      </c>
+      <c r="Q20" s="52">
+        <v>4087.8099999999995</v>
+      </c>
+      <c r="R20" s="53">
+        <v>0.7049783650571096</v>
+      </c>
+      <c r="S20" s="54">
+        <v>125.39</v>
+      </c>
+      <c r="T20" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U20" s="54">
+        <v>90.64</v>
+      </c>
+      <c r="V20" s="53">
+        <v>0.7228646622537682</v>
+      </c>
       <c r="W20" s="53"/>
-      <c r="X20" s="55"/>
-      <c r="Y20" s="55"/>
-      <c r="Z20" s="53"/>
-      <c r="AA20" s="56"/>
+      <c r="X20" s="55">
+        <v>117.328345323741</v>
+      </c>
+      <c r="Y20" s="55">
+        <v>63.27846478985563</v>
+      </c>
+      <c r="Z20" s="53">
+        <v>0.3398</v>
+      </c>
+      <c r="AA20" s="56">
+        <v>0.2885</v>
+      </c>
       <c r="AB20" s="57"/>
       <c r="AD20" s="35"/>
       <c r="AE20" s="35"/>
@@ -10955,30 +11087,74 @@
       <c r="C27" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D27" s="55"/>
-      <c r="E27" s="55"/>
-      <c r="F27" s="52"/>
-      <c r="G27" s="53"/>
-      <c r="H27" s="52"/>
-      <c r="I27" s="52"/>
-      <c r="J27" s="52"/>
-      <c r="K27" s="52"/>
-      <c r="L27" s="52"/>
-      <c r="M27" s="53"/>
+      <c r="D27" s="55">
+        <v>150850.82</v>
+      </c>
+      <c r="E27" s="55">
+        <v>144370.8</v>
+      </c>
+      <c r="F27" s="52">
+        <v>6480.020000000019</v>
+      </c>
+      <c r="G27" s="53">
+        <v>0.042956478459978</v>
+      </c>
+      <c r="H27" s="52">
+        <v>102178.42</v>
+      </c>
+      <c r="I27" s="52">
+        <v>89222.05</v>
+      </c>
+      <c r="J27" s="52">
+        <v>62464.86</v>
+      </c>
+      <c r="K27" s="52">
+        <v>58984</v>
+      </c>
+      <c r="L27" s="52">
+        <v>3480.8600000000006</v>
+      </c>
+      <c r="M27" s="53">
+        <v>0.05572509087509362</v>
+      </c>
       <c r="N27" s="53"/>
-      <c r="O27" s="52"/>
-      <c r="P27" s="52"/>
-      <c r="Q27" s="52"/>
-      <c r="R27" s="53"/>
-      <c r="S27" s="54"/>
-      <c r="T27" s="54"/>
-      <c r="U27" s="54"/>
-      <c r="V27" s="53"/>
+      <c r="O27" s="52">
+        <v>39713.56</v>
+      </c>
+      <c r="P27" s="52">
+        <v>30238.05</v>
+      </c>
+      <c r="Q27" s="52">
+        <v>9475.509999999998</v>
+      </c>
+      <c r="R27" s="53">
+        <v>0.23859633837913294</v>
+      </c>
+      <c r="S27" s="54">
+        <v>795.22</v>
+      </c>
+      <c r="T27" s="54">
+        <v>615</v>
+      </c>
+      <c r="U27" s="54">
+        <v>180.22000000000003</v>
+      </c>
+      <c r="V27" s="53">
+        <v>0.22662910892583188</v>
+      </c>
       <c r="W27" s="53"/>
-      <c r="X27" s="55"/>
-      <c r="Y27" s="55"/>
-      <c r="Z27" s="53"/>
-      <c r="AA27" s="56"/>
+      <c r="X27" s="55">
+        <v>89.67276422764228</v>
+      </c>
+      <c r="Y27" s="55">
+        <v>61.20621468124544</v>
+      </c>
+      <c r="Z27" s="53">
+        <v>0.382</v>
+      </c>
+      <c r="AA27" s="56">
+        <v>0.3227</v>
+      </c>
       <c r="AB27" s="57"/>
       <c r="AD27" s="35"/>
       <c r="AE27" s="35"/>
@@ -11318,30 +11494,74 @@
       <c r="C34" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D34" s="52"/>
-      <c r="E34" s="52"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="53"/>
-      <c r="H34" s="52"/>
-      <c r="I34" s="65"/>
-      <c r="J34" s="52"/>
-      <c r="K34" s="52"/>
-      <c r="L34" s="52"/>
-      <c r="M34" s="53"/>
+      <c r="D34" s="52">
+        <v>396422.03</v>
+      </c>
+      <c r="E34" s="52">
+        <v>259347.71</v>
+      </c>
+      <c r="F34" s="52">
+        <v>137074.32000000004</v>
+      </c>
+      <c r="G34" s="53">
+        <v>0.3457787651205964</v>
+      </c>
+      <c r="H34" s="52">
+        <v>327431.12</v>
+      </c>
+      <c r="I34" s="65">
+        <v>223659.54</v>
+      </c>
+      <c r="J34" s="52">
+        <v>271519.78</v>
+      </c>
+      <c r="K34" s="52">
+        <v>197370.72</v>
+      </c>
+      <c r="L34" s="52">
+        <v>74149.06000000003</v>
+      </c>
+      <c r="M34" s="53">
+        <v>0.27308898084699396</v>
+      </c>
       <c r="N34" s="53"/>
-      <c r="O34" s="52"/>
-      <c r="P34" s="52"/>
-      <c r="Q34" s="52"/>
-      <c r="R34" s="53"/>
-      <c r="S34" s="54"/>
-      <c r="T34" s="54"/>
-      <c r="U34" s="54"/>
-      <c r="V34" s="53"/>
+      <c r="O34" s="52">
+        <v>55911.34</v>
+      </c>
+      <c r="P34" s="52">
+        <v>26288.82</v>
+      </c>
+      <c r="Q34" s="52">
+        <v>29622.519999999997</v>
+      </c>
+      <c r="R34" s="53">
+        <v>0.5298123779540966</v>
+      </c>
+      <c r="S34" s="54">
+        <v>1120.27</v>
+      </c>
+      <c r="T34" s="54">
+        <v>607.75</v>
+      </c>
+      <c r="U34" s="54">
+        <v>512.52</v>
+      </c>
+      <c r="V34" s="53">
+        <v>0.4574968534371178</v>
+      </c>
       <c r="W34" s="53"/>
-      <c r="X34" s="55"/>
-      <c r="Y34" s="55"/>
-      <c r="Z34" s="53"/>
-      <c r="AA34" s="56"/>
+      <c r="X34" s="55">
+        <v>58.721793500617025</v>
+      </c>
+      <c r="Y34" s="55">
+        <v>61.5841822414239</v>
+      </c>
+      <c r="Z34" s="53">
+        <v>0.1376</v>
+      </c>
+      <c r="AA34" s="56">
+        <v>0.174</v>
+      </c>
       <c r="AB34" s="57"/>
       <c r="AD34" s="35"/>
       <c r="AE34" s="35"/>
@@ -11681,30 +11901,74 @@
       <c r="C41" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D41" s="52"/>
-      <c r="E41" s="52"/>
-      <c r="F41" s="52"/>
-      <c r="G41" s="53"/>
-      <c r="H41" s="52"/>
-      <c r="I41" s="52"/>
-      <c r="J41" s="52"/>
-      <c r="K41" s="52"/>
-      <c r="L41" s="52"/>
-      <c r="M41" s="53"/>
+      <c r="D41" s="52">
+        <v>128258.5</v>
+      </c>
+      <c r="E41" s="52">
+        <v>53944.83</v>
+      </c>
+      <c r="F41" s="52">
+        <v>74313.67</v>
+      </c>
+      <c r="G41" s="53">
+        <v>0.5794054195238522</v>
+      </c>
+      <c r="H41" s="52">
+        <v>94098.32</v>
+      </c>
+      <c r="I41" s="52">
+        <v>49261.61</v>
+      </c>
+      <c r="J41" s="52">
+        <v>69042.09000000001</v>
+      </c>
+      <c r="K41" s="52">
+        <v>35683.74</v>
+      </c>
+      <c r="L41" s="52">
+        <v>33358.35000000001</v>
+      </c>
+      <c r="M41" s="53">
+        <v>0.4831596204576079</v>
+      </c>
       <c r="N41" s="53"/>
-      <c r="O41" s="52"/>
-      <c r="P41" s="52"/>
-      <c r="Q41" s="52"/>
-      <c r="R41" s="53"/>
-      <c r="S41" s="54"/>
-      <c r="T41" s="54"/>
-      <c r="U41" s="54"/>
-      <c r="V41" s="53"/>
+      <c r="O41" s="52">
+        <v>25056.23</v>
+      </c>
+      <c r="P41" s="52">
+        <v>13577.87</v>
+      </c>
+      <c r="Q41" s="52">
+        <v>11478.359999999999</v>
+      </c>
+      <c r="R41" s="53">
+        <v>0.45810403241030273</v>
+      </c>
+      <c r="S41" s="54">
+        <v>501.83</v>
+      </c>
+      <c r="T41" s="54">
+        <v>299.5</v>
+      </c>
+      <c r="U41" s="54">
+        <v>202.32999999999998</v>
+      </c>
+      <c r="V41" s="53">
+        <v>0.40318434529621583</v>
+      </c>
       <c r="W41" s="53"/>
-      <c r="X41" s="55"/>
-      <c r="Y41" s="55"/>
-      <c r="Z41" s="53"/>
-      <c r="AA41" s="56"/>
+      <c r="X41" s="55">
+        <v>15.63679465776294</v>
+      </c>
+      <c r="Y41" s="55">
+        <v>68.07122423898531</v>
+      </c>
+      <c r="Z41" s="53">
+        <v>0.0868</v>
+      </c>
+      <c r="AA41" s="56">
+        <v>0.2663</v>
+      </c>
       <c r="AB41" s="57"/>
       <c r="AD41" s="35"/>
       <c r="AE41" s="35"/>
@@ -12046,30 +12310,74 @@
       <c r="C48" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D48" s="52"/>
-      <c r="E48" s="52"/>
-      <c r="F48" s="52"/>
-      <c r="G48" s="53"/>
-      <c r="H48" s="52"/>
-      <c r="I48" s="52"/>
-      <c r="J48" s="52"/>
-      <c r="K48" s="52"/>
-      <c r="L48" s="52"/>
-      <c r="M48" s="53"/>
+      <c r="D48" s="52">
+        <v>65693.36</v>
+      </c>
+      <c r="E48" s="52">
+        <v>33326.49</v>
+      </c>
+      <c r="F48" s="52">
+        <v>32366.870000000003</v>
+      </c>
+      <c r="G48" s="53">
+        <v>0.49269621769993194</v>
+      </c>
+      <c r="H48" s="52">
+        <v>50582.37</v>
+      </c>
+      <c r="I48" s="52">
+        <v>25196.36</v>
+      </c>
+      <c r="J48" s="52">
+        <v>39438.990000000005</v>
+      </c>
+      <c r="K48" s="52">
+        <v>20036.420000000002</v>
+      </c>
+      <c r="L48" s="52">
+        <v>19402.570000000003</v>
+      </c>
+      <c r="M48" s="53">
+        <v>0.49196417048205343</v>
+      </c>
       <c r="N48" s="53"/>
-      <c r="O48" s="52"/>
-      <c r="P48" s="52"/>
-      <c r="Q48" s="52"/>
-      <c r="R48" s="53"/>
-      <c r="S48" s="54"/>
-      <c r="T48" s="54"/>
-      <c r="U48" s="54"/>
-      <c r="V48" s="53"/>
+      <c r="O48" s="52">
+        <v>11143.38</v>
+      </c>
+      <c r="P48" s="52">
+        <v>5159.94</v>
+      </c>
+      <c r="Q48" s="52">
+        <v>5983.44</v>
+      </c>
+      <c r="R48" s="53">
+        <v>0.5369501892603501</v>
+      </c>
+      <c r="S48" s="54">
+        <v>223.22</v>
+      </c>
+      <c r="T48" s="54">
+        <v>113.25</v>
+      </c>
+      <c r="U48" s="54">
+        <v>109.97</v>
+      </c>
+      <c r="V48" s="53">
+        <v>0.49265298808350505</v>
+      </c>
       <c r="W48" s="53"/>
-      <c r="X48" s="55"/>
-      <c r="Y48" s="55"/>
-      <c r="Z48" s="53"/>
-      <c r="AA48" s="56"/>
+      <c r="X48" s="55">
+        <v>71.78922737306843</v>
+      </c>
+      <c r="Y48" s="55">
+        <v>67.69550512136009</v>
+      </c>
+      <c r="Z48" s="53">
+        <v>0.244</v>
+      </c>
+      <c r="AA48" s="56">
+        <v>0.23</v>
+      </c>
       <c r="AB48" s="57"/>
       <c r="AD48" s="35"/>
       <c r="AE48" s="35"/>
@@ -12409,30 +12717,74 @@
       <c r="C55" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D55" s="52"/>
-      <c r="E55" s="52"/>
-      <c r="F55" s="52"/>
-      <c r="G55" s="53"/>
-      <c r="H55" s="52"/>
-      <c r="I55" s="52"/>
-      <c r="J55" s="52"/>
-      <c r="K55" s="52"/>
-      <c r="L55" s="52"/>
-      <c r="M55" s="53"/>
+      <c r="D55" s="52">
+        <v>155296.79</v>
+      </c>
+      <c r="E55" s="52">
+        <v>127814.48</v>
+      </c>
+      <c r="F55" s="52">
+        <v>27482.310000000012</v>
+      </c>
+      <c r="G55" s="53">
+        <v>0.176966375158173</v>
+      </c>
+      <c r="H55" s="52">
+        <v>109364.97</v>
+      </c>
+      <c r="I55" s="52">
+        <v>96483.38</v>
+      </c>
+      <c r="J55" s="52">
+        <v>75135.01000000001</v>
+      </c>
+      <c r="K55" s="52">
+        <v>71221.34</v>
+      </c>
+      <c r="L55" s="52">
+        <v>3913.670000000013</v>
+      </c>
+      <c r="M55" s="53">
+        <v>0.05208850042077604</v>
+      </c>
       <c r="N55" s="53"/>
-      <c r="O55" s="52"/>
-      <c r="P55" s="52"/>
-      <c r="Q55" s="52"/>
-      <c r="R55" s="53"/>
-      <c r="S55" s="54"/>
-      <c r="T55" s="54"/>
-      <c r="U55" s="54"/>
-      <c r="V55" s="53"/>
+      <c r="O55" s="52">
+        <v>34229.96</v>
+      </c>
+      <c r="P55" s="52">
+        <v>25262.04</v>
+      </c>
+      <c r="Q55" s="52">
+        <v>8967.919999999998</v>
+      </c>
+      <c r="R55" s="53">
+        <v>0.2619903733454552</v>
+      </c>
+      <c r="S55" s="54">
+        <v>685.48</v>
+      </c>
+      <c r="T55" s="54">
+        <v>533.75</v>
+      </c>
+      <c r="U55" s="54">
+        <v>151.73000000000002</v>
+      </c>
+      <c r="V55" s="53">
+        <v>0.22134854408589605</v>
+      </c>
       <c r="W55" s="53"/>
-      <c r="X55" s="55"/>
-      <c r="Y55" s="55"/>
-      <c r="Z55" s="53"/>
-      <c r="AA55" s="56"/>
+      <c r="X55" s="55">
+        <v>58.699953161592504</v>
+      </c>
+      <c r="Y55" s="55">
+        <v>67.00679527854935</v>
+      </c>
+      <c r="Z55" s="53">
+        <v>0.2451</v>
+      </c>
+      <c r="AA55" s="56">
+        <v>0.2958</v>
+      </c>
       <c r="AB55" s="57"/>
       <c r="AD55" s="35"/>
       <c r="AE55" s="35"/>
@@ -12772,30 +13124,74 @@
       <c r="C62" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D62" s="52"/>
-      <c r="E62" s="52"/>
-      <c r="F62" s="52"/>
-      <c r="G62" s="53"/>
-      <c r="H62" s="52"/>
-      <c r="I62" s="52"/>
-      <c r="J62" s="52"/>
-      <c r="K62" s="52"/>
-      <c r="L62" s="52"/>
-      <c r="M62" s="53"/>
+      <c r="D62" s="52">
+        <v>20420.56</v>
+      </c>
+      <c r="E62" s="52">
+        <v>20420.56</v>
+      </c>
+      <c r="F62" s="52">
+        <v>0</v>
+      </c>
+      <c r="G62" s="53">
+        <v>0</v>
+      </c>
+      <c r="H62" s="52">
+        <v>15859.68</v>
+      </c>
+      <c r="I62" s="52">
+        <v>13435.12</v>
+      </c>
+      <c r="J62" s="52">
+        <v>12689.1</v>
+      </c>
+      <c r="K62" s="52">
+        <v>11478.25</v>
+      </c>
+      <c r="L62" s="52">
+        <v>1210.8500000000004</v>
+      </c>
+      <c r="M62" s="53">
+        <v>0.09542441938356545</v>
+      </c>
       <c r="N62" s="53"/>
-      <c r="O62" s="52"/>
-      <c r="P62" s="52"/>
-      <c r="Q62" s="52"/>
-      <c r="R62" s="53"/>
-      <c r="S62" s="54"/>
-      <c r="T62" s="54"/>
-      <c r="U62" s="54"/>
-      <c r="V62" s="53"/>
+      <c r="O62" s="52">
+        <v>3170.58</v>
+      </c>
+      <c r="P62" s="52">
+        <v>1956.87</v>
+      </c>
+      <c r="Q62" s="52">
+        <v>1213.71</v>
+      </c>
+      <c r="R62" s="53">
+        <v>0.38280377722687964</v>
+      </c>
+      <c r="S62" s="54">
+        <v>63.5</v>
+      </c>
+      <c r="T62" s="54">
+        <v>48.25</v>
+      </c>
+      <c r="U62" s="54">
+        <v>15.25</v>
+      </c>
+      <c r="V62" s="53">
+        <v>0.24015748031496062</v>
+      </c>
       <c r="W62" s="53"/>
-      <c r="X62" s="55"/>
-      <c r="Y62" s="55"/>
-      <c r="Z62" s="53"/>
-      <c r="AA62" s="56"/>
+      <c r="X62" s="55">
+        <v>144.7759585492228</v>
+      </c>
+      <c r="Y62" s="55">
+        <v>71.82495570677168</v>
+      </c>
+      <c r="Z62" s="53">
+        <v>0.3421</v>
+      </c>
+      <c r="AA62" s="56">
+        <v>0.2233</v>
+      </c>
       <c r="AB62" s="57"/>
       <c r="AD62" s="35"/>
       <c r="AE62" s="35"/>
@@ -13129,30 +13525,74 @@
       <c r="C69" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D69" s="52"/>
-      <c r="E69" s="52"/>
-      <c r="F69" s="52"/>
-      <c r="G69" s="53"/>
-      <c r="H69" s="52"/>
-      <c r="I69" s="52"/>
-      <c r="J69" s="52"/>
-      <c r="K69" s="52"/>
-      <c r="L69" s="52"/>
-      <c r="M69" s="53"/>
+      <c r="D69" s="52">
+        <v>47801.68</v>
+      </c>
+      <c r="E69" s="52">
+        <v>10650.43</v>
+      </c>
+      <c r="F69" s="52">
+        <v>37151.25</v>
+      </c>
+      <c r="G69" s="53">
+        <v>0.7771954876899724</v>
+      </c>
+      <c r="H69" s="52">
+        <v>35572.59</v>
+      </c>
+      <c r="I69" s="52">
+        <v>10547.08</v>
+      </c>
+      <c r="J69" s="52">
+        <v>27136.549999999996</v>
+      </c>
+      <c r="K69" s="52">
+        <v>10398.3</v>
+      </c>
+      <c r="L69" s="52">
+        <v>16738.249999999996</v>
+      </c>
+      <c r="M69" s="53">
+        <v>0.6168156969106242</v>
+      </c>
       <c r="N69" s="53"/>
-      <c r="O69" s="52"/>
-      <c r="P69" s="52"/>
-      <c r="Q69" s="52"/>
-      <c r="R69" s="53"/>
-      <c r="S69" s="54"/>
-      <c r="T69" s="54"/>
-      <c r="U69" s="54"/>
-      <c r="V69" s="53"/>
+      <c r="O69" s="52">
+        <v>8436.04</v>
+      </c>
+      <c r="P69" s="52">
+        <v>148.78</v>
+      </c>
+      <c r="Q69" s="52">
+        <v>8287.26</v>
+      </c>
+      <c r="R69" s="53">
+        <v>0.9823637630926358</v>
+      </c>
+      <c r="S69" s="54">
+        <v>169.32</v>
+      </c>
+      <c r="T69" s="54">
+        <v>2.75</v>
+      </c>
+      <c r="U69" s="54">
+        <v>166.57</v>
+      </c>
+      <c r="V69" s="53">
+        <v>0.9837585636664304</v>
+      </c>
       <c r="W69" s="53"/>
-      <c r="X69" s="55"/>
-      <c r="Y69" s="55"/>
-      <c r="Z69" s="53"/>
-      <c r="AA69" s="56"/>
+      <c r="X69" s="55">
+        <v>37.58181818181818</v>
+      </c>
+      <c r="Y69" s="55">
+        <v>72.22475431425701</v>
+      </c>
+      <c r="Z69" s="53">
+        <v>0.0097</v>
+      </c>
+      <c r="AA69" s="56">
+        <v>0.2558</v>
+      </c>
       <c r="AB69" s="57"/>
       <c r="AD69" s="35"/>
       <c r="AE69" s="35"/>
@@ -13482,30 +13922,74 @@
       <c r="C76" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D76" s="52"/>
-      <c r="E76" s="52"/>
-      <c r="F76" s="52"/>
-      <c r="G76" s="53"/>
-      <c r="H76" s="52"/>
-      <c r="I76" s="52"/>
-      <c r="J76" s="52"/>
-      <c r="K76" s="52"/>
-      <c r="L76" s="52"/>
-      <c r="M76" s="53"/>
+      <c r="D76" s="52">
+        <v>77166.16</v>
+      </c>
+      <c r="E76" s="52">
+        <v>44764.99</v>
+      </c>
+      <c r="F76" s="52">
+        <v>32401.170000000006</v>
+      </c>
+      <c r="G76" s="53">
+        <v>0.41988832928838243</v>
+      </c>
+      <c r="H76" s="52">
+        <v>54302.66</v>
+      </c>
+      <c r="I76" s="52">
+        <v>29696.65</v>
+      </c>
+      <c r="J76" s="52">
+        <v>31383.390000000003</v>
+      </c>
+      <c r="K76" s="52">
+        <v>23592.600000000002</v>
+      </c>
+      <c r="L76" s="52">
+        <v>7790.790000000001</v>
+      </c>
+      <c r="M76" s="53">
+        <v>0.24824564841465502</v>
+      </c>
       <c r="N76" s="53"/>
-      <c r="O76" s="52"/>
-      <c r="P76" s="52"/>
-      <c r="Q76" s="52"/>
-      <c r="R76" s="53"/>
-      <c r="S76" s="54"/>
-      <c r="T76" s="54"/>
-      <c r="U76" s="54"/>
-      <c r="V76" s="53"/>
+      <c r="O76" s="52">
+        <v>22919.27</v>
+      </c>
+      <c r="P76" s="52">
+        <v>6104.05</v>
+      </c>
+      <c r="Q76" s="52">
+        <v>16815.22</v>
+      </c>
+      <c r="R76" s="53">
+        <v>0.7336717094392623</v>
+      </c>
+      <c r="S76" s="54">
+        <v>470.62</v>
+      </c>
+      <c r="T76" s="54">
+        <v>120.25</v>
+      </c>
+      <c r="U76" s="54">
+        <v>350.37</v>
+      </c>
+      <c r="V76" s="53">
+        <v>0.7444859971951894</v>
+      </c>
       <c r="W76" s="53"/>
-      <c r="X76" s="55"/>
-      <c r="Y76" s="55"/>
-      <c r="Z76" s="53"/>
-      <c r="AA76" s="56"/>
+      <c r="X76" s="55">
+        <v>125.30844074844074</v>
+      </c>
+      <c r="Y76" s="55">
+        <v>48.58165977967362</v>
+      </c>
+      <c r="Z76" s="53">
+        <v>0.33659999999999995</v>
+      </c>
+      <c r="AA76" s="56">
+        <v>0.2963</v>
+      </c>
       <c r="AB76" s="57"/>
       <c r="AD76" s="35"/>
       <c r="AE76" s="35"/>
@@ -13841,30 +14325,74 @@
       <c r="C83" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D83" s="52"/>
-      <c r="E83" s="52"/>
-      <c r="F83" s="52"/>
-      <c r="G83" s="53"/>
-      <c r="H83" s="52"/>
-      <c r="I83" s="52"/>
-      <c r="J83" s="52"/>
-      <c r="K83" s="52"/>
-      <c r="L83" s="52"/>
-      <c r="M83" s="53"/>
+      <c r="D83" s="52">
+        <v>25467.84</v>
+      </c>
+      <c r="E83" s="52">
+        <v>19598.41</v>
+      </c>
+      <c r="F83" s="52">
+        <v>5869.43</v>
+      </c>
+      <c r="G83" s="53">
+        <v>0.2304643817457625</v>
+      </c>
+      <c r="H83" s="52">
+        <v>16606.83</v>
+      </c>
+      <c r="I83" s="52">
+        <v>12958.24</v>
+      </c>
+      <c r="J83" s="52">
+        <v>9659.990000000002</v>
+      </c>
+      <c r="K83" s="52">
+        <v>5354.12</v>
+      </c>
+      <c r="L83" s="52">
+        <v>4305.870000000002</v>
+      </c>
+      <c r="M83" s="53">
+        <v>0.44574269745620865</v>
+      </c>
       <c r="N83" s="53"/>
-      <c r="O83" s="52"/>
-      <c r="P83" s="52"/>
-      <c r="Q83" s="52"/>
-      <c r="R83" s="53"/>
-      <c r="S83" s="54"/>
-      <c r="T83" s="54"/>
-      <c r="U83" s="54"/>
-      <c r="V83" s="53"/>
+      <c r="O83" s="52">
+        <v>6946.84</v>
+      </c>
+      <c r="P83" s="52">
+        <v>7604.12</v>
+      </c>
+      <c r="Q83" s="52">
+        <v>-657.2799999999997</v>
+      </c>
+      <c r="R83" s="53">
+        <v>-0.09461568137455299</v>
+      </c>
+      <c r="S83" s="54">
+        <v>139.07</v>
+      </c>
+      <c r="T83" s="54">
+        <v>147.75</v>
+      </c>
+      <c r="U83" s="54">
+        <v>-8.680000000000007</v>
+      </c>
+      <c r="V83" s="53">
+        <v>-0.06241461134680382</v>
+      </c>
       <c r="W83" s="53"/>
-      <c r="X83" s="55"/>
-      <c r="Y83" s="55"/>
-      <c r="Z83" s="53"/>
-      <c r="AA83" s="56"/>
+      <c r="X83" s="55">
+        <v>44.94192893401015</v>
+      </c>
+      <c r="Y83" s="55">
+        <v>63.7162162306752</v>
+      </c>
+      <c r="Z83" s="53">
+        <v>0.33880000000000005</v>
+      </c>
+      <c r="AA83" s="56">
+        <v>0.3479</v>
+      </c>
       <c r="AB83" s="57"/>
       <c r="AD83" s="35"/>
       <c r="AE83" s="35"/>
@@ -14204,30 +14732,74 @@
       <c r="C90" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D90" s="67"/>
-      <c r="E90" s="67"/>
-      <c r="F90" s="52"/>
-      <c r="G90" s="53"/>
-      <c r="H90" s="52"/>
-      <c r="I90" s="52"/>
-      <c r="J90" s="52"/>
-      <c r="K90" s="52"/>
-      <c r="L90" s="52"/>
-      <c r="M90" s="53"/>
+      <c r="D90" s="67">
+        <v>37083.03</v>
+      </c>
+      <c r="E90" s="67">
+        <v>36381.33</v>
+      </c>
+      <c r="F90" s="52">
+        <v>701.6999999999971</v>
+      </c>
+      <c r="G90" s="53">
+        <v>0.018922401972007064</v>
+      </c>
+      <c r="H90" s="52">
+        <v>27002.93</v>
+      </c>
+      <c r="I90" s="52">
+        <v>25060.53</v>
+      </c>
+      <c r="J90" s="52">
+        <v>15440.32</v>
+      </c>
+      <c r="K90" s="52">
+        <v>13974.73</v>
+      </c>
+      <c r="L90" s="52">
+        <v>1465.5900000000001</v>
+      </c>
+      <c r="M90" s="53">
+        <v>0.09491966487741188</v>
+      </c>
       <c r="N90" s="53"/>
-      <c r="O90" s="52"/>
-      <c r="P90" s="52"/>
-      <c r="Q90" s="52"/>
-      <c r="R90" s="53"/>
-      <c r="S90" s="68"/>
-      <c r="T90" s="68"/>
-      <c r="U90" s="54"/>
-      <c r="V90" s="53"/>
+      <c r="O90" s="52">
+        <v>11562.61</v>
+      </c>
+      <c r="P90" s="52">
+        <v>11085.8</v>
+      </c>
+      <c r="Q90" s="52">
+        <v>476.8100000000013</v>
+      </c>
+      <c r="R90" s="53">
+        <v>0.041237229310683424</v>
+      </c>
+      <c r="S90" s="68">
+        <v>231.75</v>
+      </c>
+      <c r="T90" s="68">
+        <v>225.5</v>
+      </c>
+      <c r="U90" s="54">
+        <v>6.25</v>
+      </c>
+      <c r="V90" s="53">
+        <v>0.02696871628910464</v>
+      </c>
       <c r="W90" s="53"/>
-      <c r="X90" s="55"/>
-      <c r="Y90" s="55"/>
-      <c r="Z90" s="53"/>
-      <c r="AA90" s="56"/>
+      <c r="X90" s="55">
+        <v>50.20310421286031</v>
+      </c>
+      <c r="Y90" s="55">
+        <v>43.49557070636461</v>
+      </c>
+      <c r="Z90" s="53">
+        <v>0.31120000000000003</v>
+      </c>
+      <c r="AA90" s="56">
+        <v>0.2718</v>
+      </c>
       <c r="AB90" s="57"/>
       <c r="AD90" s="35"/>
       <c r="AE90" s="35"/>
@@ -14567,30 +15139,74 @@
       <c r="C97" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D97" s="52"/>
-      <c r="E97" s="52"/>
-      <c r="F97" s="52"/>
-      <c r="G97" s="53"/>
-      <c r="H97" s="52"/>
-      <c r="I97" s="52"/>
-      <c r="J97" s="52"/>
-      <c r="K97" s="52"/>
-      <c r="L97" s="52"/>
-      <c r="M97" s="53"/>
+      <c r="D97" s="52">
+        <v>26186.14</v>
+      </c>
+      <c r="E97" s="52">
+        <v>5762.27</v>
+      </c>
+      <c r="F97" s="52">
+        <v>20423.87</v>
+      </c>
+      <c r="G97" s="53">
+        <v>0.7799496222047235</v>
+      </c>
+      <c r="H97" s="52">
+        <v>19428.98</v>
+      </c>
+      <c r="I97" s="52">
+        <v>7925.81</v>
+      </c>
+      <c r="J97" s="52">
+        <v>12051.32</v>
+      </c>
+      <c r="K97" s="52">
+        <v>7679.910000000001</v>
+      </c>
+      <c r="L97" s="52">
+        <v>4371.409999999999</v>
+      </c>
+      <c r="M97" s="53">
+        <v>0.36273287905391266</v>
+      </c>
       <c r="N97" s="53"/>
-      <c r="O97" s="52"/>
-      <c r="P97" s="52"/>
-      <c r="Q97" s="52"/>
-      <c r="R97" s="53"/>
-      <c r="S97" s="54"/>
-      <c r="T97" s="54"/>
-      <c r="U97" s="54"/>
-      <c r="V97" s="53"/>
+      <c r="O97" s="52">
+        <v>7377.66</v>
+      </c>
+      <c r="P97" s="52">
+        <v>245.9</v>
+      </c>
+      <c r="Q97" s="52">
+        <v>7131.76</v>
+      </c>
+      <c r="R97" s="53">
+        <v>0.9666696486419813</v>
+      </c>
+      <c r="S97" s="54">
+        <v>147.9</v>
+      </c>
+      <c r="T97" s="54">
+        <v>5</v>
+      </c>
+      <c r="U97" s="54">
+        <v>142.9</v>
+      </c>
+      <c r="V97" s="53">
+        <v>0.9661933739012847</v>
+      </c>
       <c r="W97" s="53"/>
-      <c r="X97" s="55"/>
-      <c r="Y97" s="55"/>
-      <c r="Z97" s="53"/>
-      <c r="AA97" s="56"/>
+      <c r="X97" s="55">
+        <v>-432.70799999999997</v>
+      </c>
+      <c r="Y97" s="55">
+        <v>45.687352144692355</v>
+      </c>
+      <c r="Z97" s="53">
+        <v>-0.37549999999999994</v>
+      </c>
+      <c r="AA97" s="56">
+        <v>0.258</v>
+      </c>
       <c r="AB97" s="57"/>
       <c r="AD97" s="35"/>
       <c r="AE97" s="35"/>
@@ -14930,30 +15546,74 @@
       <c r="C104" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D104" s="52"/>
-      <c r="E104" s="69"/>
-      <c r="F104" s="52"/>
-      <c r="G104" s="53"/>
-      <c r="H104" s="52"/>
-      <c r="I104" s="52"/>
-      <c r="J104" s="52"/>
-      <c r="K104" s="52"/>
-      <c r="L104" s="52"/>
-      <c r="M104" s="53"/>
+      <c r="D104" s="52">
+        <v>32473.02</v>
+      </c>
+      <c r="E104" s="69">
+        <v>33188.03</v>
+      </c>
+      <c r="F104" s="52">
+        <v>-715.0099999999984</v>
+      </c>
+      <c r="G104" s="53">
+        <v>-0.022018586506582952</v>
+      </c>
+      <c r="H104" s="52">
+        <v>23075.07</v>
+      </c>
+      <c r="I104" s="52">
+        <v>30925.21</v>
+      </c>
+      <c r="J104" s="52">
+        <v>12691.21</v>
+      </c>
+      <c r="K104" s="52">
+        <v>15184.269999999999</v>
+      </c>
+      <c r="L104" s="52">
+        <v>-2493.0599999999995</v>
+      </c>
+      <c r="M104" s="53">
+        <v>-0.1964398981657383</v>
+      </c>
       <c r="N104" s="53"/>
-      <c r="O104" s="52"/>
-      <c r="P104" s="52"/>
-      <c r="Q104" s="52"/>
-      <c r="R104" s="53"/>
-      <c r="S104" s="54"/>
-      <c r="T104" s="54"/>
-      <c r="U104" s="54"/>
-      <c r="V104" s="53"/>
+      <c r="O104" s="52">
+        <v>10383.86</v>
+      </c>
+      <c r="P104" s="52">
+        <v>15740.94</v>
+      </c>
+      <c r="Q104" s="52">
+        <v>-5357.08</v>
+      </c>
+      <c r="R104" s="53">
+        <v>-0.5159044902377343</v>
+      </c>
+      <c r="S104" s="54">
+        <v>208.2</v>
+      </c>
+      <c r="T104" s="54">
+        <v>317.25</v>
+      </c>
+      <c r="U104" s="54">
+        <v>-109.05000000000001</v>
+      </c>
+      <c r="V104" s="53">
+        <v>-0.5237752161383286</v>
+      </c>
       <c r="W104" s="53"/>
-      <c r="X104" s="55"/>
-      <c r="Y104" s="55"/>
-      <c r="Z104" s="53"/>
-      <c r="AA104" s="56"/>
+      <c r="X104" s="55">
+        <v>7.132608353033885</v>
+      </c>
+      <c r="Y104" s="55">
+        <v>45.139084580403456</v>
+      </c>
+      <c r="Z104" s="53">
+        <v>0.0682</v>
+      </c>
+      <c r="AA104" s="56">
+        <v>0.2894</v>
+      </c>
       <c r="AB104" s="57"/>
       <c r="AD104" s="35"/>
       <c r="AE104" s="35"/>
@@ -15295,30 +15955,74 @@
       <c r="C111" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D111" s="52"/>
-      <c r="E111" s="52"/>
-      <c r="F111" s="52"/>
-      <c r="G111" s="53"/>
-      <c r="H111" s="52"/>
-      <c r="I111" s="52"/>
-      <c r="J111" s="52"/>
-      <c r="K111" s="52"/>
-      <c r="L111" s="52"/>
-      <c r="M111" s="53"/>
+      <c r="D111" s="52">
+        <v>58902.56</v>
+      </c>
+      <c r="E111" s="52">
+        <v>0</v>
+      </c>
+      <c r="F111" s="52">
+        <v>58902.56</v>
+      </c>
+      <c r="G111" s="53">
+        <v>1</v>
+      </c>
+      <c r="H111" s="52">
+        <v>37601.88</v>
+      </c>
+      <c r="I111" s="52">
+        <v>45817.77</v>
+      </c>
+      <c r="J111" s="52">
+        <v>21415.85</v>
+      </c>
+      <c r="K111" s="52">
+        <v>23939.389999999996</v>
+      </c>
+      <c r="L111" s="52">
+        <v>-2523.5399999999972</v>
+      </c>
+      <c r="M111" s="53">
+        <v>-0.11783515480356826</v>
+      </c>
       <c r="N111" s="53"/>
-      <c r="O111" s="52"/>
-      <c r="P111" s="52"/>
-      <c r="Q111" s="52"/>
-      <c r="R111" s="53"/>
-      <c r="S111" s="54"/>
-      <c r="T111" s="54"/>
-      <c r="U111" s="54"/>
-      <c r="V111" s="53"/>
+      <c r="O111" s="52">
+        <v>16186.03</v>
+      </c>
+      <c r="P111" s="52">
+        <v>21878.38</v>
+      </c>
+      <c r="Q111" s="52">
+        <v>-5692.35</v>
+      </c>
+      <c r="R111" s="53">
+        <v>-0.3516829018604315</v>
+      </c>
+      <c r="S111" s="54">
+        <v>324.19</v>
+      </c>
+      <c r="T111" s="54">
+        <v>472.75</v>
+      </c>
+      <c r="U111" s="54">
+        <v>-148.56</v>
+      </c>
+      <c r="V111" s="53">
+        <v>-0.45824979178876585</v>
+      </c>
       <c r="W111" s="53"/>
-      <c r="X111" s="55"/>
-      <c r="Y111" s="55"/>
-      <c r="Z111" s="53"/>
-      <c r="AA111" s="56"/>
+      <c r="X111" s="55">
+        <v>48.973178212585935</v>
+      </c>
+      <c r="Y111" s="55">
+        <v>65.70431400737223</v>
+      </c>
+      <c r="Z111" s="53">
+        <v>0.3357</v>
+      </c>
+      <c r="AA111" s="56">
+        <v>0.3616</v>
+      </c>
       <c r="AB111" s="57"/>
       <c r="AD111" s="35"/>
       <c r="AE111" s="35"/>
@@ -18848,30 +19552,74 @@
       <c r="C181" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D181" s="52"/>
-      <c r="E181" s="52"/>
-      <c r="F181" s="52"/>
-      <c r="G181" s="53"/>
-      <c r="H181" s="52"/>
-      <c r="I181" s="52"/>
-      <c r="J181" s="52"/>
-      <c r="K181" s="52"/>
-      <c r="L181" s="52"/>
-      <c r="M181" s="53"/>
+      <c r="D181" s="52">
+        <v>16897.53</v>
+      </c>
+      <c r="E181" s="52">
+        <v>5491.7</v>
+      </c>
+      <c r="F181" s="52">
+        <v>11405.829999999998</v>
+      </c>
+      <c r="G181" s="53">
+        <v>0.6749998372543206</v>
+      </c>
+      <c r="H181" s="52">
+        <v>9226.27</v>
+      </c>
+      <c r="I181" s="52">
+        <v>3702.78</v>
+      </c>
+      <c r="J181" s="52">
+        <v>2977.1100000000006</v>
+      </c>
+      <c r="K181" s="52">
+        <v>2335.9700000000003</v>
+      </c>
+      <c r="L181" s="52">
+        <v>641.1400000000003</v>
+      </c>
+      <c r="M181" s="53">
+        <v>0.2153565034546927</v>
+      </c>
       <c r="N181" s="53"/>
-      <c r="O181" s="52"/>
-      <c r="P181" s="52"/>
-      <c r="Q181" s="52"/>
-      <c r="R181" s="53"/>
-      <c r="S181" s="54"/>
-      <c r="T181" s="54"/>
-      <c r="U181" s="54"/>
-      <c r="V181" s="53"/>
+      <c r="O181" s="52">
+        <v>6249.16</v>
+      </c>
+      <c r="P181" s="52">
+        <v>1366.81</v>
+      </c>
+      <c r="Q181" s="52">
+        <v>4882.35</v>
+      </c>
+      <c r="R181" s="53">
+        <v>0.7812810041669601</v>
+      </c>
+      <c r="S181" s="54">
+        <v>125.17</v>
+      </c>
+      <c r="T181" s="54">
+        <v>23.75</v>
+      </c>
+      <c r="U181" s="54">
+        <v>101.42</v>
+      </c>
+      <c r="V181" s="53">
+        <v>0.8102580490532876</v>
+      </c>
       <c r="W181" s="53"/>
-      <c r="X181" s="55"/>
-      <c r="Y181" s="55"/>
-      <c r="Z181" s="53"/>
-      <c r="AA181" s="56"/>
+      <c r="X181" s="55">
+        <v>75.32294736842105</v>
+      </c>
+      <c r="Y181" s="55">
+        <v>61.286703843093385</v>
+      </c>
+      <c r="Z181" s="53">
+        <v>0.3257</v>
+      </c>
+      <c r="AA181" s="56">
+        <v>0.454</v>
+      </c>
       <c r="AB181" s="57"/>
       <c r="AD181" s="35"/>
       <c r="AE181" s="35"/>
@@ -21185,30 +21933,74 @@
       <c r="C230" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D230" s="52"/>
-      <c r="E230" s="52"/>
-      <c r="F230" s="52"/>
-      <c r="G230" s="53"/>
-      <c r="H230" s="52"/>
-      <c r="I230" s="52"/>
-      <c r="J230" s="52"/>
-      <c r="K230" s="52"/>
-      <c r="L230" s="52"/>
-      <c r="M230" s="53"/>
+      <c r="D230" s="52">
+        <v>8795.03</v>
+      </c>
+      <c r="E230" s="52">
+        <v>0</v>
+      </c>
+      <c r="F230" s="52">
+        <v>8795.03</v>
+      </c>
+      <c r="G230" s="53">
+        <v>1</v>
+      </c>
+      <c r="H230" s="52">
+        <v>6369.12</v>
+      </c>
+      <c r="I230" s="52">
+        <v>0</v>
+      </c>
+      <c r="J230" s="52">
+        <v>4527.889999999999</v>
+      </c>
+      <c r="K230" s="52">
+        <v>0</v>
+      </c>
+      <c r="L230" s="52">
+        <v>4527.889999999999</v>
+      </c>
+      <c r="M230" s="53">
+        <v>1</v>
+      </c>
       <c r="N230" s="53"/>
-      <c r="O230" s="52"/>
-      <c r="P230" s="52"/>
-      <c r="Q230" s="52"/>
-      <c r="R230" s="53"/>
-      <c r="S230" s="54"/>
-      <c r="T230" s="54"/>
-      <c r="U230" s="54"/>
-      <c r="V230" s="53"/>
+      <c r="O230" s="52">
+        <v>1841.23</v>
+      </c>
+      <c r="P230" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q230" s="52">
+        <v>1841.23</v>
+      </c>
+      <c r="R230" s="53">
+        <v>1</v>
+      </c>
+      <c r="S230" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="T230" s="54">
+        <v>0</v>
+      </c>
+      <c r="U230" s="54">
+        <v>36.92</v>
+      </c>
+      <c r="V230" s="53">
+        <v>1</v>
+      </c>
       <c r="W230" s="53"/>
-      <c r="X230" s="55"/>
-      <c r="Y230" s="55"/>
-      <c r="Z230" s="53"/>
-      <c r="AA230" s="56"/>
+      <c r="X230" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y230" s="55">
+        <v>65.70711175027087</v>
+      </c>
+      <c r="Z230" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA230" s="56">
+        <v>0.2758</v>
+      </c>
       <c r="AB230" s="57"/>
       <c r="AD230" s="35"/>
       <c r="AE230" s="35"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-07T21:15:28Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -17100,7 +17100,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>97</v>
@@ -22683,7 +22683,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD71"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -22697,7 +22697,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -22719,7 +22719,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>102</v>
       </c>
@@ -22767,7 +22767,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -22785,7 +22785,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -22832,7 +22832,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -22849,7 +22849,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -22899,7 +22899,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -22916,7 +22916,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -22959,7 +22959,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -22976,7 +22976,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23023,7 +23023,7 @@
         <v>24.375135929463628</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23040,7 +23040,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23090,7 +23090,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23107,7 +23107,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23154,7 +23154,7 @@
         <v>89.17785714285712</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23171,7 +23171,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23216,7 +23216,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23233,7 +23233,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23283,7 +23283,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23300,7 +23300,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23339,7 +23339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23356,7 +23356,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23397,7 +23397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23414,7 +23414,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -23453,7 +23453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -23470,7 +23470,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -23515,7 +23515,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -23532,7 +23532,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -23575,7 +23575,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -23592,7 +23592,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -23635,7 +23635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -23652,7 +23652,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -23699,7 +23699,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -23716,7 +23716,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -23761,7 +23761,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -23778,7 +23778,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -23821,7 +23821,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -23838,7 +23838,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -23879,7 +23879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -23896,7 +23896,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -23941,7 +23941,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -23958,7 +23958,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24001,7 +24001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24018,7 +24018,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24055,7 +24055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24072,7 +24072,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -24113,7 +24113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24130,7 +24130,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -24173,7 +24173,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24190,7 +24190,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -24232,7 +24232,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24249,7 +24249,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -24294,7 +24294,7 @@
         <v>14.333675527039448</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24311,7 +24311,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -24356,7 +24356,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24373,7 +24373,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -24418,7 +24418,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -24435,7 +24435,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -24472,7 +24472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -24489,7 +24489,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -24506,7 +24506,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -24523,7 +24523,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -24544,7 +24544,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -24561,7 +24561,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -24602,7 +24602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -24619,7 +24619,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -24664,7 +24664,7 @@
         <v>-25.71043082686644</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -24699,7 +24699,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -24716,7 +24716,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -24733,7 +24733,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>122</v>
       </c>
@@ -24768,7 +24768,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>126</v>
@@ -25151,7 +25151,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD110"/>
+  <dimension ref="A1:AB110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25162,7 +25162,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25183,7 +25183,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>127</v>
@@ -25245,7 +25245,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>143</v>
       </c>
@@ -25303,7 +25303,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25339,7 +25339,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25358,7 +25358,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25392,7 +25392,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25411,7 +25411,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -25445,7 +25445,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -25464,7 +25464,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -25502,7 +25502,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -25521,7 +25521,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -25559,7 +25559,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -25578,7 +25578,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -25616,7 +25616,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -25635,7 +25635,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -25668,7 +25668,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -25687,7 +25687,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -25720,7 +25720,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -25739,7 +25739,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -25770,7 +25770,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -25789,7 +25789,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -25824,7 +25824,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -25843,7 +25843,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -25876,7 +25876,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -25895,7 +25895,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25926,7 +25926,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -25945,7 +25945,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25977,7 +25977,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -25996,7 +25996,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -26032,7 +26032,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26051,7 +26051,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -26080,7 +26080,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26099,7 +26099,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -26130,7 +26130,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26149,7 +26149,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -26182,7 +26182,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26201,7 +26201,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -26237,7 +26237,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26256,7 +26256,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -26291,7 +26291,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26310,7 +26310,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -26340,7 +26340,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26359,7 +26359,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -26399,7 +26399,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -26418,7 +26418,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -26447,7 +26447,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -26466,7 +26466,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -26499,7 +26499,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -26518,7 +26518,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -26551,7 +26551,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -26570,7 +26570,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -26606,7 +26606,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -26625,7 +26625,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -26661,7 +26661,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -26680,7 +26680,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -26714,7 +26714,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -26733,7 +26733,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -26768,7 +26768,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -26787,7 +26787,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -26806,7 +26806,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -26825,7 +26825,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -26846,7 +26846,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -26865,7 +26865,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -26898,7 +26898,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -26917,7 +26917,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -26956,7 +26956,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -26985,7 +26985,7 @@
       <c r="P67" s="54"/>
       <c r="Q67" s="54"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27004,7 +27004,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="142"/>
       <c r="B69" s="143"/>
       <c r="C69" s="35"/>
@@ -27023,7 +27023,7 @@
       <c r="P69" s="35"/>
       <c r="Q69" s="144"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="145"/>
       <c r="B70" s="145"/>
       <c r="C70" s="145"/>
@@ -27042,7 +27042,7 @@
       <c r="P70" s="145"/>
       <c r="Q70" s="145"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="146" t="s">
         <v>147</v>
@@ -27087,7 +27087,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -27126,7 +27126,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="77" t="s">
         <v>149</v>
@@ -27155,7 +27155,7 @@
       <c r="P73" s="20"/>
       <c r="Q73" s="20"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="148" t="s">
         <v>150</v>
@@ -27200,7 +27200,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="151" t="s">
         <v>151</v>
@@ -27245,7 +27245,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
@@ -27264,7 +27264,7 @@
       <c r="P76" s="35"/>
       <c r="Q76" s="144"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="156" t="s">
         <v>152</v>
@@ -27311,7 +27311,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="161"/>
       <c r="B78" s="162" t="s">
         <v>154</v>
@@ -27356,7 +27356,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -27375,7 +27375,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="164" t="s">
         <v>155</v>
@@ -27398,7 +27398,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="167" t="s">
         <v>157</v>
@@ -27421,7 +27421,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -27444,7 +27444,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -27467,7 +27467,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -27490,7 +27490,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -27513,7 +27513,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -27536,7 +27536,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -27559,7 +27559,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -27582,7 +27582,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -27605,7 +27605,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -27628,7 +27628,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -27651,7 +27651,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -27672,7 +27672,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -27693,7 +27693,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -27714,7 +27714,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -27735,7 +27735,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -27756,7 +27756,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -27777,7 +27777,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -27798,7 +27798,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -27821,7 +27821,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -27844,7 +27844,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -27867,7 +27867,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -27890,7 +27890,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -27913,7 +27913,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -27936,7 +27936,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -27959,7 +27959,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -27978,7 +27978,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -27997,7 +27997,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19"/>
       <c r="C108" s="131"/>
@@ -28016,7 +28016,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="169"/>
       <c r="C109" s="150"/>
@@ -28035,7 +28035,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="164" t="s">
         <v>175</v>
@@ -28109,11 +28109,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>176</v>
       </c>
@@ -28145,7 +28144,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>177</v>
       </c>
@@ -28178,7 +28177,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>178</v>
       </c>
@@ -28211,7 +28210,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>179</v>
       </c>
@@ -28244,7 +28243,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>180</v>
       </c>
@@ -28277,7 +28276,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>181</v>
       </c>
@@ -28310,7 +28309,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>182</v>
       </c>
@@ -28343,7 +28342,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>183</v>
       </c>
@@ -28376,7 +28375,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28407,7 +28406,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -28438,7 +28437,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>184</v>
       </c>
@@ -28471,7 +28470,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>185</v>
       </c>
@@ -28504,7 +28503,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>186</v>
       </c>
@@ -28537,7 +28536,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>187</v>
       </c>
@@ -28570,7 +28569,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>188</v>
       </c>
@@ -28603,7 +28602,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>189</v>
       </c>
@@ -28636,7 +28635,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>190</v>
       </c>
@@ -28669,7 +28668,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>191</v>
       </c>
@@ -28702,7 +28701,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>192</v>
       </c>
@@ -28735,7 +28734,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>193</v>
       </c>
@@ -28768,7 +28767,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>194</v>
       </c>
@@ -28801,7 +28800,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>195</v>
       </c>
@@ -28834,7 +28833,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>196</v>
       </c>
@@ -28867,7 +28866,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>197</v>
       </c>
@@ -28900,7 +28899,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>198</v>
       </c>
@@ -28933,7 +28932,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>199</v>
       </c>
@@ -28966,7 +28965,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>200</v>
       </c>
@@ -28998,7 +28997,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>201</v>
       </c>
@@ -29030,7 +29029,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>202</v>
       </c>
@@ -29062,7 +29061,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>203</v>
       </c>
@@ -29094,7 +29093,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>204</v>
       </c>
@@ -29126,7 +29125,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29156,7 +29155,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29186,7 +29185,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>205</v>
       </c>
@@ -29218,7 +29217,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>206</v>
       </c>
@@ -29250,7 +29249,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>207</v>
       </c>
@@ -29282,7 +29281,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>208</v>
       </c>
@@ -29314,7 +29313,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>209</v>
       </c>
@@ -29346,7 +29345,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29376,7 +29375,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>210</v>
       </c>
@@ -29408,7 +29407,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>211</v>
       </c>
@@ -29440,7 +29439,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>212</v>
       </c>
@@ -29472,7 +29471,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>213</v>
       </c>
@@ -29504,7 +29503,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -29534,7 +29533,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -29564,7 +29563,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -29594,7 +29593,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -29624,7 +29623,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>214</v>
       </c>
@@ -29656,7 +29655,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>215</v>
       </c>
@@ -29688,7 +29687,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -29718,7 +29717,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -29748,7 +29747,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -29778,7 +29777,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -29808,7 +29807,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -29838,7 +29837,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -29933,11 +29932,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>216</v>
       </c>
@@ -29969,7 +29967,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -30000,7 +29998,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30031,7 +30029,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30062,7 +30060,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30093,7 +30091,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30124,7 +30122,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30155,7 +30153,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30186,7 +30184,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30217,7 +30215,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -30248,7 +30246,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -30279,7 +30277,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -30310,7 +30308,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -30341,7 +30339,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -30372,7 +30370,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -30403,7 +30401,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -30434,7 +30432,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -30465,7 +30463,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -30496,7 +30494,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -30527,7 +30525,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -30558,7 +30556,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -30588,7 +30586,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -30618,7 +30616,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -30648,7 +30646,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -30678,7 +30676,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -30708,7 +30706,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -30738,7 +30736,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -30768,7 +30766,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -30798,7 +30796,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -30828,7 +30826,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -30858,7 +30856,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -30888,7 +30886,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -30918,7 +30916,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -30948,7 +30946,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -30978,7 +30976,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -31008,7 +31006,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -31038,7 +31036,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>214</v>
       </c>
@@ -31070,7 +31068,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>215</v>
       </c>
@@ -31102,7 +31100,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -31132,7 +31130,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -31162,7 +31160,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -31192,7 +31190,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -31222,7 +31220,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -31252,7 +31250,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -52995,19 +52993,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -53021,7 +53019,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>223</v>
       </c>
@@ -53033,7 +53031,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>224</v>
       </c>
@@ -53044,7 +53042,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>225</v>
       </c>
@@ -53055,7 +53053,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>226</v>
       </c>
@@ -53066,13 +53064,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-07T21:22:24Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -17100,7 +17100,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>97</v>
@@ -17432,30 +17432,74 @@
       <c r="C139" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D139" s="52"/>
-      <c r="E139" s="52"/>
-      <c r="F139" s="52"/>
-      <c r="G139" s="53"/>
-      <c r="H139" s="52"/>
-      <c r="I139" s="52"/>
-      <c r="J139" s="52"/>
-      <c r="K139" s="52"/>
-      <c r="L139" s="52"/>
-      <c r="M139" s="53"/>
+      <c r="D139" s="52">
+        <v>30749.24</v>
+      </c>
+      <c r="E139" s="52">
+        <v>30749.24</v>
+      </c>
+      <c r="F139" s="52">
+        <v>0</v>
+      </c>
+      <c r="G139" s="53">
+        <v>0</v>
+      </c>
+      <c r="H139" s="52">
+        <v>22587.89</v>
+      </c>
+      <c r="I139" s="52">
+        <v>25905.23</v>
+      </c>
+      <c r="J139" s="52">
+        <v>12565.06</v>
+      </c>
+      <c r="K139" s="52">
+        <v>11805.46</v>
+      </c>
+      <c r="L139" s="52">
+        <v>759.6000000000004</v>
+      </c>
+      <c r="M139" s="53">
+        <v>0.06045335239147289</v>
+      </c>
       <c r="N139" s="53"/>
-      <c r="O139" s="52"/>
-      <c r="P139" s="52"/>
-      <c r="Q139" s="52"/>
-      <c r="R139" s="53"/>
-      <c r="S139" s="54"/>
-      <c r="T139" s="54"/>
-      <c r="U139" s="54"/>
-      <c r="V139" s="53"/>
+      <c r="O139" s="52">
+        <v>10022.83</v>
+      </c>
+      <c r="P139" s="52">
+        <v>14099.77</v>
+      </c>
+      <c r="Q139" s="52">
+        <v>-4076.9400000000005</v>
+      </c>
+      <c r="R139" s="53">
+        <v>-0.40676535469523084</v>
+      </c>
+      <c r="S139" s="54">
+        <v>200.82</v>
+      </c>
+      <c r="T139" s="54">
+        <v>283.75</v>
+      </c>
+      <c r="U139" s="54">
+        <v>-82.93</v>
+      </c>
+      <c r="V139" s="53">
+        <v>-0.4129568768050991</v>
+      </c>
       <c r="W139" s="53"/>
-      <c r="X139" s="55"/>
-      <c r="Y139" s="55"/>
-      <c r="Z139" s="53"/>
-      <c r="AA139" s="56"/>
+      <c r="X139" s="55">
+        <v>17.07140088105727</v>
+      </c>
+      <c r="Y139" s="55">
+        <v>40.64013272149188</v>
+      </c>
+      <c r="Z139" s="53">
+        <v>0.1575</v>
+      </c>
+      <c r="AA139" s="56">
+        <v>0.2654</v>
+      </c>
       <c r="AB139" s="57"/>
       <c r="AD139" s="35"/>
       <c r="AE139" s="35"/>
@@ -17785,30 +17829,74 @@
       <c r="C146" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D146" s="52"/>
-      <c r="E146" s="52"/>
-      <c r="F146" s="52"/>
-      <c r="G146" s="53"/>
-      <c r="H146" s="52"/>
-      <c r="I146" s="52"/>
-      <c r="J146" s="52"/>
-      <c r="K146" s="52"/>
-      <c r="L146" s="52"/>
-      <c r="M146" s="53"/>
+      <c r="D146" s="52">
+        <v>268228.26</v>
+      </c>
+      <c r="E146" s="52">
+        <v>9034.53</v>
+      </c>
+      <c r="F146" s="52">
+        <v>259193.73</v>
+      </c>
+      <c r="G146" s="53">
+        <v>0.9663177548853353</v>
+      </c>
+      <c r="H146" s="52">
+        <v>238611.58</v>
+      </c>
+      <c r="I146" s="52">
+        <v>6362.08</v>
+      </c>
+      <c r="J146" s="52">
+        <v>214154.25</v>
+      </c>
+      <c r="K146" s="52">
+        <v>3465.35</v>
+      </c>
+      <c r="L146" s="52">
+        <v>210688.9</v>
+      </c>
+      <c r="M146" s="53">
+        <v>0.9838184392791645</v>
+      </c>
       <c r="N146" s="53"/>
-      <c r="O146" s="52"/>
-      <c r="P146" s="52"/>
-      <c r="Q146" s="52"/>
-      <c r="R146" s="53"/>
-      <c r="S146" s="54"/>
-      <c r="T146" s="54"/>
-      <c r="U146" s="54"/>
-      <c r="V146" s="53"/>
+      <c r="O146" s="52">
+        <v>24457.33</v>
+      </c>
+      <c r="P146" s="52">
+        <v>2896.73</v>
+      </c>
+      <c r="Q146" s="52">
+        <v>21560.600000000002</v>
+      </c>
+      <c r="R146" s="53">
+        <v>0.8815598432044708</v>
+      </c>
+      <c r="S146" s="54">
+        <v>497.55</v>
+      </c>
+      <c r="T146" s="54">
+        <v>58.25</v>
+      </c>
+      <c r="U146" s="54">
+        <v>439.3</v>
+      </c>
+      <c r="V146" s="53">
+        <v>0.8829263390614008</v>
+      </c>
       <c r="W146" s="53"/>
-      <c r="X146" s="55"/>
-      <c r="Y146" s="55"/>
-      <c r="Z146" s="53"/>
-      <c r="AA146" s="56"/>
+      <c r="X146" s="55">
+        <v>45.878969957081544</v>
+      </c>
+      <c r="Y146" s="55">
+        <v>59.525035875791396</v>
+      </c>
+      <c r="Z146" s="53">
+        <v>0.2958</v>
+      </c>
+      <c r="AA146" s="56">
+        <v>0.1104</v>
+      </c>
       <c r="AB146" s="57"/>
       <c r="AD146" s="35"/>
       <c r="AE146" s="35"/>
@@ -18142,30 +18230,74 @@
       <c r="C153" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D153" s="52"/>
-      <c r="E153" s="52"/>
-      <c r="F153" s="52"/>
-      <c r="G153" s="53"/>
-      <c r="H153" s="52"/>
-      <c r="I153" s="52"/>
-      <c r="J153" s="52"/>
-      <c r="K153" s="52"/>
-      <c r="L153" s="52"/>
-      <c r="M153" s="53"/>
+      <c r="D153" s="52">
+        <v>32773.41</v>
+      </c>
+      <c r="E153" s="52">
+        <v>32773.41</v>
+      </c>
+      <c r="F153" s="52">
+        <v>0</v>
+      </c>
+      <c r="G153" s="53">
+        <v>0</v>
+      </c>
+      <c r="H153" s="52">
+        <v>22750.99</v>
+      </c>
+      <c r="I153" s="52">
+        <v>22254.11</v>
+      </c>
+      <c r="J153" s="52">
+        <v>12243.410000000002</v>
+      </c>
+      <c r="K153" s="52">
+        <v>9324.41</v>
+      </c>
+      <c r="L153" s="52">
+        <v>2919.000000000002</v>
+      </c>
+      <c r="M153" s="53">
+        <v>0.23841397127107575</v>
+      </c>
       <c r="N153" s="53"/>
-      <c r="O153" s="52"/>
-      <c r="P153" s="52"/>
-      <c r="Q153" s="52"/>
-      <c r="R153" s="53"/>
-      <c r="S153" s="54"/>
-      <c r="T153" s="54"/>
-      <c r="U153" s="54"/>
-      <c r="V153" s="53"/>
+      <c r="O153" s="52">
+        <v>10507.58</v>
+      </c>
+      <c r="P153" s="52">
+        <v>12929.7</v>
+      </c>
+      <c r="Q153" s="52">
+        <v>-2422.120000000001</v>
+      </c>
+      <c r="R153" s="53">
+        <v>-0.23051168775303169</v>
+      </c>
+      <c r="S153" s="54">
+        <v>210.6</v>
+      </c>
+      <c r="T153" s="54">
+        <v>260.75</v>
+      </c>
+      <c r="U153" s="54">
+        <v>-50.150000000000006</v>
+      </c>
+      <c r="V153" s="53">
+        <v>-0.2381291547958215</v>
+      </c>
       <c r="W153" s="53"/>
-      <c r="X153" s="55"/>
-      <c r="Y153" s="55"/>
-      <c r="Z153" s="53"/>
-      <c r="AA153" s="56"/>
+      <c r="X153" s="55">
+        <v>40.342473633748796</v>
+      </c>
+      <c r="Y153" s="55">
+        <v>47.58984852136751</v>
+      </c>
+      <c r="Z153" s="53">
+        <v>0.321</v>
+      </c>
+      <c r="AA153" s="56">
+        <v>0.3058</v>
+      </c>
       <c r="AB153" s="57"/>
       <c r="AD153" s="35"/>
       <c r="AE153" s="35"/>
@@ -18499,30 +18631,74 @@
       <c r="C160" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D160" s="52"/>
-      <c r="E160" s="52"/>
-      <c r="F160" s="52"/>
-      <c r="G160" s="53"/>
-      <c r="H160" s="52"/>
-      <c r="I160" s="52"/>
-      <c r="J160" s="52"/>
-      <c r="K160" s="52"/>
-      <c r="L160" s="52"/>
-      <c r="M160" s="53"/>
+      <c r="D160" s="52">
+        <v>17899.33</v>
+      </c>
+      <c r="E160" s="52">
+        <v>13424.5</v>
+      </c>
+      <c r="F160" s="52">
+        <v>4474.830000000002</v>
+      </c>
+      <c r="G160" s="53">
+        <v>0.24999986032996774</v>
+      </c>
+      <c r="H160" s="52">
+        <v>13919.4</v>
+      </c>
+      <c r="I160" s="52">
+        <v>10402.37</v>
+      </c>
+      <c r="J160" s="52">
+        <v>8410.93</v>
+      </c>
+      <c r="K160" s="52">
+        <v>7278.380000000001</v>
+      </c>
+      <c r="L160" s="52">
+        <v>1132.5499999999993</v>
+      </c>
+      <c r="M160" s="53">
+        <v>0.13465217282749936</v>
+      </c>
       <c r="N160" s="53"/>
-      <c r="O160" s="52"/>
-      <c r="P160" s="52"/>
-      <c r="Q160" s="52"/>
-      <c r="R160" s="53"/>
-      <c r="S160" s="54"/>
-      <c r="T160" s="54"/>
-      <c r="U160" s="54"/>
-      <c r="V160" s="53"/>
+      <c r="O160" s="52">
+        <v>5508.47</v>
+      </c>
+      <c r="P160" s="52">
+        <v>3123.99</v>
+      </c>
+      <c r="Q160" s="52">
+        <v>2384.4800000000005</v>
+      </c>
+      <c r="R160" s="53">
+        <v>0.43287519038861977</v>
+      </c>
+      <c r="S160" s="54">
+        <v>110.44</v>
+      </c>
+      <c r="T160" s="54">
+        <v>60.75</v>
+      </c>
+      <c r="U160" s="54">
+        <v>49.69</v>
+      </c>
+      <c r="V160" s="53">
+        <v>0.44992756247736326</v>
+      </c>
       <c r="W160" s="53"/>
-      <c r="X160" s="55"/>
-      <c r="Y160" s="55"/>
-      <c r="Z160" s="53"/>
-      <c r="AA160" s="56"/>
+      <c r="X160" s="55">
+        <v>49.74699588477367</v>
+      </c>
+      <c r="Y160" s="55">
+        <v>36.03704967040926</v>
+      </c>
+      <c r="Z160" s="53">
+        <v>0.22510000000000002</v>
+      </c>
+      <c r="AA160" s="56">
+        <v>0.2224</v>
+      </c>
       <c r="AB160" s="57"/>
       <c r="AD160" s="35"/>
       <c r="AE160" s="35"/>
@@ -18838,30 +19014,74 @@
       <c r="C167" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D167" s="52"/>
-      <c r="E167" s="52"/>
-      <c r="F167" s="52"/>
-      <c r="G167" s="53"/>
-      <c r="H167" s="52"/>
-      <c r="I167" s="52"/>
-      <c r="J167" s="52"/>
-      <c r="K167" s="52"/>
-      <c r="L167" s="52"/>
-      <c r="M167" s="53"/>
+      <c r="D167" s="52">
+        <v>10827.2</v>
+      </c>
+      <c r="E167" s="52">
+        <v>0</v>
+      </c>
+      <c r="F167" s="52">
+        <v>10827.2</v>
+      </c>
+      <c r="G167" s="53">
+        <v>1</v>
+      </c>
+      <c r="H167" s="52">
+        <v>7687.77</v>
+      </c>
+      <c r="I167" s="52">
+        <v>2116.21</v>
+      </c>
+      <c r="J167" s="52">
+        <v>4437.14</v>
+      </c>
+      <c r="K167" s="52">
+        <v>1029.51</v>
+      </c>
+      <c r="L167" s="52">
+        <v>3407.63</v>
+      </c>
+      <c r="M167" s="53">
+        <v>0.7679789233605431</v>
+      </c>
       <c r="N167" s="53"/>
-      <c r="O167" s="52"/>
-      <c r="P167" s="52"/>
-      <c r="Q167" s="52"/>
-      <c r="R167" s="53"/>
-      <c r="S167" s="54"/>
-      <c r="T167" s="54"/>
-      <c r="U167" s="54"/>
-      <c r="V167" s="53"/>
+      <c r="O167" s="52">
+        <v>3250.63</v>
+      </c>
+      <c r="P167" s="52">
+        <v>1086.7</v>
+      </c>
+      <c r="Q167" s="52">
+        <v>2163.9300000000003</v>
+      </c>
+      <c r="R167" s="53">
+        <v>0.6656955728581845</v>
+      </c>
+      <c r="S167" s="54">
+        <v>65.13</v>
+      </c>
+      <c r="T167" s="54">
+        <v>24.33</v>
+      </c>
+      <c r="U167" s="54">
+        <v>40.8</v>
+      </c>
+      <c r="V167" s="53">
+        <v>0.6264394288346384</v>
+      </c>
       <c r="W167" s="53"/>
-      <c r="X167" s="55"/>
-      <c r="Y167" s="55"/>
-      <c r="Z167" s="53"/>
-      <c r="AA167" s="56"/>
+      <c r="X167" s="55">
+        <v>-86.97944923962187</v>
+      </c>
+      <c r="Y167" s="55">
+        <v>48.202633430830645</v>
+      </c>
+      <c r="Z167" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA167" s="56">
+        <v>0.29</v>
+      </c>
       <c r="AB167" s="57"/>
       <c r="AD167" s="35"/>
       <c r="AE167" s="35"/>
@@ -19191,30 +19411,74 @@
       <c r="C174" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D174" s="52"/>
-      <c r="E174" s="52"/>
-      <c r="F174" s="52"/>
-      <c r="G174" s="53"/>
-      <c r="H174" s="52"/>
-      <c r="I174" s="52"/>
-      <c r="J174" s="52"/>
-      <c r="K174" s="52"/>
-      <c r="L174" s="52"/>
-      <c r="M174" s="53"/>
+      <c r="D174" s="52">
+        <v>146237.11</v>
+      </c>
+      <c r="E174" s="52">
+        <v>125386.21</v>
+      </c>
+      <c r="F174" s="52">
+        <v>20850.89999999998</v>
+      </c>
+      <c r="G174" s="53">
+        <v>0.14258282319720336</v>
+      </c>
+      <c r="H174" s="52">
+        <v>114651.87</v>
+      </c>
+      <c r="I174" s="52">
+        <v>105118.87</v>
+      </c>
+      <c r="J174" s="52">
+        <v>82888.07999999999</v>
+      </c>
+      <c r="K174" s="52">
+        <v>77768.29999999999</v>
+      </c>
+      <c r="L174" s="52">
+        <v>5119.779999999999</v>
+      </c>
+      <c r="M174" s="53">
+        <v>0.06176738561202044</v>
+      </c>
       <c r="N174" s="53"/>
-      <c r="O174" s="52"/>
-      <c r="P174" s="52"/>
-      <c r="Q174" s="52"/>
-      <c r="R174" s="53"/>
-      <c r="S174" s="54"/>
-      <c r="T174" s="54"/>
-      <c r="U174" s="54"/>
-      <c r="V174" s="53"/>
+      <c r="O174" s="52">
+        <v>31763.79</v>
+      </c>
+      <c r="P174" s="52">
+        <v>27350.57</v>
+      </c>
+      <c r="Q174" s="52">
+        <v>4413.220000000001</v>
+      </c>
+      <c r="R174" s="53">
+        <v>0.13893870976983544</v>
+      </c>
+      <c r="S174" s="54">
+        <v>659.73</v>
+      </c>
+      <c r="T174" s="54">
+        <v>548.75</v>
+      </c>
+      <c r="U174" s="54">
+        <v>110.98000000000002</v>
+      </c>
+      <c r="V174" s="53">
+        <v>0.16822033256028984</v>
+      </c>
       <c r="W174" s="53"/>
-      <c r="X174" s="55"/>
-      <c r="Y174" s="55"/>
-      <c r="Z174" s="53"/>
-      <c r="AA174" s="56"/>
+      <c r="X174" s="55">
+        <v>36.933649202733484</v>
+      </c>
+      <c r="Y174" s="55">
+        <v>47.87601261940491</v>
+      </c>
+      <c r="Z174" s="53">
+        <v>0.1616</v>
+      </c>
+      <c r="AA174" s="56">
+        <v>0.216</v>
+      </c>
       <c r="AB174" s="57"/>
       <c r="AD174" s="35"/>
       <c r="AE174" s="35"/>
@@ -19953,30 +20217,74 @@
       <c r="C188" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D188" s="52"/>
-      <c r="E188" s="52"/>
-      <c r="F188" s="52"/>
-      <c r="G188" s="53"/>
-      <c r="H188" s="52"/>
-      <c r="I188" s="52"/>
-      <c r="J188" s="52"/>
-      <c r="K188" s="52"/>
-      <c r="L188" s="52"/>
-      <c r="M188" s="53"/>
+      <c r="D188" s="52">
+        <v>20992.12</v>
+      </c>
+      <c r="E188" s="52">
+        <v>14169.68</v>
+      </c>
+      <c r="F188" s="52">
+        <v>6822.439999999999</v>
+      </c>
+      <c r="G188" s="53">
+        <v>0.32500004763692275</v>
+      </c>
+      <c r="H188" s="52">
+        <v>16299.09</v>
+      </c>
+      <c r="I188" s="52">
+        <v>9699.51</v>
+      </c>
+      <c r="J188" s="52">
+        <v>9784.33</v>
+      </c>
+      <c r="K188" s="52">
+        <v>8137.88</v>
+      </c>
+      <c r="L188" s="52">
+        <v>1646.4499999999998</v>
+      </c>
+      <c r="M188" s="53">
+        <v>0.16827416900288522</v>
+      </c>
       <c r="N188" s="53"/>
-      <c r="O188" s="52"/>
-      <c r="P188" s="52"/>
-      <c r="Q188" s="52"/>
-      <c r="R188" s="53"/>
-      <c r="S188" s="54"/>
-      <c r="T188" s="54"/>
-      <c r="U188" s="54"/>
-      <c r="V188" s="53"/>
+      <c r="O188" s="52">
+        <v>6514.76</v>
+      </c>
+      <c r="P188" s="52">
+        <v>1561.63</v>
+      </c>
+      <c r="Q188" s="52">
+        <v>4953.13</v>
+      </c>
+      <c r="R188" s="53">
+        <v>0.7602935488030257</v>
+      </c>
+      <c r="S188" s="54">
+        <v>130.62</v>
+      </c>
+      <c r="T188" s="54">
+        <v>34.75</v>
+      </c>
+      <c r="U188" s="54">
+        <v>95.87</v>
+      </c>
+      <c r="V188" s="53">
+        <v>0.7339611085591793</v>
+      </c>
       <c r="W188" s="53"/>
-      <c r="X188" s="55"/>
-      <c r="Y188" s="55"/>
-      <c r="Z188" s="53"/>
-      <c r="AA188" s="56"/>
+      <c r="X188" s="55">
+        <v>128.6379856115108</v>
+      </c>
+      <c r="Y188" s="55">
+        <v>35.92887828502527</v>
+      </c>
+      <c r="Z188" s="53">
+        <v>0.3155</v>
+      </c>
+      <c r="AA188" s="56">
+        <v>0.2236</v>
+      </c>
       <c r="AB188" s="57"/>
       <c r="AD188" s="35"/>
       <c r="AE188" s="35"/>
@@ -20304,30 +20612,74 @@
       <c r="C195" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D195" s="52"/>
-      <c r="E195" s="52"/>
-      <c r="F195" s="52"/>
-      <c r="G195" s="53"/>
-      <c r="H195" s="52"/>
-      <c r="I195" s="52"/>
-      <c r="J195" s="52"/>
-      <c r="K195" s="52"/>
-      <c r="L195" s="52"/>
-      <c r="M195" s="53"/>
+      <c r="D195" s="52">
+        <v>23770.95</v>
+      </c>
+      <c r="E195" s="52">
+        <v>10204.54</v>
+      </c>
+      <c r="F195" s="52">
+        <v>13566.41</v>
+      </c>
+      <c r="G195" s="53">
+        <v>0.5707138334816235</v>
+      </c>
+      <c r="H195" s="52">
+        <v>14310.96</v>
+      </c>
+      <c r="I195" s="52">
+        <v>6935.96</v>
+      </c>
+      <c r="J195" s="52">
+        <v>7389.339999999999</v>
+      </c>
+      <c r="K195" s="52">
+        <v>6605.05</v>
+      </c>
+      <c r="L195" s="52">
+        <v>784.289999999999</v>
+      </c>
+      <c r="M195" s="53">
+        <v>0.1061380312720756</v>
+      </c>
       <c r="N195" s="53"/>
-      <c r="O195" s="52"/>
-      <c r="P195" s="52"/>
-      <c r="Q195" s="52"/>
-      <c r="R195" s="53"/>
-      <c r="S195" s="54"/>
-      <c r="T195" s="54"/>
-      <c r="U195" s="54"/>
-      <c r="V195" s="53"/>
+      <c r="O195" s="52">
+        <v>6921.62</v>
+      </c>
+      <c r="P195" s="52">
+        <v>330.91</v>
+      </c>
+      <c r="Q195" s="52">
+        <v>6590.71</v>
+      </c>
+      <c r="R195" s="53">
+        <v>0.9521918279246766</v>
+      </c>
+      <c r="S195" s="54">
+        <v>140.15</v>
+      </c>
+      <c r="T195" s="54">
+        <v>5.75</v>
+      </c>
+      <c r="U195" s="54">
+        <v>134.4</v>
+      </c>
+      <c r="V195" s="53">
+        <v>0.9589725294327506</v>
+      </c>
       <c r="W195" s="53"/>
-      <c r="X195" s="55"/>
-      <c r="Y195" s="55"/>
-      <c r="Z195" s="53"/>
-      <c r="AA195" s="56"/>
+      <c r="X195" s="55">
+        <v>568.4486956521739</v>
+      </c>
+      <c r="Y195" s="55">
+        <v>67.49902570438813</v>
+      </c>
+      <c r="Z195" s="53">
+        <v>0.32030000000000003</v>
+      </c>
+      <c r="AA195" s="56">
+        <v>0.398</v>
+      </c>
       <c r="AB195" s="57"/>
       <c r="AD195" s="35"/>
       <c r="AE195" s="35"/>
@@ -21233,30 +21585,74 @@
       <c r="C216" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D216" s="52"/>
-      <c r="E216" s="52"/>
-      <c r="F216" s="52"/>
-      <c r="G216" s="53"/>
-      <c r="H216" s="52"/>
-      <c r="I216" s="52"/>
-      <c r="J216" s="52"/>
-      <c r="K216" s="52"/>
-      <c r="L216" s="52"/>
-      <c r="M216" s="53"/>
+      <c r="D216" s="52">
+        <v>137109.56</v>
+      </c>
+      <c r="E216" s="52">
+        <v>30174.75</v>
+      </c>
+      <c r="F216" s="52">
+        <v>106934.81</v>
+      </c>
+      <c r="G216" s="53">
+        <v>0.7799223482301307</v>
+      </c>
+      <c r="H216" s="52">
+        <v>117394.57</v>
+      </c>
+      <c r="I216" s="52">
+        <v>30594.96</v>
+      </c>
+      <c r="J216" s="52">
+        <v>99479.62000000001</v>
+      </c>
+      <c r="K216" s="52">
+        <v>30594.96</v>
+      </c>
+      <c r="L216" s="52">
+        <v>68884.66</v>
+      </c>
+      <c r="M216" s="53">
+        <v>0.692449971159922</v>
+      </c>
       <c r="N216" s="53"/>
-      <c r="O216" s="52"/>
-      <c r="P216" s="52"/>
-      <c r="Q216" s="52"/>
-      <c r="R216" s="53"/>
-      <c r="S216" s="54"/>
-      <c r="T216" s="54"/>
-      <c r="U216" s="54"/>
-      <c r="V216" s="53"/>
+      <c r="O216" s="52">
+        <v>17914.95</v>
+      </c>
+      <c r="P216" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q216" s="52">
+        <v>17914.95</v>
+      </c>
+      <c r="R216" s="53">
+        <v>1</v>
+      </c>
+      <c r="S216" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="T216" s="54">
+        <v>0</v>
+      </c>
+      <c r="U216" s="54">
+        <v>358.86</v>
+      </c>
+      <c r="V216" s="53">
+        <v>1</v>
+      </c>
       <c r="W216" s="53"/>
-      <c r="X216" s="55"/>
-      <c r="Y216" s="55"/>
-      <c r="Z216" s="53"/>
-      <c r="AA216" s="56"/>
+      <c r="X216" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y216" s="55">
+        <v>54.93783457863793</v>
+      </c>
+      <c r="Z216" s="53">
+        <v>-0.0139</v>
+      </c>
+      <c r="AA216" s="56">
+        <v>0.1438</v>
+      </c>
       <c r="AB216" s="57"/>
       <c r="AD216" s="35"/>
       <c r="AE216" s="35"/>
@@ -21586,30 +21982,74 @@
       <c r="C223" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D223" s="52"/>
-      <c r="E223" s="52"/>
-      <c r="F223" s="52"/>
-      <c r="G223" s="53"/>
-      <c r="H223" s="52"/>
-      <c r="I223" s="52"/>
-      <c r="J223" s="52"/>
-      <c r="K223" s="52"/>
-      <c r="L223" s="52"/>
-      <c r="M223" s="53"/>
+      <c r="D223" s="52">
+        <v>396453.46</v>
+      </c>
+      <c r="E223" s="52">
+        <v>306038.55</v>
+      </c>
+      <c r="F223" s="52">
+        <v>90414.91000000003</v>
+      </c>
+      <c r="G223" s="53">
+        <v>0.2280593288301735</v>
+      </c>
+      <c r="H223" s="52">
+        <v>295569.99</v>
+      </c>
+      <c r="I223" s="52">
+        <v>245307.56</v>
+      </c>
+      <c r="J223" s="52">
+        <v>178700.37</v>
+      </c>
+      <c r="K223" s="52">
+        <v>180550.95</v>
+      </c>
+      <c r="L223" s="52">
+        <v>-1850.5800000000163</v>
+      </c>
+      <c r="M223" s="53">
+        <v>-0.010355770388164369</v>
+      </c>
       <c r="N223" s="53"/>
-      <c r="O223" s="52"/>
-      <c r="P223" s="52"/>
-      <c r="Q223" s="52"/>
-      <c r="R223" s="53"/>
-      <c r="S223" s="54"/>
-      <c r="T223" s="54"/>
-      <c r="U223" s="54"/>
-      <c r="V223" s="53"/>
+      <c r="O223" s="52">
+        <v>116869.62</v>
+      </c>
+      <c r="P223" s="52">
+        <v>64756.61</v>
+      </c>
+      <c r="Q223" s="52">
+        <v>52113.009999999995</v>
+      </c>
+      <c r="R223" s="53">
+        <v>0.4459072426178848</v>
+      </c>
+      <c r="S223" s="54">
+        <v>2344.68</v>
+      </c>
+      <c r="T223" s="54">
+        <v>1377.92</v>
+      </c>
+      <c r="U223" s="54">
+        <v>966.7599999999998</v>
+      </c>
+      <c r="V223" s="53">
+        <v>0.4123206578296398</v>
+      </c>
       <c r="W223" s="53"/>
-      <c r="X223" s="55"/>
-      <c r="Y223" s="55"/>
-      <c r="Z223" s="53"/>
-      <c r="AA223" s="56"/>
+      <c r="X223" s="55">
+        <v>44.07439473989781</v>
+      </c>
+      <c r="Y223" s="55">
+        <v>43.0265399367206</v>
+      </c>
+      <c r="Z223" s="53">
+        <v>0.1984</v>
+      </c>
+      <c r="AA223" s="56">
+        <v>0.2545</v>
+      </c>
       <c r="AB223" s="57"/>
       <c r="AD223" s="35"/>
       <c r="AE223" s="35"/>
@@ -22683,7 +23123,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R71"/>
+  <dimension ref="A1:AD71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -22697,7 +23137,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -22719,7 +23159,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>102</v>
       </c>
@@ -22767,7 +23207,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -22785,7 +23225,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -22832,7 +23272,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -22849,7 +23289,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -22899,7 +23339,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -22916,7 +23356,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -22959,7 +23399,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -22976,7 +23416,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23023,7 +23463,7 @@
         <v>24.375135929463628</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23040,7 +23480,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23090,7 +23530,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23107,7 +23547,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23154,7 +23594,7 @@
         <v>89.17785714285712</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23171,7 +23611,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23216,7 +23656,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23233,7 +23673,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23283,7 +23723,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23300,7 +23740,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23339,7 +23779,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23356,7 +23796,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23397,7 +23837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23414,7 +23854,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -23453,7 +23893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -23470,7 +23910,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -23515,7 +23955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -23532,7 +23972,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -23575,7 +24015,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -23592,7 +24032,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -23635,7 +24075,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -23652,7 +24092,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -23699,7 +24139,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -23716,7 +24156,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -23761,7 +24201,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -23778,7 +24218,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -23821,7 +24261,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -23838,7 +24278,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -23879,7 +24319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -23896,7 +24336,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -23941,7 +24381,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -23958,7 +24398,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24001,7 +24441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24018,7 +24458,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24055,7 +24495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24072,7 +24512,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -24113,7 +24553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24130,7 +24570,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -24173,7 +24613,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24190,7 +24630,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -24201,10 +24641,10 @@
         <v>0</v>
       </c>
       <c r="D50" s="99">
-        <v>853.55</v>
+        <v>2116.21</v>
       </c>
       <c r="E50" s="99">
-        <v>-853.55</v>
+        <v>-2116.21</v>
       </c>
       <c r="F50" s="99"/>
       <c r="G50" s="100">
@@ -24222,7 +24662,7 @@
         <v>0</v>
       </c>
       <c r="M50" s="99">
-        <v>-853.55</v>
+        <v>-2116.21</v>
       </c>
       <c r="N50" s="98"/>
       <c r="O50" s="60">
@@ -24232,7 +24672,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24249,7 +24689,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -24260,10 +24700,10 @@
         <v>0</v>
       </c>
       <c r="D52" s="99">
-        <v>2629.5100000000093</v>
+        <v>2236.75</v>
       </c>
       <c r="E52" s="99">
-        <v>-2629.5100000000093</v>
+        <v>-2236.75</v>
       </c>
       <c r="F52" s="99"/>
       <c r="G52" s="100">
@@ -24285,16 +24725,16 @@
         <v>0</v>
       </c>
       <c r="M52" s="99">
-        <v>-3909.5100000000093</v>
+        <v>-3516.75</v>
       </c>
       <c r="N52" s="98">
         <v>-304.75</v>
       </c>
       <c r="O52" s="60">
-        <v>14.333675527039448</v>
-      </c>
-    </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>12.893675527039413</v>
+      </c>
+    </row>
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24311,7 +24751,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -24356,7 +24796,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24373,7 +24813,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -24418,7 +24858,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -24435,7 +24875,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -24472,7 +24912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -24489,7 +24929,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -24506,7 +24946,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -24523,7 +24963,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -24544,7 +24984,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -24561,7 +25001,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -24602,7 +25042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -24619,7 +25059,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -24630,14 +25070,14 @@
         <v>34650.399999999965</v>
       </c>
       <c r="D66" s="99">
-        <v>7430.429999999993</v>
+        <v>10984.75</v>
       </c>
       <c r="E66" s="99">
-        <v>27219.969999999972</v>
+        <v>23665.649999999965</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
-        <v>0.7855600512548195</v>
+        <v>0.6829834576224225</v>
       </c>
       <c r="H66" s="100">
         <v>0.256265521519856</v>
@@ -24652,19 +25092,19 @@
         <v>3200</v>
       </c>
       <c r="L66" s="100">
-        <v>0.6932090250040402</v>
+        <v>0.5906324313716432</v>
       </c>
       <c r="M66" s="99">
-        <v>24019.969999999972</v>
+        <v>20465.649999999965</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>-25.71043082686644</v>
-      </c>
-    </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>-21.90596735349207</v>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -24699,7 +25139,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -24716,7 +25156,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -24733,7 +25173,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>122</v>
       </c>
@@ -24744,22 +25184,22 @@
         <v>88818.76999999996</v>
       </c>
       <c r="D70" s="104">
-        <v>39414.08000000001</v>
+        <v>43838.3</v>
       </c>
       <c r="E70" s="105">
-        <v>49404.68999999996</v>
+        <v>44980.469999999965</v>
       </c>
       <c r="F70" s="106" t="s">
         <v>124</v>
       </c>
       <c r="G70" s="107">
-        <v>0.5562415466910877</v>
+        <v>0.5064297783002397</v>
       </c>
       <c r="H70" s="108" t="s">
         <v>125</v>
       </c>
       <c r="I70" s="109">
-        <v>-0.02733555080756062</v>
+        <v>-0.07714731919840859</v>
       </c>
       <c r="J70" s="36"/>
       <c r="K70" s="36"/>
@@ -24768,7 +25208,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>126</v>
@@ -25151,7 +25591,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB110"/>
+  <dimension ref="A1:AD110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25162,7 +25602,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25183,7 +25623,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>127</v>
@@ -25245,7 +25685,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>143</v>
       </c>
@@ -25303,7 +25743,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25339,7 +25779,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25358,7 +25798,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25392,7 +25832,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25411,7 +25851,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -25445,7 +25885,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -25464,7 +25904,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -25502,7 +25942,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -25521,7 +25961,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -25559,7 +25999,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -25578,7 +26018,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -25616,7 +26056,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -25635,7 +26075,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -25668,7 +26108,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -25687,7 +26127,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -25720,7 +26160,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -25739,7 +26179,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -25770,7 +26210,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -25789,7 +26229,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -25824,7 +26264,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -25843,7 +26283,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -25876,7 +26316,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -25895,7 +26335,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -25926,7 +26366,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -25945,7 +26385,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -25977,7 +26417,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -25996,7 +26436,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -26032,7 +26472,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26051,7 +26491,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -26080,7 +26520,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26099,7 +26539,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -26130,7 +26570,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26149,7 +26589,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -26182,7 +26622,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26201,7 +26641,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -26237,7 +26677,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26256,7 +26696,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -26291,7 +26731,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26310,7 +26750,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -26340,7 +26780,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26359,7 +26799,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -26399,7 +26839,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -26418,7 +26858,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -26447,7 +26887,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -26466,7 +26906,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -26499,7 +26939,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -26518,7 +26958,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -26529,10 +26969,10 @@
         <v>65.13</v>
       </c>
       <c r="D50" s="54">
-        <v>0</v>
+        <v>24.33</v>
       </c>
       <c r="E50" s="54">
-        <v>65.13</v>
+        <v>40.8</v>
       </c>
       <c r="F50" s="54"/>
       <c r="G50" s="54"/>
@@ -26551,7 +26991,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -26570,7 +27010,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -26606,7 +27046,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -26625,7 +27065,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -26661,7 +27101,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -26680,7 +27120,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -26714,7 +27154,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -26733,7 +27173,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -26768,7 +27208,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -26787,7 +27227,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -26806,7 +27246,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -26825,7 +27265,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -26846,7 +27286,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -26865,7 +27305,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -26898,7 +27338,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -26917,7 +27357,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -26928,10 +27368,10 @@
         <v>2344.68</v>
       </c>
       <c r="D66" s="54">
-        <v>1335</v>
+        <v>1377.92</v>
       </c>
       <c r="E66" s="54">
-        <v>1009.6799999999998</v>
+        <v>966.7599999999998</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>
@@ -26956,7 +27396,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -26985,7 +27425,7 @@
       <c r="P67" s="54"/>
       <c r="Q67" s="54"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27004,7 +27444,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="142"/>
       <c r="B69" s="143"/>
       <c r="C69" s="35"/>
@@ -27023,7 +27463,7 @@
       <c r="P69" s="35"/>
       <c r="Q69" s="144"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="145"/>
       <c r="B70" s="145"/>
       <c r="C70" s="145"/>
@@ -27042,7 +27482,7 @@
       <c r="P70" s="145"/>
       <c r="Q70" s="145"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="146" t="s">
         <v>147</v>
@@ -27087,7 +27527,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -27126,7 +27566,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="77" t="s">
         <v>149</v>
@@ -27155,7 +27595,7 @@
       <c r="P73" s="20"/>
       <c r="Q73" s="20"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="148" t="s">
         <v>150</v>
@@ -27200,7 +27640,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="151" t="s">
         <v>151</v>
@@ -27245,7 +27685,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
@@ -27264,7 +27704,7 @@
       <c r="P76" s="35"/>
       <c r="Q76" s="144"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="156" t="s">
         <v>152</v>
@@ -27311,7 +27751,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="161"/>
       <c r="B78" s="162" t="s">
         <v>154</v>
@@ -27356,7 +27796,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -27375,7 +27815,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="164" t="s">
         <v>155</v>
@@ -27398,7 +27838,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="167" t="s">
         <v>157</v>
@@ -27421,7 +27861,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -27444,7 +27884,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -27467,7 +27907,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -27490,7 +27930,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -27513,7 +27953,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -27536,7 +27976,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -27559,7 +27999,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -27582,7 +28022,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -27605,7 +28045,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -27628,7 +28068,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -27651,7 +28091,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -27672,7 +28112,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -27693,7 +28133,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -27714,7 +28154,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -27735,7 +28175,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -27756,7 +28196,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -27777,7 +28217,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -27798,7 +28238,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -27821,7 +28261,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -27844,7 +28284,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -27867,7 +28307,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -27890,7 +28330,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -27913,7 +28353,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -27936,7 +28376,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -27959,7 +28399,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -27978,7 +28418,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -27997,7 +28437,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19"/>
       <c r="C108" s="131"/>
@@ -28016,7 +28456,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="169"/>
       <c r="C109" s="150"/>
@@ -28035,7 +28475,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="164" t="s">
         <v>175</v>
@@ -28109,10 +28549,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>176</v>
       </c>
@@ -28144,7 +28585,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>177</v>
       </c>
@@ -28177,7 +28618,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>178</v>
       </c>
@@ -28210,7 +28651,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>179</v>
       </c>
@@ -28243,7 +28684,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>180</v>
       </c>
@@ -28276,7 +28717,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>181</v>
       </c>
@@ -28309,7 +28750,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>182</v>
       </c>
@@ -28342,7 +28783,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>183</v>
       </c>
@@ -28375,7 +28816,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28406,7 +28847,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -28437,7 +28878,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>184</v>
       </c>
@@ -28470,7 +28911,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>185</v>
       </c>
@@ -28503,7 +28944,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>186</v>
       </c>
@@ -28536,7 +28977,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>187</v>
       </c>
@@ -28569,7 +29010,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>188</v>
       </c>
@@ -28602,7 +29043,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>189</v>
       </c>
@@ -28635,7 +29076,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>190</v>
       </c>
@@ -28668,7 +29109,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>191</v>
       </c>
@@ -28701,7 +29142,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>192</v>
       </c>
@@ -28734,7 +29175,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>193</v>
       </c>
@@ -28767,7 +29208,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>194</v>
       </c>
@@ -28800,7 +29241,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>195</v>
       </c>
@@ -28833,7 +29274,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>196</v>
       </c>
@@ -28866,7 +29307,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>197</v>
       </c>
@@ -28899,7 +29340,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>198</v>
       </c>
@@ -28932,7 +29373,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>199</v>
       </c>
@@ -28965,7 +29406,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>200</v>
       </c>
@@ -28997,7 +29438,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>201</v>
       </c>
@@ -29029,7 +29470,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>202</v>
       </c>
@@ -29061,7 +29502,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>203</v>
       </c>
@@ -29093,7 +29534,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>204</v>
       </c>
@@ -29125,7 +29566,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29155,7 +29596,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29185,7 +29626,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>205</v>
       </c>
@@ -29217,7 +29658,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>206</v>
       </c>
@@ -29249,7 +29690,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>207</v>
       </c>
@@ -29281,7 +29722,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>208</v>
       </c>
@@ -29313,7 +29754,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>209</v>
       </c>
@@ -29345,7 +29786,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29375,7 +29816,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>210</v>
       </c>
@@ -29407,7 +29848,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>211</v>
       </c>
@@ -29439,7 +29880,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>212</v>
       </c>
@@ -29471,7 +29912,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>213</v>
       </c>
@@ -29503,7 +29944,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -29533,7 +29974,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -29563,7 +30004,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -29593,7 +30034,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -29623,7 +30064,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>214</v>
       </c>
@@ -29655,7 +30096,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>215</v>
       </c>
@@ -29687,7 +30128,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -29717,7 +30158,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -29747,7 +30188,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -29777,7 +30218,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -29807,7 +30248,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -29837,7 +30278,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -29932,10 +30373,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>216</v>
       </c>
@@ -29967,7 +30409,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -29998,7 +30440,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30029,7 +30471,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30060,7 +30502,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30091,7 +30533,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30122,7 +30564,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30153,7 +30595,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30184,7 +30626,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30215,7 +30657,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -30246,7 +30688,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -30277,7 +30719,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -30308,7 +30750,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -30339,7 +30781,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -30370,7 +30812,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -30401,7 +30843,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -30432,7 +30874,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -30463,7 +30905,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -30494,7 +30936,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -30525,7 +30967,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -30556,7 +30998,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -30586,7 +31028,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -30616,7 +31058,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -30646,7 +31088,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -30676,7 +31118,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -30706,7 +31148,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -30736,7 +31178,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -30766,7 +31208,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -30796,7 +31238,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -30826,7 +31268,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -30856,7 +31298,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -30886,7 +31328,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -30916,7 +31358,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -30946,7 +31388,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -30976,7 +31418,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -31006,7 +31448,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -31036,7 +31478,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>214</v>
       </c>
@@ -31068,7 +31510,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>215</v>
       </c>
@@ -31100,7 +31542,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -31130,7 +31572,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -31160,7 +31602,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -31190,7 +31632,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -31220,7 +31662,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -31250,7 +31692,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -52993,19 +53435,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -53019,7 +53461,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>223</v>
       </c>
@@ -53031,7 +53473,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>224</v>
       </c>
@@ -53042,7 +53484,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>225</v>
       </c>
@@ -53053,7 +53495,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>226</v>
       </c>
@@ -53064,13 +53506,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-07T21:27:59Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -16356,30 +16356,74 @@
       <c r="C118" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D118" s="52"/>
-      <c r="E118" s="52"/>
-      <c r="F118" s="52"/>
-      <c r="G118" s="53"/>
-      <c r="H118" s="52"/>
-      <c r="I118" s="52"/>
-      <c r="J118" s="52"/>
-      <c r="K118" s="52"/>
-      <c r="L118" s="52"/>
-      <c r="M118" s="53"/>
+      <c r="D118" s="52">
+        <v>21404.82</v>
+      </c>
+      <c r="E118" s="52">
+        <v>0</v>
+      </c>
+      <c r="F118" s="52">
+        <v>21404.82</v>
+      </c>
+      <c r="G118" s="53">
+        <v>1</v>
+      </c>
+      <c r="H118" s="52">
+        <v>17514.09</v>
+      </c>
+      <c r="I118" s="52">
+        <v>0</v>
+      </c>
+      <c r="J118" s="52">
+        <v>13318.880000000001</v>
+      </c>
+      <c r="K118" s="52">
+        <v>0</v>
+      </c>
+      <c r="L118" s="52">
+        <v>13318.880000000001</v>
+      </c>
+      <c r="M118" s="53">
+        <v>1</v>
+      </c>
       <c r="N118" s="53"/>
-      <c r="O118" s="52"/>
-      <c r="P118" s="52"/>
-      <c r="Q118" s="52"/>
-      <c r="R118" s="53"/>
-      <c r="S118" s="54"/>
-      <c r="T118" s="54"/>
-      <c r="U118" s="54"/>
-      <c r="V118" s="53"/>
+      <c r="O118" s="52">
+        <v>4195.21</v>
+      </c>
+      <c r="P118" s="52">
+        <v>0</v>
+      </c>
+      <c r="Q118" s="52">
+        <v>4195.21</v>
+      </c>
+      <c r="R118" s="53">
+        <v>1</v>
+      </c>
+      <c r="S118" s="54">
+        <v>84.05</v>
+      </c>
+      <c r="T118" s="54">
+        <v>0</v>
+      </c>
+      <c r="U118" s="54">
+        <v>84.05</v>
+      </c>
+      <c r="V118" s="53">
+        <v>1</v>
+      </c>
       <c r="W118" s="53"/>
-      <c r="X118" s="55"/>
-      <c r="Y118" s="55"/>
-      <c r="Z118" s="53"/>
-      <c r="AA118" s="56"/>
+      <c r="X118" s="55">
+        <v>0</v>
+      </c>
+      <c r="Y118" s="55">
+        <v>46.29062162403328</v>
+      </c>
+      <c r="Z118" s="53">
+        <v>0</v>
+      </c>
+      <c r="AA118" s="56">
+        <v>0.1818</v>
+      </c>
       <c r="AB118" s="57"/>
       <c r="AD118" s="35"/>
       <c r="AE118" s="35"/>
@@ -16709,30 +16753,74 @@
       <c r="C125" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D125" s="52"/>
-      <c r="E125" s="52"/>
-      <c r="F125" s="52"/>
-      <c r="G125" s="53"/>
-      <c r="H125" s="52"/>
-      <c r="I125" s="52"/>
-      <c r="J125" s="52"/>
-      <c r="K125" s="52"/>
-      <c r="L125" s="52"/>
-      <c r="M125" s="53"/>
+      <c r="D125" s="52">
+        <v>100987.51</v>
+      </c>
+      <c r="E125" s="52">
+        <v>67407.3</v>
+      </c>
+      <c r="F125" s="52">
+        <v>33580.20999999999</v>
+      </c>
+      <c r="G125" s="53">
+        <v>0.33251844708320855</v>
+      </c>
+      <c r="H125" s="52">
+        <v>82694.87</v>
+      </c>
+      <c r="I125" s="52">
+        <v>56814.23</v>
+      </c>
+      <c r="J125" s="52">
+        <v>68214.25</v>
+      </c>
+      <c r="K125" s="52">
+        <v>51957.8</v>
+      </c>
+      <c r="L125" s="52">
+        <v>16256.449999999997</v>
+      </c>
+      <c r="M125" s="53">
+        <v>0.23831457503380887</v>
+      </c>
       <c r="N125" s="53"/>
-      <c r="O125" s="52"/>
-      <c r="P125" s="52"/>
-      <c r="Q125" s="52"/>
-      <c r="R125" s="53"/>
-      <c r="S125" s="54"/>
-      <c r="T125" s="54"/>
-      <c r="U125" s="54"/>
-      <c r="V125" s="53"/>
+      <c r="O125" s="52">
+        <v>14480.62</v>
+      </c>
+      <c r="P125" s="52">
+        <v>4856.43</v>
+      </c>
+      <c r="Q125" s="52">
+        <v>9624.19</v>
+      </c>
+      <c r="R125" s="53">
+        <v>0.66462554780113</v>
+      </c>
+      <c r="S125" s="54">
+        <v>290.15</v>
+      </c>
+      <c r="T125" s="54">
+        <v>106</v>
+      </c>
+      <c r="U125" s="54">
+        <v>184.14999999999998</v>
+      </c>
+      <c r="V125" s="53">
+        <v>0.6346717215233499</v>
+      </c>
       <c r="W125" s="53"/>
-      <c r="X125" s="55"/>
-      <c r="Y125" s="55"/>
-      <c r="Z125" s="53"/>
-      <c r="AA125" s="56"/>
+      <c r="X125" s="55">
+        <v>99.93462264150943</v>
+      </c>
+      <c r="Y125" s="55">
+        <v>63.04545035767707</v>
+      </c>
+      <c r="Z125" s="53">
+        <v>0.1572</v>
+      </c>
+      <c r="AA125" s="56">
+        <v>0.1811</v>
+      </c>
       <c r="AB125" s="57"/>
       <c r="AD125" s="35"/>
       <c r="AE125" s="35"/>
@@ -17070,30 +17158,74 @@
       <c r="C132" s="51" t="s">
         <v>96</v>
       </c>
-      <c r="D132" s="52"/>
-      <c r="E132" s="52"/>
-      <c r="F132" s="52"/>
-      <c r="G132" s="53"/>
-      <c r="H132" s="52"/>
-      <c r="I132" s="52"/>
-      <c r="J132" s="52"/>
-      <c r="K132" s="52"/>
-      <c r="L132" s="52"/>
-      <c r="M132" s="53"/>
+      <c r="D132" s="52">
+        <v>31802.41</v>
+      </c>
+      <c r="E132" s="52">
+        <v>16498.64</v>
+      </c>
+      <c r="F132" s="52">
+        <v>15303.77</v>
+      </c>
+      <c r="G132" s="53">
+        <v>0.4812141595558324</v>
+      </c>
+      <c r="H132" s="52">
+        <v>23448.14</v>
+      </c>
+      <c r="I132" s="52">
+        <v>12360.83</v>
+      </c>
+      <c r="J132" s="52">
+        <v>15632.029999999999</v>
+      </c>
+      <c r="K132" s="52">
+        <v>11772.08</v>
+      </c>
+      <c r="L132" s="52">
+        <v>3859.949999999999</v>
+      </c>
+      <c r="M132" s="53">
+        <v>0.24692570318762178</v>
+      </c>
       <c r="N132" s="53"/>
-      <c r="O132" s="52"/>
-      <c r="P132" s="52"/>
-      <c r="Q132" s="52"/>
-      <c r="R132" s="53"/>
-      <c r="S132" s="54"/>
-      <c r="T132" s="54"/>
-      <c r="U132" s="54"/>
-      <c r="V132" s="53"/>
+      <c r="O132" s="52">
+        <v>7816.11</v>
+      </c>
+      <c r="P132" s="52">
+        <v>588.75</v>
+      </c>
+      <c r="Q132" s="52">
+        <v>7227.36</v>
+      </c>
+      <c r="R132" s="53">
+        <v>0.9246748062655208</v>
+      </c>
+      <c r="S132" s="54">
+        <v>156.69</v>
+      </c>
+      <c r="T132" s="54">
+        <v>11.5</v>
+      </c>
+      <c r="U132" s="54">
+        <v>145.19</v>
+      </c>
+      <c r="V132" s="53">
+        <v>0.9266066756015061</v>
+      </c>
       <c r="W132" s="53"/>
-      <c r="X132" s="55"/>
-      <c r="Y132" s="55"/>
-      <c r="Z132" s="53"/>
-      <c r="AA132" s="56"/>
+      <c r="X132" s="55">
+        <v>359.80956521739137</v>
+      </c>
+      <c r="Y132" s="55">
+        <v>53.31719360265494</v>
+      </c>
+      <c r="Z132" s="53">
+        <v>0.25079999999999997</v>
+      </c>
+      <c r="AA132" s="56">
+        <v>0.2627</v>
+      </c>
       <c r="AB132" s="57"/>
       <c r="AD132" s="35"/>
       <c r="AE132" s="35"/>
@@ -24289,16 +24421,16 @@
         <v>52040.560000000005</v>
       </c>
       <c r="D38" s="52">
-        <v>526.0599999999977</v>
+        <v>576.9800000000032</v>
       </c>
       <c r="E38" s="52">
-        <v>51514.50000000001</v>
+        <v>51463.58</v>
       </c>
       <c r="F38" s="52">
         <v>0</v>
       </c>
       <c r="G38" s="53">
-        <v>0.9898913462883566</v>
+        <v>0.9889128787238262</v>
       </c>
       <c r="H38" s="53">
         <v>0.1750921737769</v>
@@ -24309,10 +24441,10 @@
         <v>0</v>
       </c>
       <c r="L38" s="53">
-        <v>0.9898913462883566</v>
+        <v>0.9889128787238262</v>
       </c>
       <c r="M38" s="52">
-        <v>51514.50000000001</v>
+        <v>51463.58</v>
       </c>
       <c r="N38" s="54"/>
       <c r="O38" s="58">
@@ -25184,22 +25316,22 @@
         <v>88818.76999999996</v>
       </c>
       <c r="D70" s="104">
-        <v>43838.3</v>
+        <v>43889.220000000016</v>
       </c>
       <c r="E70" s="105">
-        <v>44980.469999999965</v>
+        <v>44929.54999999996</v>
       </c>
       <c r="F70" s="106" t="s">
         <v>124</v>
       </c>
       <c r="G70" s="107">
-        <v>0.5064297783002397</v>
+        <v>0.5058564760579322</v>
       </c>
       <c r="H70" s="108" t="s">
         <v>125</v>
       </c>
       <c r="I70" s="109">
-        <v>-0.07714731919840859</v>
+        <v>-0.07772062144071622</v>
       </c>
       <c r="J70" s="36"/>
       <c r="K70" s="36"/>
@@ -26652,10 +26784,10 @@
         <v>290.15</v>
       </c>
       <c r="D38" s="54">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E38" s="54">
-        <v>185.14999999999998</v>
+        <v>184.14999999999998</v>
       </c>
       <c r="F38" s="54"/>
       <c r="G38" s="54"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-07T21:30:29Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -17232,7 +17232,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>97</v>
@@ -23255,7 +23255,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD71"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -23269,7 +23269,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -23291,7 +23291,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>102</v>
       </c>
@@ -23339,7 +23339,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -23357,7 +23357,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -23404,7 +23404,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -23421,7 +23421,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -23471,7 +23471,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -23488,7 +23488,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -23531,7 +23531,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -23548,7 +23548,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23595,7 +23595,7 @@
         <v>24.375135929463628</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23612,7 +23612,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23662,7 +23662,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23679,7 +23679,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23726,7 +23726,7 @@
         <v>89.17785714285712</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23743,7 +23743,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23788,7 +23788,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23805,7 +23805,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23855,7 +23855,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23872,7 +23872,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23911,7 +23911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23928,7 +23928,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23969,7 +23969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23986,7 +23986,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24025,7 +24025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -24042,7 +24042,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24087,7 +24087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -24104,7 +24104,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24147,7 +24147,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -24164,7 +24164,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24207,7 +24207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -24224,7 +24224,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24271,7 +24271,7 @@
         <v>10.108588351431392</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -24288,7 +24288,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24333,7 +24333,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -24350,7 +24350,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24393,7 +24393,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -24410,7 +24410,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24451,7 +24451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -24468,7 +24468,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24513,7 +24513,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -24530,7 +24530,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24573,7 +24573,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24590,7 +24590,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24627,7 +24627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24644,7 +24644,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -24685,7 +24685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24702,7 +24702,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -24745,7 +24745,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24762,7 +24762,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -24804,7 +24804,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24821,7 +24821,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -24866,7 +24866,7 @@
         <v>12.893675527039413</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24883,7 +24883,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -24928,7 +24928,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24945,7 +24945,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -24990,7 +24990,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25007,7 +25007,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -25044,7 +25044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -25061,7 +25061,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -25078,7 +25078,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -25095,7 +25095,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -25116,7 +25116,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -25133,7 +25133,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -25174,7 +25174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -25191,7 +25191,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -25236,7 +25236,7 @@
         <v>-21.90596735349207</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -25271,7 +25271,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -25288,7 +25288,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -25305,7 +25305,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>122</v>
       </c>
@@ -25340,7 +25340,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>126</v>
@@ -25723,7 +25723,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD110"/>
+  <dimension ref="A1:AB110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25734,7 +25734,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25755,7 +25755,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>127</v>
@@ -25817,7 +25817,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>143</v>
       </c>
@@ -25875,7 +25875,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25911,7 +25911,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25930,7 +25930,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25964,7 +25964,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25983,7 +25983,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26017,7 +26017,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26036,7 +26036,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -26074,7 +26074,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -26093,7 +26093,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -26131,7 +26131,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -26150,7 +26150,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -26188,7 +26188,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -26207,7 +26207,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -26240,7 +26240,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -26259,7 +26259,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -26292,7 +26292,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -26311,7 +26311,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -26342,7 +26342,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -26361,7 +26361,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -26396,7 +26396,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -26415,7 +26415,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26448,7 +26448,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -26467,7 +26467,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26498,7 +26498,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -26517,7 +26517,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -26549,7 +26549,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -26568,7 +26568,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -26604,7 +26604,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26623,7 +26623,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -26652,7 +26652,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26671,7 +26671,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -26702,7 +26702,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26721,7 +26721,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -26754,7 +26754,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26773,7 +26773,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -26809,7 +26809,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26828,7 +26828,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -26863,7 +26863,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26882,7 +26882,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -26912,7 +26912,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26931,7 +26931,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -26971,7 +26971,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -26990,7 +26990,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27019,7 +27019,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27038,7 +27038,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -27071,7 +27071,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -27090,7 +27090,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -27123,7 +27123,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -27142,7 +27142,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -27178,7 +27178,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -27197,7 +27197,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -27233,7 +27233,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -27252,7 +27252,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -27286,7 +27286,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -27305,7 +27305,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -27340,7 +27340,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -27359,7 +27359,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -27378,7 +27378,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -27397,7 +27397,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -27418,7 +27418,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -27437,7 +27437,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -27470,7 +27470,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -27489,7 +27489,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -27528,7 +27528,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -27557,7 +27557,7 @@
       <c r="P67" s="54"/>
       <c r="Q67" s="54"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27576,7 +27576,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="142"/>
       <c r="B69" s="143"/>
       <c r="C69" s="35"/>
@@ -27595,7 +27595,7 @@
       <c r="P69" s="35"/>
       <c r="Q69" s="144"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="145"/>
       <c r="B70" s="145"/>
       <c r="C70" s="145"/>
@@ -27614,7 +27614,7 @@
       <c r="P70" s="145"/>
       <c r="Q70" s="145"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="146" t="s">
         <v>147</v>
@@ -27659,7 +27659,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -27698,7 +27698,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="77" t="s">
         <v>149</v>
@@ -27727,7 +27727,7 @@
       <c r="P73" s="20"/>
       <c r="Q73" s="20"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="148" t="s">
         <v>150</v>
@@ -27772,7 +27772,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="151" t="s">
         <v>151</v>
@@ -27817,7 +27817,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
@@ -27836,7 +27836,7 @@
       <c r="P76" s="35"/>
       <c r="Q76" s="144"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="156" t="s">
         <v>152</v>
@@ -27883,7 +27883,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="161"/>
       <c r="B78" s="162" t="s">
         <v>154</v>
@@ -27928,7 +27928,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -27947,7 +27947,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="164" t="s">
         <v>155</v>
@@ -27970,7 +27970,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="167" t="s">
         <v>157</v>
@@ -27993,7 +27993,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28016,7 +28016,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28039,7 +28039,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28062,7 +28062,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -28085,7 +28085,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -28108,7 +28108,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -28131,7 +28131,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -28154,7 +28154,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -28177,7 +28177,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -28200,7 +28200,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -28223,7 +28223,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -28244,7 +28244,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -28265,7 +28265,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -28286,7 +28286,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -28307,7 +28307,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -28328,7 +28328,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -28349,7 +28349,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -28370,7 +28370,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -28393,7 +28393,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -28416,7 +28416,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -28439,7 +28439,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -28462,7 +28462,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -28485,7 +28485,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -28508,7 +28508,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -28531,7 +28531,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -28550,7 +28550,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -28569,7 +28569,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19"/>
       <c r="C108" s="131"/>
@@ -28588,7 +28588,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="169"/>
       <c r="C109" s="150"/>
@@ -28607,7 +28607,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="164" t="s">
         <v>175</v>
@@ -28681,11 +28681,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>176</v>
       </c>
@@ -28717,7 +28716,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>177</v>
       </c>
@@ -28750,7 +28749,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>178</v>
       </c>
@@ -28783,7 +28782,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>179</v>
       </c>
@@ -28816,7 +28815,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>180</v>
       </c>
@@ -28849,7 +28848,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>181</v>
       </c>
@@ -28882,7 +28881,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>182</v>
       </c>
@@ -28915,7 +28914,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>183</v>
       </c>
@@ -28948,7 +28947,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28979,7 +28978,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29010,7 +29009,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>184</v>
       </c>
@@ -29043,7 +29042,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>185</v>
       </c>
@@ -29076,7 +29075,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>186</v>
       </c>
@@ -29109,7 +29108,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>187</v>
       </c>
@@ -29142,7 +29141,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>188</v>
       </c>
@@ -29175,7 +29174,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>189</v>
       </c>
@@ -29208,7 +29207,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>190</v>
       </c>
@@ -29241,7 +29240,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>191</v>
       </c>
@@ -29274,7 +29273,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>192</v>
       </c>
@@ -29307,7 +29306,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>193</v>
       </c>
@@ -29340,7 +29339,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>194</v>
       </c>
@@ -29373,7 +29372,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>195</v>
       </c>
@@ -29406,7 +29405,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>196</v>
       </c>
@@ -29439,7 +29438,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>197</v>
       </c>
@@ -29472,7 +29471,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>198</v>
       </c>
@@ -29505,7 +29504,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>199</v>
       </c>
@@ -29538,7 +29537,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>200</v>
       </c>
@@ -29570,7 +29569,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>201</v>
       </c>
@@ -29602,7 +29601,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>202</v>
       </c>
@@ -29634,7 +29633,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>203</v>
       </c>
@@ -29666,7 +29665,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>204</v>
       </c>
@@ -29698,7 +29697,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29728,7 +29727,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29758,7 +29757,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>205</v>
       </c>
@@ -29790,7 +29789,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>206</v>
       </c>
@@ -29822,7 +29821,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>207</v>
       </c>
@@ -29854,7 +29853,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>208</v>
       </c>
@@ -29886,7 +29885,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>209</v>
       </c>
@@ -29918,7 +29917,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29948,7 +29947,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>210</v>
       </c>
@@ -29980,7 +29979,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>211</v>
       </c>
@@ -30012,7 +30011,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>212</v>
       </c>
@@ -30044,7 +30043,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>213</v>
       </c>
@@ -30076,7 +30075,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -30106,7 +30105,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -30136,7 +30135,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -30166,7 +30165,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -30196,7 +30195,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>214</v>
       </c>
@@ -30228,7 +30227,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>215</v>
       </c>
@@ -30260,7 +30259,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -30290,7 +30289,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -30320,7 +30319,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -30350,7 +30349,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -30380,7 +30379,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -30410,7 +30409,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -30505,11 +30504,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>216</v>
       </c>
@@ -30541,7 +30539,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -30572,7 +30570,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30603,7 +30601,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30634,7 +30632,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30665,7 +30663,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30696,7 +30694,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30727,7 +30725,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30758,7 +30756,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30789,7 +30787,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -30820,7 +30818,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -30851,7 +30849,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -30882,7 +30880,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -30913,7 +30911,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -30944,7 +30942,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -30975,7 +30973,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31006,7 +31004,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31037,7 +31035,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31068,7 +31066,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31099,7 +31097,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -31130,7 +31128,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -31160,7 +31158,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -31190,7 +31188,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -31220,7 +31218,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -31250,7 +31248,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -31280,7 +31278,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -31310,7 +31308,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -31340,7 +31338,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -31370,7 +31368,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -31400,7 +31398,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -31430,7 +31428,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -31460,7 +31458,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -31490,7 +31488,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -31520,7 +31518,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -31550,7 +31548,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -31580,7 +31578,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -31610,7 +31608,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>214</v>
       </c>
@@ -31642,7 +31640,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>215</v>
       </c>
@@ -31674,7 +31672,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -31704,7 +31702,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -31734,7 +31732,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -31764,7 +31762,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -31794,7 +31792,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -31824,7 +31822,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -53567,19 +53565,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -53593,7 +53591,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>223</v>
       </c>
@@ -53605,7 +53603,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>224</v>
       </c>
@@ -53616,7 +53614,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>225</v>
       </c>
@@ -53627,7 +53625,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>226</v>
       </c>
@@ -53638,13 +53636,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-08T01:48:51Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -25894,8 +25894,12 @@
       <c r="F4" s="54">
         <v>0</v>
       </c>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
+      <c r="G4" s="54">
+        <v>0</v>
+      </c>
+      <c r="H4" s="54">
+        <v>0</v>
+      </c>
       <c r="I4" s="54"/>
       <c r="J4" s="54"/>
       <c r="K4" s="54"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-08T02:12:54Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1136" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1137" uniqueCount="227">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -6010,7 +6010,9 @@
         <v>27</v>
       </c>
       <c r="N12" s="14"/>
-      <c r="O12" s="18"/>
+      <c r="O12" s="18" t="s">
+        <v>27</v>
+      </c>
       <c r="P12" s="13" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-08T02:22:41Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1137" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1138" uniqueCount="227">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -5816,7 +5816,9 @@
       <c r="J8" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="K8" s="13"/>
+      <c r="K8" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="L8" s="13" t="s">
         <v>27</v>
       </c>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-08T20:19:56Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -10276,72 +10276,72 @@
         <v>96</v>
       </c>
       <c r="D13" s="52">
-        <v>129074.86</v>
+        <v>129996.92</v>
       </c>
       <c r="E13" s="62">
         <v>85864.08</v>
       </c>
       <c r="F13" s="52">
-        <v>43210.78</v>
+        <v>44132.84</v>
       </c>
       <c r="G13" s="53">
-        <v>0.3347730146676123</v>
+        <v>0.3394914279507545</v>
       </c>
       <c r="H13" s="52">
-        <v>101420.72</v>
+        <v>101885.52</v>
       </c>
       <c r="I13" s="52">
-        <v>79791.03</v>
+        <v>79864.19</v>
       </c>
       <c r="J13" s="52">
-        <v>83645.65</v>
+        <v>83735.42000000001</v>
       </c>
       <c r="K13" s="52">
-        <v>71604.5</v>
+        <v>71677.66</v>
       </c>
       <c r="L13" s="52">
-        <v>12041.149999999994</v>
+        <v>12057.76000000001</v>
       </c>
       <c r="M13" s="53">
-        <v>0.1439542881189876</v>
+        <v>0.14399832233480178</v>
       </c>
       <c r="N13" s="53"/>
       <c r="O13" s="52">
-        <v>17775.07</v>
+        <v>18150.1</v>
       </c>
       <c r="P13" s="52">
         <v>8186.53</v>
       </c>
       <c r="Q13" s="52">
-        <v>9588.54</v>
+        <v>9963.57</v>
       </c>
       <c r="R13" s="53">
-        <v>0.5394375380800188</v>
+        <v>0.5489540002534422</v>
       </c>
       <c r="S13" s="54">
-        <v>356.07</v>
+        <v>363.57</v>
       </c>
       <c r="T13" s="54">
         <v>168.25</v>
       </c>
       <c r="U13" s="54">
-        <v>187.82</v>
+        <v>195.32</v>
       </c>
       <c r="V13" s="53">
-        <v>0.5274805515769371</v>
+        <v>0.5372280441180516</v>
       </c>
       <c r="W13" s="53"/>
       <c r="X13" s="55">
-        <v>36.09539375928678</v>
+        <v>35.660564635958394</v>
       </c>
       <c r="Y13" s="55">
-        <v>77.66490997775718</v>
+        <v>77.32043896850674</v>
       </c>
       <c r="Z13" s="53">
-        <v>0.0707</v>
+        <v>0.0699</v>
       </c>
       <c r="AA13" s="56">
-        <v>0.2142</v>
+        <v>0.2162</v>
       </c>
       <c r="AB13" s="57"/>
       <c r="AD13" s="35"/>
@@ -11092,72 +11092,72 @@
         <v>96</v>
       </c>
       <c r="D27" s="55">
-        <v>150850.82</v>
+        <v>153553.67</v>
       </c>
       <c r="E27" s="55">
         <v>144370.8</v>
       </c>
       <c r="F27" s="52">
-        <v>6480.020000000019</v>
+        <v>9182.870000000024</v>
       </c>
       <c r="G27" s="53">
-        <v>0.042956478459978</v>
+        <v>0.05980234793476459</v>
       </c>
       <c r="H27" s="52">
-        <v>102178.42</v>
+        <v>104026.09</v>
       </c>
       <c r="I27" s="52">
-        <v>89222.05</v>
+        <v>89600.47</v>
       </c>
       <c r="J27" s="52">
-        <v>62464.86</v>
+        <v>63812.49</v>
       </c>
       <c r="K27" s="52">
-        <v>58984</v>
+        <v>59331.43</v>
       </c>
       <c r="L27" s="52">
-        <v>3480.8600000000006</v>
+        <v>4481.059999999998</v>
       </c>
       <c r="M27" s="53">
-        <v>0.05572509087509362</v>
+        <v>0.07022230287518945</v>
       </c>
       <c r="N27" s="53"/>
       <c r="O27" s="52">
-        <v>39713.56</v>
+        <v>40213.6</v>
       </c>
       <c r="P27" s="52">
-        <v>30238.05</v>
+        <v>30269.04</v>
       </c>
       <c r="Q27" s="52">
-        <v>9475.509999999998</v>
+        <v>9944.559999999998</v>
       </c>
       <c r="R27" s="53">
-        <v>0.23859633837913294</v>
+        <v>0.2472934529611872</v>
       </c>
       <c r="S27" s="54">
-        <v>795.22</v>
+        <v>805.22</v>
       </c>
       <c r="T27" s="54">
-        <v>615</v>
+        <v>615.5</v>
       </c>
       <c r="U27" s="54">
-        <v>180.22000000000003</v>
+        <v>189.72000000000003</v>
       </c>
       <c r="V27" s="53">
-        <v>0.22662910892583188</v>
+        <v>0.2356126276048782</v>
       </c>
       <c r="W27" s="53"/>
       <c r="X27" s="55">
-        <v>89.67276422764228</v>
+        <v>88.9851015434606</v>
       </c>
       <c r="Y27" s="55">
-        <v>61.20621468124544</v>
+        <v>61.50814037389784</v>
       </c>
       <c r="Z27" s="53">
-        <v>0.382</v>
+        <v>0.37939999999999996</v>
       </c>
       <c r="AA27" s="56">
-        <v>0.3227</v>
+        <v>0.3225</v>
       </c>
       <c r="AB27" s="57"/>
       <c r="AD27" s="35"/>
@@ -11499,72 +11499,72 @@
         <v>96</v>
       </c>
       <c r="D34" s="52">
-        <v>396422.03</v>
+        <v>397238.61</v>
       </c>
       <c r="E34" s="52">
         <v>259347.71</v>
       </c>
       <c r="F34" s="52">
-        <v>137074.32000000004</v>
+        <v>137890.9</v>
       </c>
       <c r="G34" s="53">
-        <v>0.3457787651205964</v>
+        <v>0.34712360915773016</v>
       </c>
       <c r="H34" s="52">
-        <v>327431.12</v>
+        <v>328046.93</v>
       </c>
       <c r="I34" s="65">
-        <v>223659.54</v>
+        <v>223743.65</v>
       </c>
       <c r="J34" s="52">
-        <v>271519.78</v>
+        <v>271925.57</v>
       </c>
       <c r="K34" s="52">
-        <v>197370.72</v>
+        <v>197386.58</v>
       </c>
       <c r="L34" s="52">
-        <v>74149.06000000003</v>
+        <v>74538.99000000002</v>
       </c>
       <c r="M34" s="53">
-        <v>0.27308898084699396</v>
+        <v>0.27411541327283057</v>
       </c>
       <c r="N34" s="53"/>
       <c r="O34" s="52">
-        <v>55911.34</v>
+        <v>56121.36</v>
       </c>
       <c r="P34" s="52">
-        <v>26288.82</v>
+        <v>26357.07</v>
       </c>
       <c r="Q34" s="52">
-        <v>29622.519999999997</v>
+        <v>29764.29</v>
       </c>
       <c r="R34" s="53">
-        <v>0.5298123779540966</v>
+        <v>0.5303558217405994</v>
       </c>
       <c r="S34" s="54">
-        <v>1120.27</v>
+        <v>1124.47</v>
       </c>
       <c r="T34" s="54">
-        <v>607.75</v>
+        <v>609</v>
       </c>
       <c r="U34" s="54">
-        <v>512.52</v>
+        <v>515.47</v>
       </c>
       <c r="V34" s="53">
-        <v>0.4574968534371178</v>
+        <v>0.4584115183152952</v>
       </c>
       <c r="W34" s="53"/>
       <c r="X34" s="55">
-        <v>58.721793500617025</v>
+        <v>58.463152709359605</v>
       </c>
       <c r="Y34" s="55">
-        <v>61.5841822414239</v>
+        <v>61.532703026350184</v>
       </c>
       <c r="Z34" s="53">
-        <v>0.1376</v>
+        <v>0.1373</v>
       </c>
       <c r="AA34" s="56">
-        <v>0.174</v>
+        <v>0.1742</v>
       </c>
       <c r="AB34" s="57"/>
       <c r="AD34" s="35"/>
@@ -11921,7 +11921,7 @@
         <v>94098.32</v>
       </c>
       <c r="I41" s="52">
-        <v>49261.61</v>
+        <v>49519.82</v>
       </c>
       <c r="J41" s="52">
         <v>69042.09000000001</v>
@@ -11940,35 +11940,35 @@
         <v>25056.23</v>
       </c>
       <c r="P41" s="52">
-        <v>13577.87</v>
+        <v>13836.08</v>
       </c>
       <c r="Q41" s="52">
-        <v>11478.359999999999</v>
+        <v>11220.15</v>
       </c>
       <c r="R41" s="53">
-        <v>0.45810403241030273</v>
+        <v>0.44779881091449114</v>
       </c>
       <c r="S41" s="54">
         <v>501.83</v>
       </c>
       <c r="T41" s="54">
-        <v>299.5</v>
+        <v>308.25</v>
       </c>
       <c r="U41" s="54">
-        <v>202.32999999999998</v>
+        <v>193.57999999999998</v>
       </c>
       <c r="V41" s="53">
-        <v>0.40318434529621583</v>
+        <v>0.38574816172807525</v>
       </c>
       <c r="W41" s="53"/>
       <c r="X41" s="55">
-        <v>15.63679465776294</v>
+        <v>14.355263584752636</v>
       </c>
       <c r="Y41" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z41" s="53">
-        <v>0.0868</v>
+        <v>0.08199999999999999</v>
       </c>
       <c r="AA41" s="56">
         <v>0.2663</v>
@@ -12737,54 +12737,54 @@
         <v>109364.97</v>
       </c>
       <c r="I55" s="52">
-        <v>96483.38</v>
+        <v>97978.14</v>
       </c>
       <c r="J55" s="52">
         <v>75135.01000000001</v>
       </c>
       <c r="K55" s="52">
-        <v>71221.34</v>
+        <v>71357.43</v>
       </c>
       <c r="L55" s="52">
-        <v>3913.670000000013</v>
+        <v>3777.5800000000163</v>
       </c>
       <c r="M55" s="53">
-        <v>0.05208850042077604</v>
+        <v>0.050277227619987215</v>
       </c>
       <c r="N55" s="53"/>
       <c r="O55" s="52">
         <v>34229.96</v>
       </c>
       <c r="P55" s="52">
-        <v>25262.04</v>
+        <v>26620.71</v>
       </c>
       <c r="Q55" s="52">
-        <v>8967.919999999998</v>
+        <v>7609.25</v>
       </c>
       <c r="R55" s="53">
-        <v>0.2619903733454552</v>
+        <v>0.22229795185270448</v>
       </c>
       <c r="S55" s="54">
         <v>685.48</v>
       </c>
       <c r="T55" s="54">
-        <v>533.75</v>
+        <v>561.5</v>
       </c>
       <c r="U55" s="54">
-        <v>151.73000000000002</v>
+        <v>123.98000000000002</v>
       </c>
       <c r="V55" s="53">
-        <v>0.22134854408589605</v>
+        <v>0.18086596253720022</v>
       </c>
       <c r="W55" s="53"/>
       <c r="X55" s="55">
-        <v>58.699953161592504</v>
+        <v>53.13684772929653</v>
       </c>
       <c r="Y55" s="55">
         <v>67.00679527854935</v>
       </c>
       <c r="Z55" s="53">
-        <v>0.2451</v>
+        <v>0.2334</v>
       </c>
       <c r="AA55" s="56">
         <v>0.2958</v>
@@ -14345,19 +14345,19 @@
         <v>16606.83</v>
       </c>
       <c r="I83" s="52">
-        <v>12958.24</v>
+        <v>11832.36</v>
       </c>
       <c r="J83" s="52">
         <v>9659.990000000002</v>
       </c>
       <c r="K83" s="52">
-        <v>5354.12</v>
+        <v>4228.240000000001</v>
       </c>
       <c r="L83" s="52">
-        <v>4305.870000000002</v>
+        <v>5431.750000000001</v>
       </c>
       <c r="M83" s="53">
-        <v>0.44574269745620865</v>
+        <v>0.5622935427469387</v>
       </c>
       <c r="N83" s="53"/>
       <c r="O83" s="52">
@@ -14386,13 +14386,13 @@
       </c>
       <c r="W83" s="53"/>
       <c r="X83" s="55">
-        <v>44.94192893401015</v>
+        <v>52.562098138747885</v>
       </c>
       <c r="Y83" s="55">
         <v>63.7162162306752</v>
       </c>
       <c r="Z83" s="53">
-        <v>0.33880000000000005</v>
+        <v>0.39630000000000004</v>
       </c>
       <c r="AA83" s="56">
         <v>0.3479</v>
@@ -15554,66 +15554,66 @@
         <v>32473.02</v>
       </c>
       <c r="E104" s="69">
-        <v>33188.03</v>
+        <v>32473.03</v>
       </c>
       <c r="F104" s="52">
-        <v>-715.0099999999984</v>
+        <v>-0.00999999999839929</v>
       </c>
       <c r="G104" s="53">
-        <v>-0.022018586506582952</v>
+        <v>-3.0794795181967334e-7</v>
       </c>
       <c r="H104" s="52">
         <v>23075.07</v>
       </c>
       <c r="I104" s="52">
-        <v>30925.21</v>
+        <v>31170.94</v>
       </c>
       <c r="J104" s="52">
         <v>12691.21</v>
       </c>
       <c r="K104" s="52">
-        <v>15184.269999999999</v>
+        <v>15089.13</v>
       </c>
       <c r="L104" s="52">
-        <v>-2493.0599999999995</v>
+        <v>-2397.92</v>
       </c>
       <c r="M104" s="53">
-        <v>-0.1964398981657383</v>
+        <v>-0.18894337104184708</v>
       </c>
       <c r="N104" s="53"/>
       <c r="O104" s="52">
         <v>10383.86</v>
       </c>
       <c r="P104" s="52">
-        <v>15740.94</v>
+        <v>16081.81</v>
       </c>
       <c r="Q104" s="52">
-        <v>-5357.08</v>
+        <v>-5697.949999999999</v>
       </c>
       <c r="R104" s="53">
-        <v>-0.5159044902377343</v>
+        <v>-0.5487313966097385</v>
       </c>
       <c r="S104" s="54">
         <v>208.2</v>
       </c>
       <c r="T104" s="54">
-        <v>317.25</v>
+        <v>324.25</v>
       </c>
       <c r="U104" s="54">
-        <v>-109.05000000000001</v>
+        <v>-116.05000000000001</v>
       </c>
       <c r="V104" s="53">
-        <v>-0.5237752161383286</v>
+        <v>-0.5573967339097023</v>
       </c>
       <c r="W104" s="53"/>
       <c r="X104" s="55">
-        <v>7.132608353033885</v>
+        <v>4.015697764070933</v>
       </c>
       <c r="Y104" s="55">
         <v>45.139084580403456</v>
       </c>
       <c r="Z104" s="53">
-        <v>0.0682</v>
+        <v>0.0401</v>
       </c>
       <c r="AA104" s="56">
         <v>0.2894</v>
@@ -16758,72 +16758,72 @@
         <v>96</v>
       </c>
       <c r="D125" s="52">
-        <v>100987.51</v>
+        <v>105896.96</v>
       </c>
       <c r="E125" s="52">
         <v>67407.3</v>
       </c>
       <c r="F125" s="52">
-        <v>33580.20999999999</v>
+        <v>38489.66</v>
       </c>
       <c r="G125" s="53">
-        <v>0.33251844708320855</v>
+        <v>0.36346331377218005</v>
       </c>
       <c r="H125" s="52">
-        <v>82694.87</v>
+        <v>85934.2</v>
       </c>
       <c r="I125" s="52">
         <v>56814.23</v>
       </c>
       <c r="J125" s="52">
-        <v>68214.25</v>
+        <v>70065.72</v>
       </c>
       <c r="K125" s="52">
         <v>51957.8</v>
       </c>
       <c r="L125" s="52">
-        <v>16256.449999999997</v>
+        <v>18107.92</v>
       </c>
       <c r="M125" s="53">
-        <v>0.23831457503380887</v>
+        <v>0.2584419313752859</v>
       </c>
       <c r="N125" s="53"/>
       <c r="O125" s="52">
-        <v>14480.62</v>
+        <v>15868.48</v>
       </c>
       <c r="P125" s="52">
         <v>4856.43</v>
       </c>
       <c r="Q125" s="52">
-        <v>9624.19</v>
+        <v>11012.05</v>
       </c>
       <c r="R125" s="53">
-        <v>0.66462554780113</v>
+        <v>0.6939574552824215</v>
       </c>
       <c r="S125" s="54">
-        <v>290.15</v>
+        <v>317.92</v>
       </c>
       <c r="T125" s="54">
         <v>106</v>
       </c>
       <c r="U125" s="54">
-        <v>184.14999999999998</v>
+        <v>211.92000000000002</v>
       </c>
       <c r="V125" s="53">
-        <v>0.6346717215233499</v>
+        <v>0.6665827881227983</v>
       </c>
       <c r="W125" s="53"/>
       <c r="X125" s="55">
         <v>99.93462264150943</v>
       </c>
       <c r="Y125" s="55">
-        <v>63.04545035767707</v>
+        <v>62.79176131227983</v>
       </c>
       <c r="Z125" s="53">
         <v>0.1572</v>
       </c>
       <c r="AA125" s="56">
-        <v>0.1811</v>
+        <v>0.1885</v>
       </c>
       <c r="AB125" s="57"/>
       <c r="AD125" s="35"/>
@@ -17236,7 +17236,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>97</v>
@@ -17584,19 +17584,19 @@
         <v>22587.89</v>
       </c>
       <c r="I139" s="52">
-        <v>25905.23</v>
+        <v>25891.86</v>
       </c>
       <c r="J139" s="52">
         <v>12565.06</v>
       </c>
       <c r="K139" s="52">
-        <v>11805.46</v>
+        <v>11792.09</v>
       </c>
       <c r="L139" s="52">
-        <v>759.6000000000004</v>
+        <v>772.9699999999993</v>
       </c>
       <c r="M139" s="53">
-        <v>0.06045335239147289</v>
+        <v>0.061517414162765585</v>
       </c>
       <c r="N139" s="53"/>
       <c r="O139" s="52">
@@ -17625,13 +17625,13 @@
       </c>
       <c r="W139" s="53"/>
       <c r="X139" s="55">
-        <v>17.07140088105727</v>
+        <v>17.118519823788546</v>
       </c>
       <c r="Y139" s="55">
         <v>40.64013272149188</v>
       </c>
       <c r="Z139" s="53">
-        <v>0.1575</v>
+        <v>0.158</v>
       </c>
       <c r="AA139" s="56">
         <v>0.2654</v>
@@ -22134,7 +22134,7 @@
         <v>295569.99</v>
       </c>
       <c r="I223" s="52">
-        <v>245307.56</v>
+        <v>246358.99</v>
       </c>
       <c r="J223" s="52">
         <v>178700.37</v>
@@ -22153,35 +22153,35 @@
         <v>116869.62</v>
       </c>
       <c r="P223" s="52">
-        <v>64756.61</v>
+        <v>65808.04</v>
       </c>
       <c r="Q223" s="52">
-        <v>52113.009999999995</v>
+        <v>51061.58</v>
       </c>
       <c r="R223" s="53">
-        <v>0.4459072426178848</v>
+        <v>0.43691063597194896</v>
       </c>
       <c r="S223" s="54">
         <v>2344.68</v>
       </c>
       <c r="T223" s="54">
-        <v>1377.92</v>
+        <v>1401.92</v>
       </c>
       <c r="U223" s="54">
-        <v>966.7599999999998</v>
+        <v>942.7599999999998</v>
       </c>
       <c r="V223" s="53">
-        <v>0.4123206578296398</v>
+        <v>0.40208471944998886</v>
       </c>
       <c r="W223" s="53"/>
       <c r="X223" s="55">
-        <v>44.07439473989781</v>
+        <v>42.56987559917827</v>
       </c>
       <c r="Y223" s="55">
         <v>43.0265399367206</v>
       </c>
       <c r="Z223" s="53">
-        <v>0.1984</v>
+        <v>0.195</v>
       </c>
       <c r="AA223" s="56">
         <v>0.2545</v>
@@ -23259,7 +23259,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R71"/>
+  <dimension ref="A1:AD71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -23273,7 +23273,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -23295,7 +23295,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>102</v>
       </c>
@@ -23343,7 +23343,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -23361,7 +23361,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -23408,7 +23408,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -23425,7 +23425,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -23436,10 +23436,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="52">
-        <v>5653.709999999992</v>
+        <v>5726.869999999995</v>
       </c>
       <c r="E6" s="52">
-        <v>-5653.709999999992</v>
+        <v>-5726.869999999995</v>
       </c>
       <c r="F6" s="52">
         <v>0</v>
@@ -23463,19 +23463,19 @@
         <v>0</v>
       </c>
       <c r="M6" s="52">
-        <v>-7526.309999999992</v>
+        <v>-7599.469999999996</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>602.1047999999994</v>
+        <v>607.9575999999996</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -23492,7 +23492,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -23535,7 +23535,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -23552,7 +23552,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23563,10 +23563,10 @@
         <v>0</v>
       </c>
       <c r="D10" s="52">
-        <v>3373.6399999999994</v>
+        <v>3752.0599999999977</v>
       </c>
       <c r="E10" s="52">
-        <v>-3373.6399999999994</v>
+        <v>-3752.0599999999977</v>
       </c>
       <c r="F10" s="52">
         <v>0</v>
@@ -23590,16 +23590,16 @@
         <v>0</v>
       </c>
       <c r="M10" s="52">
-        <v>-8293.64</v>
+        <v>-8672.059999999998</v>
       </c>
       <c r="N10" s="54">
         <v>-388.25</v>
       </c>
       <c r="O10" s="58">
-        <v>24.375135929463628</v>
-      </c>
-    </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>25.48731814842027</v>
+      </c>
+    </row>
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23616,7 +23616,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23627,10 +23627,10 @@
         <v>0</v>
       </c>
       <c r="D12" s="52">
-        <v>7314.940000000002</v>
+        <v>7399.049999999988</v>
       </c>
       <c r="E12" s="52">
-        <v>-7314.940000000002</v>
+        <v>-7399.049999999988</v>
       </c>
       <c r="F12" s="52">
         <v>3</v>
@@ -23654,19 +23654,19 @@
         <v>0</v>
       </c>
       <c r="M12" s="52">
-        <v>-9951.940000000002</v>
+        <v>-10036.049999999988</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>-144.23101449275364</v>
+        <v>-145.44999999999982</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23683,7 +23683,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23694,10 +23694,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="52">
-        <v>6987.919999999998</v>
+        <v>7246.129999999997</v>
       </c>
       <c r="E14" s="52">
-        <v>-6987.919999999998</v>
+        <v>-7246.129999999997</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
@@ -23721,16 +23721,16 @@
         <v>0</v>
       </c>
       <c r="M14" s="52">
-        <v>-9987.919999999998</v>
+        <v>-10246.129999999997</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>89.17785714285712</v>
-      </c>
-    </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>91.48330357142855</v>
+      </c>
+    </row>
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23747,7 +23747,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23792,7 +23792,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23809,7 +23809,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23820,10 +23820,10 @@
         <v>0</v>
       </c>
       <c r="D18" s="52">
-        <v>1162.87000000001</v>
+        <v>2657.6300000000047</v>
       </c>
       <c r="E18" s="52">
-        <v>-1162.87000000001</v>
+        <v>-2657.6300000000047</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
@@ -23847,19 +23847,19 @@
         <v>0</v>
       </c>
       <c r="M18" s="52">
-        <v>-9362.87000000001</v>
+        <v>-10857.630000000005</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>49.538994708994764</v>
+        <v>57.4477777777778</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23876,7 +23876,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23915,7 +23915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23932,7 +23932,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23973,7 +23973,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23990,7 +23990,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24029,7 +24029,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -24046,7 +24046,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24057,10 +24057,10 @@
         <v>0</v>
       </c>
       <c r="D26" s="52">
-        <v>0</v>
+        <v>-1125.8799999999992</v>
       </c>
       <c r="E26" s="52">
-        <v>0</v>
+        <v>1125.8799999999992</v>
       </c>
       <c r="F26" s="52">
         <v>0</v>
@@ -24082,16 +24082,16 @@
         <v>0</v>
       </c>
       <c r="M26" s="52">
-        <v>0</v>
+        <v>1125.8799999999992</v>
       </c>
       <c r="N26" s="54">
         <v>-143.25</v>
       </c>
       <c r="O26" s="58">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>-7.859546247818494</v>
+      </c>
+    </row>
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -24108,7 +24108,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24151,7 +24151,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -24168,7 +24168,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24211,7 +24211,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -24228,7 +24228,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24236,19 +24236,19 @@
         <v>45</v>
       </c>
       <c r="C32" s="52">
-        <v>0</v>
+        <v>-715</v>
       </c>
       <c r="D32" s="52">
-        <v>0</v>
+        <v>245.72999999999956</v>
       </c>
       <c r="E32" s="52">
-        <v>0</v>
+        <v>-960.7299999999996</v>
       </c>
       <c r="F32" s="52">
         <v>0</v>
       </c>
       <c r="G32" s="53">
-        <v>0</v>
+        <v>1.343678321678321</v>
       </c>
       <c r="H32" s="53">
         <v>0.283172964220222</v>
@@ -24263,19 +24263,19 @@
         <v>2560</v>
       </c>
       <c r="L32" s="53">
-        <v>0</v>
+        <v>4.924097902097902</v>
       </c>
       <c r="M32" s="52">
-        <v>-2560</v>
+        <v>-3520.7299999999996</v>
       </c>
       <c r="N32" s="54">
         <v>-317.25</v>
       </c>
       <c r="O32" s="58">
-        <v>10.108588351431392</v>
-      </c>
-    </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>13.90219151036525</v>
+      </c>
+    </row>
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -24292,7 +24292,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24337,7 +24337,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -24354,7 +24354,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24397,7 +24397,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -24414,7 +24414,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24455,7 +24455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -24472,7 +24472,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24517,7 +24517,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -24534,7 +24534,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24545,10 +24545,10 @@
         <v>0</v>
       </c>
       <c r="D42" s="52">
-        <v>0</v>
+        <v>-13.369999999998981</v>
       </c>
       <c r="E42" s="52">
-        <v>0</v>
+        <v>13.369999999998981</v>
       </c>
       <c r="F42" s="52"/>
       <c r="G42" s="53">
@@ -24568,16 +24568,16 @@
         <v>0</v>
       </c>
       <c r="M42" s="52">
-        <v>0</v>
+        <v>13.369999999998981</v>
       </c>
       <c r="N42" s="54">
         <v>-266.75</v>
       </c>
       <c r="O42" s="58">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>-0.05012183692595682</v>
+      </c>
+    </row>
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24594,7 +24594,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24631,7 +24631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24648,7 +24648,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -24689,7 +24689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24706,7 +24706,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -24749,7 +24749,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24766,7 +24766,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -24808,7 +24808,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24825,7 +24825,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -24870,7 +24870,7 @@
         <v>12.893675527039413</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24887,7 +24887,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -24932,7 +24932,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24949,7 +24949,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -24994,7 +24994,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25011,7 +25011,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -25048,7 +25048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -25065,7 +25065,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -25082,7 +25082,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -25099,7 +25099,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -25120,7 +25120,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -25137,7 +25137,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -25178,7 +25178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -25195,7 +25195,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -25206,14 +25206,14 @@
         <v>34650.399999999965</v>
       </c>
       <c r="D66" s="99">
-        <v>10984.75</v>
+        <v>12036.179999999993</v>
       </c>
       <c r="E66" s="99">
-        <v>23665.649999999965</v>
+        <v>22614.219999999972</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
-        <v>0.6829834576224225</v>
+        <v>0.6526395077690299</v>
       </c>
       <c r="H66" s="100">
         <v>0.256265521519856</v>
@@ -25228,19 +25228,19 @@
         <v>3200</v>
       </c>
       <c r="L66" s="100">
-        <v>0.5906324313716432</v>
+        <v>0.5602884815182506</v>
       </c>
       <c r="M66" s="99">
-        <v>20465.649999999965</v>
+        <v>19414.219999999972</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>-21.90596735349207</v>
-      </c>
-    </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>-20.78054054054051</v>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -25275,7 +25275,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -25292,7 +25292,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -25309,7 +25309,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>122</v>
       </c>
@@ -25317,25 +25317,25 @@
         <v>123</v>
       </c>
       <c r="C70" s="104">
-        <v>88818.76999999996</v>
+        <v>88103.76999999996</v>
       </c>
       <c r="D70" s="104">
-        <v>43889.220000000016</v>
+        <v>46335.78999999999</v>
       </c>
       <c r="E70" s="105">
-        <v>44929.54999999996</v>
+        <v>41767.97999999998</v>
       </c>
       <c r="F70" s="106" t="s">
         <v>124</v>
       </c>
       <c r="G70" s="107">
-        <v>0.5058564760579322</v>
+        <v>0.47407710248948487</v>
       </c>
       <c r="H70" s="108" t="s">
         <v>125</v>
       </c>
       <c r="I70" s="109">
-        <v>-0.07772062144071622</v>
+        <v>-0.11423597423810607</v>
       </c>
       <c r="J70" s="36"/>
       <c r="K70" s="36"/>
@@ -25344,7 +25344,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>126</v>
@@ -25727,7 +25727,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB110"/>
+  <dimension ref="A1:AD110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25738,7 +25738,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25759,7 +25759,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>127</v>
@@ -25821,7 +25821,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>143</v>
       </c>
@@ -25879,7 +25879,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25919,7 +25919,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25938,7 +25938,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25946,13 +25946,13 @@
         <v>29</v>
       </c>
       <c r="C6" s="54">
-        <v>356.07</v>
+        <v>363.57</v>
       </c>
       <c r="D6" s="54">
         <v>168.25</v>
       </c>
       <c r="E6" s="54">
-        <v>187.82</v>
+        <v>195.32</v>
       </c>
       <c r="F6" s="54"/>
       <c r="G6" s="54"/>
@@ -25972,7 +25972,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25991,7 +25991,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26025,7 +26025,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26044,7 +26044,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -26052,13 +26052,13 @@
         <v>32</v>
       </c>
       <c r="C10" s="54">
-        <v>795.22</v>
+        <v>805.22</v>
       </c>
       <c r="D10" s="54">
-        <v>615</v>
+        <v>615.5</v>
       </c>
       <c r="E10" s="54">
-        <v>180.22000000000003</v>
+        <v>189.72000000000003</v>
       </c>
       <c r="F10" s="54"/>
       <c r="G10" s="54"/>
@@ -26082,7 +26082,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -26101,7 +26101,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -26109,13 +26109,13 @@
         <v>118</v>
       </c>
       <c r="C12" s="54">
-        <v>1120.27</v>
+        <v>1124.47</v>
       </c>
       <c r="D12" s="54">
-        <v>607.75</v>
+        <v>609</v>
       </c>
       <c r="E12" s="54">
-        <v>512.52</v>
+        <v>515.47</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -26139,7 +26139,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -26158,7 +26158,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -26169,10 +26169,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>299.5</v>
+        <v>308.25</v>
       </c>
       <c r="E14" s="54">
-        <v>202.32999999999998</v>
+        <v>193.57999999999998</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -26196,7 +26196,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -26215,7 +26215,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -26248,7 +26248,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -26267,7 +26267,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -26278,10 +26278,10 @@
         <v>685.48</v>
       </c>
       <c r="D18" s="54">
-        <v>533.75</v>
+        <v>561.5</v>
       </c>
       <c r="E18" s="54">
-        <v>151.73000000000002</v>
+        <v>123.98000000000002</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -26300,7 +26300,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -26319,7 +26319,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -26350,7 +26350,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -26369,7 +26369,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -26404,7 +26404,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -26423,7 +26423,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26456,7 +26456,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -26475,7 +26475,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26506,7 +26506,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -26525,7 +26525,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -26557,7 +26557,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -26576,7 +26576,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -26612,7 +26612,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26631,7 +26631,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -26642,10 +26642,10 @@
         <v>208.2</v>
       </c>
       <c r="D32" s="54">
-        <v>317.25</v>
+        <v>324.25</v>
       </c>
       <c r="E32" s="54">
-        <v>-109.05000000000001</v>
+        <v>-116.05000000000001</v>
       </c>
       <c r="F32" s="54"/>
       <c r="G32" s="54"/>
@@ -26660,7 +26660,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26679,7 +26679,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -26710,7 +26710,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26729,7 +26729,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -26762,7 +26762,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26781,7 +26781,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -26789,13 +26789,13 @@
         <v>49</v>
       </c>
       <c r="C38" s="54">
-        <v>290.15</v>
+        <v>317.92</v>
       </c>
       <c r="D38" s="54">
         <v>106</v>
       </c>
       <c r="E38" s="54">
-        <v>184.14999999999998</v>
+        <v>211.92000000000002</v>
       </c>
       <c r="F38" s="54"/>
       <c r="G38" s="54"/>
@@ -26817,7 +26817,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26836,7 +26836,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -26871,7 +26871,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26890,7 +26890,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -26920,7 +26920,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26939,7 +26939,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -26979,7 +26979,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -26998,7 +26998,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27027,7 +27027,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27046,7 +27046,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -27079,7 +27079,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -27098,7 +27098,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -27131,7 +27131,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -27150,7 +27150,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -27186,7 +27186,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -27205,7 +27205,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -27241,7 +27241,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -27260,7 +27260,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -27294,7 +27294,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -27313,7 +27313,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -27348,7 +27348,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -27367,7 +27367,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -27386,7 +27386,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -27405,7 +27405,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>60</v>
@@ -27426,7 +27426,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -27445,7 +27445,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -27478,7 +27478,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -27497,7 +27497,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -27508,10 +27508,10 @@
         <v>2344.68</v>
       </c>
       <c r="D66" s="54">
-        <v>1377.92</v>
+        <v>1401.92</v>
       </c>
       <c r="E66" s="54">
-        <v>966.7599999999998</v>
+        <v>942.7599999999998</v>
       </c>
       <c r="F66" s="54"/>
       <c r="G66" s="54"/>
@@ -27536,7 +27536,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -27565,7 +27565,7 @@
       <c r="P67" s="54"/>
       <c r="Q67" s="54"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27584,7 +27584,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="142"/>
       <c r="B69" s="143"/>
       <c r="C69" s="35"/>
@@ -27603,7 +27603,7 @@
       <c r="P69" s="35"/>
       <c r="Q69" s="144"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="145"/>
       <c r="B70" s="145"/>
       <c r="C70" s="145"/>
@@ -27622,7 +27622,7 @@
       <c r="P70" s="145"/>
       <c r="Q70" s="145"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="146" t="s">
         <v>147</v>
@@ -27667,7 +27667,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -27706,7 +27706,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="77" t="s">
         <v>149</v>
@@ -27735,7 +27735,7 @@
       <c r="P73" s="20"/>
       <c r="Q73" s="20"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="148" t="s">
         <v>150</v>
@@ -27780,7 +27780,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="151" t="s">
         <v>151</v>
@@ -27825,7 +27825,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
@@ -27844,7 +27844,7 @@
       <c r="P76" s="35"/>
       <c r="Q76" s="144"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="156" t="s">
         <v>152</v>
@@ -27891,7 +27891,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="161"/>
       <c r="B78" s="162" t="s">
         <v>154</v>
@@ -27936,7 +27936,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -27955,7 +27955,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="164" t="s">
         <v>155</v>
@@ -27978,7 +27978,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="167" t="s">
         <v>157</v>
@@ -28001,7 +28001,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28024,7 +28024,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28047,7 +28047,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28070,7 +28070,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -28093,7 +28093,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -28116,7 +28116,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -28139,7 +28139,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -28162,7 +28162,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -28185,7 +28185,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -28208,7 +28208,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -28231,7 +28231,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -28252,7 +28252,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -28273,7 +28273,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -28294,7 +28294,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -28315,7 +28315,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -28336,7 +28336,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -28357,7 +28357,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -28378,7 +28378,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -28401,7 +28401,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -28424,7 +28424,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -28447,7 +28447,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -28470,7 +28470,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -28493,7 +28493,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -28516,7 +28516,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -28539,7 +28539,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -28558,7 +28558,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -28577,7 +28577,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19"/>
       <c r="C108" s="131"/>
@@ -28596,7 +28596,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="169"/>
       <c r="C109" s="150"/>
@@ -28615,7 +28615,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="164" t="s">
         <v>175</v>
@@ -28689,10 +28689,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>176</v>
       </c>
@@ -28724,7 +28725,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>177</v>
       </c>
@@ -28757,7 +28758,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>178</v>
       </c>
@@ -28790,7 +28791,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>179</v>
       </c>
@@ -28823,7 +28824,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>180</v>
       </c>
@@ -28856,7 +28857,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>181</v>
       </c>
@@ -28889,7 +28890,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>182</v>
       </c>
@@ -28922,7 +28923,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>183</v>
       </c>
@@ -28955,7 +28956,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28986,7 +28987,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29017,7 +29018,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>184</v>
       </c>
@@ -29050,7 +29051,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>185</v>
       </c>
@@ -29083,7 +29084,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>186</v>
       </c>
@@ -29116,7 +29117,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>187</v>
       </c>
@@ -29149,7 +29150,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>188</v>
       </c>
@@ -29182,7 +29183,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>189</v>
       </c>
@@ -29215,7 +29216,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>190</v>
       </c>
@@ -29248,7 +29249,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>191</v>
       </c>
@@ -29281,7 +29282,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>192</v>
       </c>
@@ -29314,7 +29315,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>193</v>
       </c>
@@ -29347,7 +29348,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>194</v>
       </c>
@@ -29380,7 +29381,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>195</v>
       </c>
@@ -29413,7 +29414,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>196</v>
       </c>
@@ -29446,7 +29447,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>197</v>
       </c>
@@ -29479,7 +29480,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>198</v>
       </c>
@@ -29512,7 +29513,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>199</v>
       </c>
@@ -29545,7 +29546,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>200</v>
       </c>
@@ -29577,7 +29578,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>201</v>
       </c>
@@ -29609,7 +29610,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>202</v>
       </c>
@@ -29641,7 +29642,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>203</v>
       </c>
@@ -29673,7 +29674,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>204</v>
       </c>
@@ -29705,7 +29706,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29735,7 +29736,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29765,7 +29766,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>205</v>
       </c>
@@ -29797,7 +29798,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>206</v>
       </c>
@@ -29829,7 +29830,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>207</v>
       </c>
@@ -29861,7 +29862,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>208</v>
       </c>
@@ -29893,7 +29894,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>209</v>
       </c>
@@ -29925,7 +29926,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29955,7 +29956,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>210</v>
       </c>
@@ -29987,7 +29988,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>211</v>
       </c>
@@ -30019,7 +30020,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>212</v>
       </c>
@@ -30051,7 +30052,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>213</v>
       </c>
@@ -30083,7 +30084,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -30113,7 +30114,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -30143,7 +30144,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -30173,7 +30174,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -30203,7 +30204,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>214</v>
       </c>
@@ -30235,7 +30236,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>215</v>
       </c>
@@ -30267,7 +30268,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -30297,7 +30298,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -30327,7 +30328,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -30357,7 +30358,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -30387,7 +30388,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -30417,7 +30418,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -30512,10 +30513,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>216</v>
       </c>
@@ -30547,7 +30549,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -30578,7 +30580,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30609,7 +30611,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30640,7 +30642,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30671,7 +30673,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30702,7 +30704,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30733,7 +30735,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30764,7 +30766,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30795,7 +30797,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -30826,7 +30828,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -30857,7 +30859,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -30888,7 +30890,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -30919,7 +30921,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -30950,7 +30952,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -30981,7 +30983,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31012,7 +31014,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31043,7 +31045,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31074,7 +31076,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31105,7 +31107,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -31136,7 +31138,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -31166,7 +31168,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -31196,7 +31198,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -31226,7 +31228,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -31256,7 +31258,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -31286,7 +31288,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -31316,7 +31318,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -31346,7 +31348,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -31376,7 +31378,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -31406,7 +31408,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -31436,7 +31438,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -31466,7 +31468,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -31496,7 +31498,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -31526,7 +31528,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -31556,7 +31558,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -31586,7 +31588,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -31616,7 +31618,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>214</v>
       </c>
@@ -31648,7 +31650,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>215</v>
       </c>
@@ -31680,7 +31682,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -31710,7 +31712,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -31740,7 +31742,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -31770,7 +31772,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -31800,7 +31802,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -31830,7 +31832,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -53573,19 +53575,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -53599,7 +53601,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>223</v>
       </c>
@@ -53611,7 +53613,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>224</v>
       </c>
@@ -53622,7 +53624,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>225</v>
       </c>
@@ -53633,7 +53635,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>226</v>
       </c>
@@ -53644,13 +53646,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-08T20:25:28Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -13530,72 +13530,72 @@
         <v>96</v>
       </c>
       <c r="D69" s="52">
-        <v>47801.68</v>
+        <v>53029.71</v>
       </c>
       <c r="E69" s="52">
         <v>10650.43</v>
       </c>
       <c r="F69" s="52">
-        <v>37151.25</v>
+        <v>42379.28</v>
       </c>
       <c r="G69" s="53">
-        <v>0.7771954876899724</v>
+        <v>0.7991610740469823</v>
       </c>
       <c r="H69" s="52">
-        <v>35572.59</v>
+        <v>39055.78</v>
       </c>
       <c r="I69" s="52">
-        <v>10547.08</v>
+        <v>16807.92</v>
       </c>
       <c r="J69" s="52">
-        <v>27136.549999999996</v>
+        <v>29537.29</v>
       </c>
       <c r="K69" s="52">
-        <v>10398.3</v>
+        <v>16659.14</v>
       </c>
       <c r="L69" s="52">
-        <v>16738.249999999996</v>
+        <v>12878.150000000001</v>
       </c>
       <c r="M69" s="53">
-        <v>0.6168156969106242</v>
+        <v>0.4359963287085579</v>
       </c>
       <c r="N69" s="53"/>
       <c r="O69" s="52">
-        <v>8436.04</v>
+        <v>9518.49</v>
       </c>
       <c r="P69" s="52">
         <v>148.78</v>
       </c>
       <c r="Q69" s="52">
-        <v>8287.26</v>
+        <v>9369.71</v>
       </c>
       <c r="R69" s="53">
-        <v>0.9823637630926358</v>
+        <v>0.9843693695113405</v>
       </c>
       <c r="S69" s="54">
-        <v>169.32</v>
+        <v>193.32</v>
       </c>
       <c r="T69" s="54">
         <v>2.75</v>
       </c>
       <c r="U69" s="54">
-        <v>166.57</v>
+        <v>190.57</v>
       </c>
       <c r="V69" s="53">
-        <v>0.9837585636664304</v>
+        <v>0.9857748810262776</v>
       </c>
       <c r="W69" s="53"/>
       <c r="X69" s="55">
-        <v>37.58181818181818</v>
+        <v>-2239.0872727272726</v>
       </c>
       <c r="Y69" s="55">
-        <v>72.22475431425701</v>
+        <v>72.28396616733912</v>
       </c>
       <c r="Z69" s="53">
-        <v>0.0097</v>
+        <v>-0.5781000000000001</v>
       </c>
       <c r="AA69" s="56">
-        <v>0.2558</v>
+        <v>0.2635</v>
       </c>
       <c r="AB69" s="57"/>
       <c r="AD69" s="35"/>
@@ -13927,72 +13927,72 @@
         <v>96</v>
       </c>
       <c r="D76" s="52">
-        <v>77166.16</v>
+        <v>77408.3</v>
       </c>
       <c r="E76" s="52">
         <v>44764.99</v>
       </c>
       <c r="F76" s="52">
-        <v>32401.170000000006</v>
+        <v>32643.310000000005</v>
       </c>
       <c r="G76" s="53">
-        <v>0.41988832928838243</v>
+        <v>0.42170296983656796</v>
       </c>
       <c r="H76" s="52">
-        <v>54302.66</v>
+        <v>54446.73</v>
       </c>
       <c r="I76" s="52">
-        <v>29696.65</v>
+        <v>31054.89</v>
       </c>
       <c r="J76" s="52">
-        <v>31383.390000000003</v>
+        <v>31451.700000000004</v>
       </c>
       <c r="K76" s="52">
-        <v>23592.600000000002</v>
+        <v>23776.52</v>
       </c>
       <c r="L76" s="52">
-        <v>7790.790000000001</v>
+        <v>7675.180000000004</v>
       </c>
       <c r="M76" s="53">
-        <v>0.24824564841465502</v>
+        <v>0.24403068832527344</v>
       </c>
       <c r="N76" s="53"/>
       <c r="O76" s="52">
-        <v>22919.27</v>
+        <v>22995.03</v>
       </c>
       <c r="P76" s="52">
-        <v>6104.05</v>
+        <v>7278.37</v>
       </c>
       <c r="Q76" s="52">
-        <v>16815.22</v>
+        <v>15716.66</v>
       </c>
       <c r="R76" s="53">
-        <v>0.7336717094392623</v>
+        <v>0.6834807347500743</v>
       </c>
       <c r="S76" s="54">
-        <v>470.62</v>
+        <v>472.14</v>
       </c>
       <c r="T76" s="54">
-        <v>120.25</v>
+        <v>144.25</v>
       </c>
       <c r="U76" s="54">
-        <v>350.37</v>
+        <v>327.89</v>
       </c>
       <c r="V76" s="53">
-        <v>0.7444859971951894</v>
+        <v>0.6944762146820859</v>
       </c>
       <c r="W76" s="53"/>
       <c r="X76" s="55">
-        <v>125.30844074844074</v>
+        <v>95.04402079722703</v>
       </c>
       <c r="Y76" s="55">
-        <v>48.58165977967362</v>
+        <v>48.63296805100184</v>
       </c>
       <c r="Z76" s="53">
-        <v>0.33659999999999995</v>
+        <v>0.3063</v>
       </c>
       <c r="AA76" s="56">
-        <v>0.2963</v>
+        <v>0.2966</v>
       </c>
       <c r="AB76" s="57"/>
       <c r="AD76" s="35"/>
@@ -23943,10 +23943,10 @@
         <v>0</v>
       </c>
       <c r="D22" s="52">
-        <v>565.6499999999996</v>
+        <v>6826.489999999998</v>
       </c>
       <c r="E22" s="52">
-        <v>-565.6499999999996</v>
+        <v>-6826.489999999998</v>
       </c>
       <c r="F22" s="52">
         <v>3</v>
@@ -23966,7 +23966,7 @@
         <v>0</v>
       </c>
       <c r="M22" s="52">
-        <v>-562.6499999999996</v>
+        <v>-6823.489999999998</v>
       </c>
       <c r="N22" s="54"/>
       <c r="O22" s="58">
@@ -24001,10 +24001,10 @@
         <v>0</v>
       </c>
       <c r="D24" s="52">
-        <v>-2222.279999999999</v>
+        <v>-864.0400000000009</v>
       </c>
       <c r="E24" s="52">
-        <v>2222.279999999999</v>
+        <v>864.0400000000009</v>
       </c>
       <c r="F24" s="52">
         <v>3</v>
@@ -24022,7 +24022,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="52">
-        <v>2225.279999999999</v>
+        <v>867.0400000000009</v>
       </c>
       <c r="N24" s="54"/>
       <c r="O24" s="58">
@@ -25320,22 +25320,22 @@
         <v>88103.76999999996</v>
       </c>
       <c r="D70" s="104">
-        <v>46335.78999999999</v>
+        <v>53954.86999999998</v>
       </c>
       <c r="E70" s="105">
-        <v>41767.97999999998</v>
+        <v>34148.89999999998</v>
       </c>
       <c r="F70" s="106" t="s">
         <v>124</v>
       </c>
       <c r="G70" s="107">
-        <v>0.47407710248948487</v>
+        <v>0.38759862375923293</v>
       </c>
       <c r="H70" s="108" t="s">
         <v>125</v>
       </c>
       <c r="I70" s="109">
-        <v>-0.11423597423810607</v>
+        <v>-0.20071445296835796</v>
       </c>
       <c r="J70" s="36"/>
       <c r="K70" s="36"/>
@@ -26377,13 +26377,13 @@
         <v>39</v>
       </c>
       <c r="C22" s="54">
-        <v>169.32</v>
+        <v>193.32</v>
       </c>
       <c r="D22" s="54">
         <v>2.75</v>
       </c>
       <c r="E22" s="54">
-        <v>166.57</v>
+        <v>190.57</v>
       </c>
       <c r="F22" s="54"/>
       <c r="G22" s="54"/>
@@ -26431,13 +26431,13 @@
         <v>40</v>
       </c>
       <c r="C24" s="54">
-        <v>470.62</v>
+        <v>472.14</v>
       </c>
       <c r="D24" s="54">
-        <v>120.25</v>
+        <v>144.25</v>
       </c>
       <c r="E24" s="54">
-        <v>350.37</v>
+        <v>327.89</v>
       </c>
       <c r="F24" s="54"/>
       <c r="G24" s="54"/>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-08T20:57:10Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1138" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1139" uniqueCount="227">
   <si>
     <t xml:space="preserve">                        Updated Job Spreadsheet</t>
   </si>
@@ -197,6 +197,9 @@
     <t xml:space="preserve">Major Hornbrook </t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>NA</t>
   </si>
   <si>
@@ -249,9 +252,6 @@
   </si>
   <si>
     <t>224 Cashel St - Eastern WC Block Reno</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Week</t>
@@ -6859,9 +6859,11 @@
       <c r="O32" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="P32" s="18"/>
+      <c r="P32" s="18" t="s">
+        <v>46</v>
+      </c>
       <c r="Q32" s="15" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="R32" s="13"/>
       <c r="S32" s="13"/>
@@ -6916,7 +6918,7 @@
         <v>8840</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C34" s="13" t="s">
         <v>42</v>
@@ -6986,7 +6988,7 @@
         <v>8769</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
@@ -7054,7 +7056,7 @@
         <v>7901</v>
       </c>
       <c r="B38" s="25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C38" s="13"/>
       <c r="D38" s="13"/>
@@ -7122,7 +7124,7 @@
         <v>8923</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C40" s="13"/>
       <c r="D40" s="13"/>
@@ -7190,7 +7192,7 @@
         <v>7864</v>
       </c>
       <c r="B42" s="25" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C42" s="13"/>
       <c r="D42" s="13"/>
@@ -7258,7 +7260,7 @@
         <v>7912</v>
       </c>
       <c r="B44" s="25" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C44" s="13" t="s">
         <v>42</v>
@@ -7340,7 +7342,7 @@
         <v>8360</v>
       </c>
       <c r="B46" s="28" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C46" s="29" t="s">
         <v>42</v>
@@ -7432,7 +7434,7 @@
         <v>8337</v>
       </c>
       <c r="B48" s="21" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C48" s="13"/>
       <c r="D48" s="13"/>
@@ -7500,7 +7502,7 @@
         <v>9240</v>
       </c>
       <c r="B50" s="21" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C50" s="29"/>
       <c r="D50" s="29"/>
@@ -7568,7 +7570,7 @@
         <v>7428</v>
       </c>
       <c r="B52" s="21" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C52" s="29" t="s">
         <v>42</v>
@@ -7656,7 +7658,7 @@
         <v>9351</v>
       </c>
       <c r="B54" s="21" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C54" s="29" t="s">
         <v>42</v>
@@ -7726,7 +7728,7 @@
         <v>7429</v>
       </c>
       <c r="B56" s="21" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C56" s="29" t="s">
         <v>42</v>
@@ -7816,7 +7818,7 @@
         <v>9508</v>
       </c>
       <c r="B58" s="21" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C58" s="29" t="s">
         <v>42</v>
@@ -7974,7 +7976,7 @@
     <row r="62" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="27"/>
       <c r="B62" s="21" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C62" s="29"/>
       <c r="D62" s="29"/>
@@ -8042,7 +8044,7 @@
         <v>8946</v>
       </c>
       <c r="B64" s="21" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C64" s="29" t="s">
         <v>26</v>
@@ -8140,7 +8142,7 @@
         <v>8308</v>
       </c>
       <c r="B66" s="21" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C66" s="29" t="s">
         <v>42</v>
@@ -8218,10 +8220,10 @@
         <v>8530</v>
       </c>
       <c r="B68" s="21" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C68" s="29" t="s">
-        <v>64</v>
+        <v>46</v>
       </c>
       <c r="D68" s="29"/>
       <c r="E68" s="13"/>
@@ -15778,7 +15780,7 @@
         <v>8840</v>
       </c>
       <c r="B109" s="20" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C109" s="51" t="s">
         <v>92</v>
@@ -16187,7 +16189,7 @@
         <v>8769</v>
       </c>
       <c r="B116" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C116" s="51" t="s">
         <v>92</v>
@@ -16584,7 +16586,7 @@
         <v>7901</v>
       </c>
       <c r="B123" s="20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C123" s="51" t="s">
         <v>92</v>
@@ -16983,7 +16985,7 @@
         <v>8923</v>
       </c>
       <c r="B130" s="20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C130" s="51" t="s">
         <v>92</v>
@@ -17236,7 +17238,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>97</v>
@@ -17389,7 +17391,7 @@
         <v>7864</v>
       </c>
       <c r="B137" s="20" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C137" s="51" t="s">
         <v>92</v>
@@ -17796,7 +17798,7 @@
         <v>7912</v>
       </c>
       <c r="B144" s="20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C144" s="51" t="s">
         <v>92</v>
@@ -18189,7 +18191,7 @@
         <v>8360</v>
       </c>
       <c r="B151" s="74" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C151" s="51" t="s">
         <v>92</v>
@@ -18594,7 +18596,7 @@
         <v>8337</v>
       </c>
       <c r="B158" s="20" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C158" s="51" t="s">
         <v>92</v>
@@ -18993,7 +18995,7 @@
         <v>9240</v>
       </c>
       <c r="B165" s="20" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C165" s="51" t="s">
         <v>92</v>
@@ -19374,7 +19376,7 @@
         <v>7428</v>
       </c>
       <c r="B172" s="19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C172" s="51" t="s">
         <v>92</v>
@@ -19775,7 +19777,7 @@
         <v>9351</v>
       </c>
       <c r="B179" s="19" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C179" s="51" t="s">
         <v>92</v>
@@ -20180,7 +20182,7 @@
         <v>7429</v>
       </c>
       <c r="B186" s="19" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C186" s="51" t="s">
         <v>92</v>
@@ -20579,7 +20581,7 @@
         <v>9508</v>
       </c>
       <c r="B193" s="20" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C193" s="51" t="s">
         <v>92</v>
@@ -21267,7 +21269,7 @@
     <row r="207" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A207" s="19"/>
       <c r="B207" s="19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C207" s="51" t="s">
         <v>92</v>
@@ -21552,7 +21554,7 @@
         <v>8946</v>
       </c>
       <c r="B214" s="77" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C214" s="51" t="s">
         <v>92</v>
@@ -21945,7 +21947,7 @@
         <v>8308</v>
       </c>
       <c r="B221" s="19" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C221" s="51" t="s">
         <v>92</v>
@@ -22344,7 +22346,7 @@
         <v>8530</v>
       </c>
       <c r="B228" s="19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C228" s="51" t="s">
         <v>92</v>
@@ -23259,7 +23261,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD71"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -23273,7 +23275,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -23295,7 +23297,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>102</v>
       </c>
@@ -23343,7 +23345,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -23361,7 +23363,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -23408,7 +23410,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -23425,7 +23427,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -23475,7 +23477,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -23492,7 +23494,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -23535,7 +23537,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -23552,7 +23554,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23599,7 +23601,7 @@
         <v>25.48731814842027</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23616,7 +23618,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23666,7 +23668,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23683,7 +23685,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23730,7 +23732,7 @@
         <v>91.48330357142855</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23747,7 +23749,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23792,7 +23794,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23809,7 +23811,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23859,7 +23861,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23876,7 +23878,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23915,7 +23917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23932,7 +23934,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23973,7 +23975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23990,7 +23992,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24029,7 +24031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -24046,7 +24048,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24091,7 +24093,7 @@
         <v>-7.859546247818494</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -24108,7 +24110,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24151,7 +24153,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -24168,7 +24170,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24211,7 +24213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -24228,7 +24230,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24275,7 +24277,7 @@
         <v>13.90219151036525</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -24292,12 +24294,12 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
       <c r="B34" s="54" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C34" s="52">
         <v>0</v>
@@ -24337,7 +24339,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -24354,12 +24356,12 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
       <c r="B36" s="54" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C36" s="52">
         <v>0</v>
@@ -24397,7 +24399,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -24414,12 +24416,12 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
       <c r="B38" s="54" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C38" s="52">
         <v>52040.560000000005</v>
@@ -24455,7 +24457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -24472,12 +24474,12 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
       <c r="B40" s="54" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C40" s="52">
         <v>2127.8099999999995</v>
@@ -24517,7 +24519,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -24534,12 +24536,12 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
       <c r="B42" s="54" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C42" s="52">
         <v>0</v>
@@ -24577,7 +24579,7 @@
         <v>-0.05012183692595682</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24594,12 +24596,12 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
       <c r="B44" s="54" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C44" s="52">
         <v>0</v>
@@ -24631,7 +24633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24648,12 +24650,12 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
       <c r="B46" s="98" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C46" s="99">
         <v>0</v>
@@ -24689,7 +24691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24706,12 +24708,12 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
       <c r="B48" s="98" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C48" s="99">
         <v>0</v>
@@ -24749,7 +24751,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24766,12 +24768,12 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
       <c r="B50" s="98" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C50" s="99">
         <v>0</v>
@@ -24808,7 +24810,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24825,12 +24827,12 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
       <c r="B52" s="98" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C52" s="99">
         <v>0</v>
@@ -24870,7 +24872,7 @@
         <v>12.893675527039413</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24887,12 +24889,12 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
       <c r="B54" s="98" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C54" s="99">
         <v>0</v>
@@ -24932,7 +24934,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24949,12 +24951,12 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
       <c r="B56" s="98" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C56" s="99">
         <v>0</v>
@@ -24994,7 +24996,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25011,12 +25013,12 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
       <c r="B58" s="98" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C58" s="99">
         <v>0</v>
@@ -25048,7 +25050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -25065,7 +25067,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -25082,7 +25084,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -25099,10 +25101,10 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C62" s="99"/>
       <c r="D62" s="99"/>
@@ -25120,7 +25122,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -25137,12 +25139,12 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
       <c r="B64" s="98" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C64" s="99">
         <v>0</v>
@@ -25178,7 +25180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -25195,12 +25197,12 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
       <c r="B66" s="98" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C66" s="99">
         <v>34650.399999999965</v>
@@ -25240,7 +25242,7 @@
         <v>-20.78054054054051</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -25275,7 +25277,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -25292,7 +25294,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -25309,7 +25311,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>122</v>
       </c>
@@ -25344,7 +25346,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>126</v>
@@ -25727,7 +25729,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD110"/>
+  <dimension ref="A1:AB110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25738,7 +25740,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25759,7 +25761,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>127</v>
@@ -25821,7 +25823,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>143</v>
       </c>
@@ -25879,7 +25881,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25919,7 +25921,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25938,7 +25940,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25972,7 +25974,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25991,7 +25993,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26025,7 +26027,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26044,7 +26046,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -26082,7 +26084,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -26101,7 +26103,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -26139,7 +26141,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -26158,7 +26160,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -26196,7 +26198,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -26215,7 +26217,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -26248,7 +26250,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -26267,7 +26269,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -26300,7 +26302,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -26319,7 +26321,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -26350,7 +26352,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -26369,7 +26371,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -26404,7 +26406,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -26423,7 +26425,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26456,7 +26458,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -26475,7 +26477,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26506,7 +26508,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -26525,7 +26527,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -26557,7 +26559,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -26576,7 +26578,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -26612,7 +26614,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26631,7 +26633,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -26660,7 +26662,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26679,12 +26681,12 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C34" s="54">
         <v>324.19</v>
@@ -26710,7 +26712,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26729,12 +26731,12 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C36" s="54">
         <v>84.05</v>
@@ -26762,7 +26764,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26781,12 +26783,12 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
       <c r="B38" s="20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C38" s="54">
         <v>317.92</v>
@@ -26817,7 +26819,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26836,12 +26838,12 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
       <c r="B40" s="20" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C40" s="54">
         <v>156.69</v>
@@ -26871,7 +26873,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26890,12 +26892,12 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
       <c r="B42" s="20" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C42" s="54">
         <v>200.82</v>
@@ -26920,7 +26922,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26939,12 +26941,12 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
       <c r="B44" s="20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C44" s="54">
         <v>497.55</v>
@@ -26979,7 +26981,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -26998,12 +27000,12 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
       <c r="B46" s="75" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C46" s="54">
         <v>210.6</v>
@@ -27027,7 +27029,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27046,12 +27048,12 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
       <c r="B48" s="20" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C48" s="54">
         <v>110.44</v>
@@ -27079,7 +27081,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -27098,12 +27100,12 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
       <c r="B50" s="20" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C50" s="54">
         <v>65.13</v>
@@ -27131,7 +27133,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -27150,12 +27152,12 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
       <c r="B52" s="20" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C52" s="54">
         <v>659.73</v>
@@ -27186,7 +27188,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -27205,12 +27207,12 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
       <c r="B54" s="20" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C54" s="54">
         <v>125.17</v>
@@ -27241,7 +27243,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -27260,12 +27262,12 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
       <c r="B56" s="20" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C56" s="54">
         <v>130.62</v>
@@ -27294,7 +27296,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -27313,12 +27315,12 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
       <c r="B58" s="20" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C58" s="54">
         <v>140.15</v>
@@ -27348,7 +27350,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -27367,7 +27369,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -27386,7 +27388,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -27405,10 +27407,10 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C62" s="54"/>
       <c r="D62" s="54"/>
@@ -27426,7 +27428,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -27445,12 +27447,12 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
       <c r="B64" s="20" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C64" s="54">
         <v>358.86</v>
@@ -27478,7 +27480,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -27497,12 +27499,12 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C66" s="54">
         <v>2344.68</v>
@@ -27536,7 +27538,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -27565,7 +27567,7 @@
       <c r="P67" s="54"/>
       <c r="Q67" s="54"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27584,7 +27586,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="142"/>
       <c r="B69" s="143"/>
       <c r="C69" s="35"/>
@@ -27603,7 +27605,7 @@
       <c r="P69" s="35"/>
       <c r="Q69" s="144"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="145"/>
       <c r="B70" s="145"/>
       <c r="C70" s="145"/>
@@ -27622,7 +27624,7 @@
       <c r="P70" s="145"/>
       <c r="Q70" s="145"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="146" t="s">
         <v>147</v>
@@ -27667,7 +27669,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -27706,7 +27708,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="77" t="s">
         <v>149</v>
@@ -27735,7 +27737,7 @@
       <c r="P73" s="20"/>
       <c r="Q73" s="20"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="148" t="s">
         <v>150</v>
@@ -27780,7 +27782,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="151" t="s">
         <v>151</v>
@@ -27825,7 +27827,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
@@ -27844,7 +27846,7 @@
       <c r="P76" s="35"/>
       <c r="Q76" s="144"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="156" t="s">
         <v>152</v>
@@ -27891,7 +27893,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="161"/>
       <c r="B78" s="162" t="s">
         <v>154</v>
@@ -27936,7 +27938,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -27955,7 +27957,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="164" t="s">
         <v>155</v>
@@ -27978,7 +27980,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="167" t="s">
         <v>157</v>
@@ -28001,7 +28003,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28024,7 +28026,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28047,7 +28049,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28070,7 +28072,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -28093,7 +28095,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -28116,7 +28118,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -28139,7 +28141,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -28162,7 +28164,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -28185,7 +28187,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -28208,7 +28210,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -28231,7 +28233,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -28252,7 +28254,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -28273,7 +28275,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -28294,7 +28296,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -28315,7 +28317,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -28336,7 +28338,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -28357,7 +28359,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -28378,7 +28380,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -28401,7 +28403,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -28424,7 +28426,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -28447,7 +28449,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -28470,7 +28472,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -28493,7 +28495,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -28516,7 +28518,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -28539,7 +28541,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -28558,7 +28560,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -28577,7 +28579,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19"/>
       <c r="C108" s="131"/>
@@ -28596,7 +28598,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="169"/>
       <c r="C109" s="150"/>
@@ -28615,7 +28617,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="164" t="s">
         <v>175</v>
@@ -28689,11 +28691,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>176</v>
       </c>
@@ -28725,7 +28726,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>177</v>
       </c>
@@ -28758,7 +28759,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>178</v>
       </c>
@@ -28791,7 +28792,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>179</v>
       </c>
@@ -28824,7 +28825,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>180</v>
       </c>
@@ -28857,7 +28858,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>181</v>
       </c>
@@ -28890,7 +28891,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>182</v>
       </c>
@@ -28923,7 +28924,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>183</v>
       </c>
@@ -28956,7 +28957,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28987,7 +28988,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29018,7 +29019,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>184</v>
       </c>
@@ -29051,7 +29052,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>185</v>
       </c>
@@ -29084,7 +29085,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>186</v>
       </c>
@@ -29117,7 +29118,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>187</v>
       </c>
@@ -29150,7 +29151,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>188</v>
       </c>
@@ -29183,7 +29184,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>189</v>
       </c>
@@ -29216,7 +29217,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>190</v>
       </c>
@@ -29249,7 +29250,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>191</v>
       </c>
@@ -29282,7 +29283,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>192</v>
       </c>
@@ -29315,7 +29316,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>193</v>
       </c>
@@ -29348,7 +29349,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>194</v>
       </c>
@@ -29381,7 +29382,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>195</v>
       </c>
@@ -29414,7 +29415,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>196</v>
       </c>
@@ -29447,7 +29448,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>197</v>
       </c>
@@ -29480,7 +29481,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>198</v>
       </c>
@@ -29513,7 +29514,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>199</v>
       </c>
@@ -29546,7 +29547,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>200</v>
       </c>
@@ -29578,7 +29579,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>201</v>
       </c>
@@ -29610,7 +29611,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>202</v>
       </c>
@@ -29642,7 +29643,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>203</v>
       </c>
@@ -29674,7 +29675,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>204</v>
       </c>
@@ -29706,7 +29707,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29736,7 +29737,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29766,7 +29767,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>205</v>
       </c>
@@ -29798,7 +29799,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>206</v>
       </c>
@@ -29830,7 +29831,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>207</v>
       </c>
@@ -29862,7 +29863,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>208</v>
       </c>
@@ -29894,7 +29895,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>209</v>
       </c>
@@ -29926,7 +29927,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29956,7 +29957,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>210</v>
       </c>
@@ -29988,7 +29989,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>211</v>
       </c>
@@ -30020,7 +30021,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>212</v>
       </c>
@@ -30052,7 +30053,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>213</v>
       </c>
@@ -30084,7 +30085,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -30114,7 +30115,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -30144,7 +30145,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -30174,7 +30175,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -30204,7 +30205,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>214</v>
       </c>
@@ -30236,7 +30237,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>215</v>
       </c>
@@ -30268,7 +30269,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -30298,7 +30299,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -30328,7 +30329,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -30358,7 +30359,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -30388,7 +30389,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -30418,7 +30419,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -30513,11 +30514,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>216</v>
       </c>
@@ -30549,7 +30549,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -30580,7 +30580,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30611,7 +30611,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30642,7 +30642,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30673,7 +30673,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30704,7 +30704,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30735,7 +30735,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30766,7 +30766,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30797,7 +30797,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -30828,7 +30828,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -30859,7 +30859,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -30890,7 +30890,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -30921,7 +30921,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -30952,7 +30952,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -30983,7 +30983,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31014,7 +31014,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31045,7 +31045,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31076,7 +31076,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31107,7 +31107,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -31138,7 +31138,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -31168,7 +31168,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -31198,7 +31198,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -31228,7 +31228,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -31258,7 +31258,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -31288,7 +31288,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -31318,7 +31318,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -31348,7 +31348,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -31378,7 +31378,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -31408,7 +31408,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -31438,7 +31438,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -31468,7 +31468,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -31498,7 +31498,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -31528,7 +31528,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -31558,7 +31558,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -31588,7 +31588,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -31618,7 +31618,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>214</v>
       </c>
@@ -31650,7 +31650,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>215</v>
       </c>
@@ -31682,7 +31682,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -31712,7 +31712,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -31742,7 +31742,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -31772,7 +31772,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -31802,7 +31802,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -31832,7 +31832,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -53575,19 +53575,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -53601,7 +53601,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>223</v>
       </c>
@@ -53613,7 +53613,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>224</v>
       </c>
@@ -53624,7 +53624,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>225</v>
       </c>
@@ -53635,7 +53635,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>226</v>
       </c>
@@ -53646,13 +53646,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-08T21:05:20Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -17238,7 +17238,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>97</v>
@@ -23261,7 +23261,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R71"/>
+  <dimension ref="A1:AD71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -23275,7 +23275,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -23297,7 +23297,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>102</v>
       </c>
@@ -23345,7 +23345,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -23363,7 +23363,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -23410,7 +23410,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -23427,7 +23427,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -23477,7 +23477,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -23494,7 +23494,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -23537,7 +23537,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -23554,7 +23554,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23601,7 +23601,7 @@
         <v>25.48731814842027</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23618,7 +23618,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23668,7 +23668,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23685,7 +23685,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23732,7 +23732,7 @@
         <v>91.48330357142855</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23749,7 +23749,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23794,7 +23794,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23811,7 +23811,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23861,7 +23861,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23878,7 +23878,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23917,7 +23917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23934,7 +23934,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23975,7 +23975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23992,7 +23992,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24031,7 +24031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -24048,7 +24048,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24093,7 +24093,7 @@
         <v>-7.859546247818494</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -24110,7 +24110,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24153,7 +24153,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -24170,7 +24170,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24213,7 +24213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -24230,7 +24230,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24277,7 +24277,7 @@
         <v>13.90219151036525</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -24294,7 +24294,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24339,7 +24339,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -24356,7 +24356,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24399,7 +24399,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -24416,7 +24416,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24457,7 +24457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -24474,7 +24474,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24519,7 +24519,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -24536,7 +24536,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24579,7 +24579,7 @@
         <v>-0.05012183692595682</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24596,7 +24596,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24633,7 +24633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24650,7 +24650,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -24691,7 +24691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24708,7 +24708,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -24751,7 +24751,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24768,7 +24768,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -24810,7 +24810,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24827,7 +24827,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -24872,7 +24872,7 @@
         <v>12.893675527039413</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24889,7 +24889,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -24934,7 +24934,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24951,7 +24951,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -24996,7 +24996,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25013,7 +25013,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -25050,7 +25050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -25067,7 +25067,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -25084,7 +25084,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -25101,7 +25101,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>61</v>
@@ -25122,7 +25122,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -25139,7 +25139,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -25180,7 +25180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -25197,7 +25197,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -25242,7 +25242,7 @@
         <v>-20.78054054054051</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -25277,7 +25277,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -25294,7 +25294,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -25311,7 +25311,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>122</v>
       </c>
@@ -25346,7 +25346,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>126</v>
@@ -25729,7 +25729,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB110"/>
+  <dimension ref="A1:AD110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25740,7 +25740,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25761,7 +25761,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>127</v>
@@ -25823,7 +25823,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>143</v>
       </c>
@@ -25881,7 +25881,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25921,7 +25921,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25940,7 +25940,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25974,7 +25974,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25993,7 +25993,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26027,7 +26027,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26046,7 +26046,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -26084,7 +26084,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -26103,7 +26103,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -26141,7 +26141,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -26160,7 +26160,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -26198,7 +26198,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -26217,7 +26217,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -26250,7 +26250,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -26269,7 +26269,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -26302,7 +26302,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -26321,7 +26321,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -26352,7 +26352,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -26371,7 +26371,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -26406,7 +26406,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -26425,7 +26425,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26458,7 +26458,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -26477,7 +26477,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26508,7 +26508,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -26527,7 +26527,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -26559,7 +26559,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -26578,7 +26578,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -26614,7 +26614,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26633,7 +26633,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -26662,7 +26662,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26681,7 +26681,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -26712,7 +26712,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26731,7 +26731,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -26764,7 +26764,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26783,7 +26783,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -26819,7 +26819,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26838,7 +26838,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -26873,7 +26873,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26892,7 +26892,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -26922,7 +26922,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26941,7 +26941,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -26981,7 +26981,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -27000,7 +27000,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27029,7 +27029,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27048,7 +27048,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -27081,7 +27081,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -27100,7 +27100,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -27133,7 +27133,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -27152,7 +27152,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -27188,7 +27188,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -27207,7 +27207,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -27243,7 +27243,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -27262,7 +27262,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -27296,7 +27296,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -27315,7 +27315,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -27350,7 +27350,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -27369,7 +27369,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -27388,7 +27388,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -27407,7 +27407,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>61</v>
@@ -27428,7 +27428,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -27447,7 +27447,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -27480,7 +27480,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -27499,7 +27499,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -27538,7 +27538,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -27567,7 +27567,7 @@
       <c r="P67" s="54"/>
       <c r="Q67" s="54"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27586,7 +27586,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="142"/>
       <c r="B69" s="143"/>
       <c r="C69" s="35"/>
@@ -27605,7 +27605,7 @@
       <c r="P69" s="35"/>
       <c r="Q69" s="144"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="145"/>
       <c r="B70" s="145"/>
       <c r="C70" s="145"/>
@@ -27624,7 +27624,7 @@
       <c r="P70" s="145"/>
       <c r="Q70" s="145"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="146" t="s">
         <v>147</v>
@@ -27669,7 +27669,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -27708,7 +27708,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="77" t="s">
         <v>149</v>
@@ -27737,7 +27737,7 @@
       <c r="P73" s="20"/>
       <c r="Q73" s="20"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="148" t="s">
         <v>150</v>
@@ -27782,7 +27782,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="151" t="s">
         <v>151</v>
@@ -27827,7 +27827,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
@@ -27846,7 +27846,7 @@
       <c r="P76" s="35"/>
       <c r="Q76" s="144"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="156" t="s">
         <v>152</v>
@@ -27893,7 +27893,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A78" s="161"/>
       <c r="B78" s="162" t="s">
         <v>154</v>
@@ -27938,7 +27938,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -27957,7 +27957,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="164" t="s">
         <v>155</v>
@@ -27980,7 +27980,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="167" t="s">
         <v>157</v>
@@ -28003,7 +28003,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28026,7 +28026,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28049,7 +28049,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28072,7 +28072,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -28095,7 +28095,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -28118,7 +28118,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -28141,7 +28141,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -28164,7 +28164,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -28187,7 +28187,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -28210,7 +28210,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -28233,7 +28233,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -28254,7 +28254,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -28275,7 +28275,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -28296,7 +28296,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -28317,7 +28317,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -28338,7 +28338,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -28359,7 +28359,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -28380,7 +28380,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -28403,7 +28403,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -28426,7 +28426,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -28449,7 +28449,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -28472,7 +28472,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -28495,7 +28495,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -28518,7 +28518,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -28541,7 +28541,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -28560,7 +28560,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -28579,7 +28579,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19"/>
       <c r="C108" s="131"/>
@@ -28598,7 +28598,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="169"/>
       <c r="C109" s="150"/>
@@ -28617,7 +28617,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="164" t="s">
         <v>175</v>
@@ -28691,10 +28691,11 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>176</v>
       </c>
@@ -28726,7 +28727,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>177</v>
       </c>
@@ -28759,7 +28760,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>178</v>
       </c>
@@ -28792,7 +28793,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>179</v>
       </c>
@@ -28825,7 +28826,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>180</v>
       </c>
@@ -28858,7 +28859,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>181</v>
       </c>
@@ -28891,7 +28892,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>182</v>
       </c>
@@ -28924,7 +28925,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>183</v>
       </c>
@@ -28957,7 +28958,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28988,7 +28989,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29019,7 +29020,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>184</v>
       </c>
@@ -29052,7 +29053,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>185</v>
       </c>
@@ -29085,7 +29086,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>186</v>
       </c>
@@ -29118,7 +29119,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>187</v>
       </c>
@@ -29151,7 +29152,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>188</v>
       </c>
@@ -29184,7 +29185,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>189</v>
       </c>
@@ -29217,7 +29218,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>190</v>
       </c>
@@ -29250,7 +29251,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>191</v>
       </c>
@@ -29283,7 +29284,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>192</v>
       </c>
@@ -29316,7 +29317,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>193</v>
       </c>
@@ -29349,7 +29350,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>194</v>
       </c>
@@ -29382,7 +29383,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>195</v>
       </c>
@@ -29415,7 +29416,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>196</v>
       </c>
@@ -29448,7 +29449,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>197</v>
       </c>
@@ -29481,7 +29482,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>198</v>
       </c>
@@ -29514,7 +29515,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>199</v>
       </c>
@@ -29547,7 +29548,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>200</v>
       </c>
@@ -29579,7 +29580,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>201</v>
       </c>
@@ -29611,7 +29612,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>202</v>
       </c>
@@ -29643,7 +29644,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>203</v>
       </c>
@@ -29675,7 +29676,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>204</v>
       </c>
@@ -29707,7 +29708,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29737,7 +29738,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29767,7 +29768,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>205</v>
       </c>
@@ -29799,7 +29800,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>206</v>
       </c>
@@ -29831,7 +29832,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>207</v>
       </c>
@@ -29863,7 +29864,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>208</v>
       </c>
@@ -29895,7 +29896,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>209</v>
       </c>
@@ -29927,7 +29928,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29957,7 +29958,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>210</v>
       </c>
@@ -29989,7 +29990,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>211</v>
       </c>
@@ -30021,7 +30022,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>212</v>
       </c>
@@ -30053,7 +30054,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>213</v>
       </c>
@@ -30085,7 +30086,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -30115,7 +30116,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -30145,7 +30146,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -30175,7 +30176,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -30205,7 +30206,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>214</v>
       </c>
@@ -30237,7 +30238,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>215</v>
       </c>
@@ -30269,7 +30270,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -30299,7 +30300,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -30329,7 +30330,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -30359,7 +30360,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -30389,7 +30390,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -30419,7 +30420,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -30514,10 +30515,11 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:AC45"/>
+  <dimension ref="A1:AD45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>216</v>
       </c>
@@ -30549,7 +30551,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -30580,7 +30582,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30611,7 +30613,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30642,7 +30644,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30673,7 +30675,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30704,7 +30706,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30735,7 +30737,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30766,7 +30768,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30797,7 +30799,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -30828,7 +30830,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -30859,7 +30861,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -30890,7 +30892,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -30921,7 +30923,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -30952,7 +30954,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -30983,7 +30985,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31014,7 +31016,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31045,7 +31047,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31076,7 +31078,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31107,7 +31109,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -31138,7 +31140,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -31168,7 +31170,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -31198,7 +31200,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -31228,7 +31230,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -31258,7 +31260,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -31288,7 +31290,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -31318,7 +31320,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -31348,7 +31350,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -31378,7 +31380,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -31408,7 +31410,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -31438,7 +31440,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -31468,7 +31470,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -31498,7 +31500,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -31528,7 +31530,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -31558,7 +31560,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -31588,7 +31590,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -31618,7 +31620,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>214</v>
       </c>
@@ -31650,7 +31652,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>215</v>
       </c>
@@ -31682,7 +31684,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -31712,7 +31714,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -31742,7 +31744,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -31772,7 +31774,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -31802,7 +31804,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -31832,7 +31834,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -53575,19 +53577,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:AD9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -53601,7 +53603,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>223</v>
       </c>
@@ -53613,7 +53615,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>224</v>
       </c>
@@ -53624,7 +53626,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>225</v>
       </c>
@@ -53635,7 +53637,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>226</v>
       </c>
@@ -53646,13 +53648,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-09T00:20:42Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -17238,7 +17238,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>97</v>
@@ -23261,7 +23261,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD71"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -23275,7 +23275,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -23297,7 +23297,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>102</v>
       </c>
@@ -23345,7 +23345,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -23363,7 +23363,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -23410,7 +23410,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -23427,7 +23427,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -23444,7 +23444,7 @@
         <v>-5726.869999999995</v>
       </c>
       <c r="F6" s="52">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G6" s="53">
         <v>0</v>
@@ -23477,7 +23477,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -23494,7 +23494,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -23537,7 +23537,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -23554,7 +23554,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23601,7 +23601,7 @@
         <v>25.48731814842027</v>
       </c>
     </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23618,7 +23618,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23668,7 +23668,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23685,7 +23685,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23732,7 +23732,7 @@
         <v>91.48330357142855</v>
       </c>
     </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23749,7 +23749,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23794,7 +23794,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23811,7 +23811,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23861,7 +23861,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23878,7 +23878,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23917,7 +23917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23934,7 +23934,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23975,7 +23975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23992,7 +23992,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24031,7 +24031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -24048,7 +24048,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24093,7 +24093,7 @@
         <v>-7.859546247818494</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -24110,7 +24110,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24153,7 +24153,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -24170,7 +24170,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24213,7 +24213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -24230,7 +24230,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24277,7 +24277,7 @@
         <v>13.90219151036525</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -24294,7 +24294,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24339,7 +24339,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -24356,7 +24356,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24399,7 +24399,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -24416,7 +24416,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24457,7 +24457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -24474,7 +24474,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24519,7 +24519,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -24536,7 +24536,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24579,7 +24579,7 @@
         <v>-0.05012183692595682</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24596,7 +24596,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24633,7 +24633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24650,7 +24650,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -24691,7 +24691,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24708,7 +24708,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -24751,7 +24751,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24768,7 +24768,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -24810,7 +24810,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24827,7 +24827,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -24872,7 +24872,7 @@
         <v>12.893675527039413</v>
       </c>
     </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24889,7 +24889,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -24934,7 +24934,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24951,7 +24951,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -24996,7 +24996,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25013,7 +25013,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -25050,7 +25050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -25067,7 +25067,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -25084,7 +25084,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -25101,7 +25101,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>61</v>
@@ -25122,7 +25122,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -25139,7 +25139,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -25180,7 +25180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -25197,7 +25197,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -25242,7 +25242,7 @@
         <v>-20.78054054054051</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -25277,7 +25277,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -25294,7 +25294,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -25311,7 +25311,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>122</v>
       </c>
@@ -25346,7 +25346,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>126</v>
@@ -25729,7 +25729,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD110"/>
+  <dimension ref="A1:AB110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25740,7 +25740,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25761,7 +25761,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>127</v>
@@ -25823,7 +25823,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>143</v>
       </c>
@@ -25881,7 +25881,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25921,7 +25921,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25940,7 +25940,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25974,7 +25974,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25993,7 +25993,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26027,7 +26027,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26046,7 +26046,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -26084,7 +26084,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -26103,7 +26103,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -26141,7 +26141,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -26160,7 +26160,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -26198,7 +26198,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -26217,7 +26217,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -26250,7 +26250,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -26269,7 +26269,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -26302,7 +26302,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -26321,7 +26321,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -26352,7 +26352,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -26371,7 +26371,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -26406,7 +26406,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r="C23" s="134"/>
@@ -26425,7 +26425,7 @@
       <c r="P23" s="134"/>
       <c r="Q23" s="137"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -26458,7 +26458,7 @@
       <c r="P24" s="54"/>
       <c r="Q24" s="131"/>
     </row>
-    <row r="25" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="66"/>
       <c r="B25" s="66"/>
       <c r="C25" s="66"/>
@@ -26477,7 +26477,7 @@
       <c r="P25" s="66"/>
       <c r="Q25" s="66"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -26508,7 +26508,7 @@
       <c r="P26" s="54"/>
       <c r="Q26" s="131"/>
     </row>
-    <row r="27" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="61"/>
       <c r="B27" s="61"/>
       <c r="C27" s="61"/>
@@ -26527,7 +26527,7 @@
       <c r="P27" s="61"/>
       <c r="Q27" s="61"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -26559,7 +26559,7 @@
       <c r="Q28" s="131"/>
       <c r="S28" s="138"/>
     </row>
-    <row r="29" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="61"/>
       <c r="B29" s="61"/>
       <c r="C29" s="61"/>
@@ -26578,7 +26578,7 @@
       <c r="P29" s="61"/>
       <c r="Q29" s="61"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -26614,7 +26614,7 @@
       <c r="Q30" s="131"/>
       <c r="S30" s="139"/>
     </row>
-    <row r="31" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="61"/>
       <c r="B31" s="61"/>
       <c r="C31" s="61"/>
@@ -26633,7 +26633,7 @@
       <c r="P31" s="61"/>
       <c r="Q31" s="61"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -26662,7 +26662,7 @@
       <c r="P32" s="54"/>
       <c r="Q32" s="131"/>
     </row>
-    <row r="33" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="61"/>
       <c r="B33" s="61"/>
       <c r="C33" s="61"/>
@@ -26681,7 +26681,7 @@
       <c r="P33" s="61"/>
       <c r="Q33" s="61"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -26712,7 +26712,7 @@
       <c r="P34" s="54"/>
       <c r="Q34" s="131"/>
     </row>
-    <row r="35" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="61"/>
       <c r="B35" s="61"/>
       <c r="C35" s="61"/>
@@ -26731,7 +26731,7 @@
       <c r="P35" s="61"/>
       <c r="Q35" s="61"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -26764,7 +26764,7 @@
       <c r="P36" s="54"/>
       <c r="Q36" s="131"/>
     </row>
-    <row r="37" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="61"/>
       <c r="B37" s="61"/>
       <c r="C37" s="61"/>
@@ -26783,7 +26783,7 @@
       <c r="P37" s="61"/>
       <c r="Q37" s="61"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -26819,7 +26819,7 @@
       <c r="Q38" s="131"/>
       <c r="S38" s="139"/>
     </row>
-    <row r="39" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="61"/>
       <c r="B39" s="61"/>
       <c r="C39" s="61"/>
@@ -26838,7 +26838,7 @@
       <c r="P39" s="61"/>
       <c r="Q39" s="61"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -26873,7 +26873,7 @@
       <c r="P40" s="54"/>
       <c r="Q40" s="131"/>
     </row>
-    <row r="41" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="61"/>
       <c r="B41" s="61"/>
       <c r="C41" s="61"/>
@@ -26892,7 +26892,7 @@
       <c r="P41" s="61"/>
       <c r="Q41" s="61"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -26922,7 +26922,7 @@
       <c r="Q42" s="131"/>
       <c r="S42" s="139"/>
     </row>
-    <row r="43" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="61"/>
       <c r="B43" s="61"/>
       <c r="C43" s="61"/>
@@ -26941,7 +26941,7 @@
       <c r="P43" s="61"/>
       <c r="Q43" s="61"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -26981,7 +26981,7 @@
       </c>
       <c r="S44" s="139"/>
     </row>
-    <row r="45" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="61"/>
       <c r="B45" s="61"/>
       <c r="C45" s="61"/>
@@ -27000,7 +27000,7 @@
       <c r="P45" s="61"/>
       <c r="Q45" s="61"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -27029,7 +27029,7 @@
       <c r="P46" s="98"/>
       <c r="Q46" s="140"/>
     </row>
-    <row r="47" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="61"/>
       <c r="B47" s="61"/>
       <c r="C47" s="61"/>
@@ -27048,7 +27048,7 @@
       <c r="P47" s="61"/>
       <c r="Q47" s="61"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="19">
         <v>8337</v>
       </c>
@@ -27081,7 +27081,7 @@
       <c r="P48" s="54"/>
       <c r="Q48" s="131"/>
     </row>
-    <row r="49" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="61"/>
       <c r="B49" s="61"/>
       <c r="C49" s="61"/>
@@ -27100,7 +27100,7 @@
       <c r="P49" s="61"/>
       <c r="Q49" s="61"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="19">
         <v>9240</v>
       </c>
@@ -27133,7 +27133,7 @@
       <c r="P50" s="54"/>
       <c r="Q50" s="131"/>
     </row>
-    <row r="51" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="61"/>
       <c r="B51" s="61"/>
       <c r="C51" s="61"/>
@@ -27152,7 +27152,7 @@
       <c r="P51" s="61"/>
       <c r="Q51" s="61"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" s="19">
         <v>7428</v>
       </c>
@@ -27188,7 +27188,7 @@
       <c r="Q52" s="131"/>
       <c r="S52" s="139"/>
     </row>
-    <row r="53" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="61"/>
       <c r="B53" s="61"/>
       <c r="C53" s="61"/>
@@ -27207,7 +27207,7 @@
       <c r="P53" s="61"/>
       <c r="Q53" s="61"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A54" s="19">
         <v>9351</v>
       </c>
@@ -27243,7 +27243,7 @@
       <c r="Q54" s="131"/>
       <c r="S54" s="138"/>
     </row>
-    <row r="55" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="61"/>
       <c r="B55" s="61"/>
       <c r="C55" s="61"/>
@@ -27262,7 +27262,7 @@
       <c r="P55" s="61"/>
       <c r="Q55" s="61"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" s="19">
         <v>7429</v>
       </c>
@@ -27296,7 +27296,7 @@
       <c r="Q56" s="131"/>
       <c r="S56" s="139"/>
     </row>
-    <row r="57" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="57" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="61"/>
       <c r="B57" s="61"/>
       <c r="C57" s="61"/>
@@ -27315,7 +27315,7 @@
       <c r="P57" s="61"/>
       <c r="Q57" s="61"/>
     </row>
-    <row r="58" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="58" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="19">
         <v>9508</v>
       </c>
@@ -27350,7 +27350,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="59" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="61"/>
       <c r="B59" s="61"/>
       <c r="C59" s="61"/>
@@ -27369,7 +27369,7 @@
       <c r="P59" s="61"/>
       <c r="Q59" s="61"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="19"/>
       <c r="B60" s="20"/>
       <c r="C60" s="54"/>
@@ -27388,7 +27388,7 @@
       <c r="P60" s="54"/>
       <c r="Q60" s="131"/>
     </row>
-    <row r="61" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="61" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="61"/>
       <c r="B61" s="61"/>
       <c r="C61" s="61"/>
@@ -27407,7 +27407,7 @@
       <c r="P61" s="61"/>
       <c r="Q61" s="61"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="19"/>
       <c r="B62" s="20" t="s">
         <v>61</v>
@@ -27428,7 +27428,7 @@
       <c r="P62" s="54"/>
       <c r="Q62" s="131"/>
     </row>
-    <row r="63" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="63" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="61"/>
       <c r="B63" s="61"/>
       <c r="C63" s="61"/>
@@ -27447,7 +27447,7 @@
       <c r="P63" s="61"/>
       <c r="Q63" s="61"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="19">
         <v>8946</v>
       </c>
@@ -27480,7 +27480,7 @@
       </c>
       <c r="Q64" s="131"/>
     </row>
-    <row r="65" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="65" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="61"/>
       <c r="B65" s="61"/>
       <c r="C65" s="61"/>
@@ -27499,7 +27499,7 @@
       <c r="P65" s="61"/>
       <c r="Q65" s="61"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="19">
         <v>8308</v>
       </c>
@@ -27538,7 +27538,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="67" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="19">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -27567,7 +27567,7 @@
       <c r="P67" s="54"/>
       <c r="Q67" s="54"/>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="142"/>
       <c r="B68" s="143"/>
       <c r="C68" s="35"/>
@@ -27586,7 +27586,7 @@
       <c r="P68" s="35"/>
       <c r="Q68" s="144"/>
     </row>
-    <row r="69" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="69" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="142"/>
       <c r="B69" s="143"/>
       <c r="C69" s="35"/>
@@ -27605,7 +27605,7 @@
       <c r="P69" s="35"/>
       <c r="Q69" s="144"/>
     </row>
-    <row r="70" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="70" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="145"/>
       <c r="B70" s="145"/>
       <c r="C70" s="145"/>
@@ -27624,7 +27624,7 @@
       <c r="P70" s="145"/>
       <c r="Q70" s="145"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="142"/>
       <c r="B71" s="146" t="s">
         <v>147</v>
@@ -27669,7 +27669,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="72" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="72" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="142"/>
       <c r="B72" s="77" t="s">
         <v>148</v>
@@ -27708,7 +27708,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="73" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="73" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="142"/>
       <c r="B73" s="77" t="s">
         <v>149</v>
@@ -27737,7 +27737,7 @@
       <c r="P73" s="20"/>
       <c r="Q73" s="20"/>
     </row>
-    <row r="74" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="74" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="142"/>
       <c r="B74" s="148" t="s">
         <v>150</v>
@@ -27782,7 +27782,7 @@
         <v>1478.4</v>
       </c>
     </row>
-    <row r="75" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="75" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="142"/>
       <c r="B75" s="151" t="s">
         <v>151</v>
@@ -27827,7 +27827,7 @@
         <v>-828.4</v>
       </c>
     </row>
-    <row r="76" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="76" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="142"/>
       <c r="B76" s="35"/>
       <c r="C76" s="35"/>
@@ -27846,7 +27846,7 @@
       <c r="P76" s="35"/>
       <c r="Q76" s="144"/>
     </row>
-    <row r="77" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="77" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="142"/>
       <c r="B77" s="156" t="s">
         <v>152</v>
@@ -27893,7 +27893,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="78" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="78" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="161"/>
       <c r="B78" s="162" t="s">
         <v>154</v>
@@ -27938,7 +27938,7 @@
         <v>16.5</v>
       </c>
     </row>
-    <row r="79" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="35"/>
       <c r="B79" s="35"/>
       <c r="C79" s="35"/>
@@ -27957,7 +27957,7 @@
       <c r="P79" s="35"/>
       <c r="Q79" s="35"/>
     </row>
-    <row r="80" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="80" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="35"/>
       <c r="B80" s="164" t="s">
         <v>155</v>
@@ -27980,7 +27980,7 @@
       <c r="P80" s="35"/>
       <c r="Q80" s="35"/>
     </row>
-    <row r="81" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="81" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="35"/>
       <c r="B81" s="167" t="s">
         <v>157</v>
@@ -28003,7 +28003,7 @@
       <c r="P81" s="35"/>
       <c r="Q81" s="35"/>
     </row>
-    <row r="82" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="82" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="35"/>
       <c r="B82" s="19" t="s">
         <v>158</v>
@@ -28026,7 +28026,7 @@
       <c r="P82" s="35"/>
       <c r="Q82" s="35"/>
     </row>
-    <row r="83" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="83" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="35"/>
       <c r="B83" s="19" t="s">
         <v>159</v>
@@ -28049,7 +28049,7 @@
       <c r="P83" s="35"/>
       <c r="Q83" s="35"/>
     </row>
-    <row r="84" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="84" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="35"/>
       <c r="B84" s="19" t="s">
         <v>160</v>
@@ -28072,7 +28072,7 @@
       <c r="P84" s="35"/>
       <c r="Q84" s="35"/>
     </row>
-    <row r="85" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="85" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="35"/>
       <c r="B85" s="19" t="s">
         <v>161</v>
@@ -28095,7 +28095,7 @@
       <c r="P85" s="35"/>
       <c r="Q85" s="35"/>
     </row>
-    <row r="86" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="86" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="35"/>
       <c r="B86" s="19" t="s">
         <v>162</v>
@@ -28118,7 +28118,7 @@
       <c r="P86" s="35"/>
       <c r="Q86" s="35"/>
     </row>
-    <row r="87" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="87" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="35"/>
       <c r="B87" s="19" t="s">
         <v>163</v>
@@ -28141,7 +28141,7 @@
       <c r="P87" s="35"/>
       <c r="Q87" s="35"/>
     </row>
-    <row r="88" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="88" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="35"/>
       <c r="B88" s="19" t="s">
         <v>164</v>
@@ -28164,7 +28164,7 @@
       <c r="P88" s="35"/>
       <c r="Q88" s="35"/>
     </row>
-    <row r="89" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="89" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="35"/>
       <c r="B89" s="19" t="s">
         <v>165</v>
@@ -28187,7 +28187,7 @@
       <c r="P89" s="35"/>
       <c r="Q89" s="35"/>
     </row>
-    <row r="90" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="90" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="35"/>
       <c r="B90" s="19" t="s">
         <v>166</v>
@@ -28210,7 +28210,7 @@
       <c r="P90" s="35"/>
       <c r="Q90" s="35"/>
     </row>
-    <row r="91" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="91" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="35"/>
       <c r="B91" s="19" t="s">
         <v>167</v>
@@ -28233,7 +28233,7 @@
       <c r="P91" s="35"/>
       <c r="Q91" s="35"/>
     </row>
-    <row r="92" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="92" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="35"/>
       <c r="B92" s="19"/>
       <c r="C92" s="131">
@@ -28254,7 +28254,7 @@
       <c r="P92" s="35"/>
       <c r="Q92" s="35"/>
     </row>
-    <row r="93" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="93" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="35"/>
       <c r="B93" s="19"/>
       <c r="C93" s="131">
@@ -28275,7 +28275,7 @@
       <c r="P93" s="35"/>
       <c r="Q93" s="35"/>
     </row>
-    <row r="94" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="94" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="35"/>
       <c r="B94" s="19"/>
       <c r="C94" s="131">
@@ -28296,7 +28296,7 @@
       <c r="P94" s="35"/>
       <c r="Q94" s="35"/>
     </row>
-    <row r="95" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="95" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="35"/>
       <c r="B95" s="19"/>
       <c r="C95" s="131">
@@ -28317,7 +28317,7 @@
       <c r="P95" s="35"/>
       <c r="Q95" s="35"/>
     </row>
-    <row r="96" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="96" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="35"/>
       <c r="B96" s="19"/>
       <c r="C96" s="131">
@@ -28338,7 +28338,7 @@
       <c r="P96" s="35"/>
       <c r="Q96" s="35"/>
     </row>
-    <row r="97" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="97" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="35"/>
       <c r="B97" s="19"/>
       <c r="C97" s="131">
@@ -28359,7 +28359,7 @@
       <c r="P97" s="35"/>
       <c r="Q97" s="35"/>
     </row>
-    <row r="98" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="98" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="35"/>
       <c r="B98" s="19"/>
       <c r="C98" s="131">
@@ -28380,7 +28380,7 @@
       <c r="P98" s="35"/>
       <c r="Q98" s="35"/>
     </row>
-    <row r="99" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="99" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="35"/>
       <c r="B99" s="19" t="s">
         <v>168</v>
@@ -28403,7 +28403,7 @@
       <c r="P99" s="35"/>
       <c r="Q99" s="35"/>
     </row>
-    <row r="100" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="100" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="35"/>
       <c r="B100" s="19" t="s">
         <v>169</v>
@@ -28426,7 +28426,7 @@
       <c r="P100" s="35"/>
       <c r="Q100" s="35"/>
     </row>
-    <row r="101" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="101" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="35"/>
       <c r="B101" s="19" t="s">
         <v>170</v>
@@ -28449,7 +28449,7 @@
       <c r="P101" s="35"/>
       <c r="Q101" s="35"/>
     </row>
-    <row r="102" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="102" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="35"/>
       <c r="B102" s="19" t="s">
         <v>171</v>
@@ -28472,7 +28472,7 @@
       <c r="P102" s="35"/>
       <c r="Q102" s="35"/>
     </row>
-    <row r="103" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="103" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="35"/>
       <c r="B103" s="19" t="s">
         <v>172</v>
@@ -28495,7 +28495,7 @@
       <c r="P103" s="35"/>
       <c r="Q103" s="35"/>
     </row>
-    <row r="104" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="104" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="35"/>
       <c r="B104" s="19" t="s">
         <v>173</v>
@@ -28518,7 +28518,7 @@
       <c r="P104" s="35"/>
       <c r="Q104" s="35"/>
     </row>
-    <row r="105" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="105" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="35"/>
       <c r="B105" s="19" t="s">
         <v>174</v>
@@ -28541,7 +28541,7 @@
       <c r="P105" s="35"/>
       <c r="Q105" s="35"/>
     </row>
-    <row r="106" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="106" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="35"/>
       <c r="B106" s="19"/>
       <c r="C106" s="131"/>
@@ -28560,7 +28560,7 @@
       <c r="P106" s="35"/>
       <c r="Q106" s="35"/>
     </row>
-    <row r="107" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="107" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="35"/>
       <c r="B107" s="19"/>
       <c r="C107" s="131"/>
@@ -28579,7 +28579,7 @@
       <c r="P107" s="35"/>
       <c r="Q107" s="35"/>
     </row>
-    <row r="108" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="108" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="35"/>
       <c r="B108" s="19"/>
       <c r="C108" s="131"/>
@@ -28598,7 +28598,7 @@
       <c r="P108" s="35"/>
       <c r="Q108" s="35"/>
     </row>
-    <row r="109" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="109" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="35"/>
       <c r="B109" s="169"/>
       <c r="C109" s="150"/>
@@ -28617,7 +28617,7 @@
       <c r="P109" s="35"/>
       <c r="Q109" s="35"/>
     </row>
-    <row r="110" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="110" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="35"/>
       <c r="B110" s="164" t="s">
         <v>175</v>
@@ -28691,11 +28691,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A2:AC56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>176</v>
       </c>
@@ -28727,7 +28726,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172" t="s">
         <v>177</v>
       </c>
@@ -28760,7 +28759,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174" t="s">
         <v>178</v>
       </c>
@@ -28793,7 +28792,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="175" t="s">
         <v>179</v>
       </c>
@@ -28826,7 +28825,7 @@
       <c r="AB5" s="175"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176" t="s">
         <v>180</v>
       </c>
@@ -28859,7 +28858,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="177" t="s">
         <v>181</v>
       </c>
@@ -28892,7 +28891,7 @@
       <c r="AB7" s="177"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176" t="s">
         <v>182</v>
       </c>
@@ -28925,7 +28924,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="178" t="s">
         <v>183</v>
       </c>
@@ -28958,7 +28957,7 @@
       <c r="AB9" s="178"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="179"/>
       <c r="B10" s="179"/>
       <c r="C10" s="179"/>
@@ -28989,7 +28988,7 @@
       <c r="AB10" s="179"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="180"/>
       <c r="B11" s="180"/>
       <c r="C11" s="180"/>
@@ -29020,7 +29019,7 @@
       <c r="AB11" s="180"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="181" t="s">
         <v>184</v>
       </c>
@@ -29053,7 +29052,7 @@
       <c r="AB12" s="181"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="182" t="s">
         <v>185</v>
       </c>
@@ -29086,7 +29085,7 @@
       <c r="AB13" s="182"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="183" t="s">
         <v>186</v>
       </c>
@@ -29119,7 +29118,7 @@
       <c r="AB14" s="183"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="172" t="s">
         <v>187</v>
       </c>
@@ -29152,7 +29151,7 @@
       <c r="AB15" s="172"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="184" t="s">
         <v>188</v>
       </c>
@@ -29185,7 +29184,7 @@
       <c r="AB16" s="184"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="185" t="s">
         <v>189</v>
       </c>
@@ -29218,7 +29217,7 @@
       <c r="AB17" s="185"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="186" t="s">
         <v>190</v>
       </c>
@@ -29251,7 +29250,7 @@
       <c r="AB18" s="186"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="178" t="s">
         <v>191</v>
       </c>
@@ -29284,7 +29283,7 @@
       <c r="AB19" s="178"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="187" t="s">
         <v>192</v>
       </c>
@@ -29317,7 +29316,7 @@
       <c r="AB20" s="187"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="188" t="s">
         <v>193</v>
       </c>
@@ -29350,7 +29349,7 @@
       <c r="AB21" s="188"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="188" t="s">
         <v>194</v>
       </c>
@@ -29383,7 +29382,7 @@
       <c r="AB22" s="188"/>
       <c r="AC22" s="173"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="188" t="s">
         <v>195</v>
       </c>
@@ -29416,7 +29415,7 @@
       <c r="AB23" s="188"/>
       <c r="AC23" s="173"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="188" t="s">
         <v>196</v>
       </c>
@@ -29449,7 +29448,7 @@
       <c r="AB24" s="188"/>
       <c r="AC24" s="173"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="189" t="s">
         <v>197</v>
       </c>
@@ -29482,7 +29481,7 @@
       <c r="AB25" s="189"/>
       <c r="AC25" s="173"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="181" t="s">
         <v>198</v>
       </c>
@@ -29515,7 +29514,7 @@
       <c r="AB26" s="181"/>
       <c r="AC26" s="173"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="190" t="s">
         <v>199</v>
       </c>
@@ -29548,7 +29547,7 @@
       <c r="AB27" s="190"/>
       <c r="AC27" s="173"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172" t="s">
         <v>200</v>
       </c>
@@ -29580,7 +29579,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="190" t="s">
         <v>201</v>
       </c>
@@ -29612,7 +29611,7 @@
       <c r="AA29" s="190"/>
       <c r="AB29" s="190"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="191" t="s">
         <v>202</v>
       </c>
@@ -29644,7 +29643,7 @@
       <c r="AA30" s="191"/>
       <c r="AB30" s="191"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="191" t="s">
         <v>203</v>
       </c>
@@ -29676,7 +29675,7 @@
       <c r="AA31" s="191"/>
       <c r="AB31" s="191"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="191" t="s">
         <v>204</v>
       </c>
@@ -29708,7 +29707,7 @@
       <c r="AA32" s="191"/>
       <c r="AB32" s="191"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="191"/>
       <c r="B33" s="191"/>
       <c r="C33" s="191"/>
@@ -29738,7 +29737,7 @@
       <c r="AA33" s="191"/>
       <c r="AB33" s="191"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="191"/>
       <c r="B34" s="191"/>
       <c r="C34" s="191"/>
@@ -29768,7 +29767,7 @@
       <c r="AA34" s="191"/>
       <c r="AB34" s="191"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="192" t="s">
         <v>205</v>
       </c>
@@ -29800,7 +29799,7 @@
       <c r="AA35" s="192"/>
       <c r="AB35" s="192"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="193" t="s">
         <v>206</v>
       </c>
@@ -29832,7 +29831,7 @@
       <c r="AA36" s="193"/>
       <c r="AB36" s="193"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="194" t="s">
         <v>207</v>
       </c>
@@ -29864,7 +29863,7 @@
       <c r="AA37" s="194"/>
       <c r="AB37" s="194"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="179" t="s">
         <v>208</v>
       </c>
@@ -29896,7 +29895,7 @@
       <c r="AA38" s="179"/>
       <c r="AB38" s="179"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="181" t="s">
         <v>209</v>
       </c>
@@ -29928,7 +29927,7 @@
       <c r="AA39" s="181"/>
       <c r="AB39" s="181"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="195"/>
       <c r="B40" s="195"/>
       <c r="C40" s="195"/>
@@ -29958,7 +29957,7 @@
       <c r="AA40" s="195"/>
       <c r="AB40" s="195"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="172" t="s">
         <v>210</v>
       </c>
@@ -29990,7 +29989,7 @@
       <c r="AA41" s="172"/>
       <c r="AB41" s="172"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="196" t="s">
         <v>211</v>
       </c>
@@ -30022,7 +30021,7 @@
       <c r="AA42" s="196"/>
       <c r="AB42" s="196"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="172" t="s">
         <v>212</v>
       </c>
@@ -30054,7 +30053,7 @@
       <c r="AA43" s="172"/>
       <c r="AB43" s="172"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="197" t="s">
         <v>213</v>
       </c>
@@ -30086,7 +30085,7 @@
       <c r="AA44" s="197"/>
       <c r="AB44" s="197"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="198"/>
       <c r="B45" s="198"/>
       <c r="C45" s="198"/>
@@ -30116,7 +30115,7 @@
       <c r="AA45" s="198"/>
       <c r="AB45" s="198"/>
     </row>
-    <row r="46" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="46" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A46" s="198"/>
       <c r="B46" s="198"/>
       <c r="C46" s="198"/>
@@ -30146,7 +30145,7 @@
       <c r="AA46" s="198"/>
       <c r="AB46" s="198"/>
     </row>
-    <row r="47" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="47" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A47" s="198"/>
       <c r="B47" s="198"/>
       <c r="C47" s="198"/>
@@ -30176,7 +30175,7 @@
       <c r="AA47" s="198"/>
       <c r="AB47" s="198"/>
     </row>
-    <row r="48" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="48" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A48" s="199"/>
       <c r="B48" s="199"/>
       <c r="C48" s="199"/>
@@ -30206,7 +30205,7 @@
       <c r="AA48" s="199"/>
       <c r="AB48" s="199"/>
     </row>
-    <row r="49" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="49" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A49" s="172" t="s">
         <v>214</v>
       </c>
@@ -30238,7 +30237,7 @@
       <c r="AA49" s="172"/>
       <c r="AB49" s="172"/>
     </row>
-    <row r="50" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="50" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A50" s="200" t="s">
         <v>215</v>
       </c>
@@ -30270,7 +30269,7 @@
       <c r="AA50" s="200"/>
       <c r="AB50" s="200"/>
     </row>
-    <row r="51" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="51" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A51" s="201"/>
       <c r="B51" s="201"/>
       <c r="C51" s="201"/>
@@ -30300,7 +30299,7 @@
       <c r="AA51" s="201"/>
       <c r="AB51" s="201"/>
     </row>
-    <row r="52" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="52" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A52" s="176"/>
       <c r="B52" s="176"/>
       <c r="C52" s="176"/>
@@ -30330,7 +30329,7 @@
       <c r="AA52" s="176"/>
       <c r="AB52" s="176"/>
     </row>
-    <row r="53" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="53" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A53" s="198"/>
       <c r="B53" s="198"/>
       <c r="C53" s="198"/>
@@ -30360,7 +30359,7 @@
       <c r="AA53" s="198"/>
       <c r="AB53" s="198"/>
     </row>
-    <row r="54" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="54" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A54" s="198"/>
       <c r="B54" s="198"/>
       <c r="C54" s="198"/>
@@ -30390,7 +30389,7 @@
       <c r="AA54" s="198"/>
       <c r="AB54" s="198"/>
     </row>
-    <row r="55" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="55" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A55" s="198"/>
       <c r="B55" s="198"/>
       <c r="C55" s="198"/>
@@ -30420,7 +30419,7 @@
       <c r="AA55" s="198"/>
       <c r="AB55" s="198"/>
     </row>
-    <row r="56" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="56" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A56" s="202"/>
       <c r="B56" s="202"/>
       <c r="C56" s="202"/>
@@ -30515,11 +30514,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A2:AC45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25"/>
-    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" s="171" t="s">
         <v>216</v>
       </c>
@@ -30551,7 +30549,7 @@
       <c r="AA2" s="171"/>
       <c r="AB2" s="171"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="172"/>
       <c r="B3" s="172"/>
       <c r="C3" s="172"/>
@@ -30582,7 +30580,7 @@
       <c r="AB3" s="172"/>
       <c r="AC3" s="173"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="174"/>
       <c r="B4" s="174"/>
       <c r="C4" s="174"/>
@@ -30613,7 +30611,7 @@
       <c r="AB4" s="174"/>
       <c r="AC4" s="173"/>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="203"/>
       <c r="B5" s="203"/>
       <c r="C5" s="203"/>
@@ -30644,7 +30642,7 @@
       <c r="AB5" s="203"/>
       <c r="AC5" s="173"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="176"/>
       <c r="B6" s="176"/>
       <c r="C6" s="176"/>
@@ -30675,7 +30673,7 @@
       <c r="AB6" s="176"/>
       <c r="AC6" s="173"/>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="204"/>
       <c r="B7" s="204"/>
       <c r="C7" s="204"/>
@@ -30706,7 +30704,7 @@
       <c r="AB7" s="204"/>
       <c r="AC7" s="173"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="176"/>
       <c r="B8" s="176"/>
       <c r="C8" s="176"/>
@@ -30737,7 +30735,7 @@
       <c r="AB8" s="176"/>
       <c r="AC8" s="173"/>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="205"/>
       <c r="B9" s="205"/>
       <c r="C9" s="205"/>
@@ -30768,7 +30766,7 @@
       <c r="AB9" s="205"/>
       <c r="AC9" s="173"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="206"/>
       <c r="B10" s="206"/>
       <c r="C10" s="206"/>
@@ -30799,7 +30797,7 @@
       <c r="AB10" s="206"/>
       <c r="AC10" s="173"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="172"/>
       <c r="B11" s="172"/>
       <c r="C11" s="172"/>
@@ -30830,7 +30828,7 @@
       <c r="AB11" s="172"/>
       <c r="AC11" s="173"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="207"/>
       <c r="C12" s="207"/>
@@ -30861,7 +30859,7 @@
       <c r="AB12" s="207"/>
       <c r="AC12" s="173"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="172"/>
       <c r="B13" s="172"/>
       <c r="C13" s="172"/>
@@ -30892,7 +30890,7 @@
       <c r="AB13" s="172"/>
       <c r="AC13" s="173"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="184"/>
       <c r="B14" s="184"/>
       <c r="C14" s="184"/>
@@ -30923,7 +30921,7 @@
       <c r="AB14" s="184"/>
       <c r="AC14" s="173"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="208"/>
       <c r="B15" s="208"/>
       <c r="C15" s="208"/>
@@ -30954,7 +30952,7 @@
       <c r="AB15" s="208"/>
       <c r="AC15" s="173"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="208"/>
       <c r="B16" s="208"/>
       <c r="C16" s="208"/>
@@ -30985,7 +30983,7 @@
       <c r="AB16" s="208"/>
       <c r="AC16" s="173"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="205"/>
       <c r="B17" s="205"/>
       <c r="C17" s="205"/>
@@ -31016,7 +31014,7 @@
       <c r="AB17" s="205"/>
       <c r="AC17" s="173"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="205"/>
       <c r="B18" s="205"/>
       <c r="C18" s="205"/>
@@ -31047,7 +31045,7 @@
       <c r="AB18" s="205"/>
       <c r="AC18" s="173"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="209"/>
       <c r="B19" s="209"/>
       <c r="C19" s="209"/>
@@ -31078,7 +31076,7 @@
       <c r="AB19" s="209"/>
       <c r="AC19" s="173"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="172"/>
       <c r="B20" s="172"/>
       <c r="C20" s="172"/>
@@ -31109,7 +31107,7 @@
       <c r="AB20" s="172"/>
       <c r="AC20" s="173"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="190"/>
       <c r="B21" s="190"/>
       <c r="C21" s="190"/>
@@ -31140,7 +31138,7 @@
       <c r="AB21" s="190"/>
       <c r="AC21" s="173"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A22" s="172"/>
       <c r="B22" s="172"/>
       <c r="C22" s="172"/>
@@ -31170,7 +31168,7 @@
       <c r="AA22" s="172"/>
       <c r="AB22" s="172"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A23" s="210"/>
       <c r="B23" s="210"/>
       <c r="C23" s="210"/>
@@ -31200,7 +31198,7 @@
       <c r="AA23" s="210"/>
       <c r="AB23" s="210"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A24" s="211"/>
       <c r="B24" s="211"/>
       <c r="C24" s="211"/>
@@ -31230,7 +31228,7 @@
       <c r="AA24" s="211"/>
       <c r="AB24" s="211"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A25" s="172"/>
       <c r="B25" s="172"/>
       <c r="C25" s="172"/>
@@ -31260,7 +31258,7 @@
       <c r="AA25" s="172"/>
       <c r="AB25" s="172"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A26" s="174"/>
       <c r="B26" s="174"/>
       <c r="C26" s="174"/>
@@ -31290,7 +31288,7 @@
       <c r="AA26" s="174"/>
       <c r="AB26" s="174"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A27" s="212"/>
       <c r="B27" s="212"/>
       <c r="C27" s="212"/>
@@ -31320,7 +31318,7 @@
       <c r="AA27" s="212"/>
       <c r="AB27" s="212"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A28" s="172"/>
       <c r="B28" s="172"/>
       <c r="C28" s="172"/>
@@ -31350,7 +31348,7 @@
       <c r="AA28" s="172"/>
       <c r="AB28" s="172"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A29" s="213"/>
       <c r="B29" s="213"/>
       <c r="C29" s="213"/>
@@ -31380,7 +31378,7 @@
       <c r="AA29" s="213"/>
       <c r="AB29" s="213"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A30" s="172"/>
       <c r="B30" s="172"/>
       <c r="C30" s="172"/>
@@ -31410,7 +31408,7 @@
       <c r="AA30" s="172"/>
       <c r="AB30" s="172"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A31" s="213"/>
       <c r="B31" s="213"/>
       <c r="C31" s="213"/>
@@ -31440,7 +31438,7 @@
       <c r="AA31" s="213"/>
       <c r="AB31" s="213"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A32" s="172"/>
       <c r="B32" s="172"/>
       <c r="C32" s="172"/>
@@ -31470,7 +31468,7 @@
       <c r="AA32" s="172"/>
       <c r="AB32" s="172"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A33" s="200"/>
       <c r="B33" s="200"/>
       <c r="C33" s="200"/>
@@ -31500,7 +31498,7 @@
       <c r="AA33" s="200"/>
       <c r="AB33" s="200"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A34" s="198"/>
       <c r="B34" s="198"/>
       <c r="C34" s="198"/>
@@ -31530,7 +31528,7 @@
       <c r="AA34" s="198"/>
       <c r="AB34" s="198"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A35" s="198"/>
       <c r="B35" s="198"/>
       <c r="C35" s="198"/>
@@ -31560,7 +31558,7 @@
       <c r="AA35" s="198"/>
       <c r="AB35" s="198"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="198"/>
       <c r="B36" s="198"/>
       <c r="C36" s="198"/>
@@ -31590,7 +31588,7 @@
       <c r="AA36" s="198"/>
       <c r="AB36" s="198"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A37" s="199"/>
       <c r="B37" s="199"/>
       <c r="C37" s="199"/>
@@ -31620,7 +31618,7 @@
       <c r="AA37" s="199"/>
       <c r="AB37" s="199"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A38" s="172" t="s">
         <v>214</v>
       </c>
@@ -31652,7 +31650,7 @@
       <c r="AA38" s="172"/>
       <c r="AB38" s="172"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A39" s="200" t="s">
         <v>215</v>
       </c>
@@ -31684,7 +31682,7 @@
       <c r="AA39" s="200"/>
       <c r="AB39" s="200"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A40" s="176"/>
       <c r="B40" s="176"/>
       <c r="C40" s="176"/>
@@ -31714,7 +31712,7 @@
       <c r="AA40" s="176"/>
       <c r="AB40" s="176"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A41" s="176"/>
       <c r="B41" s="176"/>
       <c r="C41" s="176"/>
@@ -31744,7 +31742,7 @@
       <c r="AA41" s="176"/>
       <c r="AB41" s="176"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A42" s="198"/>
       <c r="B42" s="198"/>
       <c r="C42" s="198"/>
@@ -31774,7 +31772,7 @@
       <c r="AA42" s="198"/>
       <c r="AB42" s="198"/>
     </row>
-    <row r="43" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="43" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A43" s="198"/>
       <c r="B43" s="198"/>
       <c r="C43" s="198"/>
@@ -31804,7 +31802,7 @@
       <c r="AA43" s="198"/>
       <c r="AB43" s="198"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A44" s="198"/>
       <c r="B44" s="198"/>
       <c r="C44" s="198"/>
@@ -31834,7 +31832,7 @@
       <c r="AA44" s="198"/>
       <c r="AB44" s="198"/>
     </row>
-    <row r="45" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="45" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A45" s="202"/>
       <c r="B45" s="202"/>
       <c r="C45" s="202"/>
@@ -53577,19 +53575,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:P9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="10.29" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="35"/>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="35">
         <v>340</v>
       </c>
@@ -53603,7 +53601,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="35" t="s">
         <v>223</v>
       </c>
@@ -53615,7 +53613,7 @@
         <v>0.0882352941176471</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="35" t="s">
         <v>224</v>
       </c>
@@ -53626,7 +53624,7 @@
         <v>95.35</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="35" t="s">
         <v>225</v>
       </c>
@@ -53637,7 +53635,7 @@
         <v>102.69</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="35" t="s">
         <v>226</v>
       </c>
@@ -53648,13 +53646,13 @@
         <v>134.82</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="35"/>
       <c r="P8" s="35">
         <v>324.19</v>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="35"/>
       <c r="P9" s="35">
         <v>415</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-09T00:29:48Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -26133,9 +26133,11 @@
         <v>320</v>
       </c>
       <c r="O12" s="86">
+        <v>0</v>
+      </c>
+      <c r="P12" s="54">
         <v>80</v>
       </c>
-      <c r="P12" s="54"/>
       <c r="Q12" s="131"/>
       <c r="S12" s="35" t="s">
         <v>145</v>

</xml_diff>

<commit_message>
Process pending data updates (2026-09-09T22:39:02Z)
</commit_message>
<xml_diff>
--- a/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
+++ b/public/Cassidy_Davies_Electrical_BPMN_Data.xlsx
@@ -10290,19 +10290,19 @@
         <v>101885.52</v>
       </c>
       <c r="I13" s="52">
-        <v>79864.19</v>
+        <v>79853.63</v>
       </c>
       <c r="J13" s="52">
         <v>83735.42000000001</v>
       </c>
       <c r="K13" s="52">
-        <v>71677.66</v>
+        <v>71667.1</v>
       </c>
       <c r="L13" s="52">
-        <v>12057.76000000001</v>
+        <v>12068.320000000007</v>
       </c>
       <c r="M13" s="53">
-        <v>0.14399832233480178</v>
+        <v>0.14412443384173634</v>
       </c>
       <c r="N13" s="53"/>
       <c r="O13" s="52">
@@ -10331,13 +10331,13 @@
       </c>
       <c r="W13" s="53"/>
       <c r="X13" s="55">
-        <v>35.660564635958394</v>
+        <v>35.72332838038633</v>
       </c>
       <c r="Y13" s="55">
         <v>77.32043896850674</v>
       </c>
       <c r="Z13" s="53">
-        <v>0.0699</v>
+        <v>0.07</v>
       </c>
       <c r="AA13" s="56">
         <v>0.2162</v>
@@ -11106,54 +11106,54 @@
         <v>104026.09</v>
       </c>
       <c r="I27" s="52">
-        <v>89600.47</v>
+        <v>90387.67</v>
       </c>
       <c r="J27" s="52">
         <v>63812.49</v>
       </c>
       <c r="K27" s="52">
-        <v>59331.43</v>
+        <v>59529.82</v>
       </c>
       <c r="L27" s="52">
-        <v>4481.059999999998</v>
+        <v>4282.669999999998</v>
       </c>
       <c r="M27" s="53">
-        <v>0.07022230287518945</v>
+        <v>0.06711335038015283</v>
       </c>
       <c r="N27" s="53"/>
       <c r="O27" s="52">
         <v>40213.6</v>
       </c>
       <c r="P27" s="52">
-        <v>30269.04</v>
+        <v>30857.85</v>
       </c>
       <c r="Q27" s="52">
-        <v>9944.559999999998</v>
+        <v>9355.75</v>
       </c>
       <c r="R27" s="53">
-        <v>0.2472934529611872</v>
+        <v>0.23265139156902143</v>
       </c>
       <c r="S27" s="54">
         <v>805.22</v>
       </c>
       <c r="T27" s="54">
-        <v>615.5</v>
+        <v>625</v>
       </c>
       <c r="U27" s="54">
-        <v>189.72000000000003</v>
+        <v>180.22000000000003</v>
       </c>
       <c r="V27" s="53">
-        <v>0.2356126276048782</v>
+        <v>0.22381460967189093</v>
       </c>
       <c r="W27" s="53"/>
       <c r="X27" s="55">
-        <v>88.9851015434606</v>
+        <v>86.373008</v>
       </c>
       <c r="Y27" s="55">
         <v>61.50814037389784</v>
       </c>
       <c r="Z27" s="53">
-        <v>0.37939999999999996</v>
+        <v>0.3739</v>
       </c>
       <c r="AA27" s="56">
         <v>0.3225</v>
@@ -11513,54 +11513,54 @@
         <v>328046.93</v>
       </c>
       <c r="I34" s="65">
-        <v>223743.65</v>
+        <v>224540.22</v>
       </c>
       <c r="J34" s="52">
         <v>271925.57</v>
       </c>
       <c r="K34" s="52">
-        <v>197386.58</v>
+        <v>197386.58000000002</v>
       </c>
       <c r="L34" s="52">
-        <v>74538.99000000002</v>
+        <v>74538.98999999999</v>
       </c>
       <c r="M34" s="53">
-        <v>0.27411541327283057</v>
+        <v>0.27411541327283045</v>
       </c>
       <c r="N34" s="53"/>
       <c r="O34" s="52">
         <v>56121.36</v>
       </c>
       <c r="P34" s="52">
-        <v>26357.07</v>
+        <v>27153.64</v>
       </c>
       <c r="Q34" s="52">
-        <v>29764.29</v>
+        <v>28967.72</v>
       </c>
       <c r="R34" s="53">
-        <v>0.5303558217405994</v>
+        <v>0.5161621172402094</v>
       </c>
       <c r="S34" s="54">
         <v>1124.47</v>
       </c>
       <c r="T34" s="54">
-        <v>609</v>
+        <v>627.75</v>
       </c>
       <c r="U34" s="54">
-        <v>515.47</v>
+        <v>496.72</v>
       </c>
       <c r="V34" s="53">
-        <v>0.4584115183152952</v>
+        <v>0.44173699609593853</v>
       </c>
       <c r="W34" s="53"/>
       <c r="X34" s="55">
-        <v>58.463152709359605</v>
+        <v>55.44801274392672</v>
       </c>
       <c r="Y34" s="55">
         <v>61.532703026350184</v>
       </c>
       <c r="Z34" s="53">
-        <v>0.1373</v>
+        <v>0.13419999999999999</v>
       </c>
       <c r="AA34" s="56">
         <v>0.1742</v>
@@ -11920,7 +11920,7 @@
         <v>94098.32</v>
       </c>
       <c r="I41" s="52">
-        <v>49519.82</v>
+        <v>50255.78</v>
       </c>
       <c r="J41" s="52">
         <v>69042.09000000001</v>
@@ -11939,35 +11939,35 @@
         <v>25056.23</v>
       </c>
       <c r="P41" s="52">
-        <v>13836.08</v>
+        <v>14572.04</v>
       </c>
       <c r="Q41" s="52">
-        <v>11220.15</v>
+        <v>10484.189999999999</v>
       </c>
       <c r="R41" s="53">
-        <v>0.44779881091449114</v>
+        <v>0.418426475172043</v>
       </c>
       <c r="S41" s="54">
         <v>501.83</v>
       </c>
       <c r="T41" s="54">
-        <v>308.25</v>
+        <v>325.75</v>
       </c>
       <c r="U41" s="54">
-        <v>193.57999999999998</v>
+        <v>176.07999999999998</v>
       </c>
       <c r="V41" s="53">
-        <v>0.38574816172807525</v>
+        <v>0.350875794591794</v>
       </c>
       <c r="W41" s="53"/>
       <c r="X41" s="55">
-        <v>14.355263584752636</v>
+        <v>11.324788948580201</v>
       </c>
       <c r="Y41" s="55">
         <v>68.07122423898531</v>
       </c>
       <c r="Z41" s="53">
-        <v>0.08199999999999999</v>
+        <v>0.0684</v>
       </c>
       <c r="AA41" s="56">
         <v>0.2663</v>
@@ -12736,54 +12736,54 @@
         <v>109364.97</v>
       </c>
       <c r="I55" s="52">
-        <v>97978.14</v>
+        <v>98837.32</v>
       </c>
       <c r="J55" s="52">
         <v>75135.01000000001</v>
       </c>
       <c r="K55" s="52">
-        <v>71357.43</v>
+        <v>71357.43000000001</v>
       </c>
       <c r="L55" s="52">
-        <v>3777.5800000000163</v>
+        <v>3777.5800000000017</v>
       </c>
       <c r="M55" s="53">
-        <v>0.050277227619987215</v>
+        <v>0.05027722761998703</v>
       </c>
       <c r="N55" s="53"/>
       <c r="O55" s="52">
         <v>34229.96</v>
       </c>
       <c r="P55" s="52">
-        <v>26620.71</v>
+        <v>27479.89</v>
       </c>
       <c r="Q55" s="52">
-        <v>7609.25</v>
+        <v>6750.07</v>
       </c>
       <c r="R55" s="53">
-        <v>0.22229795185270448</v>
+        <v>0.19719771802245753</v>
       </c>
       <c r="S55" s="54">
         <v>685.48</v>
       </c>
       <c r="T55" s="54">
-        <v>561.5</v>
+        <v>578.5</v>
       </c>
       <c r="U55" s="54">
-        <v>123.98000000000002</v>
+        <v>106.98000000000002</v>
       </c>
       <c r="V55" s="53">
-        <v>0.18086596253720022</v>
+        <v>0.15606582248935055</v>
       </c>
       <c r="W55" s="53"/>
       <c r="X55" s="55">
-        <v>53.13684772929653</v>
+        <v>50.09016421780467</v>
       </c>
       <c r="Y55" s="55">
         <v>67.00679527854935</v>
       </c>
       <c r="Z55" s="53">
-        <v>0.2334</v>
+        <v>0.2267</v>
       </c>
       <c r="AA55" s="56">
         <v>0.2958</v>
@@ -17235,7 +17235,7 @@
       <c r="AH132" s="19"/>
       <c r="AI132" s="58"/>
     </row>
-    <row r="133" ht="15" customHeight="1" spans="2:35" x14ac:dyDescent="0.25">
+    <row r="133" ht="15" customHeight="1" spans="1:35" x14ac:dyDescent="0.25">
       <c r="B133" s="20"/>
       <c r="C133" s="51" t="s">
         <v>96</v>
@@ -19562,19 +19562,19 @@
         <v>114651.87</v>
       </c>
       <c r="I174" s="52">
-        <v>105118.87</v>
+        <v>105655.21</v>
       </c>
       <c r="J174" s="52">
         <v>82888.07999999999</v>
       </c>
       <c r="K174" s="52">
-        <v>77768.29999999999</v>
+        <v>78304.64000000001</v>
       </c>
       <c r="L174" s="52">
-        <v>5119.779999999999</v>
+        <v>4583.439999999973</v>
       </c>
       <c r="M174" s="53">
-        <v>0.06176738561202044</v>
+        <v>0.055296732654441676</v>
       </c>
       <c r="N174" s="53"/>
       <c r="O174" s="52">
@@ -19603,13 +19603,13 @@
       </c>
       <c r="W174" s="53"/>
       <c r="X174" s="55">
-        <v>36.933649202733484</v>
+        <v>35.95626423690205</v>
       </c>
       <c r="Y174" s="55">
         <v>47.87601261940491</v>
       </c>
       <c r="Z174" s="53">
-        <v>0.1616</v>
+        <v>0.1574</v>
       </c>
       <c r="AA174" s="56">
         <v>0.216</v>
@@ -22118,72 +22118,72 @@
         <v>95</v>
       </c>
       <c r="D223" s="52">
-        <v>396453.46</v>
+        <v>408794.64</v>
       </c>
       <c r="E223" s="52">
         <v>306038.55</v>
       </c>
       <c r="F223" s="52">
-        <v>90414.91000000003</v>
+        <v>102756.09000000003</v>
       </c>
       <c r="G223" s="53">
-        <v>0.2280593288301735</v>
+        <v>0.25136359419976745</v>
       </c>
       <c r="H223" s="52">
-        <v>295569.99</v>
+        <v>304310.08</v>
       </c>
       <c r="I223" s="52">
-        <v>246358.99</v>
+        <v>249180.5</v>
       </c>
       <c r="J223" s="52">
-        <v>178700.37</v>
+        <v>185072.60000000003</v>
       </c>
       <c r="K223" s="52">
-        <v>180550.95</v>
+        <v>182215.95</v>
       </c>
       <c r="L223" s="52">
-        <v>-1850.5800000000163</v>
+        <v>2856.6500000000233</v>
       </c>
       <c r="M223" s="53">
-        <v>-0.010355770388164369</v>
+        <v>0.015435294041365512</v>
       </c>
       <c r="N223" s="53"/>
       <c r="O223" s="52">
-        <v>116869.62</v>
+        <v>119237.48</v>
       </c>
       <c r="P223" s="52">
-        <v>65808.04</v>
+        <v>66964.55</v>
       </c>
       <c r="Q223" s="52">
-        <v>51061.58</v>
+        <v>52272.92999999999</v>
       </c>
       <c r="R223" s="53">
-        <v>0.43691063597194896</v>
+        <v>0.4383934481003791</v>
       </c>
       <c r="S223" s="54">
-        <v>2344.68</v>
+        <v>2397.2</v>
       </c>
       <c r="T223" s="54">
-        <v>1401.92</v>
+        <v>1427.42</v>
       </c>
       <c r="U223" s="54">
-        <v>942.7599999999998</v>
+        <v>969.7799999999997</v>
       </c>
       <c r="V223" s="53">
-        <v>0.40208471944998886</v>
+        <v>0.4045469714667111</v>
       </c>
       <c r="W223" s="53"/>
       <c r="X223" s="55">
-        <v>42.56987559917827</v>
+        <v>39.832740188592005</v>
       </c>
       <c r="Y223" s="55">
-        <v>43.0265399367206</v>
+        <v>43.58608178135741</v>
       </c>
       <c r="Z223" s="53">
-        <v>0.195</v>
+        <v>0.1858</v>
       </c>
       <c r="AA223" s="56">
-        <v>0.2545</v>
+        <v>0.2556</v>
       </c>
       <c r="AB223" s="57"/>
       <c r="AD223" s="35"/>
@@ -23258,7 +23258,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R71"/>
+  <dimension ref="A1:AD71"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11.43" style="35" customWidth="1"/>
@@ -23272,7 +23272,7 @@
     <col min="15" max="15" width="16.86" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="31.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" ht="31.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="78" t="s">
         <v>0</v>
       </c>
@@ -23294,7 +23294,7 @@
       <c r="Q1" s="79"/>
       <c r="R1" s="79"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="80" t="s">
         <v>101</v>
       </c>
@@ -23342,7 +23342,7 @@
       </c>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="80"/>
       <c r="B3" s="81"/>
       <c r="C3" s="81"/>
@@ -23360,7 +23360,7 @@
       <c r="O3" s="84"/>
       <c r="P3" s="35"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="85">
         <v>7658</v>
       </c>
@@ -23407,7 +23407,7 @@
         <v>-105.77028571428589</v>
       </c>
     </row>
-    <row r="5" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="88"/>
       <c r="B5" s="89"/>
       <c r="C5" s="89"/>
@@ -23424,7 +23424,7 @@
       <c r="N5" s="89"/>
       <c r="O5" s="58"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="85">
         <v>8142</v>
       </c>
@@ -23435,10 +23435,10 @@
         <v>0</v>
       </c>
       <c r="D6" s="52">
-        <v>5726.869999999995</v>
+        <v>5716.309999999998</v>
       </c>
       <c r="E6" s="52">
-        <v>-5726.869999999995</v>
+        <v>-5716.309999999998</v>
       </c>
       <c r="F6" s="52">
         <v>7</v>
@@ -23456,25 +23456,25 @@
         <v>272.6</v>
       </c>
       <c r="K6" s="52">
-        <v>1872.6</v>
+        <v>20272.6</v>
       </c>
       <c r="L6" s="53">
         <v>0</v>
       </c>
       <c r="M6" s="52">
-        <v>-7599.469999999996</v>
+        <v>-25981.909999999996</v>
       </c>
       <c r="N6" s="54">
         <v>-52.5</v>
       </c>
       <c r="O6" s="58">
-        <v>607.9575999999996</v>
+        <v>-58.06013407821228</v>
       </c>
       <c r="Q6" s="35" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="7" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="90"/>
       <c r="B7" s="91"/>
       <c r="C7" s="91"/>
@@ -23491,7 +23491,7 @@
       <c r="N7" s="91"/>
       <c r="O7" s="58"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="85">
         <v>8824</v>
       </c>
@@ -23534,7 +23534,7 @@
         <v>50.13333333333333</v>
       </c>
     </row>
-    <row r="9" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="90"/>
       <c r="B9" s="91"/>
       <c r="C9" s="91"/>
@@ -23551,7 +23551,7 @@
       <c r="N9" s="91"/>
       <c r="O9" s="58"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="85">
         <v>8127</v>
       </c>
@@ -23562,10 +23562,10 @@
         <v>0</v>
       </c>
       <c r="D10" s="52">
-        <v>3752.0599999999977</v>
+        <v>4539.259999999995</v>
       </c>
       <c r="E10" s="52">
-        <v>-3752.0599999999977</v>
+        <v>-4539.259999999995</v>
       </c>
       <c r="F10" s="52">
         <v>0</v>
@@ -23589,16 +23589,16 @@
         <v>0</v>
       </c>
       <c r="M10" s="52">
-        <v>-8672.059999999998</v>
+        <v>-9459.259999999995</v>
       </c>
       <c r="N10" s="54">
         <v>-388.25</v>
       </c>
       <c r="O10" s="58">
-        <v>25.48731814842027</v>
-      </c>
-    </row>
-    <row r="11" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>27.80091109478323</v>
+      </c>
+    </row>
+    <row r="11" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="90"/>
       <c r="B11" s="91"/>
       <c r="C11" s="91"/>
@@ -23615,7 +23615,7 @@
       <c r="N11" s="91"/>
       <c r="O11" s="58"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="85">
         <v>8183</v>
       </c>
@@ -23626,10 +23626,10 @@
         <v>0</v>
       </c>
       <c r="D12" s="52">
-        <v>7399.049999999988</v>
+        <v>8195.619999999995</v>
       </c>
       <c r="E12" s="52">
-        <v>-7399.049999999988</v>
+        <v>-8195.619999999995</v>
       </c>
       <c r="F12" s="52">
         <v>3</v>
@@ -23653,19 +23653,19 @@
         <v>0</v>
       </c>
       <c r="M12" s="52">
-        <v>-10036.049999999988</v>
+        <v>-10832.619999999995</v>
       </c>
       <c r="N12" s="54">
         <v>53</v>
       </c>
       <c r="O12" s="58">
-        <v>-145.44999999999982</v>
+        <v>-156.99449275362312</v>
       </c>
       <c r="Q12" s="35" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="13" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="90"/>
       <c r="B13" s="91"/>
       <c r="C13" s="91"/>
@@ -23682,7 +23682,7 @@
       <c r="N13" s="91"/>
       <c r="O13" s="58"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="85">
         <v>8886</v>
       </c>
@@ -23693,10 +23693,10 @@
         <v>0</v>
       </c>
       <c r="D14" s="52">
-        <v>7246.129999999997</v>
+        <v>7982.0899999999965</v>
       </c>
       <c r="E14" s="52">
-        <v>-7246.129999999997</v>
+        <v>-7982.0899999999965</v>
       </c>
       <c r="F14" s="52">
         <v>0</v>
@@ -23720,16 +23720,16 @@
         <v>0</v>
       </c>
       <c r="M14" s="52">
-        <v>-10246.129999999997</v>
+        <v>-10982.089999999997</v>
       </c>
       <c r="N14" s="54">
         <v>-112</v>
       </c>
       <c r="O14" s="58">
-        <v>91.48330357142855</v>
-      </c>
-    </row>
-    <row r="15" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>98.05437499999996</v>
+      </c>
+    </row>
+    <row r="15" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="90"/>
       <c r="B15" s="91"/>
       <c r="C15" s="91"/>
@@ -23746,7 +23746,7 @@
       <c r="N15" s="91"/>
       <c r="O15" s="58"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="85">
         <v>8887</v>
       </c>
@@ -23791,7 +23791,7 @@
         <v>34.40668587896252</v>
       </c>
     </row>
-    <row r="17" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="90"/>
       <c r="B17" s="91"/>
       <c r="C17" s="91"/>
@@ -23808,7 +23808,7 @@
       <c r="N17" s="91"/>
       <c r="O17" s="58"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="85">
         <v>8670</v>
       </c>
@@ -23819,10 +23819,10 @@
         <v>0</v>
       </c>
       <c r="D18" s="52">
-        <v>2657.6300000000047</v>
+        <v>3516.810000000012</v>
       </c>
       <c r="E18" s="52">
-        <v>-2657.6300000000047</v>
+        <v>-3516.810000000012</v>
       </c>
       <c r="F18" s="52">
         <v>0</v>
@@ -23846,19 +23846,19 @@
         <v>0</v>
       </c>
       <c r="M18" s="52">
-        <v>-10857.630000000005</v>
+        <v>-11716.810000000012</v>
       </c>
       <c r="N18" s="54">
         <v>-269</v>
       </c>
       <c r="O18" s="58">
-        <v>57.4477777777778</v>
+        <v>61.993703703703765</v>
       </c>
       <c r="Q18" s="35" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="19" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="90"/>
       <c r="B19" s="91"/>
       <c r="C19" s="91"/>
@@ -23875,7 +23875,7 @@
       <c r="N19" s="91"/>
       <c r="O19" s="58"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="85">
         <v>8907</v>
       </c>
@@ -23914,7 +23914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="90"/>
       <c r="B21" s="91"/>
       <c r="C21" s="91"/>
@@ -23931,7 +23931,7 @@
       <c r="N21" s="91"/>
       <c r="O21" s="58"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="85">
         <v>9065</v>
       </c>
@@ -23972,7 +23972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="90"/>
       <c r="B23" s="91"/>
       <c r="C23" s="91"/>
@@ -23989,7 +23989,7 @@
       <c r="N23" s="91"/>
       <c r="O23" s="58"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" s="19">
         <v>9259</v>
       </c>
@@ -24028,7 +24028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" s="94"/>
       <c r="B25" s="95"/>
       <c r="C25" s="95"/>
@@ -24045,7 +24045,7 @@
       <c r="N25" s="95"/>
       <c r="O25" s="58"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" s="19">
         <v>8352</v>
       </c>
@@ -24090,7 +24090,7 @@
         <v>-7.859546247818494</v>
       </c>
     </row>
-    <row r="27" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" s="90"/>
       <c r="B27" s="91"/>
       <c r="C27" s="91"/>
@@ -24107,7 +24107,7 @@
       <c r="N27" s="91"/>
       <c r="O27" s="58"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" s="19">
         <v>8234</v>
       </c>
@@ -24150,7 +24150,7 @@
         <v>-6.366734006734025</v>
       </c>
     </row>
-    <row r="29" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" s="90"/>
       <c r="B29" s="91"/>
       <c r="C29" s="91"/>
@@ -24167,7 +24167,7 @@
       <c r="N29" s="91"/>
       <c r="O29" s="58"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" s="19">
         <v>8214</v>
       </c>
@@ -24210,7 +24210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" s="90"/>
       <c r="B31" s="91"/>
       <c r="C31" s="91"/>
@@ -24227,7 +24227,7 @@
       <c r="N31" s="91"/>
       <c r="O31" s="58"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" s="19">
         <v>6792</v>
       </c>
@@ -24274,7 +24274,7 @@
         <v>13.90219151036525</v>
       </c>
     </row>
-    <row r="33" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A33" s="90"/>
       <c r="B33" s="91"/>
       <c r="C33" s="91"/>
@@ -24291,7 +24291,7 @@
       <c r="N33" s="91"/>
       <c r="O33" s="58"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A34" s="19">
         <v>8840</v>
       </c>
@@ -24336,7 +24336,7 @@
         <v>4.512234432234419</v>
       </c>
     </row>
-    <row r="35" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A35" s="90"/>
       <c r="B35" s="91"/>
       <c r="C35" s="91"/>
@@ -24353,7 +24353,7 @@
       <c r="N35" s="91"/>
       <c r="O35" s="58"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A36" s="19">
         <v>8769</v>
       </c>
@@ -24396,7 +24396,7 @@
         <v>-40</v>
       </c>
     </row>
-    <row r="37" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A37" s="90"/>
       <c r="B37" s="91"/>
       <c r="C37" s="91"/>
@@ -24413,7 +24413,7 @@
       <c r="N37" s="91"/>
       <c r="O37" s="58"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A38" s="19">
         <v>7901</v>
       </c>
@@ -24454,7 +24454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A39" s="90"/>
       <c r="B39" s="91"/>
       <c r="C39" s="91"/>
@@ -24471,7 +24471,7 @@
       <c r="N39" s="91"/>
       <c r="O39" s="58"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A40" s="19">
         <v>8923</v>
       </c>
@@ -24516,7 +24516,7 @@
         <v>-1063.9049999999997</v>
       </c>
     </row>
-    <row r="41" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A41" s="90"/>
       <c r="B41" s="91"/>
       <c r="C41" s="91"/>
@@ -24533,7 +24533,7 @@
       <c r="N41" s="91"/>
       <c r="O41" s="58"/>
     </row>
-    <row r="42" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A42" s="19">
         <v>7864</v>
       </c>
@@ -24576,7 +24576,7 @@
         <v>-0.05012183692595682</v>
       </c>
     </row>
-    <row r="43" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A43" s="90"/>
       <c r="B43" s="91"/>
       <c r="C43" s="91"/>
@@ -24593,7 +24593,7 @@
       <c r="N43" s="91"/>
       <c r="O43" s="58"/>
     </row>
-    <row r="44" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A44" s="19">
         <v>7912</v>
       </c>
@@ -24630,7 +24630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A45" s="90"/>
       <c r="B45" s="91"/>
       <c r="C45" s="91"/>
@@ -24647,7 +24647,7 @@
       <c r="N45" s="96"/>
       <c r="O45" s="97"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A46" s="59">
         <v>8360</v>
       </c>
@@ -24688,7 +24688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A47" s="90"/>
       <c r="B47" s="91"/>
       <c r="C47" s="91"/>
@@ -24705,7 +24705,7 @@
       <c r="N47" s="96"/>
       <c r="O47" s="97"/>
     </row>
-    <row r="48" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A48" s="59">
         <v>8337</v>
       </c>
@@ -24748,7 +24748,7 @@
         <v>56.53631284916201</v>
       </c>
     </row>
-    <row r="49" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A49" s="90"/>
       <c r="B49" s="91"/>
       <c r="C49" s="91"/>
@@ -24765,7 +24765,7 @@
       <c r="N49" s="96"/>
       <c r="O49" s="97"/>
     </row>
-    <row r="50" ht="15.75" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="50" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A50" s="59">
         <v>9240</v>
       </c>
@@ -24807,7 +24807,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="51" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A51" s="90"/>
       <c r="B51" s="91"/>
       <c r="C51" s="91"/>
@@ -24824,7 +24824,7 @@
       <c r="N51" s="96"/>
       <c r="O51" s="97"/>
     </row>
-    <row r="52" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A52" s="101">
         <v>7428</v>
       </c>
@@ -24835,10 +24835,10 @@
         <v>0</v>
       </c>
       <c r="D52" s="99">
-        <v>2236.75</v>
+        <v>2773.090000000011</v>
       </c>
       <c r="E52" s="99">
-        <v>-2236.75</v>
+        <v>-2773.090000000011</v>
       </c>
       <c r="F52" s="99"/>
       <c r="G52" s="100">
@@ -24860,16 +24860,16 @@
         <v>0</v>
       </c>
       <c r="M52" s="99">
-        <v>-3516.75</v>
+        <v>-4053.090000000011</v>
       </c>
       <c r="N52" s="98">
         <v>-304.75</v>
       </c>
       <c r="O52" s="60">
-        <v>12.893675527039413</v>
-      </c>
-    </row>
-    <row r="53" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>14.860091659028456</v>
+      </c>
+    </row>
+    <row r="53" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A53" s="90"/>
       <c r="B53" s="91"/>
       <c r="C53" s="91"/>
@@ -24886,7 +24886,7 @@
       <c r="N53" s="96"/>
       <c r="O53" s="97"/>
     </row>
-    <row r="54" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A54" s="59">
         <v>9351</v>
       </c>
@@ -24931,7 +24931,7 @@
         <v>-134.73684210526315</v>
       </c>
     </row>
-    <row r="55" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A55" s="90"/>
       <c r="B55" s="91"/>
       <c r="C55" s="91"/>
@@ -24948,7 +24948,7 @@
       <c r="N55" s="96"/>
       <c r="O55" s="97"/>
     </row>
-    <row r="56" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A56" s="59">
         <v>7429</v>
       </c>
@@ -24993,7 +24993,7 @@
         <v>242.69662921348313</v>
       </c>
     </row>
-    <row r="57" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A57" s="90"/>
       <c r="B57" s="91"/>
       <c r="C57" s="91"/>
@@ -25010,7 +25010,7 @@
       <c r="N57" s="96"/>
       <c r="O57" s="97"/>
     </row>
-    <row r="58" ht="15.75" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" ht="15.75" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A58" s="59">
         <v>9508</v>
       </c>
@@ -25047,7 +25047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A59" s="90"/>
       <c r="B59" s="91"/>
       <c r="C59" s="91"/>
@@ -25064,7 +25064,7 @@
       <c r="N59" s="96"/>
       <c r="O59" s="97"/>
     </row>
-    <row r="60" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A60" s="59"/>
       <c r="B60" s="98"/>
       <c r="C60" s="99"/>
@@ -25081,7 +25081,7 @@
       <c r="N60" s="98"/>
       <c r="O60" s="60"/>
     </row>
-    <row r="61" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A61" s="90"/>
       <c r="B61" s="91"/>
       <c r="C61" s="91"/>
@@ -25098,7 +25098,7 @@
       <c r="N61" s="96"/>
       <c r="O61" s="97"/>
     </row>
-    <row r="62" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A62" s="59"/>
       <c r="B62" s="98" t="s">
         <v>60</v>
@@ -25119,7 +25119,7 @@
       <c r="N62" s="98"/>
       <c r="O62" s="60"/>
     </row>
-    <row r="63" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A63" s="90"/>
       <c r="B63" s="91"/>
       <c r="C63" s="91"/>
@@ -25136,7 +25136,7 @@
       <c r="N63" s="96"/>
       <c r="O63" s="97"/>
     </row>
-    <row r="64" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A64" s="59">
         <v>8946</v>
       </c>
@@ -25177,7 +25177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" ht="7.5" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" ht="7.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A65" s="90"/>
       <c r="B65" s="91"/>
       <c r="C65" s="91"/>
@@ -25194,7 +25194,7 @@
       <c r="N65" s="96"/>
       <c r="O65" s="97"/>
     </row>
-    <row r="66" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A66" s="102">
         <v>8308</v>
       </c>
@@ -25205,14 +25205,14 @@
         <v>34650.399999999965</v>
       </c>
       <c r="D66" s="99">
-        <v>12036.179999999993</v>
+        <v>14857.690000000002</v>
       </c>
       <c r="E66" s="99">
-        <v>22614.219999999972</v>
+        <v>19792.709999999963</v>
       </c>
       <c r="F66" s="99"/>
       <c r="G66" s="100">
-        <v>0.6526395077690299</v>
+        <v>0.5712115877450183</v>
       </c>
       <c r="H66" s="100">
         <v>0.256265521519856</v>
@@ -25227,19 +25227,19 @@
         <v>3200</v>
       </c>
       <c r="L66" s="100">
-        <v>0.5602884815182506</v>
+        <v>0.478860561494239</v>
       </c>
       <c r="M66" s="99">
-        <v>19414.219999999972</v>
+        <v>16592.709999999963</v>
       </c>
       <c r="N66" s="98">
         <v>-1014.25</v>
       </c>
       <c r="O66" s="60">
-        <v>-20.78054054054051</v>
-      </c>
-    </row>
-    <row r="67" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+        <v>-17.7604602622424</v>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A67" s="102">
         <f>'Main Sheet'!A68</f>
       </c>
@@ -25274,7 +25274,7 @@
         <f>SUM(M67/(N67+I67))</f>
       </c>
     </row>
-    <row r="68" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A68" s="35"/>
       <c r="B68" s="35"/>
       <c r="C68" s="36"/>
@@ -25291,7 +25291,7 @@
       <c r="N68" s="35"/>
       <c r="O68" s="36"/>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A69" s="35"/>
       <c r="B69" s="35"/>
       <c r="C69" s="36"/>
@@ -25308,7 +25308,7 @@
       <c r="N69" s="35"/>
       <c r="O69" s="35"/>
     </row>
-    <row r="70" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A70" s="49" t="s">
         <v>121</v>
       </c>
@@ -25319,22 +25319,22 @@
         <v>88103.76999999996</v>
       </c>
       <c r="D70" s="104">
-        <v>53954.86999999998</v>
+        <v>60481.07000000002</v>
       </c>
       <c r="E70" s="105">
-        <v>34148.89999999998</v>
+        <v>27622.69999999995</v>
       </c>
       <c r="F70" s="106" t="s">
         <v>123</v>
       </c>
       <c r="G70" s="107">
-        <v>0.38759862375923293</v>
+        <v>0.3135246085383175</v>
       </c>
       <c r="H70" s="108" t="s">
         <v>124</v>
       </c>
       <c r="I70" s="109">
-        <v>-0.20071445296835796</v>
+        <v>-0.48363310673311793</v>
       </c>
       <c r="J70" s="36"/>
       <c r="K70" s="36"/>
@@ -25343,7 +25343,7 @@
       <c r="N70" s="35"/>
       <c r="O70" s="35"/>
     </row>
-    <row r="71" ht="15" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A71" s="59"/>
       <c r="B71" s="98" t="s">
         <v>125</v>
@@ -25726,7 +25726,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB110"/>
+  <dimension ref="A1:AD110"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.5390625"/>
   <cols>
     <col min="1" max="1" width="11" style="35" customWidth="1"/>
@@ -25737,7 +25737,7 @@
     <col min="6" max="17" width="11.43" style="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="46.5" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="46.5" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -25758,7 +25758,7 @@
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
     </row>
-    <row r="2" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" s="115"/>
       <c r="B2" s="116" t="s">
         <v>126</v>
@@ -25820,7 +25820,7 @@
       <c r="AA2" s="120"/>
       <c r="AB2" s="121"/>
     </row>
-    <row r="3" ht="15" customHeight="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" s="122" t="s">
         <v>142</v>
       </c>
@@ -25878,7 +25878,7 @@
       <c r="AA3" s="129"/>
       <c r="AB3" s="130"/>
     </row>
-    <row r="4" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" s="19">
         <v>7658</v>
       </c>
@@ -25918,7 +25918,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" s="70"/>
       <c r="B5" s="70"/>
       <c r="C5" s="70"/>
@@ -25937,7 +25937,7 @@
       <c r="P5" s="70"/>
       <c r="Q5" s="70"/>
     </row>
-    <row r="6" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" s="19">
         <v>8142</v>
       </c>
@@ -25971,7 +25971,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="7" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" s="70"/>
       <c r="B7" s="70"/>
       <c r="C7" s="70"/>
@@ -25990,7 +25990,7 @@
       <c r="P7" s="70"/>
       <c r="Q7" s="70"/>
     </row>
-    <row r="8" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="8" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" s="19">
         <v>8824</v>
       </c>
@@ -26024,7 +26024,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="9" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" s="70"/>
       <c r="B9" s="70"/>
       <c r="C9" s="70"/>
@@ -26043,7 +26043,7 @@
       <c r="P9" s="70"/>
       <c r="Q9" s="70"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" s="19">
         <v>8127</v>
       </c>
@@ -26054,10 +26054,10 @@
         <v>805.22</v>
       </c>
       <c r="D10" s="54">
-        <v>615.5</v>
+        <v>625</v>
       </c>
       <c r="E10" s="54">
-        <v>189.72000000000003</v>
+        <v>180.22000000000003</v>
       </c>
       <c r="F10" s="54"/>
       <c r="G10" s="54"/>
@@ -26081,7 +26081,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="11" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" s="70"/>
       <c r="B11" s="70"/>
       <c r="C11" s="70"/>
@@ -26100,7 +26100,7 @@
       <c r="P11" s="70"/>
       <c r="Q11" s="70"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" s="19">
         <v>8183</v>
       </c>
@@ -26111,10 +26111,10 @@
         <v>1124.47</v>
       </c>
       <c r="D12" s="54">
-        <v>609</v>
+        <v>627.75</v>
       </c>
       <c r="E12" s="54">
-        <v>515.47</v>
+        <v>496.72</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -26140,7 +26140,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="13" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" s="61"/>
       <c r="B13" s="61"/>
       <c r="C13" s="61"/>
@@ -26159,7 +26159,7 @@
       <c r="P13" s="61"/>
       <c r="Q13" s="61"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" s="19">
         <v>8886</v>
       </c>
@@ -26170,10 +26170,10 @@
         <v>501.83</v>
       </c>
       <c r="D14" s="54">
-        <v>308.25</v>
+        <v>325.75</v>
       </c>
       <c r="E14" s="54">
-        <v>193.57999999999998</v>
+        <v>176.07999999999998</v>
       </c>
       <c r="F14" s="54"/>
       <c r="G14" s="54"/>
@@ -26197,7 +26197,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="15" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" s="61"/>
       <c r="B15" s="61"/>
       <c r="C15" s="61"/>
@@ -26216,7 +26216,7 @@
       <c r="P15" s="61"/>
       <c r="Q15" s="61"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" s="19">
         <v>8887</v>
       </c>
@@ -26249,7 +26249,7 @@
       <c r="P16" s="54"/>
       <c r="Q16" s="131"/>
     </row>
-    <row r="17" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="17" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" s="132"/>
       <c r="B17" s="132"/>
       <c r="C17" s="132"/>
@@ -26268,7 +26268,7 @@
       <c r="P17" s="132"/>
       <c r="Q17" s="132"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" s="19">
         <v>8670</v>
       </c>
@@ -26279,10 +26279,10 @@
         <v>685.48</v>
       </c>
       <c r="D18" s="54">
-        <v>561.5</v>
+        <v>578.5</v>
       </c>
       <c r="E18" s="54">
-        <v>123.98000000000002</v>
+        <v>106.98000000000002</v>
       </c>
       <c r="F18" s="54"/>
       <c r="G18" s="54"/>
@@ -26301,7 +26301,7 @@
       <c r="P18" s="54"/>
       <c r="Q18" s="131"/>
     </row>
-    <row r="19" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="19" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" s="61"/>
       <c r="B19" s="61"/>
       <c r="C19" s="61"/>
@@ -26320,7 +26320,7 @@
       <c r="P19" s="61"/>
       <c r="Q19" s="61"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" s="19">
         <v>8907</v>
       </c>
@@ -26351,7 +26351,7 @@
       <c r="P20" s="54"/>
       <c r="Q20" s="131"/>
     </row>
-    <row r="21" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="21" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" s="61"/>
       <c r="B21" s="61"/>
       <c r="C21" s="61"/>
@@ -26370,7 +26370,7 @@
       <c r="P21" s="61"/>
       <c r="Q21" s="61"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" s="19">
         <v>9065</v>
       </c>
@@ -26405,7 +26405,7 @@
       <c r="P22" s="54"/>
       <c r="Q22" s="131"/>
     </row>
-    <row r="23" ht="6" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="23" ht="6" customHeight="1" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" s="133"/>
       <c r="B23" s="134"/>
       <c r